<commit_message>
Add F-001/F-002 briefs, F-002 spec, and prioritization run reports
Feature-prioritization pipeline output for the first scoring batch:

- briefs/: F-001 (Adhere to a Design System) and F-002 (customer-wide
  baseline system prompt) feature briefs authored via /write-feature-brief.
- specs/F-002-customer-system-prompt.md: formal spec derived from the
  F-002 brief (REQ-F002-### namespace; 5 open rulings flagged in §11).
- feature-value-scoring.xlsx: F-001 and F-002 scored (research agent) and
  Prioritized; F-002 human-gate scores + strategic override applied.
- .prioritization-runs/*/report.md: decision/override audit trail. Binary
  xlsx run snapshots are gitignored (.prioritization-runs/**/*.xlsx).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\derek\anythingllm-admin-console\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{04B528F0-6422-4112-AD0B-FC4DAC2A8A58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33F89561-A4FF-47B3-9A3B-74F1A29AA77B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="211">
   <si>
     <t>FEATURE VALUE SCORING FRAMEWORK</t>
   </si>
@@ -348,304 +348,331 @@
     <t>F-001</t>
   </si>
   <si>
-    <t>briefs/F-001-csv-import.md</t>
+    <t>Human</t>
+  </si>
+  <si>
+    <t>DATA DICTIONARY - machine-readable field contract for agents</t>
+  </si>
+  <si>
+    <t>Column (Scoring sheet)</t>
+  </si>
+  <si>
+    <t>field_id</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Allowed Values / Range</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>A: Feature ID</t>
+  </si>
+  <si>
+    <t>feature_id</t>
+  </si>
+  <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>Unique, pattern F-###</t>
+  </si>
+  <si>
+    <t>Stable identifier; used to join to the feature brief</t>
+  </si>
+  <si>
+    <t>B: Feature Name</t>
+  </si>
+  <si>
+    <t>feature_name</t>
+  </si>
+  <si>
+    <t>Free text</t>
+  </si>
+  <si>
+    <t>Short human-readable name</t>
+  </si>
+  <si>
+    <t>C: Brief Reference</t>
+  </si>
+  <si>
+    <t>brief_ref</t>
+  </si>
+  <si>
+    <t>Path or URL</t>
+  </si>
+  <si>
+    <t>Link to the feature brief document the score is based on</t>
+  </si>
+  <si>
+    <t>D: Status</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>enum</t>
+  </si>
+  <si>
+    <t>Idea | Brief Drafted | Scored | Prioritized | Deferred | Rejected</t>
+  </si>
+  <si>
+    <t>Human / Prioritization agent</t>
+  </si>
+  <si>
+    <t>Lifecycle state; prioritization agent may advance Scored -&gt; Prioritized</t>
+  </si>
+  <si>
+    <t>E: Scored By</t>
+  </si>
+  <si>
+    <t>scored_by</t>
+  </si>
+  <si>
+    <t>Human | Market Research Agent | Hybrid</t>
+  </si>
+  <si>
+    <t>Scorer</t>
+  </si>
+  <si>
+    <t>Provenance of the scores in this row</t>
+  </si>
+  <si>
+    <t>F: Date Scored</t>
+  </si>
+  <si>
+    <t>date_scored</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>ISO 8601 (YYYY-MM-DD)</t>
+  </si>
+  <si>
+    <t>When scores were last updated; prioritizer may discount stale rows</t>
+  </si>
+  <si>
+    <t>G: Reach</t>
+  </si>
+  <si>
+    <t>reach</t>
+  </si>
+  <si>
+    <t>integer</t>
+  </si>
+  <si>
+    <t>1-5 (Rubric sheet)</t>
+  </si>
+  <si>
+    <t>Human / Research agent</t>
+  </si>
+  <si>
+    <t>Share of users affected and frequency of exposure</t>
+  </si>
+  <si>
+    <t>H: User Value</t>
+  </si>
+  <si>
+    <t>user_value</t>
+  </si>
+  <si>
+    <t>Depth of pain relieved or capability gained per affected user</t>
+  </si>
+  <si>
+    <t>I: Business Value</t>
+  </si>
+  <si>
+    <t>business_value</t>
+  </si>
+  <si>
+    <t>Revenue, retention, cost, or market-access impact</t>
+  </si>
+  <si>
+    <t>J: Strategic Alignment</t>
+  </si>
+  <si>
+    <t>strategic_alignment</t>
+  </si>
+  <si>
+    <t>Fit with product vision; deliberately human-owned</t>
+  </si>
+  <si>
+    <t>K: Time Sensitivity</t>
+  </si>
+  <si>
+    <t>time_sensitivity</t>
+  </si>
+  <si>
+    <t>Decay of value if shipping is delayed</t>
+  </si>
+  <si>
+    <t>L: Confidence</t>
+  </si>
+  <si>
+    <t>confidence</t>
+  </si>
+  <si>
+    <t>Strength of evidence behind the value scores</t>
+  </si>
+  <si>
+    <t>M: Effort</t>
+  </si>
+  <si>
+    <t>effort</t>
+  </si>
+  <si>
+    <t>Human (engineering)</t>
+  </si>
+  <si>
+    <t>Total delivery cost incl. design, QA, maintenance</t>
+  </si>
+  <si>
+    <t>N: Risk</t>
+  </si>
+  <si>
+    <t>risk</t>
+  </si>
+  <si>
+    <t>Technical/market/reversibility risk</t>
+  </si>
+  <si>
+    <t>O: Evidence &amp; Sources</t>
+  </si>
+  <si>
+    <t>evidence_sources</t>
+  </si>
+  <si>
+    <t>Free text; citations required for agent-scored rows</t>
+  </si>
+  <si>
+    <t>What the scores are based on; research agents MUST cite sources</t>
+  </si>
+  <si>
+    <t>P: Rationale Notes</t>
+  </si>
+  <si>
+    <t>rationale_notes</t>
+  </si>
+  <si>
+    <t>Reasoning behind judgment calls and any dissent</t>
+  </si>
+  <si>
+    <t>Q: Weighted Value</t>
+  </si>
+  <si>
+    <t>weighted_value</t>
+  </si>
+  <si>
+    <t>formula</t>
+  </si>
+  <si>
+    <t>0.00-5.00</t>
+  </si>
+  <si>
+    <t>Formula - do not edit</t>
+  </si>
+  <si>
+    <t>SUMPRODUCT of value dimensions and Config weights</t>
+  </si>
+  <si>
+    <t>R: Confidence Mult</t>
+  </si>
+  <si>
+    <t>confidence_multiplier</t>
+  </si>
+  <si>
+    <t>0.50-1.00</t>
+  </si>
+  <si>
+    <t>Lookup from Config confidence map</t>
+  </si>
+  <si>
+    <t>S: Risk Factor</t>
+  </si>
+  <si>
+    <t>risk_factor</t>
+  </si>
+  <si>
+    <t>0.60-1.00</t>
+  </si>
+  <si>
+    <t>Lookup from Config risk map</t>
+  </si>
+  <si>
+    <t>T: Priority Score</t>
+  </si>
+  <si>
+    <t>priority_score</t>
+  </si>
+  <si>
+    <t>0-100</t>
+  </si>
+  <si>
+    <t>Weighted Value x Confidence Mult x Risk Factor / Effort x 20</t>
+  </si>
+  <si>
+    <t>U: Rank</t>
+  </si>
+  <si>
+    <t>rank</t>
+  </si>
+  <si>
+    <t>1-N</t>
+  </si>
+  <si>
+    <t>Descending rank of Priority Score across scored rows</t>
+  </si>
+  <si>
+    <t>Adhere to a Design System</t>
+  </si>
+  <si>
+    <t>briefs/F-001-adhere-to-design-system.md</t>
+  </si>
+  <si>
+    <t>Prioritized</t>
+  </si>
+  <si>
+    <t>Market Research Agent</t>
+  </si>
+  <si>
+    <t>VERIFIED IN-REPO (2026-07-07): Read briefs/F-001-adhere-to-design-system.md and confirmed every current-state baseline claim exactly against source: web/src/index.css = 723 lines with 30 CSS custom-property definitions and dual theming (:root dark default + [data-theme='light'] + @media prefers-color-scheme:light); exactly 143 className= usages across 22 .tsx files; five independent feature areas (diagnostics, raweditor, settings, users, workspaces under web/src/features/); exactly three shared components (DangerConfirm, ErrorBanner, SetNotSetBadge in web/src/components/). ANALOGOUS INDUSTRY BENCHMARKS (WebSearch 2026-07-07, general-category / low project-specificity): Sparkbox "Value of Design Systems" (dev efficiency ~47%), Figma internal (34% faster task completion with system), Atlassian (up to 65% dev-time reduction), and ROI syntheses (lollypop.design, netguru, Smashing Magazine 2022) citing 135-170% 5-yr ROI and ~34% of dev cycles spent recreating components. COULD NOT VERIFY: Claude Design project at https://claude.ai/design/p/4c97b85d-5482-401b-b1b3-12df2a9d8d66 returned HTTP 403 (auth-gated) - its actual contents (tokens vs. full component set, light+dark coverage, mapping to console patterns) remain unverified; claude_design MCP re-import/sync cadence unverified. NO PROJECT-SPECIFIC DEMAND EVIDENCE: per the environment limitation, no support-ticket system, operator interviews, or usage-analytics dashboard exists for this internal tool - operator pain and payoff magnitude are unmeasured. Internal operator base size unconfirmed; October 2026 GTM hard-vs-soft status unconfirmed.</t>
+  </si>
+  <si>
+    <t>REACH=5 - the console is a staff-only operator tool where the target-user population IS the internal operator base; every operator works across all five feature areas and is exposed to the governing design system on essentially every session (&gt;70% of target users in core daily workflows). Small absolute audience does not lower the target-population fraction, which the anchor measures. USER_VALUE=2 - scored for the actual users (operators), not developers. Visual/interaction inconsistency is a coherence/cosmetic issue with an easy workaround (operators complete their jobs on the current surface); there is zero evidence of measurable operator task-pain (no tickets/interviews/analytics). Honestly minor convenience, not removal of a frequent significant pain - resisting the temptation to score the developer/maintenance benefit here (that belongs to business_value). BUSINESS_VALUE=3 - the credible payoff is a cost/velocity play (reusable tokens+components lowering per-screen build/change cost and styling-maintenance churn), which the anchor rates as a measurable effect on cost. Analogous benchmarks support a real cost/velocity effect, so this clears 2; but it is NOT a revenue/expansion/churn driver (internal, non-customer-facing tool) so it does not reach 4, and the absolute cost base is small (5 areas, 3 shared components, 723-line CSS). Landed at the low end of 3. TIME_SENSITIVITY=3 - October 2026 GTM is ~3 months out and the retrofit surface compounds with every ad-hoc screen shipped before adoption, giving a meaningful advantage to shipping this year (anchor 3). Withheld 4 (references a competitive/market window, whereas this is internal-readiness, and the GTM is an unconfirmed soft target); withheld 5 (no confirmed hard gate). CONFIDENCE=2 - the current-state baseline is fully verified and there are multiple dated analogous benchmarks, but the two most value-determining legs lack project-specific evidence: (a) operator pain (user_value) rests on codebase observation + conviction with no tickets/interviews/analytics, and (b) payoff magnitude for THIS small console rests only on general-category benchmarks the brief itself flags as low-specificity. The design system to be adopted could not be inspected (403). Per the no-inflation rule, honest value + confidence=2 is the correct encoding; did not round up to 3 because the benchmarks argue the category, not this tool.</t>
+  </si>
+  <si>
+    <t>F-002</t>
+  </si>
+  <si>
+    <t>F-003</t>
+  </si>
+  <si>
+    <t>Set a customer specific system prompt</t>
+  </si>
+  <si>
+    <t>Set a workspace level system prompt</t>
+  </si>
+  <si>
+    <t>briefs/F-002-customer-system-prompt.md</t>
   </si>
   <si>
     <t>Scored</t>
   </si>
   <si>
-    <t>Human</t>
-  </si>
-  <si>
-    <t>2026-07-05</t>
-  </si>
-  <si>
-    <t>Support tickets Q1-Q2 2026 (42 requests); competitor X shipped equivalent in May</t>
-  </si>
-  <si>
-    <t>Frequent onboarding blocker for mid-market accounts; effort moderate due to validation edge cases</t>
-  </si>
-  <si>
-    <t>DATA DICTIONARY - machine-readable field contract for agents</t>
-  </si>
-  <si>
-    <t>Column (Scoring sheet)</t>
-  </si>
-  <si>
-    <t>field_id</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Allowed Values / Range</t>
-  </si>
-  <si>
-    <t>Owner</t>
-  </si>
-  <si>
-    <t>Description</t>
-  </si>
-  <si>
-    <t>A: Feature ID</t>
-  </si>
-  <si>
-    <t>feature_id</t>
-  </si>
-  <si>
-    <t>string</t>
-  </si>
-  <si>
-    <t>Unique, pattern F-###</t>
-  </si>
-  <si>
-    <t>Stable identifier; used to join to the feature brief</t>
-  </si>
-  <si>
-    <t>B: Feature Name</t>
-  </si>
-  <si>
-    <t>feature_name</t>
-  </si>
-  <si>
-    <t>Free text</t>
-  </si>
-  <si>
-    <t>Short human-readable name</t>
-  </si>
-  <si>
-    <t>C: Brief Reference</t>
-  </si>
-  <si>
-    <t>brief_ref</t>
-  </si>
-  <si>
-    <t>Path or URL</t>
-  </si>
-  <si>
-    <t>Link to the feature brief document the score is based on</t>
-  </si>
-  <si>
-    <t>D: Status</t>
-  </si>
-  <si>
-    <t>status</t>
-  </si>
-  <si>
-    <t>enum</t>
-  </si>
-  <si>
-    <t>Idea | Brief Drafted | Scored | Prioritized | Deferred | Rejected</t>
-  </si>
-  <si>
-    <t>Human / Prioritization agent</t>
-  </si>
-  <si>
-    <t>Lifecycle state; prioritization agent may advance Scored -&gt; Prioritized</t>
-  </si>
-  <si>
-    <t>E: Scored By</t>
-  </si>
-  <si>
-    <t>scored_by</t>
-  </si>
-  <si>
-    <t>Human | Market Research Agent | Hybrid</t>
-  </si>
-  <si>
-    <t>Scorer</t>
-  </si>
-  <si>
-    <t>Provenance of the scores in this row</t>
-  </si>
-  <si>
-    <t>F: Date Scored</t>
-  </si>
-  <si>
-    <t>date_scored</t>
-  </si>
-  <si>
-    <t>date</t>
-  </si>
-  <si>
-    <t>ISO 8601 (YYYY-MM-DD)</t>
-  </si>
-  <si>
-    <t>When scores were last updated; prioritizer may discount stale rows</t>
-  </si>
-  <si>
-    <t>G: Reach</t>
-  </si>
-  <si>
-    <t>reach</t>
-  </si>
-  <si>
-    <t>integer</t>
-  </si>
-  <si>
-    <t>1-5 (Rubric sheet)</t>
-  </si>
-  <si>
-    <t>Human / Research agent</t>
-  </si>
-  <si>
-    <t>Share of users affected and frequency of exposure</t>
-  </si>
-  <si>
-    <t>H: User Value</t>
-  </si>
-  <si>
-    <t>user_value</t>
-  </si>
-  <si>
-    <t>Depth of pain relieved or capability gained per affected user</t>
-  </si>
-  <si>
-    <t>I: Business Value</t>
-  </si>
-  <si>
-    <t>business_value</t>
-  </si>
-  <si>
-    <t>Revenue, retention, cost, or market-access impact</t>
-  </si>
-  <si>
-    <t>J: Strategic Alignment</t>
-  </si>
-  <si>
-    <t>strategic_alignment</t>
-  </si>
-  <si>
-    <t>Fit with product vision; deliberately human-owned</t>
-  </si>
-  <si>
-    <t>K: Time Sensitivity</t>
-  </si>
-  <si>
-    <t>time_sensitivity</t>
-  </si>
-  <si>
-    <t>Decay of value if shipping is delayed</t>
-  </si>
-  <si>
-    <t>L: Confidence</t>
-  </si>
-  <si>
-    <t>confidence</t>
-  </si>
-  <si>
-    <t>Strength of evidence behind the value scores</t>
-  </si>
-  <si>
-    <t>M: Effort</t>
-  </si>
-  <si>
-    <t>effort</t>
-  </si>
-  <si>
-    <t>Human (engineering)</t>
-  </si>
-  <si>
-    <t>Total delivery cost incl. design, QA, maintenance</t>
-  </si>
-  <si>
-    <t>N: Risk</t>
-  </si>
-  <si>
-    <t>risk</t>
-  </si>
-  <si>
-    <t>Technical/market/reversibility risk</t>
-  </si>
-  <si>
-    <t>O: Evidence &amp; Sources</t>
-  </si>
-  <si>
-    <t>evidence_sources</t>
-  </si>
-  <si>
-    <t>Free text; citations required for agent-scored rows</t>
-  </si>
-  <si>
-    <t>What the scores are based on; research agents MUST cite sources</t>
-  </si>
-  <si>
-    <t>P: Rationale Notes</t>
-  </si>
-  <si>
-    <t>rationale_notes</t>
-  </si>
-  <si>
-    <t>Reasoning behind judgment calls and any dissent</t>
-  </si>
-  <si>
-    <t>Q: Weighted Value</t>
-  </si>
-  <si>
-    <t>weighted_value</t>
-  </si>
-  <si>
-    <t>formula</t>
-  </si>
-  <si>
-    <t>0.00-5.00</t>
-  </si>
-  <si>
-    <t>Formula - do not edit</t>
-  </si>
-  <si>
-    <t>SUMPRODUCT of value dimensions and Config weights</t>
-  </si>
-  <si>
-    <t>R: Confidence Mult</t>
-  </si>
-  <si>
-    <t>confidence_multiplier</t>
-  </si>
-  <si>
-    <t>0.50-1.00</t>
-  </si>
-  <si>
-    <t>Lookup from Config confidence map</t>
-  </si>
-  <si>
-    <t>S: Risk Factor</t>
-  </si>
-  <si>
-    <t>risk_factor</t>
-  </si>
-  <si>
-    <t>0.60-1.00</t>
-  </si>
-  <si>
-    <t>Lookup from Config risk map</t>
-  </si>
-  <si>
-    <t>T: Priority Score</t>
-  </si>
-  <si>
-    <t>priority_score</t>
-  </si>
-  <si>
-    <t>0-100</t>
-  </si>
-  <si>
-    <t>Weighted Value x Confidence Mult x Risk Factor / Effort x 20</t>
-  </si>
-  <si>
-    <t>U: Rank</t>
-  </si>
-  <si>
-    <t>rank</t>
-  </si>
-  <si>
-    <t>1-N</t>
-  </si>
-  <si>
-    <t>Descending rank of Priority Score across scored rows</t>
-  </si>
-  <si>
-    <t>Adhere to a Design System</t>
+    <t>2026-07-07</t>
+  </si>
+  <si>
+    <t>VERIFIED INTERNAL (repo read 2026-07-07): (1) web/src/features/workspaces/WorkspaceSettings.tsx lines 347-354 - the per-workspace "System prompt (blank = inherit)" textarea exists today; there is no above-workspace scope, confirming the "no baseline mechanism" problem statement. (2) bff/src/engine/mappers.ts lines 64-82 (WORKSPACE_FIELD_MAP) - systemPrompt maps 1:1 to a single engine field openAiPrompt; there is literally one prompt field per workspace and no native base+workspace layering, confirming the brief's central open question that a tamper-proof/enforced baseline is NOT achievable through this channel. (3) docs/anythingllm-surface.md lines 197-234 - confirms /system/default-system-prompt (native instance-level default) is session-auth-only and a "hard boundary at the API layer," unreachable under the console's API-key custody model; the console-managed fan-out route is the only option. All three brief leads re-verified as accurate. ANALOGOUS EXTERNAL (WebSearch 2026-07-07, directional only): Technavio - Enterprise Prompt Management Platforms market +USD 2.44B 2026-2030 at 32.5% CAGR; Gartner-cited AI-governance-platform spend ~USD 492M in 2026 rising past USD 1B by 2030; market shifting toward structured prompt governance and centralized control. These establish that centralized prompt/guardrail governance is a real, growing enterprise need. COUNTER-EVIDENCE: industry best-practice for real enforcement is a gateway-plus-guardrails architecture (policy enforced OUTSIDE the model call), not single-prompt-field storage (Galileo/Maxim/CSA 2025-2026) - corroborating that F-002's single-field approach is best-effort, not true enforcement. COULD NOT VERIFY: no support-ticket system, sales CRM, or usage-analytics dashboard exists for this internal tool, so zero direct demand signal for THIS feature; the brief itself states no discovery scan was run. Workspaces-per-customer count (bounds reach/effort) is unverifiable - an open question in the brief. The "governance as a selling point" business claim is entirely unverified against any sales evidence.</t>
+  </si>
+  <si>
+    <t>REACH (3): Scored against the STAFF OPERATORS who configure the feature (the console is staff-only per surface doc; customers never touch it), not the end-user chat population whose experience the prompt shapes. Absolute operator headcount is small and the config action is infrequent/high-leverage, but establishing a baseline persona/guardrail is a task essentially every customer onboarding would touch - "regular use" within the operator setup workflow, landing at the 15-40% regular-use anchor. Note: if scored against the effect population (every end-user chat across all workspaces) it would be 5; deliberately not, because the anchor measures the feature's USERS and this is a configuration control. USER_VALUE (3): The workaround exists today and is clumsy - manually re-typing the same baseline into each workspace's systemPrompt textarea and policing drift by hand (verified the textarea is the only mechanism). F-002 removes that clumsiness = solid 3. Not 4 because (a) pain frequency scales with workspaces-per-customer, which is unknown, and (b) the "safety guardrail" job-to-be-done is only partially delivered - the verified single-field engine model means the baseline can be silently clobbered by a per-workspace edit, so the strongest value claim (an enforced guardrail) is not realizable through this channel. BUSINESS_VALUE (2): Internal operator tool; revenue/retention effect is indirect. Industry data shows governance is a growing differentiator, but there is no CRM/sales evidence customers ask for it (brief admits this), and the enforcement gap weakens the "governance selling point." Indirect/small effect = 2, not 3, because a measurable conversion/retention effect is asserted, not evidenced. TIME_SENSITIVITY (3): October 2026 GTM is ~3 months out but a SOFT internal readiness target, not a hard external deadline (no regulation/contract binds this feature), so not 4 or 5. The genuine pressure is the compounding-retrofit argument (prompts set before this exists must be retrofitted later) - real but modest. "Meaningful advantage to shipping this year" = 3. CONFIDENCE (2): Structural/feasibility facts are strongly verified in-repo, but every VALUE score rests on reasoning plus analogous industry benchmarks, not on any direct demand data for this feature - inaccessible by environment constraint and ungathered by admission. Per the cap rule and honest thinness, confidence is 2 (single-data-point/analogous-anecdote tier), not 3.</t>
   </si>
 </sst>
 </file>
@@ -655,7 +682,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -726,6 +753,14 @@
       <name val="Arial"/>
       <charset val="1"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -783,10 +818,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -836,8 +872,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="5" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1575,7 +1616,7 @@
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="2" max="2" width="41.7265625" customWidth="1"/>
     <col min="3" max="3" width="24" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
@@ -1666,54 +1707,54 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:21" ht="42" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:21" ht="409.5" x14ac:dyDescent="0.35">
       <c r="A4" s="18" t="s">
         <v>101</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>102</v>
+        <v>197</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>103</v>
+        <v>198</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>104</v>
-      </c>
-      <c r="F4" s="18" t="s">
-        <v>105</v>
+        <v>199</v>
+      </c>
+      <c r="F4" s="26">
+        <v>46210</v>
       </c>
       <c r="G4" s="19">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H4" s="19">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I4" s="19">
         <v>3</v>
       </c>
       <c r="J4" s="19">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K4" s="19">
+        <v>3</v>
+      </c>
+      <c r="L4" s="19">
         <v>2</v>
       </c>
-      <c r="L4" s="19">
-        <v>4</v>
-      </c>
       <c r="M4" s="19">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N4" s="19">
-        <v>2</v>
-      </c>
-      <c r="O4" s="20" t="s">
-        <v>106</v>
+        <v>1</v>
+      </c>
+      <c r="O4" s="25" t="s">
+        <v>200</v>
       </c>
       <c r="P4" s="20" t="s">
-        <v>107</v>
+        <v>201</v>
       </c>
       <c r="Q4" s="21">
         <f>IF(COUNT(G4:K4)&lt;5,"",ROUND(G4*Config!$B$4+H4*Config!$B$5+I4*Config!$B$6+J4*Config!$B$7+K4*Config!$B$8,2))</f>
@@ -1721,47 +1762,100 @@
       </c>
       <c r="R4" s="21">
         <f>IF(L4="","",VLOOKUP(L4,Config!$A$12:$B$16,2,0))</f>
-        <v>0.9</v>
+        <v>0.65</v>
       </c>
       <c r="S4" s="21">
         <f>IF(N4="","",VLOOKUP(N4,Config!$D$12:$E$16,2,0))</f>
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="T4" s="22">
         <f t="shared" ref="T4:T35" si="0">IF(OR(Q4="",R4="",S4="",M4=""),"",ROUND(Q4*R4*S4/M4*20,1))</f>
-        <v>19.2</v>
+        <v>46.2</v>
       </c>
       <c r="U4" s="23">
         <f t="shared" ref="U4:U35" si="1">IF(T4="","",RANK(T4,$T$4:$T$53))</f>
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A5" s="18"/>
-      <c r="B5" s="18"/>
-      <c r="C5" s="18"/>
-      <c r="D5" s="18"/>
-      <c r="E5" s="18"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="19"/>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
-      <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
-      <c r="L5" s="19"/>
-      <c r="M5" s="19"/>
-      <c r="N5" s="19"/>
-      <c r="O5" s="20"/>
-      <c r="P5" s="20"/>
-      <c r="Q5" s="21"/>
-      <c r="R5" s="21"/>
-      <c r="S5" s="21"/>
-      <c r="T5" s="22"/>
-      <c r="U5" s="23"/>
+    <row r="5" spans="1:21" ht="409.5" x14ac:dyDescent="0.35">
+      <c r="A5" s="18" t="s">
+        <v>202</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="C5" s="18" t="s">
+        <v>206</v>
+      </c>
+      <c r="D5" s="18" t="inlineStr">
+        <is>
+          <t>Prioritized</t>
+        </is>
+      </c>
+      <c r="E5" s="18" t="s">
+        <v>199</v>
+      </c>
+      <c r="F5" s="18" t="s">
+        <v>208</v>
+      </c>
+      <c r="G5" s="19">
+        <v>3</v>
+      </c>
+      <c r="H5" s="19">
+        <v>3</v>
+      </c>
+      <c r="I5" s="19">
+        <v>2</v>
+      </c>
+      <c r="J5" s="19">
+        <v>4</v>
+      </c>
+      <c r="K5" s="19">
+        <v>3</v>
+      </c>
+      <c r="L5" s="19">
+        <v>2</v>
+      </c>
+      <c r="M5" s="19">
+        <v>2</v>
+      </c>
+      <c r="N5" s="19">
+        <v>2</v>
+      </c>
+      <c r="O5" s="20" t="s">
+        <v>209</v>
+      </c>
+      <c r="P5" s="20" t="s">
+        <v>210</v>
+      </c>
+      <c r="Q5" s="21">
+        <f>IF(COUNT(G5:K5)&lt;5,"",ROUND(G5*Config!$B$4+H5*Config!$B$5+I5*Config!$B$6+J5*Config!$B$7+K5*Config!$B$8,2))</f>
+        <v>2.95</v>
+      </c>
+      <c r="R5" s="21">
+        <f>IF(L5="","",VLOOKUP(L5,Config!$A$12:$B$16,2,0))</f>
+        <v>0.65</v>
+      </c>
+      <c r="S5" s="21">
+        <f>IF(N5="","",VLOOKUP(N5,Config!$D$12:$E$16,2,0))</f>
+        <v>0.9</v>
+      </c>
+      <c r="T5" s="22">
+        <f>IF(OR(Q5="",R5="",S5="",M5=""),"",ROUND(Q5*R5*S5/M5*20,1))</f>
+        <v>17.3</v>
+      </c>
+      <c r="U5" s="23">
+        <f>IF(T5="","",RANK(T5,$T$4:$T$53))</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A6" s="18"/>
-      <c r="B6" s="18"/>
+      <c r="A6" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>205</v>
+      </c>
       <c r="C6" s="18"/>
       <c r="D6" s="18"/>
       <c r="E6" s="18"/>
@@ -1776,11 +1870,26 @@
       <c r="N6" s="19"/>
       <c r="O6" s="20"/>
       <c r="P6" s="20"/>
-      <c r="Q6" s="21"/>
-      <c r="R6" s="21"/>
-      <c r="S6" s="21"/>
-      <c r="T6" s="22"/>
-      <c r="U6" s="23"/>
+      <c r="Q6" s="21" t="str">
+        <f>IF(COUNT(G6:K6)&lt;5,"",ROUND(G6*Config!$B$4+H6*Config!$B$5+I6*Config!$B$6+J6*Config!$B$7+K6*Config!$B$8,2))</f>
+        <v/>
+      </c>
+      <c r="R6" s="21" t="str">
+        <f>IF(L6="","",VLOOKUP(L6,Config!$A$12:$B$16,2,0))</f>
+        <v/>
+      </c>
+      <c r="S6" s="21" t="str">
+        <f>IF(N6="","",VLOOKUP(N6,Config!$D$12:$E$16,2,0))</f>
+        <v/>
+      </c>
+      <c r="T6" s="22" t="str">
+        <f>IF(OR(Q6="",R6="",S6="",M6=""),"",ROUND(Q6*R6*S6/M6*20,1))</f>
+        <v/>
+      </c>
+      <c r="U6" s="23" t="str">
+        <f>IF(T6="","",RANK(T6,$T$4:$T$53))</f>
+        <v/>
+      </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.35">
       <c r="A7" s="18"/>
@@ -2914,11 +3023,11 @@
         <v/>
       </c>
       <c r="T36" s="22" t="str">
-        <f t="shared" ref="T36:T67" si="2">IF(OR(Q36="",R36="",S36="",M36=""),"",ROUND(Q36*R36*S36/M36*20,1))</f>
+        <f t="shared" ref="T36:T53" si="2">IF(OR(Q36="",R36="",S36="",M36=""),"",ROUND(Q36*R36*S36/M36*20,1))</f>
         <v/>
       </c>
       <c r="U36" s="23" t="str">
-        <f t="shared" ref="U36:U67" si="3">IF(T36="","",RANK(T36,$T$4:$T$53))</f>
+        <f t="shared" ref="U36:U53" si="3">IF(T36="","",RANK(T36,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
@@ -3583,8 +3692,14 @@
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink ref="O4" r:id="rId1" display="https://www.toptal.com/designers/design-systems/benefits-of-design-system" xr:uid="{8A9458DF-571D-4A70-8D55-70230E9370DE}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <ignoredErrors>
+    <ignoredError sqref="Q4" formulaRange="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
@@ -3603,447 +3718,447 @@
   <sheetData>
     <row r="1" spans="1:6" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="B3" s="24" t="s">
+        <v>105</v>
+      </c>
+      <c r="C3" s="24" t="s">
+        <v>106</v>
+      </c>
+      <c r="D3" s="24" t="s">
+        <v>107</v>
+      </c>
+      <c r="E3" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="F3" s="24" t="s">
         <v>109</v>
-      </c>
-      <c r="B3" s="24" t="s">
-        <v>110</v>
-      </c>
-      <c r="C3" s="24" t="s">
-        <v>111</v>
-      </c>
-      <c r="D3" s="24" t="s">
-        <v>112</v>
-      </c>
-      <c r="E3" s="24" t="s">
-        <v>113</v>
-      </c>
-      <c r="F3" s="24" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="16" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="16" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="C5" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="D5" s="16" t="s">
         <v>117</v>
       </c>
-      <c r="D5" s="16" t="s">
-        <v>122</v>
-      </c>
       <c r="E5" s="16" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="16" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="E6" s="16" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F6" s="16" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="28" x14ac:dyDescent="0.35">
       <c r="A7" s="16" t="s">
+        <v>123</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>124</v>
+      </c>
+      <c r="C7" s="16" t="s">
+        <v>125</v>
+      </c>
+      <c r="D7" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="F7" s="16" t="s">
         <v>128</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>129</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>130</v>
-      </c>
-      <c r="D7" s="16" t="s">
-        <v>131</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>132</v>
-      </c>
-      <c r="F7" s="16" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="16" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="E8" s="16" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="F8" s="16" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="16" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="E9" s="16" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" s="16" t="s">
+        <v>139</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>142</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>143</v>
+      </c>
+      <c r="F10" s="16" t="s">
         <v>144</v>
-      </c>
-      <c r="B10" s="16" t="s">
-        <v>145</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>146</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>147</v>
-      </c>
-      <c r="E10" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="F10" s="16" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" s="16" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B11" s="16" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="D11" s="16" t="s">
+        <v>142</v>
+      </c>
+      <c r="E11" s="16" t="s">
+        <v>143</v>
+      </c>
+      <c r="F11" s="16" t="s">
         <v>147</v>
-      </c>
-      <c r="E11" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="F11" s="16" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A12" s="16" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="C12" s="16" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="E12" s="16" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" s="16" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="C13" s="16" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A14" s="16" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" s="16" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="C15" s="16" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="E15" s="16" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="F15" s="16" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" s="16" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="C16" s="16" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="F16" s="16" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A17" s="16" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F17" s="16" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="28" x14ac:dyDescent="0.35">
       <c r="A18" s="16" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="C18" s="16" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="D18" s="16" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="F18" s="16" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A19" s="16" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="C19" s="16" t="s">
+        <v>112</v>
+      </c>
+      <c r="D19" s="16" t="s">
         <v>117</v>
       </c>
-      <c r="D19" s="16" t="s">
-        <v>122</v>
-      </c>
       <c r="E19" s="16" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="F19" s="16" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A20" s="16" t="s">
+        <v>174</v>
+      </c>
+      <c r="B20" s="16" t="s">
+        <v>175</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>176</v>
+      </c>
+      <c r="D20" s="16" t="s">
+        <v>177</v>
+      </c>
+      <c r="E20" s="16" t="s">
+        <v>178</v>
+      </c>
+      <c r="F20" s="16" t="s">
         <v>179</v>
-      </c>
-      <c r="B20" s="16" t="s">
-        <v>180</v>
-      </c>
-      <c r="C20" s="16" t="s">
-        <v>181</v>
-      </c>
-      <c r="D20" s="16" t="s">
-        <v>182</v>
-      </c>
-      <c r="E20" s="16" t="s">
-        <v>183</v>
-      </c>
-      <c r="F20" s="16" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A21" s="16" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="E21" s="16" t="s">
+        <v>178</v>
+      </c>
+      <c r="F21" s="16" t="s">
         <v>183</v>
-      </c>
-      <c r="F21" s="16" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A22" s="16" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="C22" s="16" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="F22" s="16" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A23" s="16" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C23" s="16" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="E23" s="16" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="F23" s="16" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A24" s="16" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C24" s="16" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="D24" s="16" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="E24" s="16" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="F24" s="16" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Score and prioritize F-003/F-004; record 2026-07-07 prioritization run
Research scores + human-owned dimensions for F-003 (priority 20.5) and F-004
(10.0); all four features now Prioritized (F-004's effort-buried flag resolved by a
human commit ruling). Adds the run report/decision audit trail; the binary xlsx
snapshot stays gitignored.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\derek\anythingllm-admin-console\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33F89561-A4FF-47B3-9A3B-74F1A29AA77B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8B12C57-3F65-47D0-B462-E418F4A4A0F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="219">
   <si>
     <t>FEATURE VALUE SCORING FRAMEWORK</t>
   </si>
@@ -663,16 +663,40 @@
     <t>briefs/F-002-customer-system-prompt.md</t>
   </si>
   <si>
+    <t>2026-07-07</t>
+  </si>
+  <si>
+    <t>VERIFIED INTERNAL (repo read 2026-07-07): (1) web/src/features/workspaces/WorkspaceSettings.tsx lines 347-354 - the per-workspace "System prompt (blank = inherit)" textarea exists today; there is no above-workspace scope, confirming the "no baseline mechanism" problem statement. (2) bff/src/engine/mappers.ts lines 64-82 (WORKSPACE_FIELD_MAP) - systemPrompt maps 1:1 to a single engine field openAiPrompt; there is literally one prompt field per workspace and no native base+workspace layering, confirming the brief's central open question that a tamper-proof/enforced baseline is NOT achievable through this channel. (3) docs/anythingllm-surface.md lines 197-234 - confirms /system/default-system-prompt (native instance-level default) is session-auth-only and a "hard boundary at the API layer," unreachable under the console's API-key custody model; the console-managed fan-out route is the only option. All three brief leads re-verified as accurate. ANALOGOUS EXTERNAL (WebSearch 2026-07-07, directional only): Technavio - Enterprise Prompt Management Platforms market +USD 2.44B 2026-2030 at 32.5% CAGR; Gartner-cited AI-governance-platform spend ~USD 492M in 2026 rising past USD 1B by 2030; market shifting toward structured prompt governance and centralized control. These establish that centralized prompt/guardrail governance is a real, growing enterprise need. COUNTER-EVIDENCE: industry best-practice for real enforcement is a gateway-plus-guardrails architecture (policy enforced OUTSIDE the model call), not single-prompt-field storage (Galileo/Maxim/CSA 2025-2026) - corroborating that F-002's single-field approach is best-effort, not true enforcement. COULD NOT VERIFY: no support-ticket system, sales CRM, or usage-analytics dashboard exists for this internal tool, so zero direct demand signal for THIS feature; the brief itself states no discovery scan was run. Workspaces-per-customer count (bounds reach/effort) is unverifiable - an open question in the brief. The "governance as a selling point" business claim is entirely unverified against any sales evidence.</t>
+  </si>
+  <si>
+    <t>REACH (3): Scored against the STAFF OPERATORS who configure the feature (the console is staff-only per surface doc; customers never touch it), not the end-user chat population whose experience the prompt shapes. Absolute operator headcount is small and the config action is infrequent/high-leverage, but establishing a baseline persona/guardrail is a task essentially every customer onboarding would touch - "regular use" within the operator setup workflow, landing at the 15-40% regular-use anchor. Note: if scored against the effect population (every end-user chat across all workspaces) it would be 5; deliberately not, because the anchor measures the feature's USERS and this is a configuration control. USER_VALUE (3): The workaround exists today and is clumsy - manually re-typing the same baseline into each workspace's systemPrompt textarea and policing drift by hand (verified the textarea is the only mechanism). F-002 removes that clumsiness = solid 3. Not 4 because (a) pain frequency scales with workspaces-per-customer, which is unknown, and (b) the "safety guardrail" job-to-be-done is only partially delivered - the verified single-field engine model means the baseline can be silently clobbered by a per-workspace edit, so the strongest value claim (an enforced guardrail) is not realizable through this channel. BUSINESS_VALUE (2): Internal operator tool; revenue/retention effect is indirect. Industry data shows governance is a growing differentiator, but there is no CRM/sales evidence customers ask for it (brief admits this), and the enforcement gap weakens the "governance selling point." Indirect/small effect = 2, not 3, because a measurable conversion/retention effect is asserted, not evidenced. TIME_SENSITIVITY (3): October 2026 GTM is ~3 months out but a SOFT internal readiness target, not a hard external deadline (no regulation/contract binds this feature), so not 4 or 5. The genuine pressure is the compounding-retrofit argument (prompts set before this exists must be retrofitted later) - real but modest. "Meaningful advantage to shipping this year" = 3. CONFIDENCE (2): Structural/feasibility facts are strongly verified in-repo, but every VALUE score rests on reasoning plus analogous industry benchmarks, not on any direct demand data for this feature - inaccessible by environment constraint and ungathered by admission. Per the cap rule and honest thinness, confidence is 2 (single-data-point/analogous-anecdote tier), not 3.</t>
+  </si>
+  <si>
+    <t>F-004</t>
+  </si>
+  <si>
+    <t>Implement a proper production ready eventbus to replace the inproc bus currently in use</t>
+  </si>
+  <si>
+    <t>briefs/F-003-workspace-system-prompt.md</t>
+  </si>
+  <si>
     <t>Scored</t>
   </si>
   <si>
-    <t>2026-07-07</t>
-  </si>
-  <si>
-    <t>VERIFIED INTERNAL (repo read 2026-07-07): (1) web/src/features/workspaces/WorkspaceSettings.tsx lines 347-354 - the per-workspace "System prompt (blank = inherit)" textarea exists today; there is no above-workspace scope, confirming the "no baseline mechanism" problem statement. (2) bff/src/engine/mappers.ts lines 64-82 (WORKSPACE_FIELD_MAP) - systemPrompt maps 1:1 to a single engine field openAiPrompt; there is literally one prompt field per workspace and no native base+workspace layering, confirming the brief's central open question that a tamper-proof/enforced baseline is NOT achievable through this channel. (3) docs/anythingllm-surface.md lines 197-234 - confirms /system/default-system-prompt (native instance-level default) is session-auth-only and a "hard boundary at the API layer," unreachable under the console's API-key custody model; the console-managed fan-out route is the only option. All three brief leads re-verified as accurate. ANALOGOUS EXTERNAL (WebSearch 2026-07-07, directional only): Technavio - Enterprise Prompt Management Platforms market +USD 2.44B 2026-2030 at 32.5% CAGR; Gartner-cited AI-governance-platform spend ~USD 492M in 2026 rising past USD 1B by 2030; market shifting toward structured prompt governance and centralized control. These establish that centralized prompt/guardrail governance is a real, growing enterprise need. COUNTER-EVIDENCE: industry best-practice for real enforcement is a gateway-plus-guardrails architecture (policy enforced OUTSIDE the model call), not single-prompt-field storage (Galileo/Maxim/CSA 2025-2026) - corroborating that F-002's single-field approach is best-effort, not true enforcement. COULD NOT VERIFY: no support-ticket system, sales CRM, or usage-analytics dashboard exists for this internal tool, so zero direct demand signal for THIS feature; the brief itself states no discovery scan was run. Workspaces-per-customer count (bounds reach/effort) is unverifiable - an open question in the brief. The "governance as a selling point" business claim is entirely unverified against any sales evidence.</t>
-  </si>
-  <si>
-    <t>REACH (3): Scored against the STAFF OPERATORS who configure the feature (the console is staff-only per surface doc; customers never touch it), not the end-user chat population whose experience the prompt shapes. Absolute operator headcount is small and the config action is infrequent/high-leverage, but establishing a baseline persona/guardrail is a task essentially every customer onboarding would touch - "regular use" within the operator setup workflow, landing at the 15-40% regular-use anchor. Note: if scored against the effect population (every end-user chat across all workspaces) it would be 5; deliberately not, because the anchor measures the feature's USERS and this is a configuration control. USER_VALUE (3): The workaround exists today and is clumsy - manually re-typing the same baseline into each workspace's systemPrompt textarea and policing drift by hand (verified the textarea is the only mechanism). F-002 removes that clumsiness = solid 3. Not 4 because (a) pain frequency scales with workspaces-per-customer, which is unknown, and (b) the "safety guardrail" job-to-be-done is only partially delivered - the verified single-field engine model means the baseline can be silently clobbered by a per-workspace edit, so the strongest value claim (an enforced guardrail) is not realizable through this channel. BUSINESS_VALUE (2): Internal operator tool; revenue/retention effect is indirect. Industry data shows governance is a growing differentiator, but there is no CRM/sales evidence customers ask for it (brief admits this), and the enforcement gap weakens the "governance selling point." Indirect/small effect = 2, not 3, because a measurable conversion/retention effect is asserted, not evidenced. TIME_SENSITIVITY (3): October 2026 GTM is ~3 months out but a SOFT internal readiness target, not a hard external deadline (no regulation/contract binds this feature), so not 4 or 5. The genuine pressure is the compounding-retrofit argument (prompts set before this exists must be retrofitted later) - real but modest. "Meaningful advantage to shipping this year" = 3. CONFIDENCE (2): Structural/feasibility facts are strongly verified in-repo, but every VALUE score rests on reasoning plus analogous industry benchmarks, not on any direct demand data for this feature - inaccessible by environment constraint and ungathered by admission. Per the cap rule and honest thinness, confidence is 2 (single-data-point/analogous-anecdote tier), not 3.</t>
+    <t>Re-verified in-repo 2026-07-07: web/src/features/workspaces/WorkspaceSettings.tsx ~347-354 (lone 'System prompt (blank=inherit)' textarea); bff/src/engine/mappers.ts:74,104 + engine-types.ts:17,41 (systemPrompt-&gt;single engine openAiPrompt, no native layering); docs/anythingllm-surface.md:58,214,216 (one prompt field; native Default System Prompt/Prompt Variables session-auth = out-of-scope holds); specs/F-002-customer-system-prompt.md (baseline+sentinel/remainder/drift model, reserves per-workspace prompting for F-003; F-002 spec exists but not yet built); DangerConfirm.tsx/ErrorBanner.tsx exist; REQ-098 specs/admin-console.md:966. Rubric sheet3. No support/CRM/analytics or discovery-scan signal (internal tool).</t>
+  </si>
+  <si>
+    <t>reach=3 (&lt;25 staff operators; workspace-prompt config regular but infrequent, per F-002 logic); user_value=3 (removes clumsy manual baseline/workspace reconciliation on one opaque field, but pain contingent on unbuilt F-002 and unmeasured); business_value=2 (internal tool, indirect governance-completeness value, no sales evidence); time_sensitivity=3 (soft Oct-2026 GTM, compounding retrofit, no hard deadline); confidence=2 (structural facts verified in-repo but all value scores rest on conviction, no demand data/benchmark, plus F-002 dependency).</t>
+  </si>
+  <si>
+    <t>briefs/F-004-production-event-bus.md</t>
+  </si>
+  <si>
+    <t>bff/src/config.ts:50 (inproc default); bff/src/events/bus.ts:16-34 (InProcessBus default + OutboxRelayBus enqueue-only stub, 'later slice' comment); bff/src/store/repositories/outbox.repo.ts:34 listUnpublished has zero callers (no drain worker); grep: no .emitter.on / getEventBus consumers = zero subscribers; bff/src/events/catalog.ts + emitter.ts (contract built); docs/design/04-cross-cutting.md:74-76 &amp; 06-risks.md:70 (relay deferred/open); specs/admin-console.md REQ-029; no incident/demand/analytics signal in-repo.</t>
+  </si>
+  <si>
+    <t>[Human] A robust stable reliable eventbus is needed for actual customer use and I may as well be developing on a real eventbus as soon as possible.  ||  [Research 2026-07-07] reach=4 (delivery backbone for the entire admin.* event spine (17 event types, core cross-cutting) but consumer population latent/empty today so not 5); user_value=4 (unlocks a currently-impossible JTBD: durable cross-process at-least-once delivery + audit reliability, held below 5 since no consumer verified waiting); business_value=3 (production-readiness/compliance + tech-debt avoidance, no evidenced revenue/churn driver, internal infra); time_sensitivity=3 (GTM-linked ~3mo window but inproc is deployable and no consumer proven blocked); confidence=2 (structural gap validated with file:line citations but value/demand/urgency rest on conviction, zero usage/incident/demand evidence).</t>
   </si>
 </sst>
 </file>
@@ -1787,16 +1811,14 @@
       <c r="C5" s="18" t="s">
         <v>206</v>
       </c>
-      <c r="D5" s="18" t="inlineStr">
-        <is>
-          <t>Prioritized</t>
-        </is>
+      <c r="D5" s="18" t="s">
+        <v>198</v>
       </c>
       <c r="E5" s="18" t="s">
         <v>199</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G5" s="19">
         <v>3</v>
@@ -1823,10 +1845,10 @@
         <v>2</v>
       </c>
       <c r="O5" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="P5" s="20" t="s">
         <v>209</v>
-      </c>
-      <c r="P5" s="20" t="s">
-        <v>210</v>
       </c>
       <c r="Q5" s="21">
         <f>IF(COUNT(G5:K5)&lt;5,"",ROUND(G5*Config!$B$4+H5*Config!$B$5+I5*Config!$B$6+J5*Config!$B$7+K5*Config!$B$8,2))</f>
@@ -1846,87 +1868,147 @@
       </c>
       <c r="U5" s="23">
         <f>IF(T5="","",RANK(T5,$T$4:$T$53))</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.35">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" ht="308" x14ac:dyDescent="0.35">
       <c r="A6" s="18" t="s">
         <v>203</v>
       </c>
       <c r="B6" s="18" t="s">
         <v>205</v>
       </c>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="19"/>
-      <c r="H6" s="19"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="19"/>
-      <c r="K6" s="19"/>
-      <c r="L6" s="19"/>
-      <c r="M6" s="19"/>
-      <c r="N6" s="19"/>
-      <c r="O6" s="20"/>
-      <c r="P6" s="20"/>
-      <c r="Q6" s="21" t="str">
+      <c r="C6" s="18" t="s">
+        <v>212</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>198</v>
+      </c>
+      <c r="E6" s="18" t="s">
+        <v>199</v>
+      </c>
+      <c r="F6" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="G6" s="19">
+        <v>3</v>
+      </c>
+      <c r="H6" s="19">
+        <v>3</v>
+      </c>
+      <c r="I6" s="19">
+        <v>2</v>
+      </c>
+      <c r="J6" s="19">
+        <v>5</v>
+      </c>
+      <c r="K6" s="19">
+        <v>3</v>
+      </c>
+      <c r="L6" s="19">
+        <v>2</v>
+      </c>
+      <c r="M6" s="19">
+        <v>2</v>
+      </c>
+      <c r="N6" s="19">
+        <v>1</v>
+      </c>
+      <c r="O6" s="20" t="s">
+        <v>214</v>
+      </c>
+      <c r="P6" s="20" t="s">
+        <v>215</v>
+      </c>
+      <c r="Q6" s="21">
         <f>IF(COUNT(G6:K6)&lt;5,"",ROUND(G6*Config!$B$4+H6*Config!$B$5+I6*Config!$B$6+J6*Config!$B$7+K6*Config!$B$8,2))</f>
-        <v/>
-      </c>
-      <c r="R6" s="21" t="str">
+        <v>3.15</v>
+      </c>
+      <c r="R6" s="21">
         <f>IF(L6="","",VLOOKUP(L6,Config!$A$12:$B$16,2,0))</f>
-        <v/>
-      </c>
-      <c r="S6" s="21" t="str">
+        <v>0.65</v>
+      </c>
+      <c r="S6" s="21">
         <f>IF(N6="","",VLOOKUP(N6,Config!$D$12:$E$16,2,0))</f>
-        <v/>
-      </c>
-      <c r="T6" s="22" t="str">
+        <v>1</v>
+      </c>
+      <c r="T6" s="22">
         <f>IF(OR(Q6="",R6="",S6="",M6=""),"",ROUND(Q6*R6*S6/M6*20,1))</f>
-        <v/>
-      </c>
-      <c r="U6" s="23" t="str">
+        <v>20.5</v>
+      </c>
+      <c r="U6" s="23">
         <f>IF(T6="","",RANK(T6,$T$4:$T$53))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A7" s="18"/>
-      <c r="B7" s="18"/>
-      <c r="C7" s="18"/>
-      <c r="D7" s="18"/>
-      <c r="E7" s="18"/>
-      <c r="F7" s="18"/>
-      <c r="G7" s="19"/>
-      <c r="H7" s="19"/>
-      <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="19"/>
-      <c r="L7" s="19"/>
-      <c r="M7" s="19"/>
-      <c r="N7" s="19"/>
-      <c r="O7" s="20"/>
-      <c r="P7" s="20"/>
-      <c r="Q7" s="21" t="str">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" ht="350" x14ac:dyDescent="0.35">
+      <c r="A7" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="D7" s="18" t="s">
+        <v>198</v>
+      </c>
+      <c r="E7" s="18" t="s">
+        <v>199</v>
+      </c>
+      <c r="F7" s="18" t="s">
+        <v>207</v>
+      </c>
+      <c r="G7" s="19">
+        <v>4</v>
+      </c>
+      <c r="H7" s="19">
+        <v>4</v>
+      </c>
+      <c r="I7" s="19">
+        <v>3</v>
+      </c>
+      <c r="J7" s="19">
+        <v>5</v>
+      </c>
+      <c r="K7" s="19">
+        <v>3</v>
+      </c>
+      <c r="L7" s="19">
+        <v>2</v>
+      </c>
+      <c r="M7" s="19">
+        <v>4</v>
+      </c>
+      <c r="N7" s="19">
+        <v>3</v>
+      </c>
+      <c r="O7" s="20" t="s">
+        <v>217</v>
+      </c>
+      <c r="P7" s="20" t="s">
+        <v>218</v>
+      </c>
+      <c r="Q7" s="21">
         <f>IF(COUNT(G7:K7)&lt;5,"",ROUND(G7*Config!$B$4+H7*Config!$B$5+I7*Config!$B$6+J7*Config!$B$7+K7*Config!$B$8,2))</f>
-        <v/>
-      </c>
-      <c r="R7" s="21" t="str">
+        <v>3.85</v>
+      </c>
+      <c r="R7" s="21">
         <f>IF(L7="","",VLOOKUP(L7,Config!$A$12:$B$16,2,0))</f>
-        <v/>
-      </c>
-      <c r="S7" s="21" t="str">
+        <v>0.65</v>
+      </c>
+      <c r="S7" s="21">
         <f>IF(N7="","",VLOOKUP(N7,Config!$D$12:$E$16,2,0))</f>
-        <v/>
-      </c>
-      <c r="T7" s="22" t="str">
+        <v>0.8</v>
+      </c>
+      <c r="T7" s="22">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="U7" s="23" t="str">
+        <v>10</v>
+      </c>
+      <c r="U7" s="23">
         <f t="shared" si="1"/>
-        <v/>
+        <v>4</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Sync workbook validations with defect-era Data Dictionary
- Status dropdown now offers the full 12-value lifecycle enum (was the
  stale pre-defect 6-value list)
- feature_id row in the Data Dictionary documents the D-### pattern
- New dropdowns: Item Type (Feature/Defect), Defect Source
  (Customer-Reported/Internal), and a 1-5 whole-number check on Severity

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -521,10 +521,10 @@
     <t xml:space="preserve">string</t>
   </si>
   <si>
-    <t xml:space="preserve">Unique, pattern F-###</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stable identifier; used to join to the feature brief</t>
+    <t xml:space="preserve">Unique, pattern F-### (Feature) or D-### (Defect)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stable identifier; used to join to the feature brief (Feature) or defect/bug report (Defect)</t>
   </si>
   <si>
     <t xml:space="preserve">B: Feature Name</t>
@@ -983,7 +983,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="21">
+  <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1007,13 +1007,13 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+  </cellStyleXfs>
+  <cellXfs count="31">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-  </cellStyleXfs>
-  <cellXfs count="30">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1029,47 +1029,47 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1093,11 +1093,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1105,7 +1105,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1125,23 +1125,22 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="170" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="15" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="*unknown*" xfId="20" builtinId="8"/>
   </cellStyles>
   <colors>
     <indexedColors>
@@ -1389,130 +1388,130 @@
   <dimension ref="A1:A27"/>
   <sheetFormatPr defaultColWidth="8.63671875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="110"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="110"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-    </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2"/>
-    </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3"/>
+    </row>
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="2" t="s">
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="2"/>
-    </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3"/>
+    </row>
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="2" t="s">
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+    <row r="22" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
+    <row r="23" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
+    <row r="24" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
+    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
+    <row r="27" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1535,241 +1534,241 @@
   <dimension ref="A1:J23"/>
   <sheetFormatPr defaultColWidth="8.63671875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="6"/>
-    </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="s">
+      <c r="B3" s="7"/>
+    </row>
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="9" t="n">
         <v>0.2</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="s">
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="9" t="n">
         <v>0.25</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="s">
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="8" t="n">
+      <c r="B6" s="9" t="n">
         <v>0.25</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="s">
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="8" t="n">
+      <c r="B7" s="9" t="n">
         <v>0.2</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="s">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="8" t="n">
+      <c r="B8" s="9" t="n">
         <v>0.1</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="s">
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="10" t="str">
+      <c r="B9" s="11" t="str">
         <f aca="false">IF(SUM(B4:B8)=1,"OK","ERROR: weights must sum to 100%")</f>
         <v>OK</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B11" s="6"/>
-      <c r="D11" s="5" t="s">
+      <c r="B11" s="7"/>
+      <c r="D11" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E11" s="6"/>
-      <c r="G11" s="5" t="s">
+      <c r="E11" s="7"/>
+      <c r="G11" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="I11" s="6" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="n">
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="B12" s="12" t="n">
+      <c r="B12" s="13" t="n">
         <v>0.5</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="D12" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="G12" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="H12" s="13" t="n">
+      <c r="H12" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="I12" s="11" t="n">
+      <c r="I12" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="J12" s="12" t="n">
+      <c r="J12" s="13" t="n">
         <v>0.8</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="n">
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B13" s="12" t="n">
+      <c r="B13" s="13" t="n">
         <v>0.65</v>
       </c>
-      <c r="D13" s="11" t="n">
+      <c r="D13" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="13" t="n">
         <v>0.9</v>
       </c>
-      <c r="G13" s="11" t="n">
+      <c r="G13" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="H13" s="13" t="n">
+      <c r="H13" s="14" t="n">
         <v>30</v>
       </c>
-      <c r="I13" s="11" t="n">
+      <c r="I13" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="J13" s="12" t="n">
+      <c r="J13" s="13" t="n">
         <v>0.9</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="n">
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="B14" s="12" t="n">
+      <c r="B14" s="13" t="n">
         <v>0.8</v>
       </c>
-      <c r="D14" s="11" t="n">
+      <c r="D14" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="12" t="n">
+      <c r="E14" s="13" t="n">
         <v>0.8</v>
       </c>
-      <c r="G14" s="11" t="n">
+      <c r="G14" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="H14" s="13" t="n">
+      <c r="H14" s="14" t="n">
         <v>55</v>
       </c>
-      <c r="I14" s="11" t="n">
+      <c r="I14" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="J14" s="12" t="n">
+      <c r="J14" s="13" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="n">
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B15" s="12" t="n">
+      <c r="B15" s="13" t="n">
         <v>0.9</v>
       </c>
-      <c r="D15" s="11" t="n">
+      <c r="D15" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E15" s="13" t="n">
         <v>0.7</v>
       </c>
-      <c r="G15" s="11" t="n">
+      <c r="G15" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="H15" s="13" t="n">
+      <c r="H15" s="14" t="n">
         <v>80</v>
       </c>
-      <c r="I15" s="11" t="n">
+      <c r="I15" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="J15" s="12" t="n">
+      <c r="J15" s="13" t="n">
         <v>1.1</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="n">
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="12" t="n">
+      <c r="B16" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="D16" s="11" t="n">
+      <c r="D16" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="E16" s="12" t="n">
+      <c r="E16" s="13" t="n">
         <v>0.6</v>
       </c>
-      <c r="G16" s="11" t="n">
+      <c r="G16" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="H16" s="13" t="n">
+      <c r="H16" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="I16" s="11" t="n">
+      <c r="I16" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="J16" s="12" t="n">
+      <c r="J16" s="13" t="n">
         <v>1.2</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="15" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="15" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="14" t="s">
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="15" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="s">
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="15" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="14" t="s">
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="15" t="s">
         <v>39</v>
       </c>
     </row>
@@ -1792,212 +1791,212 @@
   <dimension ref="A1:F12"/>
   <sheetFormatPr defaultColWidth="8.63671875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="1" width="34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="15" t="s">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="15" t="s">
+      <c r="C3" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="D3" s="15" t="s">
+      <c r="D3" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="16" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="18" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="E4" s="18" t="s">
         <v>50</v>
       </c>
-      <c r="F4" s="17" t="s">
+      <c r="F4" s="18" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="C5" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="D5" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="E5" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="F5" s="17" t="s">
+      <c r="F5" s="18" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="F6" s="17" t="s">
+      <c r="F6" s="18" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="F7" s="17" t="s">
+      <c r="F7" s="18" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="D8" s="17" t="s">
+      <c r="D8" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="E8" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="F8" s="17" t="s">
+      <c r="F8" s="18" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="17" t="s">
         <v>72</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="D9" s="17" t="s">
+      <c r="D9" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="E9" s="17" t="s">
+      <c r="E9" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="F9" s="17" t="s">
+      <c r="F9" s="18" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="D10" s="17" t="s">
+      <c r="D10" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="E10" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="F10" s="17" t="s">
+      <c r="F10" s="18" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="D11" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="F11" s="17" t="s">
+      <c r="F11" s="18" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="18" t="s">
+    <row r="12" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="3" t="s">
         <v>95</v>
       </c>
     </row>
@@ -2020,2190 +2019,2202 @@
   <dimension ref="A1:X53"/>
   <sheetFormatPr defaultColWidth="8.63671875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="41.73"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="9" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="17" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="22" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="41.73"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="9" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="15" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="17" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="22" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="14" t="s">
+    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="15" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="20" t="s">
         <v>98</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="20" t="s">
         <v>99</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="C3" s="20" t="s">
         <v>100</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="D3" s="20" t="s">
         <v>101</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="G3" s="19" t="s">
+      <c r="G3" s="20" t="s">
         <v>104</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="I3" s="19" t="s">
+      <c r="I3" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="J3" s="19" t="s">
+      <c r="J3" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="K3" s="19" t="s">
+      <c r="K3" s="20" t="s">
         <v>108</v>
       </c>
-      <c r="L3" s="19" t="s">
+      <c r="L3" s="20" t="s">
         <v>109</v>
       </c>
-      <c r="M3" s="19" t="s">
+      <c r="M3" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="N3" s="19" t="s">
+      <c r="N3" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="O3" s="19" t="s">
+      <c r="O3" s="20" t="s">
         <v>112</v>
       </c>
-      <c r="P3" s="19" t="s">
+      <c r="P3" s="20" t="s">
         <v>113</v>
       </c>
-      <c r="Q3" s="19" t="s">
+      <c r="Q3" s="20" t="s">
         <v>114</v>
       </c>
-      <c r="R3" s="19" t="s">
+      <c r="R3" s="20" t="s">
         <v>115</v>
       </c>
-      <c r="S3" s="19" t="s">
+      <c r="S3" s="20" t="s">
         <v>116</v>
       </c>
-      <c r="T3" s="19" t="s">
+      <c r="T3" s="20" t="s">
         <v>117</v>
       </c>
-      <c r="U3" s="19" t="s">
+      <c r="U3" s="20" t="s">
         <v>118</v>
       </c>
-      <c r="V3" s="19" t="s">
+      <c r="V3" s="20" t="s">
         <v>119</v>
       </c>
-      <c r="W3" s="19" t="s">
+      <c r="W3" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="X3" s="19" t="s">
+      <c r="X3" s="20" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="409.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="B4" s="20" t="s">
+      <c r="B4" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="C4" s="20" t="s">
+      <c r="C4" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="D4" s="20" t="s">
+      <c r="D4" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="E4" s="20" t="s">
+      <c r="E4" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="F4" s="21" t="n">
+      <c r="F4" s="22" t="n">
         <v>46210</v>
       </c>
-      <c r="G4" s="22" t="n">
+      <c r="G4" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="H4" s="22" t="n">
+      <c r="H4" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="I4" s="22" t="n">
+      <c r="I4" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="J4" s="22" t="n">
+      <c r="J4" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="K4" s="22" t="n">
+      <c r="K4" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="L4" s="22" t="n">
+      <c r="L4" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="M4" s="22" t="n">
+      <c r="M4" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="N4" s="22" t="n">
+      <c r="N4" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="O4" s="23" t="s">
+      <c r="O4" s="24" t="s">
         <v>127</v>
       </c>
-      <c r="P4" s="24" t="s">
+      <c r="P4" s="25" t="s">
         <v>128</v>
       </c>
-      <c r="Q4" s="25" t="n">
+      <c r="Q4" s="26" t="n">
         <f aca="false">IF(V4="Defect","",IF(COUNT(G4:K4)&lt;5,"",ROUND(G4*Config!$B$4+H4*Config!$B$5+I4*Config!$B$6+J4*Config!$B$7+K4*Config!$B$8,2)))</f>
         <v>3.55</v>
       </c>
-      <c r="R4" s="25" t="n">
+      <c r="R4" s="26" t="n">
         <f aca="false">IF(L4="","",VLOOKUP(L4,Config!$A$12:$B$16,2,0))</f>
         <v>0.65</v>
       </c>
-      <c r="S4" s="25" t="n">
+      <c r="S4" s="26" t="n">
         <f aca="false">IF(N4="","",VLOOKUP(N4,Config!$D$12:$E$16,2,0))</f>
         <v>1</v>
       </c>
-      <c r="T4" s="26" t="n">
+      <c r="T4" s="27" t="n">
         <f aca="false">IF(V4="Defect",IF(OR(X4="",G4="",R4=""),"",ROUND(MIN(100,VLOOKUP(X4,Config!$G$12:$H$16,2,0)*VLOOKUP(G4,Config!$I$12:$J$16,2,0)*R4),1)),IF(OR(Q4="",R4="",S4="",M4=""),"",ROUND(Q4*R4*S4/M4*20,1)))</f>
         <v>46.2</v>
       </c>
-      <c r="U4" s="27" t="n">
+      <c r="U4" s="28" t="n">
         <f aca="false">IF(T4="","",RANK(T4,$T$4:$T$53))</f>
         <v>2</v>
       </c>
-      <c r="V4" s="20" t="s">
+      <c r="V4" s="21" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="409.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
+      <c r="A5" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="D5" s="20" t="s">
+      <c r="D5" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="E5" s="20" t="s">
+      <c r="E5" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="F5" s="20" t="s">
+      <c r="F5" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="G5" s="22" t="n">
+      <c r="G5" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="H5" s="22" t="n">
+      <c r="H5" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="I5" s="22" t="n">
+      <c r="I5" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="J5" s="22" t="n">
+      <c r="J5" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="K5" s="22" t="n">
+      <c r="K5" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="L5" s="22" t="n">
+      <c r="L5" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="M5" s="22" t="n">
+      <c r="M5" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="N5" s="22" t="n">
+      <c r="N5" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="O5" s="24" t="s">
+      <c r="O5" s="25" t="s">
         <v>134</v>
       </c>
-      <c r="P5" s="24" t="s">
+      <c r="P5" s="25" t="s">
         <v>135</v>
       </c>
-      <c r="Q5" s="25" t="n">
+      <c r="Q5" s="26" t="n">
         <f aca="false">IF(V5="Defect","",IF(COUNT(G5:K5)&lt;5,"",ROUND(G5*Config!$B$4+H5*Config!$B$5+I5*Config!$B$6+J5*Config!$B$7+K5*Config!$B$8,2)))</f>
         <v>2.95</v>
       </c>
-      <c r="R5" s="25" t="n">
+      <c r="R5" s="26" t="n">
         <f aca="false">IF(L5="","",VLOOKUP(L5,Config!$A$12:$B$16,2,0))</f>
         <v>0.65</v>
       </c>
-      <c r="S5" s="25" t="n">
+      <c r="S5" s="26" t="n">
         <f aca="false">IF(N5="","",VLOOKUP(N5,Config!$D$12:$E$16,2,0))</f>
         <v>0.9</v>
       </c>
-      <c r="T5" s="26" t="n">
+      <c r="T5" s="27" t="n">
         <f aca="false">IF(V5="Defect",IF(OR(X5="",G5="",R5=""),"",ROUND(MIN(100,VLOOKUP(X5,Config!$G$12:$H$16,2,0)*VLOOKUP(G5,Config!$I$12:$J$16,2,0)*R5),1)),IF(OR(Q5="",R5="",S5="",M5=""),"",ROUND(Q5*R5*S5/M5*20,1)))</f>
         <v>17.3</v>
       </c>
-      <c r="U5" s="27" t="n">
+      <c r="U5" s="28" t="n">
         <f aca="false">IF(T5="","",RANK(T5,$T$4:$T$53))</f>
         <v>4</v>
       </c>
-      <c r="V5" s="20" t="s">
+      <c r="V5" s="21" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="307.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20" t="s">
+      <c r="A6" s="21" t="s">
         <v>136</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="C6" s="20" t="s">
+      <c r="C6" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="E6" s="20" t="s">
+      <c r="E6" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="F6" s="20" t="s">
+      <c r="F6" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="G6" s="22" t="n">
+      <c r="G6" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="H6" s="22" t="n">
+      <c r="H6" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="I6" s="22" t="n">
+      <c r="I6" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="J6" s="22" t="n">
+      <c r="J6" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="K6" s="22" t="n">
+      <c r="K6" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="L6" s="22" t="n">
+      <c r="L6" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="M6" s="22" t="n">
+      <c r="M6" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="N6" s="22" t="n">
+      <c r="N6" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="O6" s="24" t="s">
+      <c r="O6" s="25" t="s">
         <v>139</v>
       </c>
-      <c r="P6" s="24" t="s">
+      <c r="P6" s="25" t="s">
         <v>140</v>
       </c>
-      <c r="Q6" s="25" t="n">
+      <c r="Q6" s="26" t="n">
         <f aca="false">IF(V6="Defect","",IF(COUNT(G6:K6)&lt;5,"",ROUND(G6*Config!$B$4+H6*Config!$B$5+I6*Config!$B$6+J6*Config!$B$7+K6*Config!$B$8,2)))</f>
         <v>3.15</v>
       </c>
-      <c r="R6" s="25" t="n">
+      <c r="R6" s="26" t="n">
         <f aca="false">IF(L6="","",VLOOKUP(L6,Config!$A$12:$B$16,2,0))</f>
         <v>0.65</v>
       </c>
-      <c r="S6" s="25" t="n">
+      <c r="S6" s="26" t="n">
         <f aca="false">IF(N6="","",VLOOKUP(N6,Config!$D$12:$E$16,2,0))</f>
         <v>1</v>
       </c>
-      <c r="T6" s="26" t="n">
+      <c r="T6" s="27" t="n">
         <f aca="false">IF(V6="Defect",IF(OR(X6="",G6="",R6=""),"",ROUND(MIN(100,VLOOKUP(X6,Config!$G$12:$H$16,2,0)*VLOOKUP(G6,Config!$I$12:$J$16,2,0)*R6),1)),IF(OR(Q6="",R6="",S6="",M6=""),"",ROUND(Q6*R6*S6/M6*20,1)))</f>
         <v>20.5</v>
       </c>
-      <c r="U6" s="27" t="n">
+      <c r="U6" s="28" t="n">
         <f aca="false">IF(T6="","",RANK(T6,$T$4:$T$53))</f>
         <v>3</v>
       </c>
-      <c r="V6" s="20" t="s">
+      <c r="V6" s="21" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="349.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="21" t="s">
         <v>142</v>
       </c>
-      <c r="C7" s="20" t="s">
+      <c r="C7" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="E7" s="20" t="s">
+      <c r="E7" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="F7" s="20" t="s">
+      <c r="F7" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="G7" s="22" t="n">
+      <c r="G7" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="H7" s="22" t="n">
+      <c r="H7" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="I7" s="22" t="n">
+      <c r="I7" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="J7" s="22" t="n">
+      <c r="J7" s="23" t="n">
         <v>5</v>
       </c>
-      <c r="K7" s="22" t="n">
+      <c r="K7" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="L7" s="22" t="n">
+      <c r="L7" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="M7" s="22" t="n">
+      <c r="M7" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="N7" s="22" t="n">
+      <c r="N7" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="O7" s="24" t="s">
+      <c r="O7" s="25" t="s">
         <v>144</v>
       </c>
-      <c r="P7" s="24" t="s">
+      <c r="P7" s="25" t="s">
         <v>145</v>
       </c>
-      <c r="Q7" s="25" t="n">
+      <c r="Q7" s="26" t="n">
         <f aca="false">IF(V7="Defect","",IF(COUNT(G7:K7)&lt;5,"",ROUND(G7*Config!$B$4+H7*Config!$B$5+I7*Config!$B$6+J7*Config!$B$7+K7*Config!$B$8,2)))</f>
         <v>3.85</v>
       </c>
-      <c r="R7" s="25" t="n">
+      <c r="R7" s="26" t="n">
         <f aca="false">IF(L7="","",VLOOKUP(L7,Config!$A$12:$B$16,2,0))</f>
         <v>0.65</v>
       </c>
-      <c r="S7" s="25" t="n">
+      <c r="S7" s="26" t="n">
         <f aca="false">IF(N7="","",VLOOKUP(N7,Config!$D$12:$E$16,2,0))</f>
         <v>0.8</v>
       </c>
-      <c r="T7" s="26" t="n">
+      <c r="T7" s="27" t="n">
         <f aca="false">IF(V7="Defect",IF(OR(X7="",G7="",R7=""),"",ROUND(MIN(100,VLOOKUP(X7,Config!$G$12:$H$16,2,0)*VLOOKUP(G7,Config!$I$12:$J$16,2,0)*R7),1)),IF(OR(Q7="",R7="",S7="",M7=""),"",ROUND(Q7*R7*S7/M7*20,1)))</f>
         <v>10</v>
       </c>
-      <c r="U7" s="27" t="n">
+      <c r="U7" s="28" t="n">
         <f aca="false">IF(T7="","",RANK(T7,$T$4:$T$53))</f>
         <v>5</v>
       </c>
-      <c r="V7" s="20" t="s">
+      <c r="V7" s="21" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="20" t="s">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="C8" s="20" t="s">
+      <c r="C8" s="21" t="s">
         <v>148</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E8" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="F8" s="28" t="n">
+      <c r="F8" s="29" t="n">
         <v>46214</v>
       </c>
-      <c r="G8" s="20" t="n">
+      <c r="G8" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="H8" s="22"/>
-      <c r="I8" s="22"/>
-      <c r="J8" s="22"/>
-      <c r="K8" s="22"/>
-      <c r="L8" s="20" t="n">
+      <c r="H8" s="23"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="23"/>
+      <c r="K8" s="23"/>
+      <c r="L8" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="M8" s="22"/>
-      <c r="N8" s="22"/>
-      <c r="O8" s="20" t="s">
+      <c r="M8" s="23"/>
+      <c r="N8" s="23"/>
+      <c r="O8" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="P8" s="20" t="s">
+      <c r="P8" s="21" t="s">
         <v>152</v>
       </c>
-      <c r="Q8" s="25" t="str">
+      <c r="Q8" s="26" t="str">
         <f aca="false">IF(V8="Defect","",IF(COUNT(G8:K8)&lt;5,"",ROUND(G8*Config!$B$4+H8*Config!$B$5+I8*Config!$B$6+J8*Config!$B$7+K8*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R8" s="25" t="n">
+      <c r="R8" s="26" t="n">
         <f aca="false">IF(L8="","",VLOOKUP(L8,Config!$A$12:$B$16,2,0))</f>
         <v>0.8</v>
       </c>
-      <c r="S8" s="25" t="str">
+      <c r="S8" s="26" t="str">
         <f aca="false">IF(N8="","",VLOOKUP(N8,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T8" s="26" t="n">
+      <c r="T8" s="27" t="n">
         <f aca="false">IF(V8="Defect",IF(OR(X8="",G8="",R8=""),"",ROUND(MIN(100,VLOOKUP(X8,Config!$G$12:$H$16,2,0)*VLOOKUP(G8,Config!$I$12:$J$16,2,0)*R8),1)),IF(OR(Q8="",R8="",S8="",M8=""),"",ROUND(Q8*R8*S8/M8*20,1)))</f>
         <v>64</v>
       </c>
-      <c r="U8" s="27" t="n">
+      <c r="U8" s="28" t="n">
         <f aca="false">IF(T8="","",RANK(T8,$T$4:$T$53))</f>
         <v>1</v>
       </c>
-      <c r="V8" s="20" t="s">
+      <c r="V8" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="W8" s="20" t="s">
+      <c r="W8" s="21" t="s">
         <v>154</v>
       </c>
-      <c r="X8" s="20" t="n">
+      <c r="X8" s="21" t="n">
         <v>4</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="20"/>
-      <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="22"/>
-      <c r="H9" s="22"/>
-      <c r="I9" s="22"/>
-      <c r="J9" s="22"/>
-      <c r="K9" s="22"/>
-      <c r="L9" s="22"/>
-      <c r="M9" s="22"/>
-      <c r="N9" s="22"/>
-      <c r="O9" s="24"/>
-      <c r="P9" s="24"/>
-      <c r="Q9" s="25" t="str">
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="21"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="23"/>
+      <c r="H9" s="23"/>
+      <c r="I9" s="23"/>
+      <c r="J9" s="23"/>
+      <c r="K9" s="23"/>
+      <c r="L9" s="23"/>
+      <c r="M9" s="23"/>
+      <c r="N9" s="23"/>
+      <c r="O9" s="25"/>
+      <c r="P9" s="25"/>
+      <c r="Q9" s="26" t="str">
         <f aca="false">IF(V9="Defect","",IF(COUNT(G9:K9)&lt;5,"",ROUND(G9*Config!$B$4+H9*Config!$B$5+I9*Config!$B$6+J9*Config!$B$7+K9*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R9" s="25" t="str">
+      <c r="R9" s="26" t="str">
         <f aca="false">IF(L9="","",VLOOKUP(L9,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S9" s="25" t="str">
+      <c r="S9" s="26" t="str">
         <f aca="false">IF(N9="","",VLOOKUP(N9,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T9" s="26" t="str">
+      <c r="T9" s="27" t="str">
         <f aca="false">IF(V9="Defect",IF(OR(X9="",G9="",R9=""),"",ROUND(MIN(100,VLOOKUP(X9,Config!$G$12:$H$16,2,0)*VLOOKUP(G9,Config!$I$12:$J$16,2,0)*R9),1)),IF(OR(Q9="",R9="",S9="",M9=""),"",ROUND(Q9*R9*S9/M9*20,1)))</f>
         <v/>
       </c>
-      <c r="U9" s="27" t="str">
+      <c r="U9" s="28" t="str">
         <f aca="false">IF(T9="","",RANK(T9,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20"/>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="22"/>
-      <c r="H10" s="22"/>
-      <c r="I10" s="22"/>
-      <c r="J10" s="22"/>
-      <c r="K10" s="22"/>
-      <c r="L10" s="22"/>
-      <c r="M10" s="22"/>
-      <c r="N10" s="22"/>
-      <c r="O10" s="24"/>
-      <c r="P10" s="24"/>
-      <c r="Q10" s="25" t="str">
+    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="21"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="23"/>
+      <c r="H10" s="23"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="23"/>
+      <c r="K10" s="23"/>
+      <c r="L10" s="23"/>
+      <c r="M10" s="23"/>
+      <c r="N10" s="23"/>
+      <c r="O10" s="25"/>
+      <c r="P10" s="25"/>
+      <c r="Q10" s="26" t="str">
         <f aca="false">IF(V10="Defect","",IF(COUNT(G10:K10)&lt;5,"",ROUND(G10*Config!$B$4+H10*Config!$B$5+I10*Config!$B$6+J10*Config!$B$7+K10*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R10" s="25" t="str">
+      <c r="R10" s="26" t="str">
         <f aca="false">IF(L10="","",VLOOKUP(L10,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S10" s="25" t="str">
+      <c r="S10" s="26" t="str">
         <f aca="false">IF(N10="","",VLOOKUP(N10,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T10" s="26" t="str">
+      <c r="T10" s="27" t="str">
         <f aca="false">IF(V10="Defect",IF(OR(X10="",G10="",R10=""),"",ROUND(MIN(100,VLOOKUP(X10,Config!$G$12:$H$16,2,0)*VLOOKUP(G10,Config!$I$12:$J$16,2,0)*R10),1)),IF(OR(Q10="",R10="",S10="",M10=""),"",ROUND(Q10*R10*S10/M10*20,1)))</f>
         <v/>
       </c>
-      <c r="U10" s="27" t="str">
+      <c r="U10" s="28" t="str">
         <f aca="false">IF(T10="","",RANK(T10,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="22"/>
-      <c r="H11" s="22"/>
-      <c r="I11" s="22"/>
-      <c r="J11" s="22"/>
-      <c r="K11" s="22"/>
-      <c r="L11" s="22"/>
-      <c r="M11" s="22"/>
-      <c r="N11" s="22"/>
-      <c r="O11" s="24"/>
-      <c r="P11" s="24"/>
-      <c r="Q11" s="25" t="str">
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="21"/>
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="23"/>
+      <c r="H11" s="23"/>
+      <c r="I11" s="23"/>
+      <c r="J11" s="23"/>
+      <c r="K11" s="23"/>
+      <c r="L11" s="23"/>
+      <c r="M11" s="23"/>
+      <c r="N11" s="23"/>
+      <c r="O11" s="25"/>
+      <c r="P11" s="25"/>
+      <c r="Q11" s="26" t="str">
         <f aca="false">IF(V11="Defect","",IF(COUNT(G11:K11)&lt;5,"",ROUND(G11*Config!$B$4+H11*Config!$B$5+I11*Config!$B$6+J11*Config!$B$7+K11*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R11" s="25" t="str">
+      <c r="R11" s="26" t="str">
         <f aca="false">IF(L11="","",VLOOKUP(L11,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S11" s="25" t="str">
+      <c r="S11" s="26" t="str">
         <f aca="false">IF(N11="","",VLOOKUP(N11,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T11" s="26" t="str">
+      <c r="T11" s="27" t="str">
         <f aca="false">IF(V11="Defect",IF(OR(X11="",G11="",R11=""),"",ROUND(MIN(100,VLOOKUP(X11,Config!$G$12:$H$16,2,0)*VLOOKUP(G11,Config!$I$12:$J$16,2,0)*R11),1)),IF(OR(Q11="",R11="",S11="",M11=""),"",ROUND(Q11*R11*S11/M11*20,1)))</f>
         <v/>
       </c>
-      <c r="U11" s="27" t="str">
+      <c r="U11" s="28" t="str">
         <f aca="false">IF(T11="","",RANK(T11,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="20"/>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="22"/>
-      <c r="I12" s="22"/>
-      <c r="J12" s="22"/>
-      <c r="K12" s="22"/>
-      <c r="L12" s="22"/>
-      <c r="M12" s="22"/>
-      <c r="N12" s="22"/>
-      <c r="O12" s="24"/>
-      <c r="P12" s="24"/>
-      <c r="Q12" s="25" t="str">
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="21"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="23"/>
+      <c r="H12" s="23"/>
+      <c r="I12" s="23"/>
+      <c r="J12" s="23"/>
+      <c r="K12" s="23"/>
+      <c r="L12" s="23"/>
+      <c r="M12" s="23"/>
+      <c r="N12" s="23"/>
+      <c r="O12" s="25"/>
+      <c r="P12" s="25"/>
+      <c r="Q12" s="26" t="str">
         <f aca="false">IF(V12="Defect","",IF(COUNT(G12:K12)&lt;5,"",ROUND(G12*Config!$B$4+H12*Config!$B$5+I12*Config!$B$6+J12*Config!$B$7+K12*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R12" s="25" t="str">
+      <c r="R12" s="26" t="str">
         <f aca="false">IF(L12="","",VLOOKUP(L12,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S12" s="25" t="str">
+      <c r="S12" s="26" t="str">
         <f aca="false">IF(N12="","",VLOOKUP(N12,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T12" s="26" t="str">
+      <c r="T12" s="27" t="str">
         <f aca="false">IF(V12="Defect",IF(OR(X12="",G12="",R12=""),"",ROUND(MIN(100,VLOOKUP(X12,Config!$G$12:$H$16,2,0)*VLOOKUP(G12,Config!$I$12:$J$16,2,0)*R12),1)),IF(OR(Q12="",R12="",S12="",M12=""),"",ROUND(Q12*R12*S12/M12*20,1)))</f>
         <v/>
       </c>
-      <c r="U12" s="27" t="str">
+      <c r="U12" s="28" t="str">
         <f aca="false">IF(T12="","",RANK(T12,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20"/>
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="22"/>
-      <c r="H13" s="22"/>
-      <c r="I13" s="22"/>
-      <c r="J13" s="22"/>
-      <c r="K13" s="22"/>
-      <c r="L13" s="22"/>
-      <c r="M13" s="22"/>
-      <c r="N13" s="22"/>
-      <c r="O13" s="24"/>
-      <c r="P13" s="24"/>
-      <c r="Q13" s="25" t="str">
+    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="21"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="21"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="23"/>
+      <c r="H13" s="23"/>
+      <c r="I13" s="23"/>
+      <c r="J13" s="23"/>
+      <c r="K13" s="23"/>
+      <c r="L13" s="23"/>
+      <c r="M13" s="23"/>
+      <c r="N13" s="23"/>
+      <c r="O13" s="25"/>
+      <c r="P13" s="25"/>
+      <c r="Q13" s="26" t="str">
         <f aca="false">IF(V13="Defect","",IF(COUNT(G13:K13)&lt;5,"",ROUND(G13*Config!$B$4+H13*Config!$B$5+I13*Config!$B$6+J13*Config!$B$7+K13*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R13" s="25" t="str">
+      <c r="R13" s="26" t="str">
         <f aca="false">IF(L13="","",VLOOKUP(L13,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S13" s="25" t="str">
+      <c r="S13" s="26" t="str">
         <f aca="false">IF(N13="","",VLOOKUP(N13,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T13" s="26" t="str">
+      <c r="T13" s="27" t="str">
         <f aca="false">IF(V13="Defect",IF(OR(X13="",G13="",R13=""),"",ROUND(MIN(100,VLOOKUP(X13,Config!$G$12:$H$16,2,0)*VLOOKUP(G13,Config!$I$12:$J$16,2,0)*R13),1)),IF(OR(Q13="",R13="",S13="",M13=""),"",ROUND(Q13*R13*S13/M13*20,1)))</f>
         <v/>
       </c>
-      <c r="U13" s="27" t="str">
+      <c r="U13" s="28" t="str">
         <f aca="false">IF(T13="","",RANK(T13,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="22"/>
-      <c r="H14" s="22"/>
-      <c r="I14" s="22"/>
-      <c r="J14" s="22"/>
-      <c r="K14" s="22"/>
-      <c r="L14" s="22"/>
-      <c r="M14" s="22"/>
-      <c r="N14" s="22"/>
-      <c r="O14" s="24"/>
-      <c r="P14" s="24"/>
-      <c r="Q14" s="25" t="str">
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="21"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="23"/>
+      <c r="I14" s="23"/>
+      <c r="J14" s="23"/>
+      <c r="K14" s="23"/>
+      <c r="L14" s="23"/>
+      <c r="M14" s="23"/>
+      <c r="N14" s="23"/>
+      <c r="O14" s="25"/>
+      <c r="P14" s="25"/>
+      <c r="Q14" s="26" t="str">
         <f aca="false">IF(V14="Defect","",IF(COUNT(G14:K14)&lt;5,"",ROUND(G14*Config!$B$4+H14*Config!$B$5+I14*Config!$B$6+J14*Config!$B$7+K14*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R14" s="25" t="str">
+      <c r="R14" s="26" t="str">
         <f aca="false">IF(L14="","",VLOOKUP(L14,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S14" s="25" t="str">
+      <c r="S14" s="26" t="str">
         <f aca="false">IF(N14="","",VLOOKUP(N14,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T14" s="26" t="str">
+      <c r="T14" s="27" t="str">
         <f aca="false">IF(V14="Defect",IF(OR(X14="",G14="",R14=""),"",ROUND(MIN(100,VLOOKUP(X14,Config!$G$12:$H$16,2,0)*VLOOKUP(G14,Config!$I$12:$J$16,2,0)*R14),1)),IF(OR(Q14="",R14="",S14="",M14=""),"",ROUND(Q14*R14*S14/M14*20,1)))</f>
         <v/>
       </c>
-      <c r="U14" s="27" t="str">
+      <c r="U14" s="28" t="str">
         <f aca="false">IF(T14="","",RANK(T14,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20"/>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="22"/>
-      <c r="I15" s="22"/>
-      <c r="J15" s="22"/>
-      <c r="K15" s="22"/>
-      <c r="L15" s="22"/>
-      <c r="M15" s="22"/>
-      <c r="N15" s="22"/>
-      <c r="O15" s="24"/>
-      <c r="P15" s="24"/>
-      <c r="Q15" s="25" t="str">
+    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="21"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="21"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="23"/>
+      <c r="H15" s="23"/>
+      <c r="I15" s="23"/>
+      <c r="J15" s="23"/>
+      <c r="K15" s="23"/>
+      <c r="L15" s="23"/>
+      <c r="M15" s="23"/>
+      <c r="N15" s="23"/>
+      <c r="O15" s="25"/>
+      <c r="P15" s="25"/>
+      <c r="Q15" s="26" t="str">
         <f aca="false">IF(V15="Defect","",IF(COUNT(G15:K15)&lt;5,"",ROUND(G15*Config!$B$4+H15*Config!$B$5+I15*Config!$B$6+J15*Config!$B$7+K15*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R15" s="25" t="str">
+      <c r="R15" s="26" t="str">
         <f aca="false">IF(L15="","",VLOOKUP(L15,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S15" s="25" t="str">
+      <c r="S15" s="26" t="str">
         <f aca="false">IF(N15="","",VLOOKUP(N15,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T15" s="26" t="str">
+      <c r="T15" s="27" t="str">
         <f aca="false">IF(V15="Defect",IF(OR(X15="",G15="",R15=""),"",ROUND(MIN(100,VLOOKUP(X15,Config!$G$12:$H$16,2,0)*VLOOKUP(G15,Config!$I$12:$J$16,2,0)*R15),1)),IF(OR(Q15="",R15="",S15="",M15=""),"",ROUND(Q15*R15*S15/M15*20,1)))</f>
         <v/>
       </c>
-      <c r="U15" s="27" t="str">
+      <c r="U15" s="28" t="str">
         <f aca="false">IF(T15="","",RANK(T15,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="20"/>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="22"/>
-      <c r="H16" s="22"/>
-      <c r="I16" s="22"/>
-      <c r="J16" s="22"/>
-      <c r="K16" s="22"/>
-      <c r="L16" s="22"/>
-      <c r="M16" s="22"/>
-      <c r="N16" s="22"/>
-      <c r="O16" s="24"/>
-      <c r="P16" s="24"/>
-      <c r="Q16" s="25" t="str">
+    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="21"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="21"/>
+      <c r="F16" s="21"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="23"/>
+      <c r="K16" s="23"/>
+      <c r="L16" s="23"/>
+      <c r="M16" s="23"/>
+      <c r="N16" s="23"/>
+      <c r="O16" s="25"/>
+      <c r="P16" s="25"/>
+      <c r="Q16" s="26" t="str">
         <f aca="false">IF(V16="Defect","",IF(COUNT(G16:K16)&lt;5,"",ROUND(G16*Config!$B$4+H16*Config!$B$5+I16*Config!$B$6+J16*Config!$B$7+K16*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R16" s="25" t="str">
+      <c r="R16" s="26" t="str">
         <f aca="false">IF(L16="","",VLOOKUP(L16,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S16" s="25" t="str">
+      <c r="S16" s="26" t="str">
         <f aca="false">IF(N16="","",VLOOKUP(N16,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T16" s="26" t="str">
+      <c r="T16" s="27" t="str">
         <f aca="false">IF(V16="Defect",IF(OR(X16="",G16="",R16=""),"",ROUND(MIN(100,VLOOKUP(X16,Config!$G$12:$H$16,2,0)*VLOOKUP(G16,Config!$I$12:$J$16,2,0)*R16),1)),IF(OR(Q16="",R16="",S16="",M16=""),"",ROUND(Q16*R16*S16/M16*20,1)))</f>
         <v/>
       </c>
-      <c r="U16" s="27" t="str">
+      <c r="U16" s="28" t="str">
         <f aca="false">IF(T16="","",RANK(T16,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="20"/>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="20"/>
-      <c r="G17" s="22"/>
-      <c r="H17" s="22"/>
-      <c r="I17" s="22"/>
-      <c r="J17" s="22"/>
-      <c r="K17" s="22"/>
-      <c r="L17" s="22"/>
-      <c r="M17" s="22"/>
-      <c r="N17" s="22"/>
-      <c r="O17" s="24"/>
-      <c r="P17" s="24"/>
-      <c r="Q17" s="25" t="str">
+    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="21"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="21"/>
+      <c r="F17" s="21"/>
+      <c r="G17" s="23"/>
+      <c r="H17" s="23"/>
+      <c r="I17" s="23"/>
+      <c r="J17" s="23"/>
+      <c r="K17" s="23"/>
+      <c r="L17" s="23"/>
+      <c r="M17" s="23"/>
+      <c r="N17" s="23"/>
+      <c r="O17" s="25"/>
+      <c r="P17" s="25"/>
+      <c r="Q17" s="26" t="str">
         <f aca="false">IF(V17="Defect","",IF(COUNT(G17:K17)&lt;5,"",ROUND(G17*Config!$B$4+H17*Config!$B$5+I17*Config!$B$6+J17*Config!$B$7+K17*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R17" s="25" t="str">
+      <c r="R17" s="26" t="str">
         <f aca="false">IF(L17="","",VLOOKUP(L17,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S17" s="25" t="str">
+      <c r="S17" s="26" t="str">
         <f aca="false">IF(N17="","",VLOOKUP(N17,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T17" s="26" t="str">
+      <c r="T17" s="27" t="str">
         <f aca="false">IF(V17="Defect",IF(OR(X17="",G17="",R17=""),"",ROUND(MIN(100,VLOOKUP(X17,Config!$G$12:$H$16,2,0)*VLOOKUP(G17,Config!$I$12:$J$16,2,0)*R17),1)),IF(OR(Q17="",R17="",S17="",M17=""),"",ROUND(Q17*R17*S17/M17*20,1)))</f>
         <v/>
       </c>
-      <c r="U17" s="27" t="str">
+      <c r="U17" s="28" t="str">
         <f aca="false">IF(T17="","",RANK(T17,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="20"/>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="22"/>
-      <c r="H18" s="22"/>
-      <c r="I18" s="22"/>
-      <c r="J18" s="22"/>
-      <c r="K18" s="22"/>
-      <c r="L18" s="22"/>
-      <c r="M18" s="22"/>
-      <c r="N18" s="22"/>
-      <c r="O18" s="24"/>
-      <c r="P18" s="24"/>
-      <c r="Q18" s="25" t="str">
+    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="21"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="21"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="23"/>
+      <c r="H18" s="23"/>
+      <c r="I18" s="23"/>
+      <c r="J18" s="23"/>
+      <c r="K18" s="23"/>
+      <c r="L18" s="23"/>
+      <c r="M18" s="23"/>
+      <c r="N18" s="23"/>
+      <c r="O18" s="25"/>
+      <c r="P18" s="25"/>
+      <c r="Q18" s="26" t="str">
         <f aca="false">IF(V18="Defect","",IF(COUNT(G18:K18)&lt;5,"",ROUND(G18*Config!$B$4+H18*Config!$B$5+I18*Config!$B$6+J18*Config!$B$7+K18*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R18" s="25" t="str">
+      <c r="R18" s="26" t="str">
         <f aca="false">IF(L18="","",VLOOKUP(L18,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S18" s="25" t="str">
+      <c r="S18" s="26" t="str">
         <f aca="false">IF(N18="","",VLOOKUP(N18,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T18" s="26" t="str">
+      <c r="T18" s="27" t="str">
         <f aca="false">IF(V18="Defect",IF(OR(X18="",G18="",R18=""),"",ROUND(MIN(100,VLOOKUP(X18,Config!$G$12:$H$16,2,0)*VLOOKUP(G18,Config!$I$12:$J$16,2,0)*R18),1)),IF(OR(Q18="",R18="",S18="",M18=""),"",ROUND(Q18*R18*S18/M18*20,1)))</f>
         <v/>
       </c>
-      <c r="U18" s="27" t="str">
+      <c r="U18" s="28" t="str">
         <f aca="false">IF(T18="","",RANK(T18,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="20"/>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="22"/>
-      <c r="I19" s="22"/>
-      <c r="J19" s="22"/>
-      <c r="K19" s="22"/>
-      <c r="L19" s="22"/>
-      <c r="M19" s="22"/>
-      <c r="N19" s="22"/>
-      <c r="O19" s="24"/>
-      <c r="P19" s="24"/>
-      <c r="Q19" s="25" t="str">
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="21"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="23"/>
+      <c r="H19" s="23"/>
+      <c r="I19" s="23"/>
+      <c r="J19" s="23"/>
+      <c r="K19" s="23"/>
+      <c r="L19" s="23"/>
+      <c r="M19" s="23"/>
+      <c r="N19" s="23"/>
+      <c r="O19" s="25"/>
+      <c r="P19" s="25"/>
+      <c r="Q19" s="26" t="str">
         <f aca="false">IF(V19="Defect","",IF(COUNT(G19:K19)&lt;5,"",ROUND(G19*Config!$B$4+H19*Config!$B$5+I19*Config!$B$6+J19*Config!$B$7+K19*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R19" s="25" t="str">
+      <c r="R19" s="26" t="str">
         <f aca="false">IF(L19="","",VLOOKUP(L19,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S19" s="25" t="str">
+      <c r="S19" s="26" t="str">
         <f aca="false">IF(N19="","",VLOOKUP(N19,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T19" s="26" t="str">
+      <c r="T19" s="27" t="str">
         <f aca="false">IF(V19="Defect",IF(OR(X19="",G19="",R19=""),"",ROUND(MIN(100,VLOOKUP(X19,Config!$G$12:$H$16,2,0)*VLOOKUP(G19,Config!$I$12:$J$16,2,0)*R19),1)),IF(OR(Q19="",R19="",S19="",M19=""),"",ROUND(Q19*R19*S19/M19*20,1)))</f>
         <v/>
       </c>
-      <c r="U19" s="27" t="str">
+      <c r="U19" s="28" t="str">
         <f aca="false">IF(T19="","",RANK(T19,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="20"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="20"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="22"/>
-      <c r="I20" s="22"/>
-      <c r="J20" s="22"/>
-      <c r="K20" s="22"/>
-      <c r="L20" s="22"/>
-      <c r="M20" s="22"/>
-      <c r="N20" s="22"/>
-      <c r="O20" s="24"/>
-      <c r="P20" s="24"/>
-      <c r="Q20" s="25" t="str">
+    <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="21"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="21"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="23"/>
+      <c r="I20" s="23"/>
+      <c r="J20" s="23"/>
+      <c r="K20" s="23"/>
+      <c r="L20" s="23"/>
+      <c r="M20" s="23"/>
+      <c r="N20" s="23"/>
+      <c r="O20" s="25"/>
+      <c r="P20" s="25"/>
+      <c r="Q20" s="26" t="str">
         <f aca="false">IF(V20="Defect","",IF(COUNT(G20:K20)&lt;5,"",ROUND(G20*Config!$B$4+H20*Config!$B$5+I20*Config!$B$6+J20*Config!$B$7+K20*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R20" s="25" t="str">
+      <c r="R20" s="26" t="str">
         <f aca="false">IF(L20="","",VLOOKUP(L20,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S20" s="25" t="str">
+      <c r="S20" s="26" t="str">
         <f aca="false">IF(N20="","",VLOOKUP(N20,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T20" s="26" t="str">
+      <c r="T20" s="27" t="str">
         <f aca="false">IF(V20="Defect",IF(OR(X20="",G20="",R20=""),"",ROUND(MIN(100,VLOOKUP(X20,Config!$G$12:$H$16,2,0)*VLOOKUP(G20,Config!$I$12:$J$16,2,0)*R20),1)),IF(OR(Q20="",R20="",S20="",M20=""),"",ROUND(Q20*R20*S20/M20*20,1)))</f>
         <v/>
       </c>
-      <c r="U20" s="27" t="str">
+      <c r="U20" s="28" t="str">
         <f aca="false">IF(T20="","",RANK(T20,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="20"/>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
-      <c r="E21" s="20"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="22"/>
-      <c r="I21" s="22"/>
-      <c r="J21" s="22"/>
-      <c r="K21" s="22"/>
-      <c r="L21" s="22"/>
-      <c r="M21" s="22"/>
-      <c r="N21" s="22"/>
-      <c r="O21" s="24"/>
-      <c r="P21" s="24"/>
-      <c r="Q21" s="25" t="str">
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="21"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="21"/>
+      <c r="D21" s="21"/>
+      <c r="E21" s="21"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="23"/>
+      <c r="H21" s="23"/>
+      <c r="I21" s="23"/>
+      <c r="J21" s="23"/>
+      <c r="K21" s="23"/>
+      <c r="L21" s="23"/>
+      <c r="M21" s="23"/>
+      <c r="N21" s="23"/>
+      <c r="O21" s="25"/>
+      <c r="P21" s="25"/>
+      <c r="Q21" s="26" t="str">
         <f aca="false">IF(V21="Defect","",IF(COUNT(G21:K21)&lt;5,"",ROUND(G21*Config!$B$4+H21*Config!$B$5+I21*Config!$B$6+J21*Config!$B$7+K21*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R21" s="25" t="str">
+      <c r="R21" s="26" t="str">
         <f aca="false">IF(L21="","",VLOOKUP(L21,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S21" s="25" t="str">
+      <c r="S21" s="26" t="str">
         <f aca="false">IF(N21="","",VLOOKUP(N21,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T21" s="26" t="str">
+      <c r="T21" s="27" t="str">
         <f aca="false">IF(V21="Defect",IF(OR(X21="",G21="",R21=""),"",ROUND(MIN(100,VLOOKUP(X21,Config!$G$12:$H$16,2,0)*VLOOKUP(G21,Config!$I$12:$J$16,2,0)*R21),1)),IF(OR(Q21="",R21="",S21="",M21=""),"",ROUND(Q21*R21*S21/M21*20,1)))</f>
         <v/>
       </c>
-      <c r="U21" s="27" t="str">
+      <c r="U21" s="28" t="str">
         <f aca="false">IF(T21="","",RANK(T21,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="20"/>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="20"/>
-      <c r="E22" s="20"/>
-      <c r="F22" s="20"/>
-      <c r="G22" s="22"/>
-      <c r="H22" s="22"/>
-      <c r="I22" s="22"/>
-      <c r="J22" s="22"/>
-      <c r="K22" s="22"/>
-      <c r="L22" s="22"/>
-      <c r="M22" s="22"/>
-      <c r="N22" s="22"/>
-      <c r="O22" s="24"/>
-      <c r="P22" s="24"/>
-      <c r="Q22" s="25" t="str">
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="21"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="21"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="21"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="23"/>
+      <c r="H22" s="23"/>
+      <c r="I22" s="23"/>
+      <c r="J22" s="23"/>
+      <c r="K22" s="23"/>
+      <c r="L22" s="23"/>
+      <c r="M22" s="23"/>
+      <c r="N22" s="23"/>
+      <c r="O22" s="25"/>
+      <c r="P22" s="25"/>
+      <c r="Q22" s="26" t="str">
         <f aca="false">IF(V22="Defect","",IF(COUNT(G22:K22)&lt;5,"",ROUND(G22*Config!$B$4+H22*Config!$B$5+I22*Config!$B$6+J22*Config!$B$7+K22*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R22" s="25" t="str">
+      <c r="R22" s="26" t="str">
         <f aca="false">IF(L22="","",VLOOKUP(L22,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S22" s="25" t="str">
+      <c r="S22" s="26" t="str">
         <f aca="false">IF(N22="","",VLOOKUP(N22,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T22" s="26" t="str">
+      <c r="T22" s="27" t="str">
         <f aca="false">IF(V22="Defect",IF(OR(X22="",G22="",R22=""),"",ROUND(MIN(100,VLOOKUP(X22,Config!$G$12:$H$16,2,0)*VLOOKUP(G22,Config!$I$12:$J$16,2,0)*R22),1)),IF(OR(Q22="",R22="",S22="",M22=""),"",ROUND(Q22*R22*S22/M22*20,1)))</f>
         <v/>
       </c>
-      <c r="U22" s="27" t="str">
+      <c r="U22" s="28" t="str">
         <f aca="false">IF(T22="","",RANK(T22,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="20"/>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="20"/>
-      <c r="F23" s="20"/>
-      <c r="G23" s="22"/>
-      <c r="H23" s="22"/>
-      <c r="I23" s="22"/>
-      <c r="J23" s="22"/>
-      <c r="K23" s="22"/>
-      <c r="L23" s="22"/>
-      <c r="M23" s="22"/>
-      <c r="N23" s="22"/>
-      <c r="O23" s="24"/>
-      <c r="P23" s="24"/>
-      <c r="Q23" s="25" t="str">
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="21"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="23"/>
+      <c r="H23" s="23"/>
+      <c r="I23" s="23"/>
+      <c r="J23" s="23"/>
+      <c r="K23" s="23"/>
+      <c r="L23" s="23"/>
+      <c r="M23" s="23"/>
+      <c r="N23" s="23"/>
+      <c r="O23" s="25"/>
+      <c r="P23" s="25"/>
+      <c r="Q23" s="26" t="str">
         <f aca="false">IF(V23="Defect","",IF(COUNT(G23:K23)&lt;5,"",ROUND(G23*Config!$B$4+H23*Config!$B$5+I23*Config!$B$6+J23*Config!$B$7+K23*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R23" s="25" t="str">
+      <c r="R23" s="26" t="str">
         <f aca="false">IF(L23="","",VLOOKUP(L23,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S23" s="25" t="str">
+      <c r="S23" s="26" t="str">
         <f aca="false">IF(N23="","",VLOOKUP(N23,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T23" s="26" t="str">
+      <c r="T23" s="27" t="str">
         <f aca="false">IF(V23="Defect",IF(OR(X23="",G23="",R23=""),"",ROUND(MIN(100,VLOOKUP(X23,Config!$G$12:$H$16,2,0)*VLOOKUP(G23,Config!$I$12:$J$16,2,0)*R23),1)),IF(OR(Q23="",R23="",S23="",M23=""),"",ROUND(Q23*R23*S23/M23*20,1)))</f>
         <v/>
       </c>
-      <c r="U23" s="27" t="str">
+      <c r="U23" s="28" t="str">
         <f aca="false">IF(T23="","",RANK(T23,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="20"/>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="20"/>
-      <c r="E24" s="20"/>
-      <c r="F24" s="20"/>
-      <c r="G24" s="22"/>
-      <c r="H24" s="22"/>
-      <c r="I24" s="22"/>
-      <c r="J24" s="22"/>
-      <c r="K24" s="22"/>
-      <c r="L24" s="22"/>
-      <c r="M24" s="22"/>
-      <c r="N24" s="22"/>
-      <c r="O24" s="24"/>
-      <c r="P24" s="24"/>
-      <c r="Q24" s="25" t="str">
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="21"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="21"/>
+      <c r="D24" s="21"/>
+      <c r="E24" s="21"/>
+      <c r="F24" s="21"/>
+      <c r="G24" s="23"/>
+      <c r="H24" s="23"/>
+      <c r="I24" s="23"/>
+      <c r="J24" s="23"/>
+      <c r="K24" s="23"/>
+      <c r="L24" s="23"/>
+      <c r="M24" s="23"/>
+      <c r="N24" s="23"/>
+      <c r="O24" s="25"/>
+      <c r="P24" s="25"/>
+      <c r="Q24" s="26" t="str">
         <f aca="false">IF(V24="Defect","",IF(COUNT(G24:K24)&lt;5,"",ROUND(G24*Config!$B$4+H24*Config!$B$5+I24*Config!$B$6+J24*Config!$B$7+K24*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R24" s="25" t="str">
+      <c r="R24" s="26" t="str">
         <f aca="false">IF(L24="","",VLOOKUP(L24,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S24" s="25" t="str">
+      <c r="S24" s="26" t="str">
         <f aca="false">IF(N24="","",VLOOKUP(N24,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T24" s="26" t="str">
+      <c r="T24" s="27" t="str">
         <f aca="false">IF(V24="Defect",IF(OR(X24="",G24="",R24=""),"",ROUND(MIN(100,VLOOKUP(X24,Config!$G$12:$H$16,2,0)*VLOOKUP(G24,Config!$I$12:$J$16,2,0)*R24),1)),IF(OR(Q24="",R24="",S24="",M24=""),"",ROUND(Q24*R24*S24/M24*20,1)))</f>
         <v/>
       </c>
-      <c r="U24" s="27" t="str">
+      <c r="U24" s="28" t="str">
         <f aca="false">IF(T24="","",RANK(T24,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="20"/>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="20"/>
-      <c r="G25" s="22"/>
-      <c r="H25" s="22"/>
-      <c r="I25" s="22"/>
-      <c r="J25" s="22"/>
-      <c r="K25" s="22"/>
-      <c r="L25" s="22"/>
-      <c r="M25" s="22"/>
-      <c r="N25" s="22"/>
-      <c r="O25" s="24"/>
-      <c r="P25" s="24"/>
-      <c r="Q25" s="25" t="str">
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="21"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="21"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="21"/>
+      <c r="G25" s="23"/>
+      <c r="H25" s="23"/>
+      <c r="I25" s="23"/>
+      <c r="J25" s="23"/>
+      <c r="K25" s="23"/>
+      <c r="L25" s="23"/>
+      <c r="M25" s="23"/>
+      <c r="N25" s="23"/>
+      <c r="O25" s="25"/>
+      <c r="P25" s="25"/>
+      <c r="Q25" s="26" t="str">
         <f aca="false">IF(V25="Defect","",IF(COUNT(G25:K25)&lt;5,"",ROUND(G25*Config!$B$4+H25*Config!$B$5+I25*Config!$B$6+J25*Config!$B$7+K25*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R25" s="25" t="str">
+      <c r="R25" s="26" t="str">
         <f aca="false">IF(L25="","",VLOOKUP(L25,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S25" s="25" t="str">
+      <c r="S25" s="26" t="str">
         <f aca="false">IF(N25="","",VLOOKUP(N25,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T25" s="26" t="str">
+      <c r="T25" s="27" t="str">
         <f aca="false">IF(V25="Defect",IF(OR(X25="",G25="",R25=""),"",ROUND(MIN(100,VLOOKUP(X25,Config!$G$12:$H$16,2,0)*VLOOKUP(G25,Config!$I$12:$J$16,2,0)*R25),1)),IF(OR(Q25="",R25="",S25="",M25=""),"",ROUND(Q25*R25*S25/M25*20,1)))</f>
         <v/>
       </c>
-      <c r="U25" s="27" t="str">
+      <c r="U25" s="28" t="str">
         <f aca="false">IF(T25="","",RANK(T25,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="20"/>
-      <c r="B26" s="20"/>
-      <c r="C26" s="20"/>
-      <c r="D26" s="20"/>
-      <c r="E26" s="20"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="22"/>
-      <c r="H26" s="22"/>
-      <c r="I26" s="22"/>
-      <c r="J26" s="22"/>
-      <c r="K26" s="22"/>
-      <c r="L26" s="22"/>
-      <c r="M26" s="22"/>
-      <c r="N26" s="22"/>
-      <c r="O26" s="24"/>
-      <c r="P26" s="24"/>
-      <c r="Q26" s="25" t="str">
+    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="21"/>
+      <c r="B26" s="21"/>
+      <c r="C26" s="21"/>
+      <c r="D26" s="21"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="21"/>
+      <c r="G26" s="23"/>
+      <c r="H26" s="23"/>
+      <c r="I26" s="23"/>
+      <c r="J26" s="23"/>
+      <c r="K26" s="23"/>
+      <c r="L26" s="23"/>
+      <c r="M26" s="23"/>
+      <c r="N26" s="23"/>
+      <c r="O26" s="25"/>
+      <c r="P26" s="25"/>
+      <c r="Q26" s="26" t="str">
         <f aca="false">IF(V26="Defect","",IF(COUNT(G26:K26)&lt;5,"",ROUND(G26*Config!$B$4+H26*Config!$B$5+I26*Config!$B$6+J26*Config!$B$7+K26*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R26" s="25" t="str">
+      <c r="R26" s="26" t="str">
         <f aca="false">IF(L26="","",VLOOKUP(L26,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S26" s="25" t="str">
+      <c r="S26" s="26" t="str">
         <f aca="false">IF(N26="","",VLOOKUP(N26,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T26" s="26" t="str">
+      <c r="T26" s="27" t="str">
         <f aca="false">IF(V26="Defect",IF(OR(X26="",G26="",R26=""),"",ROUND(MIN(100,VLOOKUP(X26,Config!$G$12:$H$16,2,0)*VLOOKUP(G26,Config!$I$12:$J$16,2,0)*R26),1)),IF(OR(Q26="",R26="",S26="",M26=""),"",ROUND(Q26*R26*S26/M26*20,1)))</f>
         <v/>
       </c>
-      <c r="U26" s="27" t="str">
+      <c r="U26" s="28" t="str">
         <f aca="false">IF(T26="","",RANK(T26,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="20"/>
-      <c r="B27" s="20"/>
-      <c r="C27" s="20"/>
-      <c r="D27" s="20"/>
-      <c r="E27" s="20"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="22"/>
-      <c r="H27" s="22"/>
-      <c r="I27" s="22"/>
-      <c r="J27" s="22"/>
-      <c r="K27" s="22"/>
-      <c r="L27" s="22"/>
-      <c r="M27" s="22"/>
-      <c r="N27" s="22"/>
-      <c r="O27" s="24"/>
-      <c r="P27" s="24"/>
-      <c r="Q27" s="25" t="str">
+    <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="21"/>
+      <c r="B27" s="21"/>
+      <c r="C27" s="21"/>
+      <c r="D27" s="21"/>
+      <c r="E27" s="21"/>
+      <c r="F27" s="21"/>
+      <c r="G27" s="23"/>
+      <c r="H27" s="23"/>
+      <c r="I27" s="23"/>
+      <c r="J27" s="23"/>
+      <c r="K27" s="23"/>
+      <c r="L27" s="23"/>
+      <c r="M27" s="23"/>
+      <c r="N27" s="23"/>
+      <c r="O27" s="25"/>
+      <c r="P27" s="25"/>
+      <c r="Q27" s="26" t="str">
         <f aca="false">IF(V27="Defect","",IF(COUNT(G27:K27)&lt;5,"",ROUND(G27*Config!$B$4+H27*Config!$B$5+I27*Config!$B$6+J27*Config!$B$7+K27*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R27" s="25" t="str">
+      <c r="R27" s="26" t="str">
         <f aca="false">IF(L27="","",VLOOKUP(L27,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S27" s="25" t="str">
+      <c r="S27" s="26" t="str">
         <f aca="false">IF(N27="","",VLOOKUP(N27,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T27" s="26" t="str">
+      <c r="T27" s="27" t="str">
         <f aca="false">IF(V27="Defect",IF(OR(X27="",G27="",R27=""),"",ROUND(MIN(100,VLOOKUP(X27,Config!$G$12:$H$16,2,0)*VLOOKUP(G27,Config!$I$12:$J$16,2,0)*R27),1)),IF(OR(Q27="",R27="",S27="",M27=""),"",ROUND(Q27*R27*S27/M27*20,1)))</f>
         <v/>
       </c>
-      <c r="U27" s="27" t="str">
+      <c r="U27" s="28" t="str">
         <f aca="false">IF(T27="","",RANK(T27,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="20"/>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="20"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="20"/>
-      <c r="G28" s="22"/>
-      <c r="H28" s="22"/>
-      <c r="I28" s="22"/>
-      <c r="J28" s="22"/>
-      <c r="K28" s="22"/>
-      <c r="L28" s="22"/>
-      <c r="M28" s="22"/>
-      <c r="N28" s="22"/>
-      <c r="O28" s="24"/>
-      <c r="P28" s="24"/>
-      <c r="Q28" s="25" t="str">
+    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="21"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="23"/>
+      <c r="H28" s="23"/>
+      <c r="I28" s="23"/>
+      <c r="J28" s="23"/>
+      <c r="K28" s="23"/>
+      <c r="L28" s="23"/>
+      <c r="M28" s="23"/>
+      <c r="N28" s="23"/>
+      <c r="O28" s="25"/>
+      <c r="P28" s="25"/>
+      <c r="Q28" s="26" t="str">
         <f aca="false">IF(V28="Defect","",IF(COUNT(G28:K28)&lt;5,"",ROUND(G28*Config!$B$4+H28*Config!$B$5+I28*Config!$B$6+J28*Config!$B$7+K28*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R28" s="25" t="str">
+      <c r="R28" s="26" t="str">
         <f aca="false">IF(L28="","",VLOOKUP(L28,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S28" s="25" t="str">
+      <c r="S28" s="26" t="str">
         <f aca="false">IF(N28="","",VLOOKUP(N28,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T28" s="26" t="str">
+      <c r="T28" s="27" t="str">
         <f aca="false">IF(V28="Defect",IF(OR(X28="",G28="",R28=""),"",ROUND(MIN(100,VLOOKUP(X28,Config!$G$12:$H$16,2,0)*VLOOKUP(G28,Config!$I$12:$J$16,2,0)*R28),1)),IF(OR(Q28="",R28="",S28="",M28=""),"",ROUND(Q28*R28*S28/M28*20,1)))</f>
         <v/>
       </c>
-      <c r="U28" s="27" t="str">
+      <c r="U28" s="28" t="str">
         <f aca="false">IF(T28="","",RANK(T28,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="20"/>
-      <c r="B29" s="20"/>
-      <c r="C29" s="20"/>
-      <c r="D29" s="20"/>
-      <c r="E29" s="20"/>
-      <c r="F29" s="20"/>
-      <c r="G29" s="22"/>
-      <c r="H29" s="22"/>
-      <c r="I29" s="22"/>
-      <c r="J29" s="22"/>
-      <c r="K29" s="22"/>
-      <c r="L29" s="22"/>
-      <c r="M29" s="22"/>
-      <c r="N29" s="22"/>
-      <c r="O29" s="24"/>
-      <c r="P29" s="24"/>
-      <c r="Q29" s="25" t="str">
+    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="21"/>
+      <c r="B29" s="21"/>
+      <c r="C29" s="21"/>
+      <c r="D29" s="21"/>
+      <c r="E29" s="21"/>
+      <c r="F29" s="21"/>
+      <c r="G29" s="23"/>
+      <c r="H29" s="23"/>
+      <c r="I29" s="23"/>
+      <c r="J29" s="23"/>
+      <c r="K29" s="23"/>
+      <c r="L29" s="23"/>
+      <c r="M29" s="23"/>
+      <c r="N29" s="23"/>
+      <c r="O29" s="25"/>
+      <c r="P29" s="25"/>
+      <c r="Q29" s="26" t="str">
         <f aca="false">IF(V29="Defect","",IF(COUNT(G29:K29)&lt;5,"",ROUND(G29*Config!$B$4+H29*Config!$B$5+I29*Config!$B$6+J29*Config!$B$7+K29*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R29" s="25" t="str">
+      <c r="R29" s="26" t="str">
         <f aca="false">IF(L29="","",VLOOKUP(L29,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S29" s="25" t="str">
+      <c r="S29" s="26" t="str">
         <f aca="false">IF(N29="","",VLOOKUP(N29,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T29" s="26" t="str">
+      <c r="T29" s="27" t="str">
         <f aca="false">IF(V29="Defect",IF(OR(X29="",G29="",R29=""),"",ROUND(MIN(100,VLOOKUP(X29,Config!$G$12:$H$16,2,0)*VLOOKUP(G29,Config!$I$12:$J$16,2,0)*R29),1)),IF(OR(Q29="",R29="",S29="",M29=""),"",ROUND(Q29*R29*S29/M29*20,1)))</f>
         <v/>
       </c>
-      <c r="U29" s="27" t="str">
+      <c r="U29" s="28" t="str">
         <f aca="false">IF(T29="","",RANK(T29,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="20"/>
-      <c r="B30" s="20"/>
-      <c r="C30" s="20"/>
-      <c r="D30" s="20"/>
-      <c r="E30" s="20"/>
-      <c r="F30" s="20"/>
-      <c r="G30" s="22"/>
-      <c r="H30" s="22"/>
-      <c r="I30" s="22"/>
-      <c r="J30" s="22"/>
-      <c r="K30" s="22"/>
-      <c r="L30" s="22"/>
-      <c r="M30" s="22"/>
-      <c r="N30" s="22"/>
-      <c r="O30" s="24"/>
-      <c r="P30" s="24"/>
-      <c r="Q30" s="25" t="str">
+    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="21"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="21"/>
+      <c r="D30" s="21"/>
+      <c r="E30" s="21"/>
+      <c r="F30" s="21"/>
+      <c r="G30" s="23"/>
+      <c r="H30" s="23"/>
+      <c r="I30" s="23"/>
+      <c r="J30" s="23"/>
+      <c r="K30" s="23"/>
+      <c r="L30" s="23"/>
+      <c r="M30" s="23"/>
+      <c r="N30" s="23"/>
+      <c r="O30" s="25"/>
+      <c r="P30" s="25"/>
+      <c r="Q30" s="26" t="str">
         <f aca="false">IF(V30="Defect","",IF(COUNT(G30:K30)&lt;5,"",ROUND(G30*Config!$B$4+H30*Config!$B$5+I30*Config!$B$6+J30*Config!$B$7+K30*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R30" s="25" t="str">
+      <c r="R30" s="26" t="str">
         <f aca="false">IF(L30="","",VLOOKUP(L30,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S30" s="25" t="str">
+      <c r="S30" s="26" t="str">
         <f aca="false">IF(N30="","",VLOOKUP(N30,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T30" s="26" t="str">
+      <c r="T30" s="27" t="str">
         <f aca="false">IF(V30="Defect",IF(OR(X30="",G30="",R30=""),"",ROUND(MIN(100,VLOOKUP(X30,Config!$G$12:$H$16,2,0)*VLOOKUP(G30,Config!$I$12:$J$16,2,0)*R30),1)),IF(OR(Q30="",R30="",S30="",M30=""),"",ROUND(Q30*R30*S30/M30*20,1)))</f>
         <v/>
       </c>
-      <c r="U30" s="27" t="str">
+      <c r="U30" s="28" t="str">
         <f aca="false">IF(T30="","",RANK(T30,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="20"/>
-      <c r="B31" s="20"/>
-      <c r="C31" s="20"/>
-      <c r="D31" s="20"/>
-      <c r="E31" s="20"/>
-      <c r="F31" s="20"/>
-      <c r="G31" s="22"/>
-      <c r="H31" s="22"/>
-      <c r="I31" s="22"/>
-      <c r="J31" s="22"/>
-      <c r="K31" s="22"/>
-      <c r="L31" s="22"/>
-      <c r="M31" s="22"/>
-      <c r="N31" s="22"/>
-      <c r="O31" s="24"/>
-      <c r="P31" s="24"/>
-      <c r="Q31" s="25" t="str">
+    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="21"/>
+      <c r="B31" s="21"/>
+      <c r="C31" s="21"/>
+      <c r="D31" s="21"/>
+      <c r="E31" s="21"/>
+      <c r="F31" s="21"/>
+      <c r="G31" s="23"/>
+      <c r="H31" s="23"/>
+      <c r="I31" s="23"/>
+      <c r="J31" s="23"/>
+      <c r="K31" s="23"/>
+      <c r="L31" s="23"/>
+      <c r="M31" s="23"/>
+      <c r="N31" s="23"/>
+      <c r="O31" s="25"/>
+      <c r="P31" s="25"/>
+      <c r="Q31" s="26" t="str">
         <f aca="false">IF(V31="Defect","",IF(COUNT(G31:K31)&lt;5,"",ROUND(G31*Config!$B$4+H31*Config!$B$5+I31*Config!$B$6+J31*Config!$B$7+K31*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R31" s="25" t="str">
+      <c r="R31" s="26" t="str">
         <f aca="false">IF(L31="","",VLOOKUP(L31,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S31" s="25" t="str">
+      <c r="S31" s="26" t="str">
         <f aca="false">IF(N31="","",VLOOKUP(N31,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T31" s="26" t="str">
+      <c r="T31" s="27" t="str">
         <f aca="false">IF(V31="Defect",IF(OR(X31="",G31="",R31=""),"",ROUND(MIN(100,VLOOKUP(X31,Config!$G$12:$H$16,2,0)*VLOOKUP(G31,Config!$I$12:$J$16,2,0)*R31),1)),IF(OR(Q31="",R31="",S31="",M31=""),"",ROUND(Q31*R31*S31/M31*20,1)))</f>
         <v/>
       </c>
-      <c r="U31" s="27" t="str">
+      <c r="U31" s="28" t="str">
         <f aca="false">IF(T31="","",RANK(T31,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="20"/>
-      <c r="B32" s="20"/>
-      <c r="C32" s="20"/>
-      <c r="D32" s="20"/>
-      <c r="E32" s="20"/>
-      <c r="F32" s="20"/>
-      <c r="G32" s="22"/>
-      <c r="H32" s="22"/>
-      <c r="I32" s="22"/>
-      <c r="J32" s="22"/>
-      <c r="K32" s="22"/>
-      <c r="L32" s="22"/>
-      <c r="M32" s="22"/>
-      <c r="N32" s="22"/>
-      <c r="O32" s="24"/>
-      <c r="P32" s="24"/>
-      <c r="Q32" s="25" t="str">
+    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="21"/>
+      <c r="B32" s="21"/>
+      <c r="C32" s="21"/>
+      <c r="D32" s="21"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="21"/>
+      <c r="G32" s="23"/>
+      <c r="H32" s="23"/>
+      <c r="I32" s="23"/>
+      <c r="J32" s="23"/>
+      <c r="K32" s="23"/>
+      <c r="L32" s="23"/>
+      <c r="M32" s="23"/>
+      <c r="N32" s="23"/>
+      <c r="O32" s="25"/>
+      <c r="P32" s="25"/>
+      <c r="Q32" s="26" t="str">
         <f aca="false">IF(V32="Defect","",IF(COUNT(G32:K32)&lt;5,"",ROUND(G32*Config!$B$4+H32*Config!$B$5+I32*Config!$B$6+J32*Config!$B$7+K32*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R32" s="25" t="str">
+      <c r="R32" s="26" t="str">
         <f aca="false">IF(L32="","",VLOOKUP(L32,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S32" s="25" t="str">
+      <c r="S32" s="26" t="str">
         <f aca="false">IF(N32="","",VLOOKUP(N32,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T32" s="26" t="str">
+      <c r="T32" s="27" t="str">
         <f aca="false">IF(V32="Defect",IF(OR(X32="",G32="",R32=""),"",ROUND(MIN(100,VLOOKUP(X32,Config!$G$12:$H$16,2,0)*VLOOKUP(G32,Config!$I$12:$J$16,2,0)*R32),1)),IF(OR(Q32="",R32="",S32="",M32=""),"",ROUND(Q32*R32*S32/M32*20,1)))</f>
         <v/>
       </c>
-      <c r="U32" s="27" t="str">
+      <c r="U32" s="28" t="str">
         <f aca="false">IF(T32="","",RANK(T32,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="20"/>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
-      <c r="D33" s="20"/>
-      <c r="E33" s="20"/>
-      <c r="F33" s="20"/>
-      <c r="G33" s="22"/>
-      <c r="H33" s="22"/>
-      <c r="I33" s="22"/>
-      <c r="J33" s="22"/>
-      <c r="K33" s="22"/>
-      <c r="L33" s="22"/>
-      <c r="M33" s="22"/>
-      <c r="N33" s="22"/>
-      <c r="O33" s="24"/>
-      <c r="P33" s="24"/>
-      <c r="Q33" s="25" t="str">
+    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="21"/>
+      <c r="B33" s="21"/>
+      <c r="C33" s="21"/>
+      <c r="D33" s="21"/>
+      <c r="E33" s="21"/>
+      <c r="F33" s="21"/>
+      <c r="G33" s="23"/>
+      <c r="H33" s="23"/>
+      <c r="I33" s="23"/>
+      <c r="J33" s="23"/>
+      <c r="K33" s="23"/>
+      <c r="L33" s="23"/>
+      <c r="M33" s="23"/>
+      <c r="N33" s="23"/>
+      <c r="O33" s="25"/>
+      <c r="P33" s="25"/>
+      <c r="Q33" s="26" t="str">
         <f aca="false">IF(V33="Defect","",IF(COUNT(G33:K33)&lt;5,"",ROUND(G33*Config!$B$4+H33*Config!$B$5+I33*Config!$B$6+J33*Config!$B$7+K33*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R33" s="25" t="str">
+      <c r="R33" s="26" t="str">
         <f aca="false">IF(L33="","",VLOOKUP(L33,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S33" s="25" t="str">
+      <c r="S33" s="26" t="str">
         <f aca="false">IF(N33="","",VLOOKUP(N33,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T33" s="26" t="str">
+      <c r="T33" s="27" t="str">
         <f aca="false">IF(V33="Defect",IF(OR(X33="",G33="",R33=""),"",ROUND(MIN(100,VLOOKUP(X33,Config!$G$12:$H$16,2,0)*VLOOKUP(G33,Config!$I$12:$J$16,2,0)*R33),1)),IF(OR(Q33="",R33="",S33="",M33=""),"",ROUND(Q33*R33*S33/M33*20,1)))</f>
         <v/>
       </c>
-      <c r="U33" s="27" t="str">
+      <c r="U33" s="28" t="str">
         <f aca="false">IF(T33="","",RANK(T33,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="20"/>
-      <c r="B34" s="20"/>
-      <c r="C34" s="20"/>
-      <c r="D34" s="20"/>
-      <c r="E34" s="20"/>
-      <c r="F34" s="20"/>
-      <c r="G34" s="22"/>
-      <c r="H34" s="22"/>
-      <c r="I34" s="22"/>
-      <c r="J34" s="22"/>
-      <c r="K34" s="22"/>
-      <c r="L34" s="22"/>
-      <c r="M34" s="22"/>
-      <c r="N34" s="22"/>
-      <c r="O34" s="24"/>
-      <c r="P34" s="24"/>
-      <c r="Q34" s="25" t="str">
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="21"/>
+      <c r="B34" s="21"/>
+      <c r="C34" s="21"/>
+      <c r="D34" s="21"/>
+      <c r="E34" s="21"/>
+      <c r="F34" s="21"/>
+      <c r="G34" s="23"/>
+      <c r="H34" s="23"/>
+      <c r="I34" s="23"/>
+      <c r="J34" s="23"/>
+      <c r="K34" s="23"/>
+      <c r="L34" s="23"/>
+      <c r="M34" s="23"/>
+      <c r="N34" s="23"/>
+      <c r="O34" s="25"/>
+      <c r="P34" s="25"/>
+      <c r="Q34" s="26" t="str">
         <f aca="false">IF(V34="Defect","",IF(COUNT(G34:K34)&lt;5,"",ROUND(G34*Config!$B$4+H34*Config!$B$5+I34*Config!$B$6+J34*Config!$B$7+K34*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R34" s="25" t="str">
+      <c r="R34" s="26" t="str">
         <f aca="false">IF(L34="","",VLOOKUP(L34,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S34" s="25" t="str">
+      <c r="S34" s="26" t="str">
         <f aca="false">IF(N34="","",VLOOKUP(N34,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T34" s="26" t="str">
+      <c r="T34" s="27" t="str">
         <f aca="false">IF(V34="Defect",IF(OR(X34="",G34="",R34=""),"",ROUND(MIN(100,VLOOKUP(X34,Config!$G$12:$H$16,2,0)*VLOOKUP(G34,Config!$I$12:$J$16,2,0)*R34),1)),IF(OR(Q34="",R34="",S34="",M34=""),"",ROUND(Q34*R34*S34/M34*20,1)))</f>
         <v/>
       </c>
-      <c r="U34" s="27" t="str">
+      <c r="U34" s="28" t="str">
         <f aca="false">IF(T34="","",RANK(T34,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="20"/>
-      <c r="B35" s="20"/>
-      <c r="C35" s="20"/>
-      <c r="D35" s="20"/>
-      <c r="E35" s="20"/>
-      <c r="F35" s="20"/>
-      <c r="G35" s="22"/>
-      <c r="H35" s="22"/>
-      <c r="I35" s="22"/>
-      <c r="J35" s="22"/>
-      <c r="K35" s="22"/>
-      <c r="L35" s="22"/>
-      <c r="M35" s="22"/>
-      <c r="N35" s="22"/>
-      <c r="O35" s="24"/>
-      <c r="P35" s="24"/>
-      <c r="Q35" s="25" t="str">
+    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="21"/>
+      <c r="B35" s="21"/>
+      <c r="C35" s="21"/>
+      <c r="D35" s="21"/>
+      <c r="E35" s="21"/>
+      <c r="F35" s="21"/>
+      <c r="G35" s="23"/>
+      <c r="H35" s="23"/>
+      <c r="I35" s="23"/>
+      <c r="J35" s="23"/>
+      <c r="K35" s="23"/>
+      <c r="L35" s="23"/>
+      <c r="M35" s="23"/>
+      <c r="N35" s="23"/>
+      <c r="O35" s="25"/>
+      <c r="P35" s="25"/>
+      <c r="Q35" s="26" t="str">
         <f aca="false">IF(V35="Defect","",IF(COUNT(G35:K35)&lt;5,"",ROUND(G35*Config!$B$4+H35*Config!$B$5+I35*Config!$B$6+J35*Config!$B$7+K35*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R35" s="25" t="str">
+      <c r="R35" s="26" t="str">
         <f aca="false">IF(L35="","",VLOOKUP(L35,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S35" s="25" t="str">
+      <c r="S35" s="26" t="str">
         <f aca="false">IF(N35="","",VLOOKUP(N35,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T35" s="26" t="str">
+      <c r="T35" s="27" t="str">
         <f aca="false">IF(V35="Defect",IF(OR(X35="",G35="",R35=""),"",ROUND(MIN(100,VLOOKUP(X35,Config!$G$12:$H$16,2,0)*VLOOKUP(G35,Config!$I$12:$J$16,2,0)*R35),1)),IF(OR(Q35="",R35="",S35="",M35=""),"",ROUND(Q35*R35*S35/M35*20,1)))</f>
         <v/>
       </c>
-      <c r="U35" s="27" t="str">
+      <c r="U35" s="28" t="str">
         <f aca="false">IF(T35="","",RANK(T35,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="20"/>
-      <c r="B36" s="20"/>
-      <c r="C36" s="20"/>
-      <c r="D36" s="20"/>
-      <c r="E36" s="20"/>
-      <c r="F36" s="20"/>
-      <c r="G36" s="22"/>
-      <c r="H36" s="22"/>
-      <c r="I36" s="22"/>
-      <c r="J36" s="22"/>
-      <c r="K36" s="22"/>
-      <c r="L36" s="22"/>
-      <c r="M36" s="22"/>
-      <c r="N36" s="22"/>
-      <c r="O36" s="24"/>
-      <c r="P36" s="24"/>
-      <c r="Q36" s="25" t="str">
+    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="21"/>
+      <c r="B36" s="21"/>
+      <c r="C36" s="21"/>
+      <c r="D36" s="21"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="21"/>
+      <c r="G36" s="23"/>
+      <c r="H36" s="23"/>
+      <c r="I36" s="23"/>
+      <c r="J36" s="23"/>
+      <c r="K36" s="23"/>
+      <c r="L36" s="23"/>
+      <c r="M36" s="23"/>
+      <c r="N36" s="23"/>
+      <c r="O36" s="25"/>
+      <c r="P36" s="25"/>
+      <c r="Q36" s="26" t="str">
         <f aca="false">IF(V36="Defect","",IF(COUNT(G36:K36)&lt;5,"",ROUND(G36*Config!$B$4+H36*Config!$B$5+I36*Config!$B$6+J36*Config!$B$7+K36*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R36" s="25" t="str">
+      <c r="R36" s="26" t="str">
         <f aca="false">IF(L36="","",VLOOKUP(L36,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S36" s="25" t="str">
+      <c r="S36" s="26" t="str">
         <f aca="false">IF(N36="","",VLOOKUP(N36,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T36" s="26" t="str">
+      <c r="T36" s="27" t="str">
         <f aca="false">IF(V36="Defect",IF(OR(X36="",G36="",R36=""),"",ROUND(MIN(100,VLOOKUP(X36,Config!$G$12:$H$16,2,0)*VLOOKUP(G36,Config!$I$12:$J$16,2,0)*R36),1)),IF(OR(Q36="",R36="",S36="",M36=""),"",ROUND(Q36*R36*S36/M36*20,1)))</f>
         <v/>
       </c>
-      <c r="U36" s="27" t="str">
+      <c r="U36" s="28" t="str">
         <f aca="false">IF(T36="","",RANK(T36,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="20"/>
-      <c r="B37" s="20"/>
-      <c r="C37" s="20"/>
-      <c r="D37" s="20"/>
-      <c r="E37" s="20"/>
-      <c r="F37" s="20"/>
-      <c r="G37" s="22"/>
-      <c r="H37" s="22"/>
-      <c r="I37" s="22"/>
-      <c r="J37" s="22"/>
-      <c r="K37" s="22"/>
-      <c r="L37" s="22"/>
-      <c r="M37" s="22"/>
-      <c r="N37" s="22"/>
-      <c r="O37" s="24"/>
-      <c r="P37" s="24"/>
-      <c r="Q37" s="25" t="str">
+    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="21"/>
+      <c r="B37" s="21"/>
+      <c r="C37" s="21"/>
+      <c r="D37" s="21"/>
+      <c r="E37" s="21"/>
+      <c r="F37" s="21"/>
+      <c r="G37" s="23"/>
+      <c r="H37" s="23"/>
+      <c r="I37" s="23"/>
+      <c r="J37" s="23"/>
+      <c r="K37" s="23"/>
+      <c r="L37" s="23"/>
+      <c r="M37" s="23"/>
+      <c r="N37" s="23"/>
+      <c r="O37" s="25"/>
+      <c r="P37" s="25"/>
+      <c r="Q37" s="26" t="str">
         <f aca="false">IF(V37="Defect","",IF(COUNT(G37:K37)&lt;5,"",ROUND(G37*Config!$B$4+H37*Config!$B$5+I37*Config!$B$6+J37*Config!$B$7+K37*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R37" s="25" t="str">
+      <c r="R37" s="26" t="str">
         <f aca="false">IF(L37="","",VLOOKUP(L37,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S37" s="25" t="str">
+      <c r="S37" s="26" t="str">
         <f aca="false">IF(N37="","",VLOOKUP(N37,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T37" s="26" t="str">
+      <c r="T37" s="27" t="str">
         <f aca="false">IF(V37="Defect",IF(OR(X37="",G37="",R37=""),"",ROUND(MIN(100,VLOOKUP(X37,Config!$G$12:$H$16,2,0)*VLOOKUP(G37,Config!$I$12:$J$16,2,0)*R37),1)),IF(OR(Q37="",R37="",S37="",M37=""),"",ROUND(Q37*R37*S37/M37*20,1)))</f>
         <v/>
       </c>
-      <c r="U37" s="27" t="str">
+      <c r="U37" s="28" t="str">
         <f aca="false">IF(T37="","",RANK(T37,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="20"/>
-      <c r="B38" s="20"/>
-      <c r="C38" s="20"/>
-      <c r="D38" s="20"/>
-      <c r="E38" s="20"/>
-      <c r="F38" s="20"/>
-      <c r="G38" s="22"/>
-      <c r="H38" s="22"/>
-      <c r="I38" s="22"/>
-      <c r="J38" s="22"/>
-      <c r="K38" s="22"/>
-      <c r="L38" s="22"/>
-      <c r="M38" s="22"/>
-      <c r="N38" s="22"/>
-      <c r="O38" s="24"/>
-      <c r="P38" s="24"/>
-      <c r="Q38" s="25" t="str">
+    <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="21"/>
+      <c r="B38" s="21"/>
+      <c r="C38" s="21"/>
+      <c r="D38" s="21"/>
+      <c r="E38" s="21"/>
+      <c r="F38" s="21"/>
+      <c r="G38" s="23"/>
+      <c r="H38" s="23"/>
+      <c r="I38" s="23"/>
+      <c r="J38" s="23"/>
+      <c r="K38" s="23"/>
+      <c r="L38" s="23"/>
+      <c r="M38" s="23"/>
+      <c r="N38" s="23"/>
+      <c r="O38" s="25"/>
+      <c r="P38" s="25"/>
+      <c r="Q38" s="26" t="str">
         <f aca="false">IF(V38="Defect","",IF(COUNT(G38:K38)&lt;5,"",ROUND(G38*Config!$B$4+H38*Config!$B$5+I38*Config!$B$6+J38*Config!$B$7+K38*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R38" s="25" t="str">
+      <c r="R38" s="26" t="str">
         <f aca="false">IF(L38="","",VLOOKUP(L38,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S38" s="25" t="str">
+      <c r="S38" s="26" t="str">
         <f aca="false">IF(N38="","",VLOOKUP(N38,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T38" s="26" t="str">
+      <c r="T38" s="27" t="str">
         <f aca="false">IF(V38="Defect",IF(OR(X38="",G38="",R38=""),"",ROUND(MIN(100,VLOOKUP(X38,Config!$G$12:$H$16,2,0)*VLOOKUP(G38,Config!$I$12:$J$16,2,0)*R38),1)),IF(OR(Q38="",R38="",S38="",M38=""),"",ROUND(Q38*R38*S38/M38*20,1)))</f>
         <v/>
       </c>
-      <c r="U38" s="27" t="str">
+      <c r="U38" s="28" t="str">
         <f aca="false">IF(T38="","",RANK(T38,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="20"/>
-      <c r="B39" s="20"/>
-      <c r="C39" s="20"/>
-      <c r="D39" s="20"/>
-      <c r="E39" s="20"/>
-      <c r="F39" s="20"/>
-      <c r="G39" s="22"/>
-      <c r="H39" s="22"/>
-      <c r="I39" s="22"/>
-      <c r="J39" s="22"/>
-      <c r="K39" s="22"/>
-      <c r="L39" s="22"/>
-      <c r="M39" s="22"/>
-      <c r="N39" s="22"/>
-      <c r="O39" s="24"/>
-      <c r="P39" s="24"/>
-      <c r="Q39" s="25" t="str">
+    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="21"/>
+      <c r="B39" s="21"/>
+      <c r="C39" s="21"/>
+      <c r="D39" s="21"/>
+      <c r="E39" s="21"/>
+      <c r="F39" s="21"/>
+      <c r="G39" s="23"/>
+      <c r="H39" s="23"/>
+      <c r="I39" s="23"/>
+      <c r="J39" s="23"/>
+      <c r="K39" s="23"/>
+      <c r="L39" s="23"/>
+      <c r="M39" s="23"/>
+      <c r="N39" s="23"/>
+      <c r="O39" s="25"/>
+      <c r="P39" s="25"/>
+      <c r="Q39" s="26" t="str">
         <f aca="false">IF(V39="Defect","",IF(COUNT(G39:K39)&lt;5,"",ROUND(G39*Config!$B$4+H39*Config!$B$5+I39*Config!$B$6+J39*Config!$B$7+K39*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R39" s="25" t="str">
+      <c r="R39" s="26" t="str">
         <f aca="false">IF(L39="","",VLOOKUP(L39,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S39" s="25" t="str">
+      <c r="S39" s="26" t="str">
         <f aca="false">IF(N39="","",VLOOKUP(N39,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T39" s="26" t="str">
+      <c r="T39" s="27" t="str">
         <f aca="false">IF(V39="Defect",IF(OR(X39="",G39="",R39=""),"",ROUND(MIN(100,VLOOKUP(X39,Config!$G$12:$H$16,2,0)*VLOOKUP(G39,Config!$I$12:$J$16,2,0)*R39),1)),IF(OR(Q39="",R39="",S39="",M39=""),"",ROUND(Q39*R39*S39/M39*20,1)))</f>
         <v/>
       </c>
-      <c r="U39" s="27" t="str">
+      <c r="U39" s="28" t="str">
         <f aca="false">IF(T39="","",RANK(T39,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="20"/>
-      <c r="B40" s="20"/>
-      <c r="C40" s="20"/>
-      <c r="D40" s="20"/>
-      <c r="E40" s="20"/>
-      <c r="F40" s="20"/>
-      <c r="G40" s="22"/>
-      <c r="H40" s="22"/>
-      <c r="I40" s="22"/>
-      <c r="J40" s="22"/>
-      <c r="K40" s="22"/>
-      <c r="L40" s="22"/>
-      <c r="M40" s="22"/>
-      <c r="N40" s="22"/>
-      <c r="O40" s="24"/>
-      <c r="P40" s="24"/>
-      <c r="Q40" s="25" t="str">
+    <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="21"/>
+      <c r="B40" s="21"/>
+      <c r="C40" s="21"/>
+      <c r="D40" s="21"/>
+      <c r="E40" s="21"/>
+      <c r="F40" s="21"/>
+      <c r="G40" s="23"/>
+      <c r="H40" s="23"/>
+      <c r="I40" s="23"/>
+      <c r="J40" s="23"/>
+      <c r="K40" s="23"/>
+      <c r="L40" s="23"/>
+      <c r="M40" s="23"/>
+      <c r="N40" s="23"/>
+      <c r="O40" s="25"/>
+      <c r="P40" s="25"/>
+      <c r="Q40" s="26" t="str">
         <f aca="false">IF(V40="Defect","",IF(COUNT(G40:K40)&lt;5,"",ROUND(G40*Config!$B$4+H40*Config!$B$5+I40*Config!$B$6+J40*Config!$B$7+K40*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R40" s="25" t="str">
+      <c r="R40" s="26" t="str">
         <f aca="false">IF(L40="","",VLOOKUP(L40,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S40" s="25" t="str">
+      <c r="S40" s="26" t="str">
         <f aca="false">IF(N40="","",VLOOKUP(N40,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T40" s="26" t="str">
+      <c r="T40" s="27" t="str">
         <f aca="false">IF(V40="Defect",IF(OR(X40="",G40="",R40=""),"",ROUND(MIN(100,VLOOKUP(X40,Config!$G$12:$H$16,2,0)*VLOOKUP(G40,Config!$I$12:$J$16,2,0)*R40),1)),IF(OR(Q40="",R40="",S40="",M40=""),"",ROUND(Q40*R40*S40/M40*20,1)))</f>
         <v/>
       </c>
-      <c r="U40" s="27" t="str">
+      <c r="U40" s="28" t="str">
         <f aca="false">IF(T40="","",RANK(T40,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="20"/>
-      <c r="B41" s="20"/>
-      <c r="C41" s="20"/>
-      <c r="D41" s="20"/>
-      <c r="E41" s="20"/>
-      <c r="F41" s="20"/>
-      <c r="G41" s="22"/>
-      <c r="H41" s="22"/>
-      <c r="I41" s="22"/>
-      <c r="J41" s="22"/>
-      <c r="K41" s="22"/>
-      <c r="L41" s="22"/>
-      <c r="M41" s="22"/>
-      <c r="N41" s="22"/>
-      <c r="O41" s="24"/>
-      <c r="P41" s="24"/>
-      <c r="Q41" s="25" t="str">
+    <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="21"/>
+      <c r="B41" s="21"/>
+      <c r="C41" s="21"/>
+      <c r="D41" s="21"/>
+      <c r="E41" s="21"/>
+      <c r="F41" s="21"/>
+      <c r="G41" s="23"/>
+      <c r="H41" s="23"/>
+      <c r="I41" s="23"/>
+      <c r="J41" s="23"/>
+      <c r="K41" s="23"/>
+      <c r="L41" s="23"/>
+      <c r="M41" s="23"/>
+      <c r="N41" s="23"/>
+      <c r="O41" s="25"/>
+      <c r="P41" s="25"/>
+      <c r="Q41" s="26" t="str">
         <f aca="false">IF(V41="Defect","",IF(COUNT(G41:K41)&lt;5,"",ROUND(G41*Config!$B$4+H41*Config!$B$5+I41*Config!$B$6+J41*Config!$B$7+K41*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R41" s="25" t="str">
+      <c r="R41" s="26" t="str">
         <f aca="false">IF(L41="","",VLOOKUP(L41,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S41" s="25" t="str">
+      <c r="S41" s="26" t="str">
         <f aca="false">IF(N41="","",VLOOKUP(N41,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T41" s="26" t="str">
+      <c r="T41" s="27" t="str">
         <f aca="false">IF(V41="Defect",IF(OR(X41="",G41="",R41=""),"",ROUND(MIN(100,VLOOKUP(X41,Config!$G$12:$H$16,2,0)*VLOOKUP(G41,Config!$I$12:$J$16,2,0)*R41),1)),IF(OR(Q41="",R41="",S41="",M41=""),"",ROUND(Q41*R41*S41/M41*20,1)))</f>
         <v/>
       </c>
-      <c r="U41" s="27" t="str">
+      <c r="U41" s="28" t="str">
         <f aca="false">IF(T41="","",RANK(T41,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="20"/>
-      <c r="B42" s="20"/>
-      <c r="C42" s="20"/>
-      <c r="D42" s="20"/>
-      <c r="E42" s="20"/>
-      <c r="F42" s="20"/>
-      <c r="G42" s="22"/>
-      <c r="H42" s="22"/>
-      <c r="I42" s="22"/>
-      <c r="J42" s="22"/>
-      <c r="K42" s="22"/>
-      <c r="L42" s="22"/>
-      <c r="M42" s="22"/>
-      <c r="N42" s="22"/>
-      <c r="O42" s="24"/>
-      <c r="P42" s="24"/>
-      <c r="Q42" s="25" t="str">
+    <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="21"/>
+      <c r="B42" s="21"/>
+      <c r="C42" s="21"/>
+      <c r="D42" s="21"/>
+      <c r="E42" s="21"/>
+      <c r="F42" s="21"/>
+      <c r="G42" s="23"/>
+      <c r="H42" s="23"/>
+      <c r="I42" s="23"/>
+      <c r="J42" s="23"/>
+      <c r="K42" s="23"/>
+      <c r="L42" s="23"/>
+      <c r="M42" s="23"/>
+      <c r="N42" s="23"/>
+      <c r="O42" s="25"/>
+      <c r="P42" s="25"/>
+      <c r="Q42" s="26" t="str">
         <f aca="false">IF(V42="Defect","",IF(COUNT(G42:K42)&lt;5,"",ROUND(G42*Config!$B$4+H42*Config!$B$5+I42*Config!$B$6+J42*Config!$B$7+K42*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R42" s="25" t="str">
+      <c r="R42" s="26" t="str">
         <f aca="false">IF(L42="","",VLOOKUP(L42,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S42" s="25" t="str">
+      <c r="S42" s="26" t="str">
         <f aca="false">IF(N42="","",VLOOKUP(N42,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T42" s="26" t="str">
+      <c r="T42" s="27" t="str">
         <f aca="false">IF(V42="Defect",IF(OR(X42="",G42="",R42=""),"",ROUND(MIN(100,VLOOKUP(X42,Config!$G$12:$H$16,2,0)*VLOOKUP(G42,Config!$I$12:$J$16,2,0)*R42),1)),IF(OR(Q42="",R42="",S42="",M42=""),"",ROUND(Q42*R42*S42/M42*20,1)))</f>
         <v/>
       </c>
-      <c r="U42" s="27" t="str">
+      <c r="U42" s="28" t="str">
         <f aca="false">IF(T42="","",RANK(T42,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="20"/>
-      <c r="B43" s="20"/>
-      <c r="C43" s="20"/>
-      <c r="D43" s="20"/>
-      <c r="E43" s="20"/>
-      <c r="F43" s="20"/>
-      <c r="G43" s="22"/>
-      <c r="H43" s="22"/>
-      <c r="I43" s="22"/>
-      <c r="J43" s="22"/>
-      <c r="K43" s="22"/>
-      <c r="L43" s="22"/>
-      <c r="M43" s="22"/>
-      <c r="N43" s="22"/>
-      <c r="O43" s="24"/>
-      <c r="P43" s="24"/>
-      <c r="Q43" s="25" t="str">
+    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="21"/>
+      <c r="B43" s="21"/>
+      <c r="C43" s="21"/>
+      <c r="D43" s="21"/>
+      <c r="E43" s="21"/>
+      <c r="F43" s="21"/>
+      <c r="G43" s="23"/>
+      <c r="H43" s="23"/>
+      <c r="I43" s="23"/>
+      <c r="J43" s="23"/>
+      <c r="K43" s="23"/>
+      <c r="L43" s="23"/>
+      <c r="M43" s="23"/>
+      <c r="N43" s="23"/>
+      <c r="O43" s="25"/>
+      <c r="P43" s="25"/>
+      <c r="Q43" s="26" t="str">
         <f aca="false">IF(V43="Defect","",IF(COUNT(G43:K43)&lt;5,"",ROUND(G43*Config!$B$4+H43*Config!$B$5+I43*Config!$B$6+J43*Config!$B$7+K43*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R43" s="25" t="str">
+      <c r="R43" s="26" t="str">
         <f aca="false">IF(L43="","",VLOOKUP(L43,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S43" s="25" t="str">
+      <c r="S43" s="26" t="str">
         <f aca="false">IF(N43="","",VLOOKUP(N43,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T43" s="26" t="str">
+      <c r="T43" s="27" t="str">
         <f aca="false">IF(V43="Defect",IF(OR(X43="",G43="",R43=""),"",ROUND(MIN(100,VLOOKUP(X43,Config!$G$12:$H$16,2,0)*VLOOKUP(G43,Config!$I$12:$J$16,2,0)*R43),1)),IF(OR(Q43="",R43="",S43="",M43=""),"",ROUND(Q43*R43*S43/M43*20,1)))</f>
         <v/>
       </c>
-      <c r="U43" s="27" t="str">
+      <c r="U43" s="28" t="str">
         <f aca="false">IF(T43="","",RANK(T43,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="20"/>
-      <c r="B44" s="20"/>
-      <c r="C44" s="20"/>
-      <c r="D44" s="20"/>
-      <c r="E44" s="20"/>
-      <c r="F44" s="20"/>
-      <c r="G44" s="22"/>
-      <c r="H44" s="22"/>
-      <c r="I44" s="22"/>
-      <c r="J44" s="22"/>
-      <c r="K44" s="22"/>
-      <c r="L44" s="22"/>
-      <c r="M44" s="22"/>
-      <c r="N44" s="22"/>
-      <c r="O44" s="24"/>
-      <c r="P44" s="24"/>
-      <c r="Q44" s="25" t="str">
+    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="21"/>
+      <c r="B44" s="21"/>
+      <c r="C44" s="21"/>
+      <c r="D44" s="21"/>
+      <c r="E44" s="21"/>
+      <c r="F44" s="21"/>
+      <c r="G44" s="23"/>
+      <c r="H44" s="23"/>
+      <c r="I44" s="23"/>
+      <c r="J44" s="23"/>
+      <c r="K44" s="23"/>
+      <c r="L44" s="23"/>
+      <c r="M44" s="23"/>
+      <c r="N44" s="23"/>
+      <c r="O44" s="25"/>
+      <c r="P44" s="25"/>
+      <c r="Q44" s="26" t="str">
         <f aca="false">IF(V44="Defect","",IF(COUNT(G44:K44)&lt;5,"",ROUND(G44*Config!$B$4+H44*Config!$B$5+I44*Config!$B$6+J44*Config!$B$7+K44*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R44" s="25" t="str">
+      <c r="R44" s="26" t="str">
         <f aca="false">IF(L44="","",VLOOKUP(L44,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S44" s="25" t="str">
+      <c r="S44" s="26" t="str">
         <f aca="false">IF(N44="","",VLOOKUP(N44,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T44" s="26" t="str">
+      <c r="T44" s="27" t="str">
         <f aca="false">IF(V44="Defect",IF(OR(X44="",G44="",R44=""),"",ROUND(MIN(100,VLOOKUP(X44,Config!$G$12:$H$16,2,0)*VLOOKUP(G44,Config!$I$12:$J$16,2,0)*R44),1)),IF(OR(Q44="",R44="",S44="",M44=""),"",ROUND(Q44*R44*S44/M44*20,1)))</f>
         <v/>
       </c>
-      <c r="U44" s="27" t="str">
+      <c r="U44" s="28" t="str">
         <f aca="false">IF(T44="","",RANK(T44,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="20"/>
-      <c r="B45" s="20"/>
-      <c r="C45" s="20"/>
-      <c r="D45" s="20"/>
-      <c r="E45" s="20"/>
-      <c r="F45" s="20"/>
-      <c r="G45" s="22"/>
-      <c r="H45" s="22"/>
-      <c r="I45" s="22"/>
-      <c r="J45" s="22"/>
-      <c r="K45" s="22"/>
-      <c r="L45" s="22"/>
-      <c r="M45" s="22"/>
-      <c r="N45" s="22"/>
-      <c r="O45" s="24"/>
-      <c r="P45" s="24"/>
-      <c r="Q45" s="25" t="str">
+    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="21"/>
+      <c r="B45" s="21"/>
+      <c r="C45" s="21"/>
+      <c r="D45" s="21"/>
+      <c r="E45" s="21"/>
+      <c r="F45" s="21"/>
+      <c r="G45" s="23"/>
+      <c r="H45" s="23"/>
+      <c r="I45" s="23"/>
+      <c r="J45" s="23"/>
+      <c r="K45" s="23"/>
+      <c r="L45" s="23"/>
+      <c r="M45" s="23"/>
+      <c r="N45" s="23"/>
+      <c r="O45" s="25"/>
+      <c r="P45" s="25"/>
+      <c r="Q45" s="26" t="str">
         <f aca="false">IF(V45="Defect","",IF(COUNT(G45:K45)&lt;5,"",ROUND(G45*Config!$B$4+H45*Config!$B$5+I45*Config!$B$6+J45*Config!$B$7+K45*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R45" s="25" t="str">
+      <c r="R45" s="26" t="str">
         <f aca="false">IF(L45="","",VLOOKUP(L45,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S45" s="25" t="str">
+      <c r="S45" s="26" t="str">
         <f aca="false">IF(N45="","",VLOOKUP(N45,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T45" s="26" t="str">
+      <c r="T45" s="27" t="str">
         <f aca="false">IF(V45="Defect",IF(OR(X45="",G45="",R45=""),"",ROUND(MIN(100,VLOOKUP(X45,Config!$G$12:$H$16,2,0)*VLOOKUP(G45,Config!$I$12:$J$16,2,0)*R45),1)),IF(OR(Q45="",R45="",S45="",M45=""),"",ROUND(Q45*R45*S45/M45*20,1)))</f>
         <v/>
       </c>
-      <c r="U45" s="27" t="str">
+      <c r="U45" s="28" t="str">
         <f aca="false">IF(T45="","",RANK(T45,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="20"/>
-      <c r="B46" s="20"/>
-      <c r="C46" s="20"/>
-      <c r="D46" s="20"/>
-      <c r="E46" s="20"/>
-      <c r="F46" s="20"/>
-      <c r="G46" s="22"/>
-      <c r="H46" s="22"/>
-      <c r="I46" s="22"/>
-      <c r="J46" s="22"/>
-      <c r="K46" s="22"/>
-      <c r="L46" s="22"/>
-      <c r="M46" s="22"/>
-      <c r="N46" s="22"/>
-      <c r="O46" s="24"/>
-      <c r="P46" s="24"/>
-      <c r="Q46" s="25" t="str">
+    <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="21"/>
+      <c r="B46" s="21"/>
+      <c r="C46" s="21"/>
+      <c r="D46" s="21"/>
+      <c r="E46" s="21"/>
+      <c r="F46" s="21"/>
+      <c r="G46" s="23"/>
+      <c r="H46" s="23"/>
+      <c r="I46" s="23"/>
+      <c r="J46" s="23"/>
+      <c r="K46" s="23"/>
+      <c r="L46" s="23"/>
+      <c r="M46" s="23"/>
+      <c r="N46" s="23"/>
+      <c r="O46" s="25"/>
+      <c r="P46" s="25"/>
+      <c r="Q46" s="26" t="str">
         <f aca="false">IF(V46="Defect","",IF(COUNT(G46:K46)&lt;5,"",ROUND(G46*Config!$B$4+H46*Config!$B$5+I46*Config!$B$6+J46*Config!$B$7+K46*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R46" s="25" t="str">
+      <c r="R46" s="26" t="str">
         <f aca="false">IF(L46="","",VLOOKUP(L46,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S46" s="25" t="str">
+      <c r="S46" s="26" t="str">
         <f aca="false">IF(N46="","",VLOOKUP(N46,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T46" s="26" t="str">
+      <c r="T46" s="27" t="str">
         <f aca="false">IF(V46="Defect",IF(OR(X46="",G46="",R46=""),"",ROUND(MIN(100,VLOOKUP(X46,Config!$G$12:$H$16,2,0)*VLOOKUP(G46,Config!$I$12:$J$16,2,0)*R46),1)),IF(OR(Q46="",R46="",S46="",M46=""),"",ROUND(Q46*R46*S46/M46*20,1)))</f>
         <v/>
       </c>
-      <c r="U46" s="27" t="str">
+      <c r="U46" s="28" t="str">
         <f aca="false">IF(T46="","",RANK(T46,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="20"/>
-      <c r="B47" s="20"/>
-      <c r="C47" s="20"/>
-      <c r="D47" s="20"/>
-      <c r="E47" s="20"/>
-      <c r="F47" s="20"/>
-      <c r="G47" s="22"/>
-      <c r="H47" s="22"/>
-      <c r="I47" s="22"/>
-      <c r="J47" s="22"/>
-      <c r="K47" s="22"/>
-      <c r="L47" s="22"/>
-      <c r="M47" s="22"/>
-      <c r="N47" s="22"/>
-      <c r="O47" s="24"/>
-      <c r="P47" s="24"/>
-      <c r="Q47" s="25" t="str">
+    <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="21"/>
+      <c r="B47" s="21"/>
+      <c r="C47" s="21"/>
+      <c r="D47" s="21"/>
+      <c r="E47" s="21"/>
+      <c r="F47" s="21"/>
+      <c r="G47" s="23"/>
+      <c r="H47" s="23"/>
+      <c r="I47" s="23"/>
+      <c r="J47" s="23"/>
+      <c r="K47" s="23"/>
+      <c r="L47" s="23"/>
+      <c r="M47" s="23"/>
+      <c r="N47" s="23"/>
+      <c r="O47" s="25"/>
+      <c r="P47" s="25"/>
+      <c r="Q47" s="26" t="str">
         <f aca="false">IF(V47="Defect","",IF(COUNT(G47:K47)&lt;5,"",ROUND(G47*Config!$B$4+H47*Config!$B$5+I47*Config!$B$6+J47*Config!$B$7+K47*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R47" s="25" t="str">
+      <c r="R47" s="26" t="str">
         <f aca="false">IF(L47="","",VLOOKUP(L47,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S47" s="25" t="str">
+      <c r="S47" s="26" t="str">
         <f aca="false">IF(N47="","",VLOOKUP(N47,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T47" s="26" t="str">
+      <c r="T47" s="27" t="str">
         <f aca="false">IF(V47="Defect",IF(OR(X47="",G47="",R47=""),"",ROUND(MIN(100,VLOOKUP(X47,Config!$G$12:$H$16,2,0)*VLOOKUP(G47,Config!$I$12:$J$16,2,0)*R47),1)),IF(OR(Q47="",R47="",S47="",M47=""),"",ROUND(Q47*R47*S47/M47*20,1)))</f>
         <v/>
       </c>
-      <c r="U47" s="27" t="str">
+      <c r="U47" s="28" t="str">
         <f aca="false">IF(T47="","",RANK(T47,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="20"/>
-      <c r="B48" s="20"/>
-      <c r="C48" s="20"/>
-      <c r="D48" s="20"/>
-      <c r="E48" s="20"/>
-      <c r="F48" s="20"/>
-      <c r="G48" s="22"/>
-      <c r="H48" s="22"/>
-      <c r="I48" s="22"/>
-      <c r="J48" s="22"/>
-      <c r="K48" s="22"/>
-      <c r="L48" s="22"/>
-      <c r="M48" s="22"/>
-      <c r="N48" s="22"/>
-      <c r="O48" s="24"/>
-      <c r="P48" s="24"/>
-      <c r="Q48" s="25" t="str">
+    <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="21"/>
+      <c r="B48" s="21"/>
+      <c r="C48" s="21"/>
+      <c r="D48" s="21"/>
+      <c r="E48" s="21"/>
+      <c r="F48" s="21"/>
+      <c r="G48" s="23"/>
+      <c r="H48" s="23"/>
+      <c r="I48" s="23"/>
+      <c r="J48" s="23"/>
+      <c r="K48" s="23"/>
+      <c r="L48" s="23"/>
+      <c r="M48" s="23"/>
+      <c r="N48" s="23"/>
+      <c r="O48" s="25"/>
+      <c r="P48" s="25"/>
+      <c r="Q48" s="26" t="str">
         <f aca="false">IF(V48="Defect","",IF(COUNT(G48:K48)&lt;5,"",ROUND(G48*Config!$B$4+H48*Config!$B$5+I48*Config!$B$6+J48*Config!$B$7+K48*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R48" s="25" t="str">
+      <c r="R48" s="26" t="str">
         <f aca="false">IF(L48="","",VLOOKUP(L48,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S48" s="25" t="str">
+      <c r="S48" s="26" t="str">
         <f aca="false">IF(N48="","",VLOOKUP(N48,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T48" s="26" t="str">
+      <c r="T48" s="27" t="str">
         <f aca="false">IF(V48="Defect",IF(OR(X48="",G48="",R48=""),"",ROUND(MIN(100,VLOOKUP(X48,Config!$G$12:$H$16,2,0)*VLOOKUP(G48,Config!$I$12:$J$16,2,0)*R48),1)),IF(OR(Q48="",R48="",S48="",M48=""),"",ROUND(Q48*R48*S48/M48*20,1)))</f>
         <v/>
       </c>
-      <c r="U48" s="27" t="str">
+      <c r="U48" s="28" t="str">
         <f aca="false">IF(T48="","",RANK(T48,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="20"/>
-      <c r="B49" s="20"/>
-      <c r="C49" s="20"/>
-      <c r="D49" s="20"/>
-      <c r="E49" s="20"/>
-      <c r="F49" s="20"/>
-      <c r="G49" s="22"/>
-      <c r="H49" s="22"/>
-      <c r="I49" s="22"/>
-      <c r="J49" s="22"/>
-      <c r="K49" s="22"/>
-      <c r="L49" s="22"/>
-      <c r="M49" s="22"/>
-      <c r="N49" s="22"/>
-      <c r="O49" s="24"/>
-      <c r="P49" s="24"/>
-      <c r="Q49" s="25" t="str">
+    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="21"/>
+      <c r="B49" s="21"/>
+      <c r="C49" s="21"/>
+      <c r="D49" s="21"/>
+      <c r="E49" s="21"/>
+      <c r="F49" s="21"/>
+      <c r="G49" s="23"/>
+      <c r="H49" s="23"/>
+      <c r="I49" s="23"/>
+      <c r="J49" s="23"/>
+      <c r="K49" s="23"/>
+      <c r="L49" s="23"/>
+      <c r="M49" s="23"/>
+      <c r="N49" s="23"/>
+      <c r="O49" s="25"/>
+      <c r="P49" s="25"/>
+      <c r="Q49" s="26" t="str">
         <f aca="false">IF(V49="Defect","",IF(COUNT(G49:K49)&lt;5,"",ROUND(G49*Config!$B$4+H49*Config!$B$5+I49*Config!$B$6+J49*Config!$B$7+K49*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R49" s="25" t="str">
+      <c r="R49" s="26" t="str">
         <f aca="false">IF(L49="","",VLOOKUP(L49,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S49" s="25" t="str">
+      <c r="S49" s="26" t="str">
         <f aca="false">IF(N49="","",VLOOKUP(N49,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T49" s="26" t="str">
+      <c r="T49" s="27" t="str">
         <f aca="false">IF(V49="Defect",IF(OR(X49="",G49="",R49=""),"",ROUND(MIN(100,VLOOKUP(X49,Config!$G$12:$H$16,2,0)*VLOOKUP(G49,Config!$I$12:$J$16,2,0)*R49),1)),IF(OR(Q49="",R49="",S49="",M49=""),"",ROUND(Q49*R49*S49/M49*20,1)))</f>
         <v/>
       </c>
-      <c r="U49" s="27" t="str">
+      <c r="U49" s="28" t="str">
         <f aca="false">IF(T49="","",RANK(T49,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="20"/>
-      <c r="B50" s="20"/>
-      <c r="C50" s="20"/>
-      <c r="D50" s="20"/>
-      <c r="E50" s="20"/>
-      <c r="F50" s="20"/>
-      <c r="G50" s="22"/>
-      <c r="H50" s="22"/>
-      <c r="I50" s="22"/>
-      <c r="J50" s="22"/>
-      <c r="K50" s="22"/>
-      <c r="L50" s="22"/>
-      <c r="M50" s="22"/>
-      <c r="N50" s="22"/>
-      <c r="O50" s="24"/>
-      <c r="P50" s="24"/>
-      <c r="Q50" s="25" t="str">
+    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="21"/>
+      <c r="B50" s="21"/>
+      <c r="C50" s="21"/>
+      <c r="D50" s="21"/>
+      <c r="E50" s="21"/>
+      <c r="F50" s="21"/>
+      <c r="G50" s="23"/>
+      <c r="H50" s="23"/>
+      <c r="I50" s="23"/>
+      <c r="J50" s="23"/>
+      <c r="K50" s="23"/>
+      <c r="L50" s="23"/>
+      <c r="M50" s="23"/>
+      <c r="N50" s="23"/>
+      <c r="O50" s="25"/>
+      <c r="P50" s="25"/>
+      <c r="Q50" s="26" t="str">
         <f aca="false">IF(V50="Defect","",IF(COUNT(G50:K50)&lt;5,"",ROUND(G50*Config!$B$4+H50*Config!$B$5+I50*Config!$B$6+J50*Config!$B$7+K50*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R50" s="25" t="str">
+      <c r="R50" s="26" t="str">
         <f aca="false">IF(L50="","",VLOOKUP(L50,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S50" s="25" t="str">
+      <c r="S50" s="26" t="str">
         <f aca="false">IF(N50="","",VLOOKUP(N50,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T50" s="26" t="str">
+      <c r="T50" s="27" t="str">
         <f aca="false">IF(V50="Defect",IF(OR(X50="",G50="",R50=""),"",ROUND(MIN(100,VLOOKUP(X50,Config!$G$12:$H$16,2,0)*VLOOKUP(G50,Config!$I$12:$J$16,2,0)*R50),1)),IF(OR(Q50="",R50="",S50="",M50=""),"",ROUND(Q50*R50*S50/M50*20,1)))</f>
         <v/>
       </c>
-      <c r="U50" s="27" t="str">
+      <c r="U50" s="28" t="str">
         <f aca="false">IF(T50="","",RANK(T50,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="20"/>
-      <c r="B51" s="20"/>
-      <c r="C51" s="20"/>
-      <c r="D51" s="20"/>
-      <c r="E51" s="20"/>
-      <c r="F51" s="20"/>
-      <c r="G51" s="22"/>
-      <c r="H51" s="22"/>
-      <c r="I51" s="22"/>
-      <c r="J51" s="22"/>
-      <c r="K51" s="22"/>
-      <c r="L51" s="22"/>
-      <c r="M51" s="22"/>
-      <c r="N51" s="22"/>
-      <c r="O51" s="24"/>
-      <c r="P51" s="24"/>
-      <c r="Q51" s="25" t="str">
+    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="21"/>
+      <c r="B51" s="21"/>
+      <c r="C51" s="21"/>
+      <c r="D51" s="21"/>
+      <c r="E51" s="21"/>
+      <c r="F51" s="21"/>
+      <c r="G51" s="23"/>
+      <c r="H51" s="23"/>
+      <c r="I51" s="23"/>
+      <c r="J51" s="23"/>
+      <c r="K51" s="23"/>
+      <c r="L51" s="23"/>
+      <c r="M51" s="23"/>
+      <c r="N51" s="23"/>
+      <c r="O51" s="25"/>
+      <c r="P51" s="25"/>
+      <c r="Q51" s="26" t="str">
         <f aca="false">IF(V51="Defect","",IF(COUNT(G51:K51)&lt;5,"",ROUND(G51*Config!$B$4+H51*Config!$B$5+I51*Config!$B$6+J51*Config!$B$7+K51*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R51" s="25" t="str">
+      <c r="R51" s="26" t="str">
         <f aca="false">IF(L51="","",VLOOKUP(L51,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S51" s="25" t="str">
+      <c r="S51" s="26" t="str">
         <f aca="false">IF(N51="","",VLOOKUP(N51,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T51" s="26" t="str">
+      <c r="T51" s="27" t="str">
         <f aca="false">IF(V51="Defect",IF(OR(X51="",G51="",R51=""),"",ROUND(MIN(100,VLOOKUP(X51,Config!$G$12:$H$16,2,0)*VLOOKUP(G51,Config!$I$12:$J$16,2,0)*R51),1)),IF(OR(Q51="",R51="",S51="",M51=""),"",ROUND(Q51*R51*S51/M51*20,1)))</f>
         <v/>
       </c>
-      <c r="U51" s="27" t="str">
+      <c r="U51" s="28" t="str">
         <f aca="false">IF(T51="","",RANK(T51,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="20"/>
-      <c r="B52" s="20"/>
-      <c r="C52" s="20"/>
-      <c r="D52" s="20"/>
-      <c r="E52" s="20"/>
-      <c r="F52" s="20"/>
-      <c r="G52" s="22"/>
-      <c r="H52" s="22"/>
-      <c r="I52" s="22"/>
-      <c r="J52" s="22"/>
-      <c r="K52" s="22"/>
-      <c r="L52" s="22"/>
-      <c r="M52" s="22"/>
-      <c r="N52" s="22"/>
-      <c r="O52" s="24"/>
-      <c r="P52" s="24"/>
-      <c r="Q52" s="25" t="str">
+    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="21"/>
+      <c r="B52" s="21"/>
+      <c r="C52" s="21"/>
+      <c r="D52" s="21"/>
+      <c r="E52" s="21"/>
+      <c r="F52" s="21"/>
+      <c r="G52" s="23"/>
+      <c r="H52" s="23"/>
+      <c r="I52" s="23"/>
+      <c r="J52" s="23"/>
+      <c r="K52" s="23"/>
+      <c r="L52" s="23"/>
+      <c r="M52" s="23"/>
+      <c r="N52" s="23"/>
+      <c r="O52" s="25"/>
+      <c r="P52" s="25"/>
+      <c r="Q52" s="26" t="str">
         <f aca="false">IF(V52="Defect","",IF(COUNT(G52:K52)&lt;5,"",ROUND(G52*Config!$B$4+H52*Config!$B$5+I52*Config!$B$6+J52*Config!$B$7+K52*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R52" s="25" t="str">
+      <c r="R52" s="26" t="str">
         <f aca="false">IF(L52="","",VLOOKUP(L52,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S52" s="25" t="str">
+      <c r="S52" s="26" t="str">
         <f aca="false">IF(N52="","",VLOOKUP(N52,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T52" s="26" t="str">
+      <c r="T52" s="27" t="str">
         <f aca="false">IF(V52="Defect",IF(OR(X52="",G52="",R52=""),"",ROUND(MIN(100,VLOOKUP(X52,Config!$G$12:$H$16,2,0)*VLOOKUP(G52,Config!$I$12:$J$16,2,0)*R52),1)),IF(OR(Q52="",R52="",S52="",M52=""),"",ROUND(Q52*R52*S52/M52*20,1)))</f>
         <v/>
       </c>
-      <c r="U52" s="27" t="str">
+      <c r="U52" s="28" t="str">
         <f aca="false">IF(T52="","",RANK(T52,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="20"/>
-      <c r="B53" s="20"/>
-      <c r="C53" s="20"/>
-      <c r="D53" s="20"/>
-      <c r="E53" s="20"/>
-      <c r="F53" s="20"/>
-      <c r="G53" s="22"/>
-      <c r="H53" s="22"/>
-      <c r="I53" s="22"/>
-      <c r="J53" s="22"/>
-      <c r="K53" s="22"/>
-      <c r="L53" s="22"/>
-      <c r="M53" s="22"/>
-      <c r="N53" s="22"/>
-      <c r="O53" s="24"/>
-      <c r="P53" s="24"/>
-      <c r="Q53" s="25" t="str">
+    <row r="53" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="21"/>
+      <c r="B53" s="21"/>
+      <c r="C53" s="21"/>
+      <c r="D53" s="21"/>
+      <c r="E53" s="21"/>
+      <c r="F53" s="21"/>
+      <c r="G53" s="23"/>
+      <c r="H53" s="23"/>
+      <c r="I53" s="23"/>
+      <c r="J53" s="23"/>
+      <c r="K53" s="23"/>
+      <c r="L53" s="23"/>
+      <c r="M53" s="23"/>
+      <c r="N53" s="23"/>
+      <c r="O53" s="25"/>
+      <c r="P53" s="25"/>
+      <c r="Q53" s="26" t="str">
         <f aca="false">IF(V53="Defect","",IF(COUNT(G53:K53)&lt;5,"",ROUND(G53*Config!$B$4+H53*Config!$B$5+I53*Config!$B$6+J53*Config!$B$7+K53*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R53" s="25" t="str">
+      <c r="R53" s="26" t="str">
         <f aca="false">IF(L53="","",VLOOKUP(L53,Config!$A$12:$B$16,2,0))</f>
         <v/>
       </c>
-      <c r="S53" s="25" t="str">
+      <c r="S53" s="26" t="str">
         <f aca="false">IF(N53="","",VLOOKUP(N53,Config!$D$12:$E$16,2,0))</f>
         <v/>
       </c>
-      <c r="T53" s="26" t="str">
+      <c r="T53" s="27" t="str">
         <f aca="false">IF(V53="Defect",IF(OR(X53="",G53="",R53=""),"",ROUND(MIN(100,VLOOKUP(X53,Config!$G$12:$H$16,2,0)*VLOOKUP(G53,Config!$I$12:$J$16,2,0)*R53),1)),IF(OR(Q53="",R53="",S53="",M53=""),"",ROUND(Q53*R53*S53/M53*20,1)))</f>
         <v/>
       </c>
-      <c r="U53" s="27" t="str">
+      <c r="U53" s="28" t="str">
         <f aca="false">IF(T53="","",RANK(T53,$T$4:$T$53))</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="6">
     <dataValidation allowBlank="true" error="Scores must be whole numbers 1-5. See Rubric sheet for anchors." errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="G4:N53" type="whole">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D4:D53" type="list">
-      <formula1>"Idea,Brief Drafted,Scored,Prioritized,Deferred,Rejected"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E4:E53" type="list">
       <formula1>"Human,Market Research Agent,Hybrid"</formula1>
       <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D4:D53" type="list">
+      <formula1>"Idea,Brief Drafted,Reported,Triaged,Scored,Prioritized,In Progress,Fixed,Verified,Deferred,Rejected,Won't Fix"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="V4:V53" type="list">
+      <formula1>"Feature,Defect"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="W4:W53" type="list">
+      <formula1>"Customer-Reported,Internal"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" prompt="Whole number 1-5; see Rubric Severity row (Defect rows only)." showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="X4:X53" type="whole">
+      <formula1>1</formula1>
+      <formula2>5</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -4227,516 +4238,516 @@
   <dimension ref="A1:F27"/>
   <sheetFormatPr defaultColWidth="8.63671875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="29" t="s">
+    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="30" t="s">
         <v>156</v>
       </c>
-      <c r="B3" s="29" t="s">
+      <c r="B3" s="30" t="s">
         <v>157</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="C3" s="30" t="s">
         <v>158</v>
       </c>
-      <c r="D3" s="29" t="s">
+      <c r="D3" s="30" t="s">
         <v>159</v>
       </c>
-      <c r="E3" s="29" t="s">
+      <c r="E3" s="30" t="s">
         <v>160</v>
       </c>
-      <c r="F3" s="29" t="s">
+      <c r="F3" s="30" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17" t="s">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="18" t="s">
         <v>162</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="D4" s="17" t="s">
+      <c r="D4" s="18" t="s">
         <v>165</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="E4" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="F4" s="17" t="s">
+      <c r="F4" s="18" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17" t="s">
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="18" t="s">
         <v>168</v>
       </c>
-      <c r="C5" s="17" t="s">
+      <c r="C5" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="D5" s="17" t="s">
+      <c r="D5" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="E5" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="F5" s="17" t="s">
+      <c r="F5" s="18" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17" t="s">
+    <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="18" t="s">
         <v>171</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="18" t="s">
         <v>172</v>
       </c>
-      <c r="C6" s="17" t="s">
+      <c r="C6" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="D6" s="17" t="s">
+      <c r="D6" s="18" t="s">
         <v>173</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="F6" s="17" t="s">
+      <c r="F6" s="18" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="18" t="s">
         <v>175</v>
       </c>
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="18" t="s">
         <v>176</v>
       </c>
-      <c r="C7" s="17" t="s">
+      <c r="C7" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="D7" s="17" t="s">
+      <c r="D7" s="18" t="s">
         <v>178</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="18" t="s">
         <v>179</v>
       </c>
-      <c r="F7" s="17" t="s">
+      <c r="F7" s="18" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="18" t="s">
         <v>181</v>
       </c>
-      <c r="B8" s="17" t="s">
+      <c r="B8" s="18" t="s">
         <v>182</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="D8" s="17" t="s">
+      <c r="D8" s="18" t="s">
         <v>183</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="E8" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="F8" s="17" t="s">
+      <c r="F8" s="18" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17" t="s">
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="18" t="s">
         <v>186</v>
       </c>
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="18" t="s">
         <v>188</v>
       </c>
-      <c r="D9" s="17" t="s">
+      <c r="D9" s="18" t="s">
         <v>189</v>
       </c>
-      <c r="E9" s="17" t="s">
+      <c r="E9" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="F9" s="17" t="s">
+      <c r="F9" s="18" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17" t="s">
+    <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="s">
         <v>191</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="18" t="s">
         <v>192</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="D10" s="17" t="s">
+      <c r="D10" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="E10" s="18" t="s">
         <v>195</v>
       </c>
-      <c r="F10" s="17" t="s">
+      <c r="F10" s="18" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17" t="s">
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="18" t="s">
         <v>197</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="18" t="s">
         <v>198</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="C11" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="D11" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" s="18" t="s">
         <v>195</v>
       </c>
-      <c r="F11" s="17" t="s">
+      <c r="F11" s="18" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17" t="s">
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="18" t="s">
         <v>200</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B12" s="18" t="s">
         <v>201</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="D12" s="17" t="s">
+      <c r="D12" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="E12" s="17" t="s">
+      <c r="E12" s="18" t="s">
         <v>195</v>
       </c>
-      <c r="F12" s="17" t="s">
+      <c r="F12" s="18" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="17" t="s">
+    <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="18" t="s">
         <v>203</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="18" t="s">
         <v>204</v>
       </c>
-      <c r="C13" s="17" t="s">
+      <c r="C13" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="D13" s="17" t="s">
+      <c r="D13" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="E13" s="17" t="s">
+      <c r="E13" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="F13" s="17" t="s">
+      <c r="F13" s="18" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17" t="s">
+    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="18" t="s">
         <v>206</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="18" t="s">
         <v>207</v>
       </c>
-      <c r="C14" s="17" t="s">
+      <c r="C14" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="D14" s="17" t="s">
+      <c r="D14" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="E14" s="17" t="s">
+      <c r="E14" s="18" t="s">
         <v>195</v>
       </c>
-      <c r="F14" s="17" t="s">
+      <c r="F14" s="18" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="17" t="s">
+    <row r="15" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="18" t="s">
         <v>209</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="B15" s="18" t="s">
         <v>210</v>
       </c>
-      <c r="C15" s="17" t="s">
+      <c r="C15" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="D15" s="17" t="s">
+      <c r="D15" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="E15" s="17" t="s">
+      <c r="E15" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="F15" s="17" t="s">
+      <c r="F15" s="18" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17" t="s">
+    <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="18" t="s">
         <v>212</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="B16" s="18" t="s">
         <v>213</v>
       </c>
-      <c r="C16" s="17" t="s">
+      <c r="C16" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="D16" s="17" t="s">
+      <c r="D16" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="E16" s="17" t="s">
+      <c r="E16" s="18" t="s">
         <v>214</v>
       </c>
-      <c r="F16" s="17" t="s">
+      <c r="F16" s="18" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="17" t="s">
+    <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="18" t="s">
         <v>216</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="18" t="s">
         <v>217</v>
       </c>
-      <c r="C17" s="17" t="s">
+      <c r="C17" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="D17" s="17" t="s">
+      <c r="D17" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="E17" s="17" t="s">
+      <c r="E17" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="F17" s="17" t="s">
+      <c r="F17" s="18" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17" t="s">
+      <c r="A18" s="18" t="s">
         <v>219</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="18" t="s">
         <v>220</v>
       </c>
-      <c r="C18" s="17" t="s">
+      <c r="C18" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="D18" s="17" t="s">
+      <c r="D18" s="18" t="s">
         <v>221</v>
       </c>
-      <c r="E18" s="17" t="s">
+      <c r="E18" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="F18" s="17" t="s">
+      <c r="F18" s="18" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="17" t="s">
+    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="18" t="s">
         <v>223</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="B19" s="18" t="s">
         <v>224</v>
       </c>
-      <c r="C19" s="17" t="s">
+      <c r="C19" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="D19" s="17" t="s">
+      <c r="D19" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="E19" s="17" t="s">
+      <c r="E19" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="F19" s="17" t="s">
+      <c r="F19" s="18" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17" t="s">
+    <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="18" t="s">
         <v>226</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B20" s="18" t="s">
         <v>227</v>
       </c>
-      <c r="C20" s="17" t="s">
+      <c r="C20" s="18" t="s">
         <v>228</v>
       </c>
-      <c r="D20" s="17" t="s">
+      <c r="D20" s="18" t="s">
         <v>229</v>
       </c>
-      <c r="E20" s="17" t="s">
+      <c r="E20" s="18" t="s">
         <v>230</v>
       </c>
-      <c r="F20" s="17" t="s">
+      <c r="F20" s="18" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="17" t="s">
+    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="18" t="s">
         <v>232</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="18" t="s">
         <v>233</v>
       </c>
-      <c r="C21" s="17" t="s">
+      <c r="C21" s="18" t="s">
         <v>228</v>
       </c>
-      <c r="D21" s="17" t="s">
+      <c r="D21" s="18" t="s">
         <v>234</v>
       </c>
-      <c r="E21" s="17" t="s">
+      <c r="E21" s="18" t="s">
         <v>230</v>
       </c>
-      <c r="F21" s="17" t="s">
+      <c r="F21" s="18" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="17" t="s">
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="18" t="s">
         <v>236</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B22" s="18" t="s">
         <v>237</v>
       </c>
-      <c r="C22" s="17" t="s">
+      <c r="C22" s="18" t="s">
         <v>228</v>
       </c>
-      <c r="D22" s="17" t="s">
+      <c r="D22" s="18" t="s">
         <v>238</v>
       </c>
-      <c r="E22" s="17" t="s">
+      <c r="E22" s="18" t="s">
         <v>230</v>
       </c>
-      <c r="F22" s="17" t="s">
+      <c r="F22" s="18" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17" t="s">
+    <row r="23" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="18" t="s">
         <v>240</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B23" s="18" t="s">
         <v>241</v>
       </c>
-      <c r="C23" s="17" t="s">
+      <c r="C23" s="18" t="s">
         <v>228</v>
       </c>
-      <c r="D23" s="17" t="s">
+      <c r="D23" s="18" t="s">
         <v>242</v>
       </c>
-      <c r="E23" s="17" t="s">
+      <c r="E23" s="18" t="s">
         <v>230</v>
       </c>
-      <c r="F23" s="17" t="s">
+      <c r="F23" s="18" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="17" t="s">
+    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="18" t="s">
         <v>244</v>
       </c>
-      <c r="B24" s="17" t="s">
+      <c r="B24" s="18" t="s">
         <v>245</v>
       </c>
-      <c r="C24" s="17" t="s">
+      <c r="C24" s="18" t="s">
         <v>228</v>
       </c>
-      <c r="D24" s="17" t="s">
+      <c r="D24" s="18" t="s">
         <v>246</v>
       </c>
-      <c r="E24" s="17" t="s">
+      <c r="E24" s="18" t="s">
         <v>230</v>
       </c>
-      <c r="F24" s="17" t="s">
+      <c r="F24" s="18" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="17" t="s">
+    <row r="25" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="18" t="s">
         <v>248</v>
       </c>
-      <c r="B25" s="17" t="s">
+      <c r="B25" s="18" t="s">
         <v>249</v>
       </c>
-      <c r="C25" s="17" t="s">
+      <c r="C25" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="D25" s="17" t="s">
+      <c r="D25" s="18" t="s">
         <v>250</v>
       </c>
-      <c r="E25" s="17" t="s">
+      <c r="E25" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="F25" s="17" t="s">
+      <c r="F25" s="18" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="17" t="s">
+    <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="18" t="s">
         <v>252</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="18" t="s">
         <v>253</v>
       </c>
-      <c r="C26" s="17" t="s">
+      <c r="C26" s="18" t="s">
         <v>177</v>
       </c>
-      <c r="D26" s="17" t="s">
+      <c r="D26" s="18" t="s">
         <v>254</v>
       </c>
-      <c r="E26" s="17" t="s">
+      <c r="E26" s="18" t="s">
         <v>255</v>
       </c>
-      <c r="F26" s="17" t="s">
+      <c r="F26" s="18" t="s">
         <v>256</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="17" t="s">
+    <row r="27" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="18" t="s">
         <v>257</v>
       </c>
-      <c r="B27" s="17" t="s">
+      <c r="B27" s="18" t="s">
         <v>258</v>
       </c>
-      <c r="C27" s="17" t="s">
+      <c r="C27" s="18" t="s">
         <v>193</v>
       </c>
-      <c r="D27" s="17" t="s">
+      <c r="D27" s="18" t="s">
         <v>194</v>
       </c>
-      <c r="E27" s="17" t="s">
+      <c r="E27" s="18" t="s">
         <v>259</v>
       </c>
-      <c r="F27" s="17" t="s">
+      <c r="F27" s="18" t="s">
         <v>260</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: add F-009 brief — console login for console-created admin users
Registers F-009 in feature-value-scoring.xlsx (status: Brief Drafted) with
the brief at briefs/F-009-console-login-for-console-created-admin-users.md.
Timing ruled ASAP by product owner: blocker for go-to-market and for testing
the console under multiple admin accounts. Scoring columns left empty for
/prioritize-features.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -3010,10 +3010,26 @@
       </c>
     </row>
     <row r="18" ht="14.25" customHeight="1">
-      <c r="A18" s="21" t="n"/>
-      <c r="B18" s="22" t="n"/>
-      <c r="C18" s="21" t="n"/>
-      <c r="D18" s="21" t="n"/>
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>F-009</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>Console login for console-created admin users</t>
+        </is>
+      </c>
+      <c r="C18" s="21" t="inlineStr">
+        <is>
+          <t>briefs/F-009-console-login-for-console-created-admin-users.md</t>
+        </is>
+      </c>
+      <c r="D18" s="21" t="inlineStr">
+        <is>
+          <t>Brief Drafted</t>
+        </is>
+      </c>
       <c r="E18" s="21" t="n"/>
       <c r="F18" s="21" t="n"/>
       <c r="G18" s="24" t="n"/>
@@ -3045,6 +3061,11 @@
       <c r="U18" s="29">
         <f>IF(T18="","",RANK(T18,$T$4:$T$52))</f>
         <v/>
+      </c>
+      <c r="V18" s="32" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
       </c>
     </row>
     <row r="19" ht="14.25" customHeight="1">

</xml_diff>

<commit_message>
chore: research scoring for F-009 and D-005 (prioritization run 2026-07-19)
Market-research-agent RESEARCH pass applied by /prioritize-features:
- F-009: reach 4, user_value 6, business_value 4, time_sensitivity 9,
  confidence 5 -> Scored (awaits human strategic_alignment/effort/risk)
- D-005: reach 1, confidence 10 -> Scored (severity 1 human-set; score 7.5)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -2880,11 +2880,19 @@
       </c>
       <c r="D16" s="21" t="inlineStr">
         <is>
-          <t>Triaged</t>
-        </is>
-      </c>
-      <c r="E16" s="21" t="n"/>
-      <c r="F16" s="21" t="n"/>
+          <t>Scored</t>
+        </is>
+      </c>
+      <c r="E16" s="21" t="inlineStr">
+        <is>
+          <t>Market Research Agent</t>
+        </is>
+      </c>
+      <c r="F16" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
       <c r="G16" s="24" t="n">
         <v>1</v>
       </c>
@@ -2894,17 +2902,23 @@
         <v>5</v>
       </c>
       <c r="K16" s="24" t="n"/>
-      <c r="L16" s="24" t="n"/>
+      <c r="L16" s="24" t="n">
+        <v>10</v>
+      </c>
       <c r="M16" s="24" t="n">
         <v>1</v>
       </c>
       <c r="N16" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="O16" s="26" t="n"/>
+      <c r="O16" s="26" t="inlineStr">
+        <is>
+          <t>GH issue dispatch-derek/admin-console#10 (gh issue view 10); re-verified 2026-07-19 by code inspection: envDump interface bff/src/engine/adapter.ts:57, impl :242-245 wrapping /system/env-dump (:243); grep '\.envDump(' bff/src -&gt; 0 callers; survives as 11 mock refs across 9 test files (bff/test/routes/*, bff/test/services/baseline.service.test.ts); fix already landed at bff/src/services/settings.service.ts:341 (getEnvDump -&gt; adapter.getSystem()).</t>
+        </is>
+      </c>
       <c r="P16" s="26" t="inlineStr">
         <is>
-          <t>[intake 2026-07-15] Found while fixing the Diagnostics 'Load env dump' 500. Root cause of that 500 was adapter.request() calling JSON.parse on the engine's non-JSON 'OK' body; fixed by sourcing getEnvDump() from GET /v1/system (bff/src/services/settings.service.ts:336). Remaining dead code: EngineAdapter.envDump interface method (bff/src/engine/adapter.ts:57) + HttpEngineAdapter.envDump impl (~:242) wrapping /system/env-dump, now uncalled by any service. Referenced only by ~8 vitest adapter mocks (test/routes/*.test.ts, test/services/baseline.service.test.ts). Removal candidate; no runtime behavior change. Engine source: anything-llm/server/endpoints/api/system/index.js:16.</t>
+          <t>reach=1 (anchor 1 'rare edge case': dead code, zero runtime callers, 0% of operators affected; original 500 already fixed by repointing getEnvDump). confidence=10 (anchor 10 'validated': exhaustive static verification of a typed codebase — whole-tree grep for call sites yields none; mocks and landed fix confirmed at cited lines).</t>
         </is>
       </c>
       <c r="Q16" s="27">
@@ -3027,21 +3041,47 @@
       </c>
       <c r="D18" s="21" t="inlineStr">
         <is>
-          <t>Brief Drafted</t>
-        </is>
-      </c>
-      <c r="E18" s="21" t="n"/>
-      <c r="F18" s="21" t="n"/>
-      <c r="G18" s="24" t="n"/>
-      <c r="H18" s="24" t="n"/>
-      <c r="I18" s="24" t="n"/>
+          <t>Scored</t>
+        </is>
+      </c>
+      <c r="E18" s="21" t="inlineStr">
+        <is>
+          <t>Market Research Agent</t>
+        </is>
+      </c>
+      <c r="F18" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="G18" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="H18" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="I18" s="24" t="n">
+        <v>4</v>
+      </c>
       <c r="J18" s="24" t="n"/>
-      <c r="K18" s="24" t="n"/>
-      <c r="L18" s="24" t="n"/>
+      <c r="K18" s="24" t="n">
+        <v>9</v>
+      </c>
+      <c r="L18" s="24" t="n">
+        <v>5</v>
+      </c>
       <c r="M18" s="24" t="n"/>
       <c r="N18" s="24" t="n"/>
-      <c r="O18" s="26" t="n"/>
-      <c r="P18" s="26" t="n"/>
+      <c r="O18" s="26" t="inlineStr">
+        <is>
+          <t>Re-verified in-repo 2026-07-19: bff/src/routes/auth.routes.ts:133 (login resolves only staffRepo.findByUsername); bff/src/services/user.service.ts:101-135 (createUser writes engine only, no staff row); bff/src/auth/bootstrap.ts:11-20 (single bootstrap account when staff count==0); web/src/features/ has no staff feature; web/src/api/client.ts:127,131 listStaff/createStaff unconsumed. Firsthand operator report 2026-07-19 (brief), single known deployment/operator. Product-owner timing ruling 2026-07-19: ASAP, go-to-market blocker gating multi-operator testing.</t>
+        </is>
+      </c>
+      <c r="P18" s="26" t="inlineStr">
+        <is>
+          <t>Scored against console operators as target population. reach=4 ('5-15% or infrequent use'; onboarding-frequency, N=1 deployment today — 3 was arguable). user_value=6 (real pain, clumsy workaround: hand-rolled POST /api/staff + silent-failure UX; held below 7 as pain is onboarding-frequency, not frequent). business_value=4 (indirect GTM precondition, explicitly unquantified — not inflated; confidence carries the uncertainty). time_sensitivity=9 (ASAP/within-quarter window; not 10 — no external hard deadline). confidence=5 (mechanism code-verified, demand side N=1, no tickets/analytics).</t>
+        </is>
+      </c>
       <c r="Q18" s="27">
         <f>IF(V18="Defect","",IF(COUNT(G18:K18)&lt;5,"",ROUND(G18*Config!$B$4+H18*Config!$B$5+I18*Config!$B$6+J18*Config!$B$7+K18*Config!$B$8,2)))</f>
         <v/>

</xml_diff>

<commit_message>
chore: prioritization run 2026-07-19 — D-005 Prioritized, F-009 held for risk sign-off
feature-prioritizer recommendations applied by /prioritize-features:
- D-005 (dead-code envDump cleanup): Scored -> Prioritized (score 7.5, rank 10)
- F-009 (console admin login): stays Scored, flagged risk>=9 (human-set risk=10)
  pending sign-off; score 7.0, rank 11

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -2880,7 +2880,7 @@
       </c>
       <c r="D16" s="21" t="inlineStr">
         <is>
-          <t>Scored</t>
+          <t>Prioritized</t>
         </is>
       </c>
       <c r="E16" s="21" t="inlineStr">
@@ -3063,15 +3063,21 @@
       <c r="I18" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="J18" s="24" t="n"/>
+      <c r="J18" s="24" t="n">
+        <v>7</v>
+      </c>
       <c r="K18" s="24" t="n">
         <v>9</v>
       </c>
       <c r="L18" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="M18" s="24" t="n"/>
-      <c r="N18" s="24" t="n"/>
+      <c r="M18" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="N18" s="24" t="n">
+        <v>10</v>
+      </c>
       <c r="O18" s="26" t="inlineStr">
         <is>
           <t>Re-verified in-repo 2026-07-19: bff/src/routes/auth.routes.ts:133 (login resolves only staffRepo.findByUsername); bff/src/services/user.service.ts:101-135 (createUser writes engine only, no staff row); bff/src/auth/bootstrap.ts:11-20 (single bootstrap account when staff count==0); web/src/features/ has no staff feature; web/src/api/client.ts:127,131 listStaff/createStaff unconsumed. Firsthand operator report 2026-07-19 (brief), single known deployment/operator. Product-owner timing ruling 2026-07-19: ASAP, go-to-market blocker gating multi-operator testing.</t>

</xml_diff>

<commit_message>
chore: F-009 risk sign-off — risk 10->5, status Prioritized
Product owner resolved the risk>=9 review flag from the 2026-07-19
prioritization run: risk revised to 5. Flag cleared; prioritizer's
recommendation applied. New priority_score 9.9, rank 9.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -3041,7 +3041,7 @@
       </c>
       <c r="D18" s="21" t="inlineStr">
         <is>
-          <t>Scored</t>
+          <t>Prioritized</t>
         </is>
       </c>
       <c r="E18" s="21" t="inlineStr">
@@ -3076,7 +3076,7 @@
         <v>7</v>
       </c>
       <c r="N18" s="24" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="O18" s="26" t="inlineStr">
         <is>
@@ -3085,7 +3085,7 @@
       </c>
       <c r="P18" s="26" t="inlineStr">
         <is>
-          <t>Scored against console operators as target population. reach=4 ('5-15% or infrequent use'; onboarding-frequency, N=1 deployment today — 3 was arguable). user_value=6 (real pain, clumsy workaround: hand-rolled POST /api/staff + silent-failure UX; held below 7 as pain is onboarding-frequency, not frequent). business_value=4 (indirect GTM precondition, explicitly unquantified — not inflated; confidence carries the uncertainty). time_sensitivity=9 (ASAP/within-quarter window; not 10 — no external hard deadline). confidence=5 (mechanism code-verified, demand side N=1, no tickets/analytics).</t>
+          <t>Scored against console operators as target population. reach=4 ('5-15% or infrequent use'; onboarding-frequency, N=1 deployment today — 3 was arguable). user_value=6 (real pain, clumsy workaround: hand-rolled POST /api/staff + silent-failure UX; held below 7 as pain is onboarding-frequency, not frequent). business_value=4 (indirect GTM precondition, explicitly unquantified — not inflated; confidence carries the uncertainty). time_sensitivity=9 (ASAP/within-quarter window; not 10 — no external hard deadline). confidence=5 (mechanism code-verified, demand side N=1, no tickets/analytics). | Human sign-off 2026-07-19 (risk&gt;=9 flag review): risk revised 10 -&gt; 5 by product owner; flag cleared; status -&gt; Prioritized.</t>
         </is>
       </c>
       <c r="Q18" s="27">

</xml_diff>

<commit_message>
docs: add F-007 and F-008 briefs; register rows as Brief Drafted
F-007 (admin-console UI i18n): market-expansion driver, GTM-tied; scoped to
the operator console per ruling — customer-web-app localization gets its own
row in its own pipeline. Includes discovery signals (0 i18n deps, >=48 inline
strings, upstream 26-locale catalog) and ux-designer reads.

F-008 (system-wide scheduled backups): covers admin-console, AnythingLLM
engine, customer-web-app, and the locally installed Ollama (models + data)
per product-owner scope rulings (quoted verbatim). Spec writer directed to
evaluate Apple Business Manager fleet management + iCloud as backup
destination for feasibility. Includes persistence-inventory discovery
signals and ux-designer reads (UI optional/deferrable; restore flow is the
risk concentration).

Scoring columns untouched; both rows ready for /prioritize-features.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -2657,10 +2657,14 @@
           <t>Multi-language and number format internationalization support in the user interface</t>
         </is>
       </c>
-      <c r="C13" s="21" t="n"/>
+      <c r="C13" s="21" t="inlineStr">
+        <is>
+          <t>briefs/F-007-ui-internationalization.md</t>
+        </is>
+      </c>
       <c r="D13" s="21" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Brief Drafted</t>
         </is>
       </c>
       <c r="E13" s="21" t="n"/>
@@ -2807,10 +2811,14 @@
           <t>System-wide backups on schedule</t>
         </is>
       </c>
-      <c r="C15" s="21" t="n"/>
+      <c r="C15" s="21" t="inlineStr">
+        <is>
+          <t>briefs/F-008-system-wide-scheduled-backups.md</t>
+        </is>
+      </c>
       <c r="D15" s="21" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Brief Drafted</t>
         </is>
       </c>
       <c r="E15" s="21" t="n"/>

</xml_diff>

<commit_message>
chore: research scoring for F-007 and F-008 (prioritization run 2026-07-19 PM)
Market-research-agent RESEARCH pass applied by /prioritize-features:
- F-007 (UI i18n): reach 2, user_value 6, business_value 8,
  time_sensitivity 3, confidence 4 -> Scored
- F-008 (scheduled backups): reach 8, user_value 6, business_value 7,
  time_sensitivity 5, confidence 6 -> Scored

Ranking paused pending human confirmation of pre-existing
strategic_alignment/effort/risk values on both rows.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -2664,29 +2664,51 @@
       </c>
       <c r="D13" s="21" t="inlineStr">
         <is>
-          <t>Brief Drafted</t>
-        </is>
-      </c>
-      <c r="E13" s="21" t="n"/>
-      <c r="F13" s="21" t="n"/>
-      <c r="G13" s="24" t="n"/>
-      <c r="H13" s="24" t="n"/>
-      <c r="I13" s="24" t="n"/>
+          <t>Scored</t>
+        </is>
+      </c>
+      <c r="E13" s="21" t="inlineStr">
+        <is>
+          <t>Market Research Agent</t>
+        </is>
+      </c>
+      <c r="F13" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="G13" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="I13" s="24" t="n">
+        <v>8</v>
+      </c>
       <c r="J13" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="K13" s="24" t="n"/>
-      <c r="L13" s="24" t="n"/>
+      <c r="K13" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="L13" s="24" t="n">
+        <v>4</v>
+      </c>
       <c r="M13" s="24" t="n">
         <v>1</v>
       </c>
       <c r="N13" s="24" t="n">
         <v>1</v>
       </c>
-      <c r="O13" s="26" t="n"/>
+      <c r="O13" s="26" t="inlineStr">
+        <is>
+          <t>Re-verified 2026-07-19: web/package.json zero i18n deps (react, react-dom, @phosphor-icons only); no locale/i18n/.po files under web/; exactly 2 default-locale format sites (DiagnosticsPage.tsx:49, BaselineEditor.tsx:110); zero explicit-Intl/navigator.language/Accept-Language across 111 TS/TSX files; 56 inline JSX text nodes matched across 21 tsx files (confirms brief's &gt;=48 lower bound). Upstream: anything-llm frontend/src/locales ~26 locale folders + translation scripts (verified); upstream issue #1371 non-English UI request (verified). Zero inbound localization requests for this fork (no ticketing channel exists; nothing in docs/README/CHANGELOG).</t>
+        </is>
+      </c>
       <c r="P13" s="26" t="inlineStr">
         <is>
-          <t>Establising the capability to support languages and number formats based on the users locale is easiest to implement at the beginning of developing a software product vs retrofitting it in later, even if there is no need to display any other language than English currently.</t>
+          <t>reach=2 (population-share floor: ~0% observed non-English operators, prospective fraction unsized/undated; DISSENT: broad whole-UI capability arguably higher — a dated market-entry commitment should trigger reach re-score upward). user_value=6 (real per-session friction for non-English operator, clumsy-not-blocking workaround). business_value=8 (table-stakes enabler of stated market expansion; not 9-10 — enabler, not the market-opener, unsized). time_sensitivity=3 (GTM-tied but NO date supplied; value decays slowly; re-score if dates arrive). confidence=4 (current-state gap code-verified, but demand hypothesis rests on upstream analogs only; zero fork-specific demand signals).</t>
         </is>
       </c>
       <c r="Q13" s="27">
@@ -2818,27 +2840,53 @@
       </c>
       <c r="D15" s="21" t="inlineStr">
         <is>
-          <t>Brief Drafted</t>
-        </is>
-      </c>
-      <c r="E15" s="21" t="n"/>
-      <c r="F15" s="21" t="n"/>
-      <c r="G15" s="24" t="n"/>
-      <c r="H15" s="24" t="n"/>
-      <c r="I15" s="24" t="n"/>
+          <t>Scored</t>
+        </is>
+      </c>
+      <c r="E15" s="21" t="inlineStr">
+        <is>
+          <t>Market Research Agent</t>
+        </is>
+      </c>
+      <c r="F15" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="G15" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="H15" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="I15" s="24" t="n">
+        <v>7</v>
+      </c>
       <c r="J15" s="24" t="n">
         <v>10</v>
       </c>
-      <c r="K15" s="24" t="n"/>
-      <c r="L15" s="24" t="n"/>
+      <c r="K15" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="L15" s="24" t="n">
+        <v>6</v>
+      </c>
       <c r="M15" s="24" t="n">
         <v>5</v>
       </c>
       <c r="N15" s="24" t="n">
         <v>8</v>
       </c>
-      <c r="O15" s="26" t="n"/>
-      <c r="P15" s="26" t="n"/>
+      <c r="O15" s="26" t="inlineStr">
+        <is>
+          <t>Re-verified 2026-07-19: zero backup/restore/snapshot/VACUUM-INTO capability in admin-console AND /home/derek/git/customer-web-app (all hits unrelated: env-dump diagnostics, vitest fixtures). settings-map.ts:39-43 Ollama managed over-the-wire only; zero references to Ollama on-disk storage in either repo. db-path.ts:8 DB_PATH default data/console.db shared by BFF+relay. Manual-backup preconditions exist in TWO runbooks (F-004:86, F-005:90) — brief's 'three' is overstated, F-002 runbook has none. git log --all: zero incident/drill history (only the brief commit itself). No deployment descriptors in either repo. Brief: briefs/F-008-system-wide-scheduled-backups.md (PO scope rulings 2026-07-19 incl. Ollama + ABM/iCloud investigation).</t>
+        </is>
+      </c>
+      <c r="P15" s="26" t="inlineStr">
+        <is>
+          <t>reach=8 (judgment placement: breadth maximal — 100% of users of all three apps bear continuous data-loss exposure — but anchors 9-10 reward active daily interaction which a background DR capability lacks; pure-breadth reading defends 9-10, reviewer may override either way). user_value=6 (catastrophic-but-latent pain; zero experienced loss events; 7-8 require frequent pain). business_value=7 (production-readiness/GTM enabler + tail-risk defense; GTM milestone unconfirmed, no incident/contract evidence for higher). time_sensitivity=5 (undated production gate; rises 6-7 if near-term GTM date confirmed). confidence=6 (gap existence code-verified ~certain; value magnitude/urgency directional with no incident history; anchored to the weaker evidence class). DISSENT: if PO confirms hard near-term GTM gate, business_value and time_sensitivity are under-scored - re-score then.</t>
+        </is>
+      </c>
       <c r="Q15" s="27">
         <f>IF(V15="Defect","",IF(COUNT(G15:K15)&lt;5,"",ROUND(G15*Config!$B$4+H15*Config!$B$5+I15*Config!$B$6+J15*Config!$B$7+K15*Config!$B$8,2)))</f>
         <v/>

</xml_diff>

<commit_message>
chore: F-007 and F-008 Scored -> Prioritized (run 2026-07-19 PM)
Human-gate values confirmed by product owner (F-007 sa7/e2/r2, F-008
sa10/e4/r7). feature-prioritizer recommendations applied:
- F-007 (UI i18n): 36.4, rank 3 — advisory flag: confirm dated GTM
  commitment behind business_value=8 before spec spend
- F-008 (scheduled backups): 22.1, rank 6 — advisory flag: sa=10
  discounted by effort/risk; revisit after ABM/iCloud scoping

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -2664,7 +2664,7 @@
       </c>
       <c r="D13" s="21" t="inlineStr">
         <is>
-          <t>Scored</t>
+          <t>Prioritized</t>
         </is>
       </c>
       <c r="E13" s="21" t="inlineStr">
@@ -2687,7 +2687,7 @@
         <v>8</v>
       </c>
       <c r="J13" s="24" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K13" s="24" t="n">
         <v>3</v>
@@ -2696,10 +2696,10 @@
         <v>4</v>
       </c>
       <c r="M13" s="24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N13" s="24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O13" s="26" t="inlineStr">
         <is>
@@ -2840,7 +2840,7 @@
       </c>
       <c r="D15" s="21" t="inlineStr">
         <is>
-          <t>Scored</t>
+          <t>Prioritized</t>
         </is>
       </c>
       <c r="E15" s="21" t="inlineStr">
@@ -2872,10 +2872,10 @@
         <v>6</v>
       </c>
       <c r="M15" s="24" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N15" s="24" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="O15" s="26" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore: fix F-006 row data — item_type Defect -> Feature
Product-owner ruling (implicit in /write-feature-brief F-006 dispatch):
F-006 is a Feature idea. Cleared Defect-only fields (severity,
defect_source) that made the row invalid for either pipeline path.
Status remains Idea pending brief.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -2545,16 +2545,8 @@
       </c>
       <c r="V11" s="32" t="inlineStr">
         <is>
-          <t>Defect</t>
-        </is>
-      </c>
-      <c r="W11" t="inlineStr">
-        <is>
-          <t>Internal</t>
-        </is>
-      </c>
-      <c r="X11" t="n">
-        <v>2</v>
+          <t>Feature</t>
+        </is>
       </c>
     </row>
     <row r="12" ht="95.25" customHeight="1">

</xml_diff>

<commit_message>
docs: add F-006 brief — local-first per-workspace LLM observability
Registers F-006 (row repaired to Feature earlier on this branch) as Brief
Drafted. Consumers: ops/capacity planning, customer-facing reporting,
troubleshooting (billing explicitly excluded). Hard zero-cloud constraint
per appliance value proposition (data stays in Canada / on device).
Discovery: no per-workspace metrics exist anywhere today; Ollama emits 6
per-request metric fields only the engine can see (the load-bearing open
question). Fleet at launch: <5 appliances. Scoring columns untouched.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -2500,13 +2500,17 @@
       </c>
       <c r="B11" s="22" t="inlineStr">
         <is>
-          <t>Implement a local-first, zero-cloud dependency observability mechanism for tracking LLM usage, performance metrics, and resource load per individual customer workspace.</t>
-        </is>
-      </c>
-      <c r="C11" s="21" t="n"/>
+          <t>Local-first per-workspace LLM observability (usage, performance, resource load)</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="inlineStr">
+        <is>
+          <t>briefs/F-006-local-first-workspace-llm-observability.md</t>
+        </is>
+      </c>
       <c r="D11" s="21" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Brief Drafted</t>
         </is>
       </c>
       <c r="E11" s="21" t="n"/>

</xml_diff>

<commit_message>
chore: research scoring for F-006 (prioritization run 2026-07-19 evening)
Market-research-agent RESEARCH pass applied by /prioritize-features:
F-006 (local-first observability): reach 6, user_value 7, business_value 5,
time_sensitivity 4, confidence 5 -> Scored. Ranking paused at human gate
(effort/risk missing; strategic_alignment=5 predates the brief).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -2510,23 +2510,49 @@
       </c>
       <c r="D11" s="21" t="inlineStr">
         <is>
-          <t>Brief Drafted</t>
-        </is>
-      </c>
-      <c r="E11" s="21" t="n"/>
-      <c r="F11" s="21" t="n"/>
-      <c r="G11" s="24" t="n"/>
-      <c r="H11" s="24" t="n"/>
-      <c r="I11" s="24" t="n"/>
+          <t>Scored</t>
+        </is>
+      </c>
+      <c r="E11" s="21" t="inlineStr">
+        <is>
+          <t>Market Research Agent</t>
+        </is>
+      </c>
+      <c r="F11" s="21" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="G11" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="H11" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="I11" s="24" t="n">
+        <v>5</v>
+      </c>
       <c r="J11" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="K11" s="24" t="n"/>
-      <c r="L11" s="24" t="n"/>
+      <c r="K11" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="L11" s="24" t="n">
+        <v>5</v>
+      </c>
       <c r="M11" s="24" t="n"/>
       <c r="N11" s="24" t="n"/>
-      <c r="O11" s="26" t="n"/>
-      <c r="P11" s="26" t="n"/>
+      <c r="O11" s="26" t="inlineStr">
+        <is>
+          <t>Re-verified in-repo 2026-07-19 (first-hand): DiagnosticsPage.tsx:1-75 (2 instance-scoped facts, 0 per-workspace/time-series); relay/metrics.ts:1-68 (relay-delivery scope only); bff+web package.json (zero telemetry/charting deps); oversight.service.ts:13-27 + mappers.ts:229-231 + engine-types.ts:97-105 (chats passed as opaque unknown[], 0 metric fields parsed); events/catalog.ts AdminEventName union = 21 config/CRUD names, none usage/perf (brief said 20; substance holds). Carried from brief (not re-fetched): engine event_logs session-auth-only + workspace_chats blob-embedded timing (docs/anythingllm-surface.md:205-219); Ollama /api/generate 6 metric fields + /api/ps (ollama docs). Human-supplied: fleet &lt;5 appliances; three-consumer framing; zero-cloud constraint (PO 2026-07-19).</t>
+        </is>
+      </c>
+      <c r="P11" s="26" t="inlineStr">
+        <is>
+          <t>reach=6 (breadth-vs-frequency tension: all 3 personas exposed per deployment, but consumption episodic — capacity periodic, reporting periodic, troubleshooting incident-driven; breadth reading could argue 7). user_value=7 (troubleshooting has NO workaround — data gone once event passes; capacity is wait-for-complaint; customer reporting is a new JTBD nudging 8, held at 7 as value diffuse across episodic cases). business_value=5 (billing/metering excluded by PO so revenue argument off the table; support/ops cost + reporting satisfaction, indirect and small at &lt;5 appliances; GTM-gate not established — brief's own ops-minimum question). time_sensitivity=4 (no date/window supplied; GTM coupling real but unquantified — re-score if launch date lands). confidence=5 (gap proven multi-source in-repo; value framing single-stakeholder, usage data structurally unavailable at this fleet size; unresolved metric-capture point bleeds feasibility uncertainty into value confidence).</t>
+        </is>
+      </c>
       <c r="Q11" s="27">
         <f>IF(V11="Defect","",IF(COUNT(G11:K11)&lt;5,"",ROUND(G11*Config!$B$4+H11*Config!$B$5+I11*Config!$B$6+J11*Config!$B$7+K11*Config!$B$8,2)))</f>
         <v/>

</xml_diff>

<commit_message>
chore: F-006 Scored -> Deferred (score 12.4, rank 11)
Human-gate values from product owner (sa 7 / effort 6 / risk 5).
feature-prioritizer recommendation applied: Deferred — gap is code-proven
but value is GTM-undated, business_value narrow at <5 appliances with
billing excluded, and the metric-capture architecture is unresolved.
Revisit when a GTM date lands or F-008 spec work settles the capture point.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -2510,7 +2510,7 @@
       </c>
       <c r="D11" s="21" t="inlineStr">
         <is>
-          <t>Scored</t>
+          <t>Deferred</t>
         </is>
       </c>
       <c r="E11" s="21" t="inlineStr">
@@ -2533,7 +2533,7 @@
         <v>5</v>
       </c>
       <c r="J11" s="24" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="K11" s="24" t="n">
         <v>4</v>
@@ -2541,8 +2541,12 @@
       <c r="L11" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="M11" s="24" t="n"/>
-      <c r="N11" s="24" t="n"/>
+      <c r="M11" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="N11" s="24" t="n">
+        <v>5</v>
+      </c>
       <c r="O11" s="26" t="inlineStr">
         <is>
           <t>Re-verified in-repo 2026-07-19 (first-hand): DiagnosticsPage.tsx:1-75 (2 instance-scoped facts, 0 per-workspace/time-series); relay/metrics.ts:1-68 (relay-delivery scope only); bff+web package.json (zero telemetry/charting deps); oversight.service.ts:13-27 + mappers.ts:229-231 + engine-types.ts:97-105 (chats passed as opaque unknown[], 0 metric fields parsed); events/catalog.ts AdminEventName union = 21 config/CRUD names, none usage/perf (brief said 20; substance holds). Carried from brief (not re-fetched): engine event_logs session-auth-only + workspace_chats blob-embedded timing (docs/anythingllm-surface.md:205-219); Ollama /api/generate 6 metric fields + /api/ps (ollama docs). Human-supplied: fleet &lt;5 appliances; three-consumer framing; zero-cloud constraint (PO 2026-07-19).</t>

</xml_diff>

<commit_message>
chore: F-006 business_value 5->6 (Hybrid re-score); Deferred -> Prioritized
Agent re-score against the revised brief (PO revenue-via-reporting ruling):
business_value 6 (anchor 6 retention/revenue class; held below 7+ pending
customer evidence); confidence unchanged at 5. Score 12.4 -> 12.9, rank 11.
Status Deferred -> Prioritized by explicit product-owner override; the
prioritizer's sequencing caveats (capture point, GTM date) remain recorded.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -2510,12 +2510,12 @@
       </c>
       <c r="D11" s="21" t="inlineStr">
         <is>
-          <t>Deferred</t>
+          <t>Prioritized</t>
         </is>
       </c>
       <c r="E11" s="21" t="inlineStr">
         <is>
-          <t>Market Research Agent</t>
+          <t>Hybrid</t>
         </is>
       </c>
       <c r="F11" s="21" t="inlineStr">
@@ -2530,7 +2530,7 @@
         <v>7</v>
       </c>
       <c r="I11" s="24" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J11" s="24" t="n">
         <v>7</v>
@@ -2549,12 +2549,12 @@
       </c>
       <c r="O11" s="26" t="inlineStr">
         <is>
-          <t>Re-verified in-repo 2026-07-19 (first-hand): DiagnosticsPage.tsx:1-75 (2 instance-scoped facts, 0 per-workspace/time-series); relay/metrics.ts:1-68 (relay-delivery scope only); bff+web package.json (zero telemetry/charting deps); oversight.service.ts:13-27 + mappers.ts:229-231 + engine-types.ts:97-105 (chats passed as opaque unknown[], 0 metric fields parsed); events/catalog.ts AdminEventName union = 21 config/CRUD names, none usage/perf (brief said 20; substance holds). Carried from brief (not re-fetched): engine event_logs session-auth-only + workspace_chats blob-embedded timing (docs/anythingllm-surface.md:205-219); Ollama /api/generate 6 metric fields + /api/ps (ollama docs). Human-supplied: fleet &lt;5 appliances; three-consumer framing; zero-cloud constraint (PO 2026-07-19).</t>
+          <t>Re-verified in-repo 2026-07-19 (first-hand): DiagnosticsPage.tsx:1-75 (2 instance-scoped facts, 0 per-workspace/time-series); relay/metrics.ts:1-68 (relay-delivery scope only); bff+web package.json (zero telemetry/charting deps); oversight.service.ts:13-27 + mappers.ts:229-231 + engine-types.ts:97-105 (chats passed as opaque unknown[], 0 metric fields parsed); events/catalog.ts AdminEventName union = 21 config/CRUD names, none usage/perf (brief said 20; substance holds). Carried from brief (not re-fetched): engine event_logs session-auth-only + workspace_chats blob-embedded timing (docs/anythingllm-surface.md:205-219); Ollama /api/generate 6 metric fields + /api/ps (ollama docs). Human-supplied: fleet &lt;5 appliances; three-consumer framing; zero-cloud constraint (PO 2026-07-19). | Addendum 2026-07-19: brief Business Rationale revised — PO verbatim ruling that observability data benefits revenue via customer-facing reports/dashboards (briefs/F-006-local-first-workspace-llm-observability.md, 'Product-owner addition, 2026-07-19' + packaged/paid-vs-included Open Question).</t>
         </is>
       </c>
       <c r="P11" s="26" t="inlineStr">
         <is>
-          <t>reach=6 (breadth-vs-frequency tension: all 3 personas exposed per deployment, but consumption episodic — capacity periodic, reporting periodic, troubleshooting incident-driven; breadth reading could argue 7). user_value=7 (troubleshooting has NO workaround — data gone once event passes; capacity is wait-for-complaint; customer reporting is a new JTBD nudging 8, held at 7 as value diffuse across episodic cases). business_value=5 (billing/metering excluded by PO so revenue argument off the table; support/ops cost + reporting satisfaction, indirect and small at &lt;5 appliances; GTM-gate not established — brief's own ops-minimum question). time_sensitivity=4 (no date/window supplied; GTM coupling real but unquantified — re-score if launch date lands). confidence=5 (gap proven multi-source in-repo; value framing single-stakeholder, usage data structurally unavailable at this fleet size; unresolved metric-capture point bleeds feasibility uncertainty into value confidence).</t>
+          <t>reach=6 (breadth-vs-frequency tension: all 3 personas exposed per deployment, but consumption episodic — capacity periodic, reporting periodic, troubleshooting incident-driven; breadth reading could argue 7). user_value=7 (troubleshooting has NO workaround — data gone once event passes; capacity is wait-for-complaint; customer reporting is a new JTBD nudging 8, held at 7 as value diffuse across episodic cases). business_value=5 (billing/metering excluded by PO so revenue argument off the table; support/ops cost + reporting satisfaction, indirect and small at &lt;5 appliances; GTM-gate not established — brief's own ops-minimum question). time_sensitivity=4 (no date/window supplied; GTM coupling real but unquantified — re-score if launch date lands). confidence=5 (gap proven multi-source in-repo; value framing single-stakeholder, usage data structurally unavailable at this fleet size; unresolved metric-capture point bleeds feasibility uncertainty into value confidence). | [re-score 2026-07-19, Hybrid] business_value 5-&gt;6: PO ruling reframes billing exclusion — metering out, but customer-facing reports/dashboards = revenue-benefiting retention capability (anchor 6 'conversion, retention, or cost'); held below 7+ (single-stakeholder hypothesis, no adoption/willingness-to-pay evidence, packaged-vs-included unresolved). Confidence unchanged at 5. | Human override 2026-07-19: Deferred -&gt; Prioritized by product owner (revenue-via-reporting thesis); prioritizer's sequencing caveats stand (capture point unresolved, GTM undated).</t>
         </is>
       </c>
       <c r="Q11" s="27">

</xml_diff>

<commit_message>
chore: mark F-010 In Progress for implement-spec run
Excludes the row from /prioritize-features while implementation is in flight.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSQAV9AspmwvxZ78jg9QNx
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="390">
   <si>
     <t xml:space="preserve">FEATURE VALUE SCORING FRAMEWORK</t>
   </si>
@@ -792,6 +792,9 @@
   </si>
   <si>
     <t xml:space="preserve">briefs/F-010-deliver-admin-events-to-customer-web-app.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In Progress</t>
   </si>
   <si>
     <t xml:space="preserve">2026-07-20</t>
@@ -3911,13 +3914,13 @@
         <v>255</v>
       </c>
       <c r="D19" s="22" t="s">
-        <v>171</v>
+        <v>256</v>
       </c>
       <c r="E19" s="22" t="s">
         <v>172</v>
       </c>
       <c r="F19" s="22" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G19" s="25" t="n">
         <v>2</v>
@@ -3944,10 +3947,10 @@
         <v>5</v>
       </c>
       <c r="O19" s="27" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="P19" s="27" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="Q19" s="28" t="n">
         <f aca="false">IF(V19="Defect","",IF(COUNT(G19:K19)&lt;5,"",ROUND(G19*Config!$B$4+H19*Config!$B$5+I19*Config!$B$6+J19*Config!$B$7+K19*Config!$B$8,2)))</f>
@@ -3975,22 +3978,22 @@
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="22" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D20" s="22" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E20" s="22" t="s">
         <v>172</v>
       </c>
       <c r="F20" s="22" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G20" s="25" t="n">
         <v>5</v>
@@ -4017,10 +4020,10 @@
         <v>6</v>
       </c>
       <c r="O20" s="27" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="P20" s="27" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="Q20" s="28" t="n">
         <f aca="false">IF(V20="Defect","",IF(COUNT(G20:K20)&lt;5,"",ROUND(G20*Config!$B$4+H20*Config!$B$5+I20*Config!$B$6+J20*Config!$B$7+K20*Config!$B$8,2)))</f>
@@ -4048,22 +4051,22 @@
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="22" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C21" s="22" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D21" s="22" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E21" s="22" t="s">
         <v>172</v>
       </c>
       <c r="F21" s="22" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G21" s="25" t="n">
         <v>5</v>
@@ -4090,10 +4093,10 @@
         <v>6</v>
       </c>
       <c r="O21" s="27" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="P21" s="27" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="Q21" s="28" t="n">
         <f aca="false">IF(V21="Defect","",IF(COUNT(G21:K21)&lt;5,"",ROUND(G21*Config!$B$4+H21*Config!$B$5+I21*Config!$B$6+J21*Config!$B$7+K21*Config!$B$8,2)))</f>
@@ -4121,22 +4124,22 @@
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="22" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E22" s="22" t="s">
         <v>172</v>
       </c>
       <c r="F22" s="22" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G22" s="25" t="n">
         <v>4</v>
@@ -4163,10 +4166,10 @@
         <v>7</v>
       </c>
       <c r="O22" s="27" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="P22" s="27" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="Q22" s="28" t="n">
         <f aca="false">IF(V22="Defect","",IF(COUNT(G22:K22)&lt;5,"",ROUND(G22*Config!$B$4+H22*Config!$B$5+I22*Config!$B$6+J22*Config!$B$7+K22*Config!$B$8,2)))</f>
@@ -4194,16 +4197,16 @@
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="22" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D23" s="22" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E23" s="22"/>
       <c r="F23" s="22"/>
@@ -4216,10 +4219,10 @@
       <c r="M23" s="25"/>
       <c r="N23" s="25"/>
       <c r="O23" s="27" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="P23" s="27" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="Q23" s="28" t="str">
         <f aca="false">IF(V23="Defect","",IF(COUNT(G23:K23)&lt;5,"",ROUND(G23*Config!$B$4+H23*Config!$B$5+I23*Config!$B$6+J23*Config!$B$7+K23*Config!$B$8,2)))</f>
@@ -5439,507 +5442,507 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="37" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B3" s="37" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C3" s="37" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D3" s="37" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E3" s="37" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F3" s="37" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="F27" s="18" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: mark F-010 Implemented (implement-spec write-back)
Full pipeline green: bff 1300/1300, relay e2e 16/16, tsc clean; security
PASS WITH NOTES, code review APPROVE WITH COMMENTS. Provenance appended to
rationale_notes; status Prioritized -> In Progress -> Implemented.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSQAV9AspmwvxZ78jg9QNx
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="389">
   <si>
     <t xml:space="preserve">FEATURE VALUE SCORING FRAMEWORK</t>
   </si>
@@ -794,16 +794,13 @@
     <t xml:space="preserve">briefs/F-010-deliver-admin-events-to-customer-web-app.md</t>
   </si>
   <si>
-    <t xml:space="preserve">In Progress</t>
-  </si>
-  <si>
     <t xml:space="preserve">2026-07-20</t>
   </si>
   <si>
     <t xml:space="preserve">RE-VERIFIED 2026-07-20 (admin-console @2da1000, cwa @6044b46). STRUCTURAL (hard, first-hand): bff/src/relay/http-peer-transport.ts sends exactly 2 headers (content-type, x-event-delivery-id, const :10); grep secret/bearer/hmac/authorization/credential across bff/src/relay/ + bff/src/events/ = 0 credential code paths; bff/src/relay/config.ts exports 8 keys, none a secret; config.ts:13-17 split/trim/filter only, 0 scheme validation; config.ts:27-34 production hard-refuse on empty peer list. bff/.env:25 EVENT_BUS_MODE=inproc, 0 EVENT_BUS_URL lines. catalog.ts = 21 admin.* names, 5 admin.user.* (:15-19) = 23.8% of NAMES (not users). CONSUMER ABSENT: 0 hits for events/ingest in cwa bff/src (41 files, 9 route modules); spec-text only (cwa specs/F-005:133,187,192,272,591). cwa workbook 2026-07-20: F-005 In Progress rank4, F-007 Deferred rank2. Runbooks: 3 exist, 0 mentions of peer/secret/rotation in any. Test surface: 20 files bff/test/relay/; delivery-id assertion at http-peer-transport.test.ts:106 is containment, not exact-header-set. DEMAND ABSENT: admin-console gh issue list --state all = 5 issues, 0 related; cwa gh issue list = 0 issues; no analytics artifacts. October 2026: 29 matches/10 md files, 0 connect the date to this row.</t>
   </si>
   <si>
-    <t xml:space="preserve">Scored 2026-07-20 by re-verification, not inherited from the brief's 2026-07-19 snapshot; nothing material changed (no merges beyond the brief commit 2da1000, no cwa commits since 6044b46). reach=2: measured affected share today is 0% (no peer configured, consumer endpoint nonexistent). Declined to score off the 23.8% admin.user.* figure - that is a share of event NAMES, not users. Calibrates equal to cwa F-007 (reach=2), the mirror-image producer-side row. user_value=5: manual dual-provisioning in cwa is a real but tolerable workaround; no frequency measurement exists, so 4 is also defensible. business_value=4: effect is real but routed entirely through another repo's work; no metric attaches on this side; no revenue/usage/demand record. time_sensitivity=6: October 2026 is an internal company goal, not external/regulatory, concrete date unpinned - anchor 9/10 excluded outright. confidence=5: evidence quality is split - structural claims are hard first-hand fact, value-side claims have zero supporting data (no analytics/tickets/interviews/benchmarks). Value not inflated to offset; multiplier carries it. AGENT DISSENT FROM BRIEF (no score impact): the row's own note reads 'Config-only on the relay side ... PLUS credential provisioning/runbook' - it already scoped credential work in, so the brief's claim that the note is contradicted is overstated; the code-path gap itself is real and confirmed. Also: brief's '0 of 7 cwa rows Implemented on the ingest side' is imprecise (F-001 IS Implemented, just not the ingest endpoint). CARRIED FOR HUMAN (no proposal): D-006's recorded reach=1 basis (inproc, empty peer list, transport inactive) would stop describing reality if F-010 puts a live peer on the wire; D-006/GH#16 record no dependency on F-010. Credential header and env-var name unnamed on both sides = most likely source of a silent 401 permanent-park loop. COULD NOT VERIFY: the 2026-07-19 product-owner rulings exist only as prose inside briefs - no ticket/issue/decision-log artifact behind them. [write-spec-from-feature-brief 2026-07-22] spec drafted at specs/F-010-deliver-admin-events-to-customer-web-app.md; 19 functional / 5 non-functional requirements; 7 of 9 open questions resolved by human ruling (Q3 GTM-date and Q7 D-006-re-exam deferred to named owners); spec-reviewer PASS WITH NOTES (rev 3).</t>
+    <t xml:space="preserve">Scored 2026-07-20 by re-verification, not inherited from the brief's 2026-07-19 snapshot; nothing material changed (no merges beyond the brief commit 2da1000, no cwa commits since 6044b46). reach=2: measured affected share today is 0% (no peer configured, consumer endpoint nonexistent). Declined to score off the 23.8% admin.user.* figure - that is a share of event NAMES, not users. Calibrates equal to cwa F-007 (reach=2), the mirror-image producer-side row. user_value=5: manual dual-provisioning in cwa is a real but tolerable workaround; no frequency measurement exists, so 4 is also defensible. business_value=4: effect is real but routed entirely through another repo's work; no metric attaches on this side; no revenue/usage/demand record. time_sensitivity=6: October 2026 is an internal company goal, not external/regulatory, concrete date unpinned - anchor 9/10 excluded outright. confidence=5: evidence quality is split - structural claims are hard first-hand fact, value-side claims have zero supporting data (no analytics/tickets/interviews/benchmarks). Value not inflated to offset; multiplier carries it. AGENT DISSENT FROM BRIEF (no score impact): the row's own note reads 'Config-only on the relay side ... PLUS credential provisioning/runbook' - it already scoped credential work in, so the brief's claim that the note is contradicted is overstated; the code-path gap itself is real and confirmed. Also: brief's '0 of 7 cwa rows Implemented on the ingest side' is imprecise (F-001 IS Implemented, just not the ingest endpoint). CARRIED FOR HUMAN (no proposal): D-006's recorded reach=1 basis (inproc, empty peer list, transport inactive) would stop describing reality if F-010 puts a live peer on the wire; D-006/GH#16 record no dependency on F-010. Credential header and env-var name unnamed on both sides = most likely source of a silent 401 permanent-park loop. COULD NOT VERIFY: the 2026-07-19 product-owner rulings exist only as prose inside briefs - no ticket/issue/decision-log artifact behind them. [write-spec-from-feature-brief 2026-07-22] spec drafted at specs/F-010-deliver-admin-events-to-customer-web-app.md; 19 functional / 5 non-functional requirements; 7 of 9 open questions resolved by human ruling (Q3 GTM-date and Q7 D-006-re-exam deferred to named owners); spec-reviewer PASS WITH NOTES (rev 3). [implement-spec 2026-07-23] implemented per specs/F-010-deliver-admin-events-to-customer-web-app.md; branch spec/f-010-deliver-admin-events-to-cwa; full suite green (bff 1300, relay e2e 16, tsc clean); security PASS WITH NOTES, code review APPROVE WITH COMMENTS.</t>
   </si>
   <si>
     <t xml:space="preserve">F-011</t>
@@ -3914,13 +3911,13 @@
         <v>255</v>
       </c>
       <c r="D19" s="22" t="s">
-        <v>256</v>
+        <v>190</v>
       </c>
       <c r="E19" s="22" t="s">
         <v>172</v>
       </c>
       <c r="F19" s="22" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G19" s="25" t="n">
         <v>2</v>
@@ -3947,10 +3944,10 @@
         <v>5</v>
       </c>
       <c r="O19" s="27" t="s">
+        <v>257</v>
+      </c>
+      <c r="P19" s="27" t="s">
         <v>258</v>
-      </c>
-      <c r="P19" s="27" t="s">
-        <v>259</v>
       </c>
       <c r="Q19" s="28" t="n">
         <f aca="false">IF(V19="Defect","",IF(COUNT(G19:K19)&lt;5,"",ROUND(G19*Config!$B$4+H19*Config!$B$5+I19*Config!$B$6+J19*Config!$B$7+K19*Config!$B$8,2)))</f>
@@ -3978,22 +3975,22 @@
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="22" t="s">
+        <v>259</v>
+      </c>
+      <c r="B20" s="23" t="s">
         <v>260</v>
       </c>
-      <c r="B20" s="23" t="s">
+      <c r="C20" s="22" t="s">
         <v>261</v>
       </c>
-      <c r="C20" s="22" t="s">
+      <c r="D20" s="22" t="s">
         <v>262</v>
-      </c>
-      <c r="D20" s="22" t="s">
-        <v>263</v>
       </c>
       <c r="E20" s="22" t="s">
         <v>172</v>
       </c>
       <c r="F20" s="22" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G20" s="25" t="n">
         <v>5</v>
@@ -4020,10 +4017,10 @@
         <v>6</v>
       </c>
       <c r="O20" s="27" t="s">
+        <v>263</v>
+      </c>
+      <c r="P20" s="27" t="s">
         <v>264</v>
-      </c>
-      <c r="P20" s="27" t="s">
-        <v>265</v>
       </c>
       <c r="Q20" s="28" t="n">
         <f aca="false">IF(V20="Defect","",IF(COUNT(G20:K20)&lt;5,"",ROUND(G20*Config!$B$4+H20*Config!$B$5+I20*Config!$B$6+J20*Config!$B$7+K20*Config!$B$8,2)))</f>
@@ -4051,22 +4048,22 @@
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="22" t="s">
+        <v>265</v>
+      </c>
+      <c r="B21" s="23" t="s">
         <v>266</v>
       </c>
-      <c r="B21" s="23" t="s">
+      <c r="C21" s="22" t="s">
         <v>267</v>
       </c>
-      <c r="C21" s="22" t="s">
-        <v>268</v>
-      </c>
       <c r="D21" s="22" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E21" s="22" t="s">
         <v>172</v>
       </c>
       <c r="F21" s="22" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G21" s="25" t="n">
         <v>5</v>
@@ -4093,10 +4090,10 @@
         <v>6</v>
       </c>
       <c r="O21" s="27" t="s">
+        <v>268</v>
+      </c>
+      <c r="P21" s="27" t="s">
         <v>269</v>
-      </c>
-      <c r="P21" s="27" t="s">
-        <v>270</v>
       </c>
       <c r="Q21" s="28" t="n">
         <f aca="false">IF(V21="Defect","",IF(COUNT(G21:K21)&lt;5,"",ROUND(G21*Config!$B$4+H21*Config!$B$5+I21*Config!$B$6+J21*Config!$B$7+K21*Config!$B$8,2)))</f>
@@ -4124,22 +4121,22 @@
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="22" t="s">
+        <v>270</v>
+      </c>
+      <c r="B22" s="23" t="s">
         <v>271</v>
       </c>
-      <c r="B22" s="23" t="s">
+      <c r="C22" s="22" t="s">
         <v>272</v>
       </c>
-      <c r="C22" s="22" t="s">
-        <v>273</v>
-      </c>
       <c r="D22" s="22" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="E22" s="22" t="s">
         <v>172</v>
       </c>
       <c r="F22" s="22" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="G22" s="25" t="n">
         <v>4</v>
@@ -4166,10 +4163,10 @@
         <v>7</v>
       </c>
       <c r="O22" s="27" t="s">
+        <v>273</v>
+      </c>
+      <c r="P22" s="27" t="s">
         <v>274</v>
-      </c>
-      <c r="P22" s="27" t="s">
-        <v>275</v>
       </c>
       <c r="Q22" s="28" t="n">
         <f aca="false">IF(V22="Defect","",IF(COUNT(G22:K22)&lt;5,"",ROUND(G22*Config!$B$4+H22*Config!$B$5+I22*Config!$B$6+J22*Config!$B$7+K22*Config!$B$8,2)))</f>
@@ -4197,16 +4194,16 @@
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="22" t="s">
+        <v>275</v>
+      </c>
+      <c r="B23" s="23" t="s">
         <v>276</v>
       </c>
-      <c r="B23" s="23" t="s">
+      <c r="C23" s="22" t="s">
         <v>277</v>
       </c>
-      <c r="C23" s="22" t="s">
+      <c r="D23" s="22" t="s">
         <v>278</v>
-      </c>
-      <c r="D23" s="22" t="s">
-        <v>279</v>
       </c>
       <c r="E23" s="22"/>
       <c r="F23" s="22"/>
@@ -4219,10 +4216,10 @@
       <c r="M23" s="25"/>
       <c r="N23" s="25"/>
       <c r="O23" s="27" t="s">
+        <v>279</v>
+      </c>
+      <c r="P23" s="27" t="s">
         <v>280</v>
-      </c>
-      <c r="P23" s="27" t="s">
-        <v>281</v>
       </c>
       <c r="Q23" s="28" t="str">
         <f aca="false">IF(V23="Defect","",IF(COUNT(G23:K23)&lt;5,"",ROUND(G23*Config!$B$4+H23*Config!$B$5+I23*Config!$B$6+J23*Config!$B$7+K23*Config!$B$8,2)))</f>
@@ -5442,507 +5439,507 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="37" t="s">
+        <v>282</v>
+      </c>
+      <c r="B3" s="37" t="s">
         <v>283</v>
       </c>
-      <c r="B3" s="37" t="s">
+      <c r="C3" s="37" t="s">
         <v>284</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="D3" s="37" t="s">
         <v>285</v>
       </c>
-      <c r="D3" s="37" t="s">
+      <c r="E3" s="37" t="s">
         <v>286</v>
       </c>
-      <c r="E3" s="37" t="s">
+      <c r="F3" s="37" t="s">
         <v>287</v>
-      </c>
-      <c r="F3" s="37" t="s">
-        <v>288</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
+        <v>288</v>
+      </c>
+      <c r="B4" s="18" t="s">
         <v>289</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="C4" s="18" t="s">
         <v>290</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="D4" s="18" t="s">
         <v>291</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="E4" s="18" t="s">
         <v>292</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="F4" s="18" t="s">
         <v>293</v>
-      </c>
-      <c r="F4" s="18" t="s">
-        <v>294</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
+        <v>294</v>
+      </c>
+      <c r="B5" s="18" t="s">
         <v>295</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="C5" s="18" t="s">
+        <v>290</v>
+      </c>
+      <c r="D5" s="18" t="s">
         <v>296</v>
       </c>
-      <c r="C5" s="18" t="s">
-        <v>291</v>
-      </c>
-      <c r="D5" s="18" t="s">
+      <c r="E5" s="18" t="s">
+        <v>292</v>
+      </c>
+      <c r="F5" s="18" t="s">
         <v>297</v>
-      </c>
-      <c r="E5" s="18" t="s">
-        <v>293</v>
-      </c>
-      <c r="F5" s="18" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
+        <v>298</v>
+      </c>
+      <c r="B6" s="18" t="s">
         <v>299</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="C6" s="18" t="s">
+        <v>290</v>
+      </c>
+      <c r="D6" s="18" t="s">
         <v>300</v>
       </c>
-      <c r="C6" s="18" t="s">
-        <v>291</v>
-      </c>
-      <c r="D6" s="18" t="s">
+      <c r="E6" s="18" t="s">
+        <v>292</v>
+      </c>
+      <c r="F6" s="18" t="s">
         <v>301</v>
-      </c>
-      <c r="E6" s="18" t="s">
-        <v>293</v>
-      </c>
-      <c r="F6" s="18" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="B7" s="18" t="s">
         <v>303</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="C7" s="18" t="s">
         <v>304</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="D7" s="18" t="s">
         <v>305</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="E7" s="18" t="s">
         <v>306</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="F7" s="18" t="s">
         <v>307</v>
-      </c>
-      <c r="F7" s="18" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
+        <v>308</v>
+      </c>
+      <c r="B8" s="18" t="s">
         <v>309</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="C8" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="D8" s="18" t="s">
         <v>310</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>305</v>
-      </c>
-      <c r="D8" s="18" t="s">
+      <c r="E8" s="18" t="s">
         <v>311</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="F8" s="18" t="s">
         <v>312</v>
-      </c>
-      <c r="F8" s="18" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
+        <v>313</v>
+      </c>
+      <c r="B9" s="18" t="s">
         <v>314</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="C9" s="18" t="s">
         <v>315</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="D9" s="18" t="s">
         <v>316</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="E9" s="18" t="s">
+        <v>311</v>
+      </c>
+      <c r="F9" s="18" t="s">
         <v>317</v>
-      </c>
-      <c r="E9" s="18" t="s">
-        <v>312</v>
-      </c>
-      <c r="F9" s="18" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
+        <v>318</v>
+      </c>
+      <c r="B10" s="18" t="s">
         <v>319</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="C10" s="18" t="s">
         <v>320</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="D10" s="18" t="s">
         <v>321</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="E10" s="18" t="s">
         <v>322</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="F10" s="18" t="s">
         <v>323</v>
-      </c>
-      <c r="F10" s="18" t="s">
-        <v>324</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="B11" s="18" t="s">
         <v>325</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="C11" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="F11" s="18" t="s">
         <v>326</v>
-      </c>
-      <c r="C11" s="18" t="s">
-        <v>321</v>
-      </c>
-      <c r="D11" s="18" t="s">
-        <v>322</v>
-      </c>
-      <c r="E11" s="18" t="s">
-        <v>323</v>
-      </c>
-      <c r="F11" s="18" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
+        <v>327</v>
+      </c>
+      <c r="B12" s="18" t="s">
         <v>328</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="C12" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="E12" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="F12" s="18" t="s">
         <v>329</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>321</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>322</v>
-      </c>
-      <c r="E12" s="18" t="s">
-        <v>323</v>
-      </c>
-      <c r="F12" s="18" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
+        <v>330</v>
+      </c>
+      <c r="B13" s="18" t="s">
         <v>331</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="C13" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>292</v>
+      </c>
+      <c r="F13" s="18" t="s">
         <v>332</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>321</v>
-      </c>
-      <c r="D13" s="18" t="s">
-        <v>322</v>
-      </c>
-      <c r="E13" s="18" t="s">
-        <v>293</v>
-      </c>
-      <c r="F13" s="18" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
+        <v>333</v>
+      </c>
+      <c r="B14" s="18" t="s">
         <v>334</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="C14" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="F14" s="18" t="s">
         <v>335</v>
-      </c>
-      <c r="C14" s="18" t="s">
-        <v>321</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>322</v>
-      </c>
-      <c r="E14" s="18" t="s">
-        <v>323</v>
-      </c>
-      <c r="F14" s="18" t="s">
-        <v>336</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
+        <v>336</v>
+      </c>
+      <c r="B15" s="18" t="s">
         <v>337</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="C15" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="E15" s="18" t="s">
+        <v>311</v>
+      </c>
+      <c r="F15" s="18" t="s">
         <v>338</v>
-      </c>
-      <c r="C15" s="18" t="s">
-        <v>321</v>
-      </c>
-      <c r="D15" s="18" t="s">
-        <v>322</v>
-      </c>
-      <c r="E15" s="18" t="s">
-        <v>312</v>
-      </c>
-      <c r="F15" s="18" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
+        <v>339</v>
+      </c>
+      <c r="B16" s="18" t="s">
         <v>340</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="C16" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="E16" s="18" t="s">
         <v>341</v>
       </c>
-      <c r="C16" s="18" t="s">
-        <v>321</v>
-      </c>
-      <c r="D16" s="18" t="s">
-        <v>322</v>
-      </c>
-      <c r="E16" s="18" t="s">
+      <c r="F16" s="18" t="s">
         <v>342</v>
-      </c>
-      <c r="F16" s="18" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
+        <v>343</v>
+      </c>
+      <c r="B17" s="18" t="s">
         <v>344</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="C17" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>292</v>
+      </c>
+      <c r="F17" s="18" t="s">
         <v>345</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>321</v>
-      </c>
-      <c r="D17" s="18" t="s">
-        <v>322</v>
-      </c>
-      <c r="E17" s="18" t="s">
-        <v>293</v>
-      </c>
-      <c r="F17" s="18" t="s">
-        <v>346</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="B18" s="18" t="s">
         <v>347</v>
       </c>
-      <c r="B18" s="18" t="s">
+      <c r="C18" s="18" t="s">
+        <v>290</v>
+      </c>
+      <c r="D18" s="18" t="s">
         <v>348</v>
       </c>
-      <c r="C18" s="18" t="s">
-        <v>291</v>
-      </c>
-      <c r="D18" s="18" t="s">
+      <c r="E18" s="18" t="s">
+        <v>311</v>
+      </c>
+      <c r="F18" s="18" t="s">
         <v>349</v>
-      </c>
-      <c r="E18" s="18" t="s">
-        <v>312</v>
-      </c>
-      <c r="F18" s="18" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
+        <v>350</v>
+      </c>
+      <c r="B19" s="18" t="s">
         <v>351</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="C19" s="18" t="s">
+        <v>290</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>296</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>311</v>
+      </c>
+      <c r="F19" s="18" t="s">
         <v>352</v>
-      </c>
-      <c r="C19" s="18" t="s">
-        <v>291</v>
-      </c>
-      <c r="D19" s="18" t="s">
-        <v>297</v>
-      </c>
-      <c r="E19" s="18" t="s">
-        <v>312</v>
-      </c>
-      <c r="F19" s="18" t="s">
-        <v>353</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
+        <v>353</v>
+      </c>
+      <c r="B20" s="18" t="s">
         <v>354</v>
       </c>
-      <c r="B20" s="18" t="s">
+      <c r="C20" s="18" t="s">
         <v>355</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="D20" s="18" t="s">
         <v>356</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="E20" s="18" t="s">
         <v>357</v>
       </c>
-      <c r="E20" s="18" t="s">
+      <c r="F20" s="18" t="s">
         <v>358</v>
-      </c>
-      <c r="F20" s="18" t="s">
-        <v>359</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
+        <v>359</v>
+      </c>
+      <c r="B21" s="18" t="s">
         <v>360</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="C21" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="D21" s="18" t="s">
         <v>361</v>
       </c>
-      <c r="C21" s="18" t="s">
-        <v>356</v>
-      </c>
-      <c r="D21" s="18" t="s">
+      <c r="E21" s="18" t="s">
+        <v>357</v>
+      </c>
+      <c r="F21" s="18" t="s">
         <v>362</v>
-      </c>
-      <c r="E21" s="18" t="s">
-        <v>358</v>
-      </c>
-      <c r="F21" s="18" t="s">
-        <v>363</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
+        <v>363</v>
+      </c>
+      <c r="B22" s="18" t="s">
         <v>364</v>
       </c>
-      <c r="B22" s="18" t="s">
+      <c r="C22" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="D22" s="18" t="s">
         <v>365</v>
       </c>
-      <c r="C22" s="18" t="s">
-        <v>356</v>
-      </c>
-      <c r="D22" s="18" t="s">
+      <c r="E22" s="18" t="s">
+        <v>357</v>
+      </c>
+      <c r="F22" s="18" t="s">
         <v>366</v>
-      </c>
-      <c r="E22" s="18" t="s">
-        <v>358</v>
-      </c>
-      <c r="F22" s="18" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
+        <v>367</v>
+      </c>
+      <c r="B23" s="18" t="s">
         <v>368</v>
       </c>
-      <c r="B23" s="18" t="s">
+      <c r="C23" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="D23" s="18" t="s">
         <v>369</v>
       </c>
-      <c r="C23" s="18" t="s">
-        <v>356</v>
-      </c>
-      <c r="D23" s="18" t="s">
+      <c r="E23" s="18" t="s">
+        <v>357</v>
+      </c>
+      <c r="F23" s="18" t="s">
         <v>370</v>
-      </c>
-      <c r="E23" s="18" t="s">
-        <v>358</v>
-      </c>
-      <c r="F23" s="18" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
+        <v>371</v>
+      </c>
+      <c r="B24" s="18" t="s">
         <v>372</v>
       </c>
-      <c r="B24" s="18" t="s">
+      <c r="C24" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="D24" s="18" t="s">
         <v>373</v>
       </c>
-      <c r="C24" s="18" t="s">
-        <v>356</v>
-      </c>
-      <c r="D24" s="18" t="s">
+      <c r="E24" s="18" t="s">
+        <v>357</v>
+      </c>
+      <c r="F24" s="18" t="s">
         <v>374</v>
-      </c>
-      <c r="E24" s="18" t="s">
-        <v>358</v>
-      </c>
-      <c r="F24" s="18" t="s">
-        <v>375</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
+        <v>375</v>
+      </c>
+      <c r="B25" s="18" t="s">
         <v>376</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="C25" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="D25" s="18" t="s">
         <v>377</v>
       </c>
-      <c r="C25" s="18" t="s">
-        <v>305</v>
-      </c>
-      <c r="D25" s="18" t="s">
+      <c r="E25" s="18" t="s">
+        <v>292</v>
+      </c>
+      <c r="F25" s="18" t="s">
         <v>378</v>
-      </c>
-      <c r="E25" s="18" t="s">
-        <v>293</v>
-      </c>
-      <c r="F25" s="18" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
+        <v>379</v>
+      </c>
+      <c r="B26" s="18" t="s">
         <v>380</v>
       </c>
-      <c r="B26" s="18" t="s">
+      <c r="C26" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="D26" s="18" t="s">
         <v>381</v>
       </c>
-      <c r="C26" s="18" t="s">
-        <v>305</v>
-      </c>
-      <c r="D26" s="18" t="s">
+      <c r="E26" s="18" t="s">
         <v>382</v>
       </c>
-      <c r="E26" s="18" t="s">
+      <c r="F26" s="18" t="s">
         <v>383</v>
-      </c>
-      <c r="F26" s="18" t="s">
-        <v>384</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="B27" s="18" t="s">
         <v>385</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="C27" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="D27" s="18" t="s">
         <v>386</v>
       </c>
-      <c r="C27" s="18" t="s">
-        <v>321</v>
-      </c>
-      <c r="D27" s="18" t="s">
+      <c r="E27" s="18" t="s">
         <v>387</v>
       </c>
-      <c r="E27" s="18" t="s">
+      <c r="F27" s="18" t="s">
         <v>388</v>
-      </c>
-      <c r="F27" s="18" t="s">
-        <v>389</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: log D-008 — relay partially-delivered-park not observable
Surfaced by F-010 Phase-6 e2e. The recordPartiallyDeliveredPark() counter
(metrics.ts:57) is in-process only — no getter/snapshot, no /metrics, no
/ready field, and setLastError writes a generic message — so operators
cannot distinguish a partially-delivered park (acked peer holds a dedupable
copy) from a never-delivered one. Predates F-010 (F-004 REQ-F004-025
machinery); REQ-F010-015 is the first to require operator observability.
Logged Reported (Internal), GH #40; severity/scoring left for triage.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSQAV9AspmwvxZ78jg9QNx
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="511" uniqueCount="389">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="394">
   <si>
     <t xml:space="preserve">FEATURE VALUE SCORING FRAMEWORK</t>
   </si>
@@ -867,6 +867,21 @@
   </si>
   <si>
     <t xml:space="preserve">Distinct from but overlapping D-006 (GH #16): D-006 = broad relay transport hardening (HMAC/mTLS + https-only enforcement), scored while the transport was inactive; this row = the concrete secret-disclosure that F-010 makes active. Surfaced as F-010 spec Open Question Q4 (scheme validation deliberately left to D-006). Minimal fix = fail-fast reject of non-https peer URLs when a credential is configured (bff/src/relay/config.ts). Severity + scoring left for triage/prioritization; triage to decide fix-here vs fold-into-D-006.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D-008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relay partially-delivered-park signal is in-process only — not observable by operators</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/dispatch-derek/admin-console/issues/40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logged 2026-07-23 (Internal); surfaced by F-010 Phase-6 e2e. recordPartiallyDeliveredPark() counter (bff/src/relay/metrics.ts:57-58, incremented at drainer.ts:71) is a process-lifetime singleton with NO exported getter/snapshot; only DB-backed gauges getBacklogCount/getRelayLagMs are wired out (index.ts:14,46-47). No /metrics endpoint, no /ready field (ready.ts exposes only eventBusUrlConfigured), and setLastError(row.id, errText(err)) (drainer.ts:80) writes a generic TransportError message that does not encode partial-vs-never-delivered. So operators cannot distinguish a partially-delivered park (acked peer holds a dedupable copy) from a never-delivered one, nor see the counter at all. Verified first-hand. GH issue #40.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Predates F-010: the counter and REQ-F004-051(e)/REQ-F004-025 partial-vs-never split are F-004 machinery; no F-004 test asserted external observability. Surfaced because REQ-F010-015 is the first requirement to state 'operators MUST be able to observe this outcome' against this counter. Observability/operability defect, not correctness (row is retained/parked, no data loss). Fix direction: expose event counters via /metrics or /ready, and/or encode partial-vs-never in the parked row's last_error. Severity + scoring left for triage. Relates to F-010 (REQ-F010-015) and F-004 (REQ-F004-025).</t>
   </si>
   <si>
     <t xml:space="preserve">DATA DICTIONARY - machine-readable field contract for agents</t>
@@ -4249,10 +4264,18 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="22"/>
-      <c r="B24" s="23"/>
-      <c r="C24" s="22"/>
-      <c r="D24" s="22"/>
+      <c r="A24" s="22" t="s">
+        <v>281</v>
+      </c>
+      <c r="B24" s="23" t="s">
+        <v>282</v>
+      </c>
+      <c r="C24" s="22" t="s">
+        <v>283</v>
+      </c>
+      <c r="D24" s="22" t="s">
+        <v>278</v>
+      </c>
       <c r="E24" s="22"/>
       <c r="F24" s="22"/>
       <c r="G24" s="25"/>
@@ -4263,8 +4286,12 @@
       <c r="L24" s="25"/>
       <c r="M24" s="25"/>
       <c r="N24" s="25"/>
-      <c r="O24" s="27"/>
-      <c r="P24" s="27"/>
+      <c r="O24" s="27" t="s">
+        <v>284</v>
+      </c>
+      <c r="P24" s="27" t="s">
+        <v>285</v>
+      </c>
       <c r="Q24" s="28" t="str">
         <f aca="false">IF(V24="Defect","",IF(COUNT(G24:K24)&lt;5,"",ROUND(G24*Config!$B$4+H24*Config!$B$5+I24*Config!$B$6+J24*Config!$B$7+K24*Config!$B$8,2)))</f>
         <v/>
@@ -4285,7 +4312,12 @@
         <f aca="false">IF(T24="","",RANK(T24,$T$4:$T$52))</f>
         <v/>
       </c>
-      <c r="V24" s="36"/>
+      <c r="V24" s="36" t="s">
+        <v>199</v>
+      </c>
+      <c r="W24" s="1" t="s">
+        <v>200</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="22"/>
@@ -5439,507 +5471,507 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="37" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="B3" s="37" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C3" s="37" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="D3" s="37" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="E3" s="37" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="F3" s="37" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="B5" s="18" t="s">
+        <v>300</v>
+      </c>
+      <c r="C5" s="18" t="s">
         <v>295</v>
       </c>
-      <c r="C5" s="18" t="s">
-        <v>290</v>
-      </c>
       <c r="D5" s="18" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="B8" s="18" t="s">
+        <v>314</v>
+      </c>
+      <c r="C8" s="18" t="s">
         <v>309</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>304</v>
-      </c>
       <c r="D8" s="18" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="D9" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="E9" s="18" t="s">
         <v>316</v>
       </c>
-      <c r="E9" s="18" t="s">
-        <v>311</v>
-      </c>
       <c r="F9" s="18" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="B11" s="18" t="s">
+        <v>330</v>
+      </c>
+      <c r="C11" s="18" t="s">
         <v>325</v>
       </c>
-      <c r="C11" s="18" t="s">
-        <v>320</v>
-      </c>
       <c r="D11" s="18" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
+        <v>332</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>333</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="E12" s="18" t="s">
         <v>327</v>
       </c>
-      <c r="B12" s="18" t="s">
-        <v>328</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>320</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>321</v>
-      </c>
-      <c r="E12" s="18" t="s">
-        <v>322</v>
-      </c>
       <c r="F12" s="18" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="B21" s="18" t="s">
+        <v>365</v>
+      </c>
+      <c r="C21" s="18" t="s">
         <v>360</v>
       </c>
-      <c r="C21" s="18" t="s">
-        <v>355</v>
-      </c>
       <c r="D21" s="18" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>369</v>
+        <v>374</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
       <c r="F27" s="18" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: triage D-007 (sev 5) and D-008 (sev 3) — human severity gate
Human triage during /prioritize-features: D-007 (cleartext secret over
http:// peers) severity 5; D-008 (partially-delivered-park not observable)
severity 3. Both advanced Reported -> Triaged for research scoring.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSQAV9AspmwvxZ78jg9QNx
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -860,7 +860,7 @@
     <t xml:space="preserve">https://github.com/dispatch-derek/admin-console/issues/39</t>
   </si>
   <si>
-    <t xml:space="preserve">Reported</t>
+    <t xml:space="preserve">Triaged</t>
   </si>
   <si>
     <t xml:space="preserve">Logged 2026-07-22 (Internal). F-010 introduces a shared-secret credential on the relay's outbound POST (header X-Event-Auth-Token / env EVENT_BUS_PEER_AUTH_TOKEN; spec specs/F-010-deliver-admin-events-to-customer-web-app.md REQ-F010-005/-007). bff/src/relay/config.ts splits/trims/filters EVENT_BUS_URL with 0 scheme validation, so http:// peer URLs are accepted (all 3 README examples at bff/src/relay/README.md are http://). Result: any http:// peer transmits the secret in cleartext on every delivery -&gt; credential disclosure -&gt; forgeable admin.user.* events into the consumer. Not live today (EVENT_BUS_MODE=inproc, no credential code path); becomes exploitable the moment F-010 ships with any http:// peer. GH issue #39.</t>
@@ -4262,6 +4262,9 @@
       <c r="W23" s="1" t="s">
         <v>200</v>
       </c>
+      <c r="X23" s="1" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="22" t="s">
@@ -4317,6 +4320,9 @@
       </c>
       <c r="W24" s="1" t="s">
         <v>200</v>
+      </c>
+      <c r="X24" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
chore: research-score D-007 (reach2/conf9) and D-008 (reach1/conf9)
market-research-agent RESEARCH role, re-verified vs main. D-007 -> priority
76 (sev5 x reach_factor 0.8 x conf 0.95); D-008 -> 39.2 (sev3 x 0.75 x 0.95).
Both status Scored. Evidence/rationale appended (provenance preserved).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSQAV9AspmwvxZ78jg9QNx
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="394">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="394">
   <si>
     <t xml:space="preserve">FEATURE VALUE SCORING FRAMEWORK</t>
   </si>
@@ -860,13 +860,13 @@
     <t xml:space="preserve">https://github.com/dispatch-derek/admin-console/issues/39</t>
   </si>
   <si>
-    <t xml:space="preserve">Triaged</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Logged 2026-07-22 (Internal). F-010 introduces a shared-secret credential on the relay's outbound POST (header X-Event-Auth-Token / env EVENT_BUS_PEER_AUTH_TOKEN; spec specs/F-010-deliver-admin-events-to-customer-web-app.md REQ-F010-005/-007). bff/src/relay/config.ts splits/trims/filters EVENT_BUS_URL with 0 scheme validation, so http:// peer URLs are accepted (all 3 README examples at bff/src/relay/README.md are http://). Result: any http:// peer transmits the secret in cleartext on every delivery -&gt; credential disclosure -&gt; forgeable admin.user.* events into the consumer. Not live today (EVENT_BUS_MODE=inproc, no credential code path); becomes exploitable the moment F-010 ships with any http:// peer. GH issue #39.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Distinct from but overlapping D-006 (GH #16): D-006 = broad relay transport hardening (HMAC/mTLS + https-only enforcement), scored while the transport was inactive; this row = the concrete secret-disclosure that F-010 makes active. Surfaced as F-010 spec Open Question Q4 (scheme validation deliberately left to D-006). Minimal fix = fail-fast reject of non-https peer URLs when a credential is configured (bff/src/relay/config.ts). Severity + scoring left for triage/prioritization; triage to decide fix-here vs fold-into-D-006.</t>
+    <t xml:space="preserve">Scored</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logged 2026-07-22 (Internal). F-010 introduces a shared-secret credential on the relay's outbound POST (header X-Event-Auth-Token / env EVENT_BUS_PEER_AUTH_TOKEN; spec specs/F-010-deliver-admin-events-to-customer-web-app.md REQ-F010-005/-007). bff/src/relay/config.ts splits/trims/filters EVENT_BUS_URL with 0 scheme validation, so http:// peer URLs are accepted (all 3 README examples at bff/src/relay/README.md are http://). Result: any http:// peer transmits the secret in cleartext on every delivery -&gt; credential disclosure -&gt; forgeable admin.user.* events into the consumer. Not live today (EVENT_BUS_MODE=inproc, no credential code path); becomes exploitable the moment F-010 ships with any http:// peer. GH issue #39. || [RESEARCH 2026-07-23 re-verified vs main, F-010 merged] config.ts: EVENT_BUS_URL split/trim/filter only, NO URL-scheme validation, http:// accepted. http-peer-transport.ts:18 AUTH_TOKEN_HEADER='X-Event-Auth-Token', :90-91 attached to every outbound POST when credential configured, :93 fetch to peer URL verbatim -&gt; http:// peer carries secret in cleartext. README.md:26,40,54 all peer examples http://; :90-92 Security caveat; :182 threat-model F2. GH #39; related D-006/#16 (https-only/mTLS, separate track). No support tickets/analytics/demand records (internal tool).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Distinct from but overlapping D-006 (GH #16): D-006 = broad relay transport hardening (HMAC/mTLS + https-only enforcement), scored while the transport was inactive; this row = the concrete secret-disclosure that F-010 makes active. Surfaced as F-010 spec Open Question Q4 (scheme validation deliberately left to D-006). Minimal fix = fail-fast reject of non-https peer URLs when a credential is configured (bff/src/relay/config.ts). Severity + scoring left for triage/prioritization; triage to decide fix-here vs fold-into-D-006. || [RESEARCH 2026-07-23] reach=2 (Rubric: &lt;5%/rare edge case): exposure gated behind bus-mode relay + http:// peer + on-path observer; https:// unaffected; nudged off floor because README ships http:// examples. confidence=9: code-certain multi-source repro (config.ts, http-peer-transport.ts:90-91, README); held below 10 for lack of a live cleartext capture. severity untouched (human=5).</t>
   </si>
   <si>
     <t xml:space="preserve">D-008</t>
@@ -878,10 +878,10 @@
     <t xml:space="preserve">https://github.com/dispatch-derek/admin-console/issues/40</t>
   </si>
   <si>
-    <t xml:space="preserve">Logged 2026-07-23 (Internal); surfaced by F-010 Phase-6 e2e. recordPartiallyDeliveredPark() counter (bff/src/relay/metrics.ts:57-58, incremented at drainer.ts:71) is a process-lifetime singleton with NO exported getter/snapshot; only DB-backed gauges getBacklogCount/getRelayLagMs are wired out (index.ts:14,46-47). No /metrics endpoint, no /ready field (ready.ts exposes only eventBusUrlConfigured), and setLastError(row.id, errText(err)) (drainer.ts:80) writes a generic TransportError message that does not encode partial-vs-never-delivered. So operators cannot distinguish a partially-delivered park (acked peer holds a dedupable copy) from a never-delivered one, nor see the counter at all. Verified first-hand. GH issue #40.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Predates F-010: the counter and REQ-F004-051(e)/REQ-F004-025 partial-vs-never split are F-004 machinery; no F-004 test asserted external observability. Surfaced because REQ-F010-015 is the first requirement to state 'operators MUST be able to observe this outcome' against this counter. Observability/operability defect, not correctness (row is retained/parked, no data loss). Fix direction: expose event counters via /metrics or /ready, and/or encode partial-vs-never in the parked row's last_error. Severity + scoring left for triage. Relates to F-010 (REQ-F010-015) and F-004 (REQ-F004-025).</t>
+    <t xml:space="preserve">Logged 2026-07-23 (Internal); surfaced by F-010 Phase-6 e2e. recordPartiallyDeliveredPark() counter (bff/src/relay/metrics.ts:57-58, incremented at drainer.ts:71) is a process-lifetime singleton with NO exported getter/snapshot; only DB-backed gauges getBacklogCount/getRelayLagMs are wired out (index.ts:14,46-47). No /metrics endpoint, no /ready field (ready.ts exposes only eventBusUrlConfigured), and setLastError(row.id, errText(err)) (drainer.ts:80) writes a generic TransportError message that does not encode partial-vs-never-delivered. So operators cannot distinguish a partially-delivered park (acked peer holds a dedupable copy) from a never-delivered one, nor see the counter at all. Verified first-hand. GH issue #40. || [RESEARCH 2026-07-23 re-verified vs main] Counter is process-lifetime singleton: metrics.ts:37-59 counters, :57-58 recordPartiallyDeliveredPark, incremented drainer.ts:71. getCounters() EXISTS at metrics.ts:66-68 but is DEAD CODE (grep: zero consumers) -&gt; counters still externally unobservable. Only DB gauges wired out: index.ts:14,46-47 (getBacklogCount, getRelayLagMs). /ready exposes no counter/park field: ready.ts:8-16,21-39. No /metrics route anywhere (grep). last_error generic: drainer.ts:80 setLastError(row.id, errText(err)); partial-vs-never captured only at recordPark drainer.ts:70-73 feeding the unobservable counter. GH #40; predates F-010 (F-004 REQ-F004-025/-051(e)); no data loss. No tickets/analytics/demand (internal tool).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Predates F-010: the counter and REQ-F004-051(e)/REQ-F004-025 partial-vs-never split are F-004 machinery; no F-004 test asserted external observability. Surfaced because REQ-F010-015 is the first requirement to state 'operators MUST be able to observe this outcome' against this counter. Observability/operability defect, not correctness (row is retained/parked, no data loss). Fix direction: expose event counters via /metrics or /ready, and/or encode partial-vs-never in the parked row's last_error. Severity + scoring left for triage. Relates to F-010 (REQ-F010-015) and F-004 (REQ-F004-025). || [RESEARCH 2026-07-23] reach=1 (Rubric: &lt;3%/rare edge case): only bites during a partially-delivered-park incident (drainer.ts:69-73 partialAck path) on an internal tool with small operator population; floor, not inflated. confidence=9: structurally provable across 4 files + negative /metrics grep; held below 10 (static inspection, not live incident repro). REMEDIATION NOTE: getCounters() already exists as dead code -&gt; fix likely just wires it to /metrics or /ready. severity untouched (human=3).</t>
   </si>
   <si>
     <t xml:space="preserve">DATA DICTIONARY - machine-readable field contract for agents</t>
@@ -2892,7 +2892,7 @@
       </c>
       <c r="U4" s="30" t="n">
         <f aca="false">IF(T4="","",RANK(T4,$T$4:$T$52))</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V4" s="22" t="s">
         <v>175</v>
@@ -2965,7 +2965,7 @@
       </c>
       <c r="U5" s="30" t="n">
         <f aca="false">IF(T5="","",RANK(T5,$T$4:$T$52))</f>
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="V5" s="22" t="s">
         <v>175</v>
@@ -3038,7 +3038,7 @@
       </c>
       <c r="U6" s="30" t="n">
         <f aca="false">IF(T6="","",RANK(T6,$T$4:$T$52))</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="V6" s="22" t="s">
         <v>175</v>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="U7" s="30" t="n">
         <f aca="false">IF(T7="","",RANK(T7,$T$4:$T$52))</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="V7" s="22" t="s">
         <v>175</v>
@@ -3184,7 +3184,7 @@
       </c>
       <c r="U8" s="30" t="n">
         <f aca="false">IF(T8="","",RANK(T8,$T$4:$T$52))</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="V8" s="33" t="s">
         <v>199</v>
@@ -3263,7 +3263,7 @@
       </c>
       <c r="U9" s="30" t="n">
         <f aca="false">IF(T9="","",RANK(T9,$T$4:$T$52))</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="V9" s="33" t="s">
         <v>175</v>
@@ -3332,7 +3332,7 @@
       </c>
       <c r="U10" s="30" t="n">
         <f aca="false">IF(T10="","",RANK(T10,$T$4:$T$52))</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="V10" s="33" t="s">
         <v>199</v>
@@ -3411,7 +3411,7 @@
       </c>
       <c r="U11" s="30" t="n">
         <f aca="false">IF(T11="","",RANK(T11,$T$4:$T$52))</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="V11" s="33" t="s">
         <v>175</v>
@@ -3553,7 +3553,7 @@
       </c>
       <c r="U13" s="30" t="n">
         <f aca="false">IF(T13="","",RANK(T13,$T$4:$T$52))</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="V13" s="33" t="s">
         <v>175</v>
@@ -3614,7 +3614,7 @@
       </c>
       <c r="U14" s="30" t="n">
         <f aca="false">IF(T14="","",RANK(T14,$T$4:$T$52))</f>
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="V14" s="33" t="s">
         <v>199</v>
@@ -3693,7 +3693,7 @@
       </c>
       <c r="U15" s="30" t="n">
         <f aca="false">IF(T15="","",RANK(T15,$T$4:$T$52))</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="V15" s="33" t="s">
         <v>175</v>
@@ -3763,7 +3763,7 @@
       </c>
       <c r="U16" s="30" t="n">
         <f aca="false">IF(T16="","",RANK(T16,$T$4:$T$52))</f>
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="V16" s="36" t="s">
         <v>199</v>
@@ -3830,7 +3830,7 @@
       </c>
       <c r="U17" s="30" t="n">
         <f aca="false">IF(T17="","",RANK(T17,$T$4:$T$52))</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="V17" s="36" t="s">
         <v>199</v>
@@ -3909,7 +3909,7 @@
       </c>
       <c r="U18" s="30" t="n">
         <f aca="false">IF(T18="","",RANK(T18,$T$4:$T$52))</f>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="V18" s="33" t="s">
         <v>175</v>
@@ -3982,7 +3982,7 @@
       </c>
       <c r="U19" s="30" t="n">
         <f aca="false">IF(T19="","",RANK(T19,$T$4:$T$52))</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="V19" s="36" t="s">
         <v>175</v>
@@ -4055,7 +4055,7 @@
       </c>
       <c r="U20" s="30" t="n">
         <f aca="false">IF(T20="","",RANK(T20,$T$4:$T$52))</f>
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="V20" s="36" t="s">
         <v>175</v>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="U21" s="30" t="n">
         <f aca="false">IF(T21="","",RANK(T21,$T$4:$T$52))</f>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="V21" s="36" t="s">
         <v>175</v>
@@ -4201,7 +4201,7 @@
       </c>
       <c r="U22" s="30" t="n">
         <f aca="false">IF(T22="","",RANK(T22,$T$4:$T$52))</f>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="V22" s="36" t="s">
         <v>175</v>
@@ -4220,14 +4220,22 @@
       <c r="D23" s="22" t="s">
         <v>278</v>
       </c>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="25"/>
+      <c r="E23" s="22" t="s">
+        <v>172</v>
+      </c>
+      <c r="F23" s="32" t="n">
+        <v>46226</v>
+      </c>
+      <c r="G23" s="25" t="n">
+        <v>2</v>
+      </c>
       <c r="H23" s="25"/>
       <c r="I23" s="25"/>
       <c r="J23" s="25"/>
       <c r="K23" s="25"/>
-      <c r="L23" s="25"/>
+      <c r="L23" s="25" t="n">
+        <v>9</v>
+      </c>
       <c r="M23" s="25"/>
       <c r="N23" s="25"/>
       <c r="O23" s="27" t="s">
@@ -4240,21 +4248,21 @@
         <f aca="false">IF(V23="Defect","",IF(COUNT(G23:K23)&lt;5,"",ROUND(G23*Config!$B$4+H23*Config!$B$5+I23*Config!$B$6+J23*Config!$B$7+K23*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R23" s="28" t="str">
+      <c r="R23" s="28" t="n">
         <f aca="false">IF(L23="","",VLOOKUP(L23,Config!$A$12:$B$21,2,0))</f>
-        <v/>
+        <v>0.95</v>
       </c>
       <c r="S23" s="28" t="str">
         <f aca="false">IF(N23="","",VLOOKUP(N23,Config!$D$12:$E$21,2,0))</f>
         <v/>
       </c>
-      <c r="T23" s="29" t="str">
+      <c r="T23" s="29" t="n">
         <f aca="false">IF(V23="Defect",IF(OR(X23="",G23="",R23=""),"",ROUND(MIN(100,VLOOKUP(X23,Config!$G$12:$H$16,2,0)*VLOOKUP(G23,Config!$I$12:$J$21,2,0)*R23),1)),IF(OR(Q23="",R23="",S23="",M23=""),"",ROUND(MIN(100,Q23*R23*S23/M23*20),1)))</f>
-        <v/>
-      </c>
-      <c r="U23" s="30" t="str">
+        <v>76</v>
+      </c>
+      <c r="U23" s="30" t="n">
         <f aca="false">IF(T23="","",RANK(T23,$T$4:$T$52))</f>
-        <v/>
+        <v>2</v>
       </c>
       <c r="V23" s="36" t="s">
         <v>199</v>
@@ -4279,14 +4287,22 @@
       <c r="D24" s="22" t="s">
         <v>278</v>
       </c>
-      <c r="E24" s="22"/>
-      <c r="F24" s="22"/>
-      <c r="G24" s="25"/>
+      <c r="E24" s="22" t="s">
+        <v>172</v>
+      </c>
+      <c r="F24" s="32" t="n">
+        <v>46226</v>
+      </c>
+      <c r="G24" s="25" t="n">
+        <v>1</v>
+      </c>
       <c r="H24" s="25"/>
       <c r="I24" s="25"/>
       <c r="J24" s="25"/>
       <c r="K24" s="25"/>
-      <c r="L24" s="25"/>
+      <c r="L24" s="25" t="n">
+        <v>9</v>
+      </c>
       <c r="M24" s="25"/>
       <c r="N24" s="25"/>
       <c r="O24" s="27" t="s">
@@ -4299,21 +4315,21 @@
         <f aca="false">IF(V24="Defect","",IF(COUNT(G24:K24)&lt;5,"",ROUND(G24*Config!$B$4+H24*Config!$B$5+I24*Config!$B$6+J24*Config!$B$7+K24*Config!$B$8,2)))</f>
         <v/>
       </c>
-      <c r="R24" s="28" t="str">
+      <c r="R24" s="28" t="n">
         <f aca="false">IF(L24="","",VLOOKUP(L24,Config!$A$12:$B$21,2,0))</f>
-        <v/>
+        <v>0.95</v>
       </c>
       <c r="S24" s="28" t="str">
         <f aca="false">IF(N24="","",VLOOKUP(N24,Config!$D$12:$E$21,2,0))</f>
         <v/>
       </c>
-      <c r="T24" s="29" t="str">
+      <c r="T24" s="29" t="n">
         <f aca="false">IF(V24="Defect",IF(OR(X24="",G24="",R24=""),"",ROUND(MIN(100,VLOOKUP(X24,Config!$G$12:$H$16,2,0)*VLOOKUP(G24,Config!$I$12:$J$21,2,0)*R24),1)),IF(OR(Q24="",R24="",S24="",M24=""),"",ROUND(MIN(100,Q24*R24*S24/M24*20),1)))</f>
-        <v/>
-      </c>
-      <c r="U24" s="30" t="str">
+        <v>39.2</v>
+      </c>
+      <c r="U24" s="30" t="n">
         <f aca="false">IF(T24="","",RANK(T24,$T$4:$T$52))</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="V24" s="36" t="s">
         <v>199</v>

</xml_diff>

<commit_message>
chore: D-007 -> Prioritized (Sev1 signoff), fix folded into D-006
Human ruling 2026-07-23: D-007 (cleartext credential over http:// peers)
prioritized after Sev1 sign-off; remediation folded into D-006 (GH #16)
as one https-only/mTLS relay-hardening effort rather than a standalone
patch.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSQAV9AspmwvxZ78jg9QNx
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="394">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="393">
   <si>
     <t xml:space="preserve">FEATURE VALUE SCORING FRAMEWORK</t>
   </si>
@@ -860,13 +860,10 @@
     <t xml:space="preserve">https://github.com/dispatch-derek/admin-console/issues/39</t>
   </si>
   <si>
-    <t xml:space="preserve">Scored</t>
-  </si>
-  <si>
     <t xml:space="preserve">Logged 2026-07-22 (Internal). F-010 introduces a shared-secret credential on the relay's outbound POST (header X-Event-Auth-Token / env EVENT_BUS_PEER_AUTH_TOKEN; spec specs/F-010-deliver-admin-events-to-customer-web-app.md REQ-F010-005/-007). bff/src/relay/config.ts splits/trims/filters EVENT_BUS_URL with 0 scheme validation, so http:// peer URLs are accepted (all 3 README examples at bff/src/relay/README.md are http://). Result: any http:// peer transmits the secret in cleartext on every delivery -&gt; credential disclosure -&gt; forgeable admin.user.* events into the consumer. Not live today (EVENT_BUS_MODE=inproc, no credential code path); becomes exploitable the moment F-010 ships with any http:// peer. GH issue #39. || [RESEARCH 2026-07-23 re-verified vs main, F-010 merged] config.ts: EVENT_BUS_URL split/trim/filter only, NO URL-scheme validation, http:// accepted. http-peer-transport.ts:18 AUTH_TOKEN_HEADER='X-Event-Auth-Token', :90-91 attached to every outbound POST when credential configured, :93 fetch to peer URL verbatim -&gt; http:// peer carries secret in cleartext. README.md:26,40,54 all peer examples http://; :90-92 Security caveat; :182 threat-model F2. GH #39; related D-006/#16 (https-only/mTLS, separate track). No support tickets/analytics/demand records (internal tool).</t>
   </si>
   <si>
-    <t xml:space="preserve">Distinct from but overlapping D-006 (GH #16): D-006 = broad relay transport hardening (HMAC/mTLS + https-only enforcement), scored while the transport was inactive; this row = the concrete secret-disclosure that F-010 makes active. Surfaced as F-010 spec Open Question Q4 (scheme validation deliberately left to D-006). Minimal fix = fail-fast reject of non-https peer URLs when a credential is configured (bff/src/relay/config.ts). Severity + scoring left for triage/prioritization; triage to decide fix-here vs fold-into-D-006. || [RESEARCH 2026-07-23] reach=2 (Rubric: &lt;5%/rare edge case): exposure gated behind bus-mode relay + http:// peer + on-path observer; https:// unaffected; nudged off floor because README ships http:// examples. confidence=9: code-certain multi-source repro (config.ts, http-peer-transport.ts:90-91, README); held below 10 for lack of a live cleartext capture. severity untouched (human=5).</t>
+    <t xml:space="preserve">Distinct from but overlapping D-006 (GH #16): D-006 = broad relay transport hardening (HMAC/mTLS + https-only enforcement), scored while the transport was inactive; this row = the concrete secret-disclosure that F-010 makes active. Surfaced as F-010 spec Open Question Q4 (scheme validation deliberately left to D-006). Minimal fix = fail-fast reject of non-https peer URLs when a credential is configured (bff/src/relay/config.ts). Severity + scoring left for triage/prioritization; triage to decide fix-here vs fold-into-D-006. || [RESEARCH 2026-07-23] reach=2 (Rubric: &lt;5%/rare edge case): exposure gated behind bus-mode relay + http:// peer + on-path observer; https:// unaffected; nudged off floor because README ships http:// examples. confidence=9: code-certain multi-source repro (config.ts, http-peer-transport.ts:90-91, README); held below 10 for lack of a live cleartext capture. severity untouched (human=5). || [human ruling 2026-07-23] Sev1 sign-off: Prioritized. Fix FOLDED INTO D-006 (GH #16) per product-owner decision — a single https-only/mTLS relay-hardening effort covers this cleartext-credential leak; do not fix D-007 as a standalone patch. See GH #39/#16.</t>
   </si>
   <si>
     <t xml:space="preserve">D-008</t>
@@ -4218,7 +4215,7 @@
         <v>277</v>
       </c>
       <c r="D23" s="22" t="s">
-        <v>278</v>
+        <v>171</v>
       </c>
       <c r="E23" s="22" t="s">
         <v>172</v>
@@ -4239,10 +4236,10 @@
       <c r="M23" s="25"/>
       <c r="N23" s="25"/>
       <c r="O23" s="27" t="s">
+        <v>278</v>
+      </c>
+      <c r="P23" s="27" t="s">
         <v>279</v>
-      </c>
-      <c r="P23" s="27" t="s">
-        <v>280</v>
       </c>
       <c r="Q23" s="28" t="str">
         <f aca="false">IF(V23="Defect","",IF(COUNT(G23:K23)&lt;5,"",ROUND(G23*Config!$B$4+H23*Config!$B$5+I23*Config!$B$6+J23*Config!$B$7+K23*Config!$B$8,2)))</f>
@@ -4276,13 +4273,13 @@
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="22" t="s">
+        <v>280</v>
+      </c>
+      <c r="B24" s="23" t="s">
         <v>281</v>
       </c>
-      <c r="B24" s="23" t="s">
+      <c r="C24" s="22" t="s">
         <v>282</v>
-      </c>
-      <c r="C24" s="22" t="s">
-        <v>283</v>
       </c>
       <c r="D24" s="22" t="s">
         <v>171</v>
@@ -4306,10 +4303,10 @@
       <c r="M24" s="25"/>
       <c r="N24" s="25"/>
       <c r="O24" s="27" t="s">
+        <v>283</v>
+      </c>
+      <c r="P24" s="27" t="s">
         <v>284</v>
-      </c>
-      <c r="P24" s="27" t="s">
-        <v>285</v>
       </c>
       <c r="Q24" s="28" t="str">
         <f aca="false">IF(V24="Defect","",IF(COUNT(G24:K24)&lt;5,"",ROUND(G24*Config!$B$4+H24*Config!$B$5+I24*Config!$B$6+J24*Config!$B$7+K24*Config!$B$8,2)))</f>
@@ -5493,507 +5490,507 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="37" t="s">
+        <v>286</v>
+      </c>
+      <c r="B3" s="37" t="s">
         <v>287</v>
       </c>
-      <c r="B3" s="37" t="s">
+      <c r="C3" s="37" t="s">
         <v>288</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="D3" s="37" t="s">
         <v>289</v>
       </c>
-      <c r="D3" s="37" t="s">
+      <c r="E3" s="37" t="s">
         <v>290</v>
       </c>
-      <c r="E3" s="37" t="s">
+      <c r="F3" s="37" t="s">
         <v>291</v>
-      </c>
-      <c r="F3" s="37" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
+        <v>292</v>
+      </c>
+      <c r="B4" s="18" t="s">
         <v>293</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="C4" s="18" t="s">
         <v>294</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="D4" s="18" t="s">
         <v>295</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="E4" s="18" t="s">
         <v>296</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="F4" s="18" t="s">
         <v>297</v>
-      </c>
-      <c r="F4" s="18" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
+        <v>298</v>
+      </c>
+      <c r="B5" s="18" t="s">
         <v>299</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="C5" s="18" t="s">
+        <v>294</v>
+      </c>
+      <c r="D5" s="18" t="s">
         <v>300</v>
       </c>
-      <c r="C5" s="18" t="s">
-        <v>295</v>
-      </c>
-      <c r="D5" s="18" t="s">
+      <c r="E5" s="18" t="s">
+        <v>296</v>
+      </c>
+      <c r="F5" s="18" t="s">
         <v>301</v>
-      </c>
-      <c r="E5" s="18" t="s">
-        <v>297</v>
-      </c>
-      <c r="F5" s="18" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
+        <v>302</v>
+      </c>
+      <c r="B6" s="18" t="s">
         <v>303</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="C6" s="18" t="s">
+        <v>294</v>
+      </c>
+      <c r="D6" s="18" t="s">
         <v>304</v>
       </c>
-      <c r="C6" s="18" t="s">
-        <v>295</v>
-      </c>
-      <c r="D6" s="18" t="s">
+      <c r="E6" s="18" t="s">
+        <v>296</v>
+      </c>
+      <c r="F6" s="18" t="s">
         <v>305</v>
-      </c>
-      <c r="E6" s="18" t="s">
-        <v>297</v>
-      </c>
-      <c r="F6" s="18" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
+        <v>306</v>
+      </c>
+      <c r="B7" s="18" t="s">
         <v>307</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="C7" s="18" t="s">
         <v>308</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="D7" s="18" t="s">
         <v>309</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="E7" s="18" t="s">
         <v>310</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="F7" s="18" t="s">
         <v>311</v>
-      </c>
-      <c r="F7" s="18" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
+        <v>312</v>
+      </c>
+      <c r="B8" s="18" t="s">
         <v>313</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="C8" s="18" t="s">
+        <v>308</v>
+      </c>
+      <c r="D8" s="18" t="s">
         <v>314</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>309</v>
-      </c>
-      <c r="D8" s="18" t="s">
+      <c r="E8" s="18" t="s">
         <v>315</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="F8" s="18" t="s">
         <v>316</v>
-      </c>
-      <c r="F8" s="18" t="s">
-        <v>317</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
+        <v>317</v>
+      </c>
+      <c r="B9" s="18" t="s">
         <v>318</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="C9" s="18" t="s">
         <v>319</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="D9" s="18" t="s">
         <v>320</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="E9" s="18" t="s">
+        <v>315</v>
+      </c>
+      <c r="F9" s="18" t="s">
         <v>321</v>
-      </c>
-      <c r="E9" s="18" t="s">
-        <v>316</v>
-      </c>
-      <c r="F9" s="18" t="s">
-        <v>322</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
+        <v>322</v>
+      </c>
+      <c r="B10" s="18" t="s">
         <v>323</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="C10" s="18" t="s">
         <v>324</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="D10" s="18" t="s">
         <v>325</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="E10" s="18" t="s">
         <v>326</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="F10" s="18" t="s">
         <v>327</v>
-      </c>
-      <c r="F10" s="18" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
+        <v>328</v>
+      </c>
+      <c r="B11" s="18" t="s">
         <v>329</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="C11" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="F11" s="18" t="s">
         <v>330</v>
-      </c>
-      <c r="C11" s="18" t="s">
-        <v>325</v>
-      </c>
-      <c r="D11" s="18" t="s">
-        <v>326</v>
-      </c>
-      <c r="E11" s="18" t="s">
-        <v>327</v>
-      </c>
-      <c r="F11" s="18" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
+        <v>331</v>
+      </c>
+      <c r="B12" s="18" t="s">
         <v>332</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="C12" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="E12" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="F12" s="18" t="s">
         <v>333</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>325</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>326</v>
-      </c>
-      <c r="E12" s="18" t="s">
-        <v>327</v>
-      </c>
-      <c r="F12" s="18" t="s">
-        <v>334</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
+        <v>334</v>
+      </c>
+      <c r="B13" s="18" t="s">
         <v>335</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="C13" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>296</v>
+      </c>
+      <c r="F13" s="18" t="s">
         <v>336</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>325</v>
-      </c>
-      <c r="D13" s="18" t="s">
-        <v>326</v>
-      </c>
-      <c r="E13" s="18" t="s">
-        <v>297</v>
-      </c>
-      <c r="F13" s="18" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
+        <v>337</v>
+      </c>
+      <c r="B14" s="18" t="s">
         <v>338</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="C14" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="F14" s="18" t="s">
         <v>339</v>
-      </c>
-      <c r="C14" s="18" t="s">
-        <v>325</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>326</v>
-      </c>
-      <c r="E14" s="18" t="s">
-        <v>327</v>
-      </c>
-      <c r="F14" s="18" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
+        <v>340</v>
+      </c>
+      <c r="B15" s="18" t="s">
         <v>341</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="C15" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="E15" s="18" t="s">
+        <v>315</v>
+      </c>
+      <c r="F15" s="18" t="s">
         <v>342</v>
-      </c>
-      <c r="C15" s="18" t="s">
-        <v>325</v>
-      </c>
-      <c r="D15" s="18" t="s">
-        <v>326</v>
-      </c>
-      <c r="E15" s="18" t="s">
-        <v>316</v>
-      </c>
-      <c r="F15" s="18" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
+        <v>343</v>
+      </c>
+      <c r="B16" s="18" t="s">
         <v>344</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="C16" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="E16" s="18" t="s">
         <v>345</v>
       </c>
-      <c r="C16" s="18" t="s">
-        <v>325</v>
-      </c>
-      <c r="D16" s="18" t="s">
-        <v>326</v>
-      </c>
-      <c r="E16" s="18" t="s">
+      <c r="F16" s="18" t="s">
         <v>346</v>
-      </c>
-      <c r="F16" s="18" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
+        <v>347</v>
+      </c>
+      <c r="B17" s="18" t="s">
         <v>348</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="C17" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>296</v>
+      </c>
+      <c r="F17" s="18" t="s">
         <v>349</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>325</v>
-      </c>
-      <c r="D17" s="18" t="s">
-        <v>326</v>
-      </c>
-      <c r="E17" s="18" t="s">
-        <v>297</v>
-      </c>
-      <c r="F17" s="18" t="s">
-        <v>350</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
+        <v>350</v>
+      </c>
+      <c r="B18" s="18" t="s">
         <v>351</v>
       </c>
-      <c r="B18" s="18" t="s">
+      <c r="C18" s="18" t="s">
+        <v>294</v>
+      </c>
+      <c r="D18" s="18" t="s">
         <v>352</v>
       </c>
-      <c r="C18" s="18" t="s">
-        <v>295</v>
-      </c>
-      <c r="D18" s="18" t="s">
+      <c r="E18" s="18" t="s">
+        <v>315</v>
+      </c>
+      <c r="F18" s="18" t="s">
         <v>353</v>
-      </c>
-      <c r="E18" s="18" t="s">
-        <v>316</v>
-      </c>
-      <c r="F18" s="18" t="s">
-        <v>354</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
+        <v>354</v>
+      </c>
+      <c r="B19" s="18" t="s">
         <v>355</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="C19" s="18" t="s">
+        <v>294</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>300</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>315</v>
+      </c>
+      <c r="F19" s="18" t="s">
         <v>356</v>
-      </c>
-      <c r="C19" s="18" t="s">
-        <v>295</v>
-      </c>
-      <c r="D19" s="18" t="s">
-        <v>301</v>
-      </c>
-      <c r="E19" s="18" t="s">
-        <v>316</v>
-      </c>
-      <c r="F19" s="18" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
+        <v>357</v>
+      </c>
+      <c r="B20" s="18" t="s">
         <v>358</v>
       </c>
-      <c r="B20" s="18" t="s">
+      <c r="C20" s="18" t="s">
         <v>359</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="D20" s="18" t="s">
         <v>360</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="E20" s="18" t="s">
         <v>361</v>
       </c>
-      <c r="E20" s="18" t="s">
+      <c r="F20" s="18" t="s">
         <v>362</v>
-      </c>
-      <c r="F20" s="18" t="s">
-        <v>363</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
+        <v>363</v>
+      </c>
+      <c r="B21" s="18" t="s">
         <v>364</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="C21" s="18" t="s">
+        <v>359</v>
+      </c>
+      <c r="D21" s="18" t="s">
         <v>365</v>
       </c>
-      <c r="C21" s="18" t="s">
-        <v>360</v>
-      </c>
-      <c r="D21" s="18" t="s">
+      <c r="E21" s="18" t="s">
+        <v>361</v>
+      </c>
+      <c r="F21" s="18" t="s">
         <v>366</v>
-      </c>
-      <c r="E21" s="18" t="s">
-        <v>362</v>
-      </c>
-      <c r="F21" s="18" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
+        <v>367</v>
+      </c>
+      <c r="B22" s="18" t="s">
         <v>368</v>
       </c>
-      <c r="B22" s="18" t="s">
+      <c r="C22" s="18" t="s">
+        <v>359</v>
+      </c>
+      <c r="D22" s="18" t="s">
         <v>369</v>
       </c>
-      <c r="C22" s="18" t="s">
-        <v>360</v>
-      </c>
-      <c r="D22" s="18" t="s">
+      <c r="E22" s="18" t="s">
+        <v>361</v>
+      </c>
+      <c r="F22" s="18" t="s">
         <v>370</v>
-      </c>
-      <c r="E22" s="18" t="s">
-        <v>362</v>
-      </c>
-      <c r="F22" s="18" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
+        <v>371</v>
+      </c>
+      <c r="B23" s="18" t="s">
         <v>372</v>
       </c>
-      <c r="B23" s="18" t="s">
+      <c r="C23" s="18" t="s">
+        <v>359</v>
+      </c>
+      <c r="D23" s="18" t="s">
         <v>373</v>
       </c>
-      <c r="C23" s="18" t="s">
-        <v>360</v>
-      </c>
-      <c r="D23" s="18" t="s">
+      <c r="E23" s="18" t="s">
+        <v>361</v>
+      </c>
+      <c r="F23" s="18" t="s">
         <v>374</v>
-      </c>
-      <c r="E23" s="18" t="s">
-        <v>362</v>
-      </c>
-      <c r="F23" s="18" t="s">
-        <v>375</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
+        <v>375</v>
+      </c>
+      <c r="B24" s="18" t="s">
         <v>376</v>
       </c>
-      <c r="B24" s="18" t="s">
+      <c r="C24" s="18" t="s">
+        <v>359</v>
+      </c>
+      <c r="D24" s="18" t="s">
         <v>377</v>
       </c>
-      <c r="C24" s="18" t="s">
-        <v>360</v>
-      </c>
-      <c r="D24" s="18" t="s">
+      <c r="E24" s="18" t="s">
+        <v>361</v>
+      </c>
+      <c r="F24" s="18" t="s">
         <v>378</v>
-      </c>
-      <c r="E24" s="18" t="s">
-        <v>362</v>
-      </c>
-      <c r="F24" s="18" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
+        <v>379</v>
+      </c>
+      <c r="B25" s="18" t="s">
         <v>380</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="C25" s="18" t="s">
+        <v>308</v>
+      </c>
+      <c r="D25" s="18" t="s">
         <v>381</v>
       </c>
-      <c r="C25" s="18" t="s">
-        <v>309</v>
-      </c>
-      <c r="D25" s="18" t="s">
+      <c r="E25" s="18" t="s">
+        <v>296</v>
+      </c>
+      <c r="F25" s="18" t="s">
         <v>382</v>
-      </c>
-      <c r="E25" s="18" t="s">
-        <v>297</v>
-      </c>
-      <c r="F25" s="18" t="s">
-        <v>383</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
+        <v>383</v>
+      </c>
+      <c r="B26" s="18" t="s">
         <v>384</v>
       </c>
-      <c r="B26" s="18" t="s">
+      <c r="C26" s="18" t="s">
+        <v>308</v>
+      </c>
+      <c r="D26" s="18" t="s">
         <v>385</v>
       </c>
-      <c r="C26" s="18" t="s">
-        <v>309</v>
-      </c>
-      <c r="D26" s="18" t="s">
+      <c r="E26" s="18" t="s">
         <v>386</v>
       </c>
-      <c r="E26" s="18" t="s">
+      <c r="F26" s="18" t="s">
         <v>387</v>
-      </c>
-      <c r="F26" s="18" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="B27" s="18" t="s">
         <v>389</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="C27" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="D27" s="18" t="s">
         <v>390</v>
       </c>
-      <c r="C27" s="18" t="s">
-        <v>325</v>
-      </c>
-      <c r="D27" s="18" t="s">
+      <c r="E27" s="18" t="s">
         <v>391</v>
       </c>
-      <c r="E27" s="18" t="s">
+      <c r="F27" s="18" t="s">
         <v>392</v>
-      </c>
-      <c r="F27" s="18" t="s">
-        <v>393</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: mark D-006 In Progress (fix-defect-or-bug, TLS-enforcement scope)
Working D-006's TLS-enforcement leg (reject non-https peer URLs when a
credential is set or in production), which also closes the folded-in D-007
Sev5 cleartext-secret leak. HMAC/mTLS and SSRF allowlist remain out of scope.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSQAV9AspmwvxZ78jg9QNx
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="394">
   <si>
     <t xml:space="preserve">FEATURE VALUE SCORING FRAMEWORK</t>
   </si>
@@ -762,6 +762,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://github.com/dispatch-derek/admin-console/issues/16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In Progress</t>
   </si>
   <si>
     <t xml:space="preserve">Re-verified 2026-07-19 (main, F-004 merged via PR #17): bff/src/relay/http-peer-transport.ts:60-67 POST sends only content-type + x-event-delivery-id, no HMAC/signature/bearer/mTLS; bff/src/relay/config.ts:13-17 EVENT_BUS_URL parsed with no scheme validation (http:// accepted); bff/.env.example:24-25 and bff/.env:25 EVENT_BUS_MODE=inproc, EVENT_BUS_URL empty -&gt; HttpPeerTransport inactive in known deployment; bff/src/config.ts:40-56 bus/inproc gating; security/F-004-review.md finding F2 [Medium] independent confirmation; GH issue #16.</t>
@@ -3783,7 +3786,7 @@
         <v>245</v>
       </c>
       <c r="D17" s="22" t="s">
-        <v>171</v>
+        <v>246</v>
       </c>
       <c r="E17" s="22" t="s">
         <v>172</v>
@@ -3804,10 +3807,10 @@
       <c r="M17" s="25"/>
       <c r="N17" s="25"/>
       <c r="O17" s="27" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="P17" s="27" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="Q17" s="28" t="str">
         <f aca="false">IF(V17="Defect","",IF(COUNT(G17:K17)&lt;5,"",ROUND(G17*Config!$B$4+H17*Config!$B$5+I17*Config!$B$6+J17*Config!$B$7+K17*Config!$B$8,2)))</f>
@@ -3841,13 +3844,13 @@
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="22" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B18" s="23" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D18" s="22" t="s">
         <v>171</v>
@@ -3883,10 +3886,10 @@
         <v>5</v>
       </c>
       <c r="O18" s="27" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="P18" s="27" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="Q18" s="28" t="n">
         <f aca="false">IF(V18="Defect","",IF(COUNT(G18:K18)&lt;5,"",ROUND(G18*Config!$B$4+H18*Config!$B$5+I18*Config!$B$6+J18*Config!$B$7+K18*Config!$B$8,2)))</f>
@@ -3914,13 +3917,13 @@
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="22" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B19" s="23" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C19" s="22" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D19" s="22" t="s">
         <v>190</v>
@@ -3929,7 +3932,7 @@
         <v>172</v>
       </c>
       <c r="F19" s="22" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G19" s="25" t="n">
         <v>2</v>
@@ -3956,10 +3959,10 @@
         <v>5</v>
       </c>
       <c r="O19" s="27" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="P19" s="27" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="Q19" s="28" t="n">
         <f aca="false">IF(V19="Defect","",IF(COUNT(G19:K19)&lt;5,"",ROUND(G19*Config!$B$4+H19*Config!$B$5+I19*Config!$B$6+J19*Config!$B$7+K19*Config!$B$8,2)))</f>
@@ -3987,22 +3990,22 @@
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="22" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D20" s="22" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E20" s="22" t="s">
         <v>172</v>
       </c>
       <c r="F20" s="22" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G20" s="25" t="n">
         <v>5</v>
@@ -4029,10 +4032,10 @@
         <v>6</v>
       </c>
       <c r="O20" s="27" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="P20" s="27" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="Q20" s="28" t="n">
         <f aca="false">IF(V20="Defect","",IF(COUNT(G20:K20)&lt;5,"",ROUND(G20*Config!$B$4+H20*Config!$B$5+I20*Config!$B$6+J20*Config!$B$7+K20*Config!$B$8,2)))</f>
@@ -4060,22 +4063,22 @@
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="22" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C21" s="22" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D21" s="22" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E21" s="22" t="s">
         <v>172</v>
       </c>
       <c r="F21" s="22" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G21" s="25" t="n">
         <v>5</v>
@@ -4102,10 +4105,10 @@
         <v>6</v>
       </c>
       <c r="O21" s="27" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="P21" s="27" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="Q21" s="28" t="n">
         <f aca="false">IF(V21="Defect","",IF(COUNT(G21:K21)&lt;5,"",ROUND(G21*Config!$B$4+H21*Config!$B$5+I21*Config!$B$6+J21*Config!$B$7+K21*Config!$B$8,2)))</f>
@@ -4133,22 +4136,22 @@
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="22" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E22" s="22" t="s">
         <v>172</v>
       </c>
       <c r="F22" s="22" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="G22" s="25" t="n">
         <v>4</v>
@@ -4175,10 +4178,10 @@
         <v>7</v>
       </c>
       <c r="O22" s="27" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="P22" s="27" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="Q22" s="28" t="n">
         <f aca="false">IF(V22="Defect","",IF(COUNT(G22:K22)&lt;5,"",ROUND(G22*Config!$B$4+H22*Config!$B$5+I22*Config!$B$6+J22*Config!$B$7+K22*Config!$B$8,2)))</f>
@@ -4206,13 +4209,13 @@
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="22" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D23" s="22" t="s">
         <v>171</v>
@@ -4236,10 +4239,10 @@
       <c r="M23" s="25"/>
       <c r="N23" s="25"/>
       <c r="O23" s="27" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="P23" s="27" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="Q23" s="28" t="str">
         <f aca="false">IF(V23="Defect","",IF(COUNT(G23:K23)&lt;5,"",ROUND(G23*Config!$B$4+H23*Config!$B$5+I23*Config!$B$6+J23*Config!$B$7+K23*Config!$B$8,2)))</f>
@@ -4273,13 +4276,13 @@
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="22" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C24" s="22" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D24" s="22" t="s">
         <v>171</v>
@@ -4303,10 +4306,10 @@
       <c r="M24" s="25"/>
       <c r="N24" s="25"/>
       <c r="O24" s="27" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="P24" s="27" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="Q24" s="28" t="str">
         <f aca="false">IF(V24="Defect","",IF(COUNT(G24:K24)&lt;5,"",ROUND(G24*Config!$B$4+H24*Config!$B$5+I24*Config!$B$6+J24*Config!$B$7+K24*Config!$B$8,2)))</f>
@@ -5490,507 +5493,507 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="37" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B3" s="37" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C3" s="37" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D3" s="37" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E3" s="37" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F3" s="37" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="F27" s="18" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: D-006 + D-007 -> Fixed (fix-defect-or-bug write-back)
D-006 TLS-enforcement leg fixed (https-only peer guard); D-007's cleartext-
secret exposure closed via the same fix per the fold-into-D-006 ruling.
Both rows -> Fixed with provenance. D-006's HMAC/mTLS + SSRF legs remain
open under the row's broader scope / GH #16.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSQAV9AspmwvxZ78jg9QNx
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -764,13 +764,13 @@
     <t xml:space="preserve">https://github.com/dispatch-derek/admin-console/issues/16</t>
   </si>
   <si>
-    <t xml:space="preserve">In Progress</t>
+    <t xml:space="preserve">Fixed</t>
   </si>
   <si>
     <t xml:space="preserve">Re-verified 2026-07-19 (main, F-004 merged via PR #17): bff/src/relay/http-peer-transport.ts:60-67 POST sends only content-type + x-event-delivery-id, no HMAC/signature/bearer/mTLS; bff/src/relay/config.ts:13-17 EVENT_BUS_URL parsed with no scheme validation (http:// accepted); bff/.env.example:24-25 and bff/.env:25 EVENT_BUS_MODE=inproc, EVENT_BUS_URL empty -&gt; HttpPeerTransport inactive in known deployment; bff/src/config.ts:40-56 bus/inproc gating; security/F-004-review.md finding F2 [Medium] independent confirmation; GH issue #16.</t>
   </si>
   <si>
-    <t xml:space="preserve">[intake 2026-07-19] Logged from F-004 Phase 7 security review (security/F-004-review.md, finding F2 [Medium]). Accepted for GTM: peers are operator-controlled endpoints on a trusted network and the peer trust model was explicitly deferred by the F-004 spec. Follow-up: HMAC body signing or mTLS, plus require https:// peers when NODE_ENV=production (allow internal http:// only behind a service mesh by opt-in). See also security review F3 (/ready bind address) and F4 (outbound SSRF allowlist). GH issue #16. | [research 2026-07-19] reach=1 (anchor 1 'rare edge case': exposure requires opting into EVENT_BUS_MODE=bus + peer URLs + http/MITM-able hop; known deployment runs inproc, ~0 operators hit it today). confidence=9 (anchor 9: absent-control confirmed by direct code read at exact lines + independent security review F2; residual unknown only that no live bus-mode deployment exercises the path). Not inflating reach to compensate severity - severity (human, 2) carries the fast-track formula by design.</t>
+    <t xml:space="preserve">[intake 2026-07-19] Logged from F-004 Phase 7 security review (security/F-004-review.md, finding F2 [Medium]). Accepted for GTM: peers are operator-controlled endpoints on a trusted network and the peer trust model was explicitly deferred by the F-004 spec. Follow-up: HMAC body signing or mTLS, plus require https:// peers when NODE_ENV=production (allow internal http:// only behind a service mesh by opt-in). See also security review F3 (/ready bind address) and F4 (outbound SSRF allowlist). GH issue #16. | [research 2026-07-19] reach=1 (anchor 1 'rare edge case': exposure requires opting into EVENT_BUS_MODE=bus + peer URLs + http/MITM-able hop; known deployment runs inproc, ~0 operators hit it today). confidence=9 (anchor 9: absent-control confirmed by direct code read at exact lines + independent security review F2; residual unknown only that no live bus-mode deployment exercises the path). Not inflating reach to compensate severity - severity (human, 2) carries the fast-track formula by design. || [fix-defect-or-bug 2026-07-23] root cause: config.ts parsed EVENT_BUS_URL with no scheme validation (http:// accepted). Fixed (TLS-enforcement leg): boot-time fail-fast rejecting non-https:// peer URLs when a credential is configured OR NODE_ENV=production (bff/src/relay/config.ts); http:// allowed only in dev w/o credential. Regression: bff/test/relay/relay-config.d006.test.ts (+ config-scheme-guard.unit.test.ts). Full suite green; security PASS, code review APPROVE. HMAC/mTLS message-auth + SSRF host-allowlist legs remain OPEN under D-006/#16.</t>
   </si>
   <si>
     <t xml:space="preserve">F-009</t>
@@ -866,7 +866,7 @@
     <t xml:space="preserve">Logged 2026-07-22 (Internal). F-010 introduces a shared-secret credential on the relay's outbound POST (header X-Event-Auth-Token / env EVENT_BUS_PEER_AUTH_TOKEN; spec specs/F-010-deliver-admin-events-to-customer-web-app.md REQ-F010-005/-007). bff/src/relay/config.ts splits/trims/filters EVENT_BUS_URL with 0 scheme validation, so http:// peer URLs are accepted (all 3 README examples at bff/src/relay/README.md are http://). Result: any http:// peer transmits the secret in cleartext on every delivery -&gt; credential disclosure -&gt; forgeable admin.user.* events into the consumer. Not live today (EVENT_BUS_MODE=inproc, no credential code path); becomes exploitable the moment F-010 ships with any http:// peer. GH issue #39. || [RESEARCH 2026-07-23 re-verified vs main, F-010 merged] config.ts: EVENT_BUS_URL split/trim/filter only, NO URL-scheme validation, http:// accepted. http-peer-transport.ts:18 AUTH_TOKEN_HEADER='X-Event-Auth-Token', :90-91 attached to every outbound POST when credential configured, :93 fetch to peer URL verbatim -&gt; http:// peer carries secret in cleartext. README.md:26,40,54 all peer examples http://; :90-92 Security caveat; :182 threat-model F2. GH #39; related D-006/#16 (https-only/mTLS, separate track). No support tickets/analytics/demand records (internal tool).</t>
   </si>
   <si>
-    <t xml:space="preserve">Distinct from but overlapping D-006 (GH #16): D-006 = broad relay transport hardening (HMAC/mTLS + https-only enforcement), scored while the transport was inactive; this row = the concrete secret-disclosure that F-010 makes active. Surfaced as F-010 spec Open Question Q4 (scheme validation deliberately left to D-006). Minimal fix = fail-fast reject of non-https peer URLs when a credential is configured (bff/src/relay/config.ts). Severity + scoring left for triage/prioritization; triage to decide fix-here vs fold-into-D-006. || [RESEARCH 2026-07-23] reach=2 (Rubric: &lt;5%/rare edge case): exposure gated behind bus-mode relay + http:// peer + on-path observer; https:// unaffected; nudged off floor because README ships http:// examples. confidence=9: code-certain multi-source repro (config.ts, http-peer-transport.ts:90-91, README); held below 10 for lack of a live cleartext capture. severity untouched (human=5). || [human ruling 2026-07-23] Sev1 sign-off: Prioritized. Fix FOLDED INTO D-006 (GH #16) per product-owner decision — a single https-only/mTLS relay-hardening effort covers this cleartext-credential leak; do not fix D-007 as a standalone patch. See GH #39/#16.</t>
+    <t xml:space="preserve">Distinct from but overlapping D-006 (GH #16): D-006 = broad relay transport hardening (HMAC/mTLS + https-only enforcement), scored while the transport was inactive; this row = the concrete secret-disclosure that F-010 makes active. Surfaced as F-010 spec Open Question Q4 (scheme validation deliberately left to D-006). Minimal fix = fail-fast reject of non-https peer URLs when a credential is configured (bff/src/relay/config.ts). Severity + scoring left for triage/prioritization; triage to decide fix-here vs fold-into-D-006. || [RESEARCH 2026-07-23] reach=2 (Rubric: &lt;5%/rare edge case): exposure gated behind bus-mode relay + http:// peer + on-path observer; https:// unaffected; nudged off floor because README ships http:// examples. confidence=9: code-certain multi-source repro (config.ts, http-peer-transport.ts:90-91, README); held below 10 for lack of a live cleartext capture. severity untouched (human=5). || [human ruling 2026-07-23] Sev1 sign-off: Prioritized. Fix FOLDED INTO D-006 (GH #16) per product-owner decision — a single https-only/mTLS relay-hardening effort covers this cleartext-credential leak; do not fix D-007 as a standalone patch. See GH #39/#16. || [fix-defect-or-bug 2026-07-23] FIXED VIA D-006: the cleartext-secret exposure is closed by D-006 https-only peer enforcement (config.ts fail-fast; the same isCredentialConfigured predicate gates both credential attachment and non-https rejection, so the secret can never traverse http://). No standalone D-007 patch, per the 2026-07-23 fold-into-D-006 ruling. GH #39.</t>
   </si>
   <si>
     <t xml:space="preserve">D-008</t>
@@ -4218,7 +4218,7 @@
         <v>278</v>
       </c>
       <c r="D23" s="22" t="s">
-        <v>171</v>
+        <v>246</v>
       </c>
       <c r="E23" s="22" t="s">
         <v>172</v>

</xml_diff>

<commit_message>
chore: mark D-008 In Progress (fix-defect-or-bug, /metrics scope)
Exposing the relay event counters via a new GET /metrics endpoint so
partially-delivered vs never-delivered parks are observable to operators.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSQAV9AspmwvxZ78jg9QNx
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="394">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="395">
   <si>
     <t xml:space="preserve">FEATURE VALUE SCORING FRAMEWORK</t>
   </si>
@@ -876,6 +876,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://github.com/dispatch-derek/admin-console/issues/40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In Progress</t>
   </si>
   <si>
     <t xml:space="preserve">Logged 2026-07-23 (Internal); surfaced by F-010 Phase-6 e2e. recordPartiallyDeliveredPark() counter (bff/src/relay/metrics.ts:57-58, incremented at drainer.ts:71) is a process-lifetime singleton with NO exported getter/snapshot; only DB-backed gauges getBacklogCount/getRelayLagMs are wired out (index.ts:14,46-47). No /metrics endpoint, no /ready field (ready.ts exposes only eventBusUrlConfigured), and setLastError(row.id, errText(err)) (drainer.ts:80) writes a generic TransportError message that does not encode partial-vs-never-delivered. So operators cannot distinguish a partially-delivered park (acked peer holds a dedupable copy) from a never-delivered one, nor see the counter at all. Verified first-hand. GH issue #40. || [RESEARCH 2026-07-23 re-verified vs main] Counter is process-lifetime singleton: metrics.ts:37-59 counters, :57-58 recordPartiallyDeliveredPark, incremented drainer.ts:71. getCounters() EXISTS at metrics.ts:66-68 but is DEAD CODE (grep: zero consumers) -&gt; counters still externally unobservable. Only DB gauges wired out: index.ts:14,46-47 (getBacklogCount, getRelayLagMs). /ready exposes no counter/park field: ready.ts:8-16,21-39. No /metrics route anywhere (grep). last_error generic: drainer.ts:80 setLastError(row.id, errText(err)); partial-vs-never captured only at recordPark drainer.ts:70-73 feeding the unobservable counter. GH #40; predates F-010 (F-004 REQ-F004-025/-051(e)); no data loss. No tickets/analytics/demand (internal tool).</t>
@@ -4285,7 +4288,7 @@
         <v>283</v>
       </c>
       <c r="D24" s="22" t="s">
-        <v>171</v>
+        <v>284</v>
       </c>
       <c r="E24" s="22" t="s">
         <v>172</v>
@@ -4306,10 +4309,10 @@
       <c r="M24" s="25"/>
       <c r="N24" s="25"/>
       <c r="O24" s="27" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="P24" s="27" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="Q24" s="28" t="str">
         <f aca="false">IF(V24="Defect","",IF(COUNT(G24:K24)&lt;5,"",ROUND(G24*Config!$B$4+H24*Config!$B$5+I24*Config!$B$6+J24*Config!$B$7+K24*Config!$B$8,2)))</f>
@@ -5493,507 +5496,507 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="37" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B3" s="37" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C3" s="37" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D3" s="37" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E3" s="37" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F3" s="37" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="F27" s="18" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: D-008 -> Fixed (fix-defect-or-bug write-back)
Relay GET /metrics endpoint surfaces the event counters; partially- vs
never-delivered parks now observable. Full suite green; security PASS WITH
NOTES, code review APPROVE WITH COMMENTS. Provenance appended.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSQAV9AspmwvxZ78jg9QNx
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="394">
   <si>
     <t xml:space="preserve">FEATURE VALUE SCORING FRAMEWORK</t>
   </si>
@@ -878,13 +878,10 @@
     <t xml:space="preserve">https://github.com/dispatch-derek/admin-console/issues/40</t>
   </si>
   <si>
-    <t xml:space="preserve">In Progress</t>
-  </si>
-  <si>
     <t xml:space="preserve">Logged 2026-07-23 (Internal); surfaced by F-010 Phase-6 e2e. recordPartiallyDeliveredPark() counter (bff/src/relay/metrics.ts:57-58, incremented at drainer.ts:71) is a process-lifetime singleton with NO exported getter/snapshot; only DB-backed gauges getBacklogCount/getRelayLagMs are wired out (index.ts:14,46-47). No /metrics endpoint, no /ready field (ready.ts exposes only eventBusUrlConfigured), and setLastError(row.id, errText(err)) (drainer.ts:80) writes a generic TransportError message that does not encode partial-vs-never-delivered. So operators cannot distinguish a partially-delivered park (acked peer holds a dedupable copy) from a never-delivered one, nor see the counter at all. Verified first-hand. GH issue #40. || [RESEARCH 2026-07-23 re-verified vs main] Counter is process-lifetime singleton: metrics.ts:37-59 counters, :57-58 recordPartiallyDeliveredPark, incremented drainer.ts:71. getCounters() EXISTS at metrics.ts:66-68 but is DEAD CODE (grep: zero consumers) -&gt; counters still externally unobservable. Only DB gauges wired out: index.ts:14,46-47 (getBacklogCount, getRelayLagMs). /ready exposes no counter/park field: ready.ts:8-16,21-39. No /metrics route anywhere (grep). last_error generic: drainer.ts:80 setLastError(row.id, errText(err)); partial-vs-never captured only at recordPark drainer.ts:70-73 feeding the unobservable counter. GH #40; predates F-010 (F-004 REQ-F004-025/-051(e)); no data loss. No tickets/analytics/demand (internal tool).</t>
   </si>
   <si>
-    <t xml:space="preserve">Predates F-010: the counter and REQ-F004-051(e)/REQ-F004-025 partial-vs-never split are F-004 machinery; no F-004 test asserted external observability. Surfaced because REQ-F010-015 is the first requirement to state 'operators MUST be able to observe this outcome' against this counter. Observability/operability defect, not correctness (row is retained/parked, no data loss). Fix direction: expose event counters via /metrics or /ready, and/or encode partial-vs-never in the parked row's last_error. Severity + scoring left for triage. Relates to F-010 (REQ-F010-015) and F-004 (REQ-F004-025). || [RESEARCH 2026-07-23] reach=1 (Rubric: &lt;3%/rare edge case): only bites during a partially-delivered-park incident (drainer.ts:69-73 partialAck path) on an internal tool with small operator population; floor, not inflated. confidence=9: structurally provable across 4 files + negative /metrics grep; held below 10 (static inspection, not live incident repro). REMEDIATION NOTE: getCounters() already exists as dead code -&gt; fix likely just wires it to /metrics or /ready. severity untouched (human=3).</t>
+    <t xml:space="preserve">Predates F-010: the counter and REQ-F004-051(e)/REQ-F004-025 partial-vs-never split are F-004 machinery; no F-004 test asserted external observability. Surfaced because REQ-F010-015 is the first requirement to state 'operators MUST be able to observe this outcome' against this counter. Observability/operability defect, not correctness (row is retained/parked, no data loss). Fix direction: expose event counters via /metrics or /ready, and/or encode partial-vs-never in the parked row's last_error. Severity + scoring left for triage. Relates to F-010 (REQ-F010-015) and F-004 (REQ-F004-025). || [RESEARCH 2026-07-23] reach=1 (Rubric: &lt;3%/rare edge case): only bites during a partially-delivered-park incident (drainer.ts:69-73 partialAck path) on an internal tool with small operator population; floor, not inflated. confidence=9: structurally provable across 4 files + negative /metrics grep; held below 10 (static inspection, not live incident repro). REMEDIATION NOTE: getCounters() already exists as dead code -&gt; fix likely just wires it to /metrics or /ready. severity untouched (human=3). || [fix-defect-or-bug 2026-07-23] root cause: getCounters() (metrics.ts) was dead code and /ready never read the event counters, so partially-vs-never-delivered parks were unobservable. Fixed: new read-only GET /metrics route on buildReadyApp (ready.ts) returning the 5 event counters + backlogCount/relayLagMs gauges as JSON; getCounters injected via ReadyDeps (index.ts). Regression: bff/test/relay/metrics-endpoint.d008.test.ts. Full suite green; security PASS WITH NOTES (unauth telemetry, tied to F-004 F3), code review APPROVE WITH COMMENTS (non-blocking: explicit /metrics field allow-list recommended).</t>
   </si>
   <si>
     <t xml:space="preserve">DATA DICTIONARY - machine-readable field contract for agents</t>
@@ -4288,7 +4285,7 @@
         <v>283</v>
       </c>
       <c r="D24" s="22" t="s">
-        <v>284</v>
+        <v>246</v>
       </c>
       <c r="E24" s="22" t="s">
         <v>172</v>
@@ -4309,10 +4306,10 @@
       <c r="M24" s="25"/>
       <c r="N24" s="25"/>
       <c r="O24" s="27" t="s">
+        <v>284</v>
+      </c>
+      <c r="P24" s="27" t="s">
         <v>285</v>
-      </c>
-      <c r="P24" s="27" t="s">
-        <v>286</v>
       </c>
       <c r="Q24" s="28" t="str">
         <f aca="false">IF(V24="Defect","",IF(COUNT(G24:K24)&lt;5,"",ROUND(G24*Config!$B$4+H24*Config!$B$5+I24*Config!$B$6+J24*Config!$B$7+K24*Config!$B$8,2)))</f>
@@ -5496,507 +5493,507 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="37" t="s">
+        <v>287</v>
+      </c>
+      <c r="B3" s="37" t="s">
         <v>288</v>
       </c>
-      <c r="B3" s="37" t="s">
+      <c r="C3" s="37" t="s">
         <v>289</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="D3" s="37" t="s">
         <v>290</v>
       </c>
-      <c r="D3" s="37" t="s">
+      <c r="E3" s="37" t="s">
         <v>291</v>
       </c>
-      <c r="E3" s="37" t="s">
+      <c r="F3" s="37" t="s">
         <v>292</v>
-      </c>
-      <c r="F3" s="37" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
+        <v>293</v>
+      </c>
+      <c r="B4" s="18" t="s">
         <v>294</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="C4" s="18" t="s">
         <v>295</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="D4" s="18" t="s">
         <v>296</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="E4" s="18" t="s">
         <v>297</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="F4" s="18" t="s">
         <v>298</v>
-      </c>
-      <c r="F4" s="18" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
+        <v>299</v>
+      </c>
+      <c r="B5" s="18" t="s">
         <v>300</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="C5" s="18" t="s">
+        <v>295</v>
+      </c>
+      <c r="D5" s="18" t="s">
         <v>301</v>
       </c>
-      <c r="C5" s="18" t="s">
-        <v>296</v>
-      </c>
-      <c r="D5" s="18" t="s">
+      <c r="E5" s="18" t="s">
+        <v>297</v>
+      </c>
+      <c r="F5" s="18" t="s">
         <v>302</v>
-      </c>
-      <c r="E5" s="18" t="s">
-        <v>298</v>
-      </c>
-      <c r="F5" s="18" t="s">
-        <v>303</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="B6" s="18" t="s">
         <v>304</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="C6" s="18" t="s">
+        <v>295</v>
+      </c>
+      <c r="D6" s="18" t="s">
         <v>305</v>
       </c>
-      <c r="C6" s="18" t="s">
-        <v>296</v>
-      </c>
-      <c r="D6" s="18" t="s">
+      <c r="E6" s="18" t="s">
+        <v>297</v>
+      </c>
+      <c r="F6" s="18" t="s">
         <v>306</v>
-      </c>
-      <c r="E6" s="18" t="s">
-        <v>298</v>
-      </c>
-      <c r="F6" s="18" t="s">
-        <v>307</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
+        <v>307</v>
+      </c>
+      <c r="B7" s="18" t="s">
         <v>308</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="C7" s="18" t="s">
         <v>309</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="D7" s="18" t="s">
         <v>310</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="E7" s="18" t="s">
         <v>311</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="F7" s="18" t="s">
         <v>312</v>
-      </c>
-      <c r="F7" s="18" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
+        <v>313</v>
+      </c>
+      <c r="B8" s="18" t="s">
         <v>314</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="C8" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="D8" s="18" t="s">
         <v>315</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>310</v>
-      </c>
-      <c r="D8" s="18" t="s">
+      <c r="E8" s="18" t="s">
         <v>316</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="F8" s="18" t="s">
         <v>317</v>
-      </c>
-      <c r="F8" s="18" t="s">
-        <v>318</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
+        <v>318</v>
+      </c>
+      <c r="B9" s="18" t="s">
         <v>319</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="C9" s="18" t="s">
         <v>320</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="D9" s="18" t="s">
         <v>321</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="E9" s="18" t="s">
+        <v>316</v>
+      </c>
+      <c r="F9" s="18" t="s">
         <v>322</v>
-      </c>
-      <c r="E9" s="18" t="s">
-        <v>317</v>
-      </c>
-      <c r="F9" s="18" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="B10" s="18" t="s">
         <v>324</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="C10" s="18" t="s">
         <v>325</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="D10" s="18" t="s">
         <v>326</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="E10" s="18" t="s">
         <v>327</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="F10" s="18" t="s">
         <v>328</v>
-      </c>
-      <c r="F10" s="18" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
+        <v>329</v>
+      </c>
+      <c r="B11" s="18" t="s">
         <v>330</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="C11" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>327</v>
+      </c>
+      <c r="F11" s="18" t="s">
         <v>331</v>
-      </c>
-      <c r="C11" s="18" t="s">
-        <v>326</v>
-      </c>
-      <c r="D11" s="18" t="s">
-        <v>327</v>
-      </c>
-      <c r="E11" s="18" t="s">
-        <v>328</v>
-      </c>
-      <c r="F11" s="18" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
+        <v>332</v>
+      </c>
+      <c r="B12" s="18" t="s">
         <v>333</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="C12" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="E12" s="18" t="s">
+        <v>327</v>
+      </c>
+      <c r="F12" s="18" t="s">
         <v>334</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>326</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>327</v>
-      </c>
-      <c r="E12" s="18" t="s">
-        <v>328</v>
-      </c>
-      <c r="F12" s="18" t="s">
-        <v>335</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
+        <v>335</v>
+      </c>
+      <c r="B13" s="18" t="s">
         <v>336</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="C13" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>297</v>
+      </c>
+      <c r="F13" s="18" t="s">
         <v>337</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>326</v>
-      </c>
-      <c r="D13" s="18" t="s">
-        <v>327</v>
-      </c>
-      <c r="E13" s="18" t="s">
-        <v>298</v>
-      </c>
-      <c r="F13" s="18" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
+        <v>338</v>
+      </c>
+      <c r="B14" s="18" t="s">
         <v>339</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="C14" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>327</v>
+      </c>
+      <c r="F14" s="18" t="s">
         <v>340</v>
-      </c>
-      <c r="C14" s="18" t="s">
-        <v>326</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>327</v>
-      </c>
-      <c r="E14" s="18" t="s">
-        <v>328</v>
-      </c>
-      <c r="F14" s="18" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
+        <v>341</v>
+      </c>
+      <c r="B15" s="18" t="s">
         <v>342</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="C15" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="E15" s="18" t="s">
+        <v>316</v>
+      </c>
+      <c r="F15" s="18" t="s">
         <v>343</v>
-      </c>
-      <c r="C15" s="18" t="s">
-        <v>326</v>
-      </c>
-      <c r="D15" s="18" t="s">
-        <v>327</v>
-      </c>
-      <c r="E15" s="18" t="s">
-        <v>317</v>
-      </c>
-      <c r="F15" s="18" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
+        <v>344</v>
+      </c>
+      <c r="B16" s="18" t="s">
         <v>345</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="C16" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="E16" s="18" t="s">
         <v>346</v>
       </c>
-      <c r="C16" s="18" t="s">
-        <v>326</v>
-      </c>
-      <c r="D16" s="18" t="s">
-        <v>327</v>
-      </c>
-      <c r="E16" s="18" t="s">
+      <c r="F16" s="18" t="s">
         <v>347</v>
-      </c>
-      <c r="F16" s="18" t="s">
-        <v>348</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
+        <v>348</v>
+      </c>
+      <c r="B17" s="18" t="s">
         <v>349</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="C17" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>297</v>
+      </c>
+      <c r="F17" s="18" t="s">
         <v>350</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>326</v>
-      </c>
-      <c r="D17" s="18" t="s">
-        <v>327</v>
-      </c>
-      <c r="E17" s="18" t="s">
-        <v>298</v>
-      </c>
-      <c r="F17" s="18" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
+        <v>351</v>
+      </c>
+      <c r="B18" s="18" t="s">
         <v>352</v>
       </c>
-      <c r="B18" s="18" t="s">
+      <c r="C18" s="18" t="s">
+        <v>295</v>
+      </c>
+      <c r="D18" s="18" t="s">
         <v>353</v>
       </c>
-      <c r="C18" s="18" t="s">
-        <v>296</v>
-      </c>
-      <c r="D18" s="18" t="s">
+      <c r="E18" s="18" t="s">
+        <v>316</v>
+      </c>
+      <c r="F18" s="18" t="s">
         <v>354</v>
-      </c>
-      <c r="E18" s="18" t="s">
-        <v>317</v>
-      </c>
-      <c r="F18" s="18" t="s">
-        <v>355</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="B19" s="18" t="s">
         <v>356</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="C19" s="18" t="s">
+        <v>295</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>301</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>316</v>
+      </c>
+      <c r="F19" s="18" t="s">
         <v>357</v>
-      </c>
-      <c r="C19" s="18" t="s">
-        <v>296</v>
-      </c>
-      <c r="D19" s="18" t="s">
-        <v>302</v>
-      </c>
-      <c r="E19" s="18" t="s">
-        <v>317</v>
-      </c>
-      <c r="F19" s="18" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
+        <v>358</v>
+      </c>
+      <c r="B20" s="18" t="s">
         <v>359</v>
       </c>
-      <c r="B20" s="18" t="s">
+      <c r="C20" s="18" t="s">
         <v>360</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="D20" s="18" t="s">
         <v>361</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="E20" s="18" t="s">
         <v>362</v>
       </c>
-      <c r="E20" s="18" t="s">
+      <c r="F20" s="18" t="s">
         <v>363</v>
-      </c>
-      <c r="F20" s="18" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
+        <v>364</v>
+      </c>
+      <c r="B21" s="18" t="s">
         <v>365</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="C21" s="18" t="s">
+        <v>360</v>
+      </c>
+      <c r="D21" s="18" t="s">
         <v>366</v>
       </c>
-      <c r="C21" s="18" t="s">
-        <v>361</v>
-      </c>
-      <c r="D21" s="18" t="s">
+      <c r="E21" s="18" t="s">
+        <v>362</v>
+      </c>
+      <c r="F21" s="18" t="s">
         <v>367</v>
-      </c>
-      <c r="E21" s="18" t="s">
-        <v>363</v>
-      </c>
-      <c r="F21" s="18" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
+        <v>368</v>
+      </c>
+      <c r="B22" s="18" t="s">
         <v>369</v>
       </c>
-      <c r="B22" s="18" t="s">
+      <c r="C22" s="18" t="s">
+        <v>360</v>
+      </c>
+      <c r="D22" s="18" t="s">
         <v>370</v>
       </c>
-      <c r="C22" s="18" t="s">
-        <v>361</v>
-      </c>
-      <c r="D22" s="18" t="s">
+      <c r="E22" s="18" t="s">
+        <v>362</v>
+      </c>
+      <c r="F22" s="18" t="s">
         <v>371</v>
-      </c>
-      <c r="E22" s="18" t="s">
-        <v>363</v>
-      </c>
-      <c r="F22" s="18" t="s">
-        <v>372</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
+        <v>372</v>
+      </c>
+      <c r="B23" s="18" t="s">
         <v>373</v>
       </c>
-      <c r="B23" s="18" t="s">
+      <c r="C23" s="18" t="s">
+        <v>360</v>
+      </c>
+      <c r="D23" s="18" t="s">
         <v>374</v>
       </c>
-      <c r="C23" s="18" t="s">
-        <v>361</v>
-      </c>
-      <c r="D23" s="18" t="s">
+      <c r="E23" s="18" t="s">
+        <v>362</v>
+      </c>
+      <c r="F23" s="18" t="s">
         <v>375</v>
-      </c>
-      <c r="E23" s="18" t="s">
-        <v>363</v>
-      </c>
-      <c r="F23" s="18" t="s">
-        <v>376</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
+        <v>376</v>
+      </c>
+      <c r="B24" s="18" t="s">
         <v>377</v>
       </c>
-      <c r="B24" s="18" t="s">
+      <c r="C24" s="18" t="s">
+        <v>360</v>
+      </c>
+      <c r="D24" s="18" t="s">
         <v>378</v>
       </c>
-      <c r="C24" s="18" t="s">
-        <v>361</v>
-      </c>
-      <c r="D24" s="18" t="s">
+      <c r="E24" s="18" t="s">
+        <v>362</v>
+      </c>
+      <c r="F24" s="18" t="s">
         <v>379</v>
-      </c>
-      <c r="E24" s="18" t="s">
-        <v>363</v>
-      </c>
-      <c r="F24" s="18" t="s">
-        <v>380</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
+        <v>380</v>
+      </c>
+      <c r="B25" s="18" t="s">
         <v>381</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="C25" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="D25" s="18" t="s">
         <v>382</v>
       </c>
-      <c r="C25" s="18" t="s">
-        <v>310</v>
-      </c>
-      <c r="D25" s="18" t="s">
+      <c r="E25" s="18" t="s">
+        <v>297</v>
+      </c>
+      <c r="F25" s="18" t="s">
         <v>383</v>
-      </c>
-      <c r="E25" s="18" t="s">
-        <v>298</v>
-      </c>
-      <c r="F25" s="18" t="s">
-        <v>384</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="B26" s="18" t="s">
         <v>385</v>
       </c>
-      <c r="B26" s="18" t="s">
+      <c r="C26" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="D26" s="18" t="s">
         <v>386</v>
       </c>
-      <c r="C26" s="18" t="s">
-        <v>310</v>
-      </c>
-      <c r="D26" s="18" t="s">
+      <c r="E26" s="18" t="s">
         <v>387</v>
       </c>
-      <c r="E26" s="18" t="s">
+      <c r="F26" s="18" t="s">
         <v>388</v>
-      </c>
-      <c r="F26" s="18" t="s">
-        <v>389</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
+        <v>389</v>
+      </c>
+      <c r="B27" s="18" t="s">
         <v>390</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="C27" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="D27" s="18" t="s">
         <v>391</v>
       </c>
-      <c r="C27" s="18" t="s">
-        <v>326</v>
-      </c>
-      <c r="D27" s="18" t="s">
+      <c r="E27" s="18" t="s">
         <v>392</v>
       </c>
-      <c r="E27" s="18" t="s">
+      <c r="F27" s="18" t="s">
         <v>393</v>
-      </c>
-      <c r="F27" s="18" t="s">
-        <v>394</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: log F-014 — dual-key signing-key rotation window (Idea)
Deferred from the D-006 HMAC hardening spec (Q7 ruling): future feature for
zero-gap relay signing-key rotation via a consumer-side dual-key acceptance
window. Status Idea; next /write-feature-brief F-014 -> /prioritize-features.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSQAV9AspmwvxZ78jg9QNx
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="394">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="398">
   <si>
     <t xml:space="preserve">FEATURE VALUE SCORING FRAMEWORK</t>
   </si>
@@ -882,6 +882,18 @@
   </si>
   <si>
     <t xml:space="preserve">Predates F-010: the counter and REQ-F004-051(e)/REQ-F004-025 partial-vs-never split are F-004 machinery; no F-004 test asserted external observability. Surfaced because REQ-F010-015 is the first requirement to state 'operators MUST be able to observe this outcome' against this counter. Observability/operability defect, not correctness (row is retained/parked, no data loss). Fix direction: expose event counters via /metrics or /ready, and/or encode partial-vs-never in the parked row's last_error. Severity + scoring left for triage. Relates to F-010 (REQ-F010-015) and F-004 (REQ-F004-025). || [RESEARCH 2026-07-23] reach=1 (Rubric: &lt;3%/rare edge case): only bites during a partially-delivered-park incident (drainer.ts:69-73 partialAck path) on an internal tool with small operator population; floor, not inflated. confidence=9: structurally provable across 4 files + negative /metrics grep; held below 10 (static inspection, not live incident repro). REMEDIATION NOTE: getCounters() already exists as dead code -&gt; fix likely just wires it to /metrics or /ready. severity untouched (human=3). || [fix-defect-or-bug 2026-07-23] root cause: getCounters() (metrics.ts) was dead code and /ready never read the event counters, so partially-vs-never-delivered parks were unobservable. Fixed: new read-only GET /metrics route on buildReadyApp (ready.ts) returning the 5 event counters + backlogCount/relayLagMs gauges as JSON; getCounters injected via ReadyDeps (index.ts). Regression: bff/test/relay/metrics-endpoint.d008.test.ts. Full suite green; security PASS WITH NOTES (unauth telemetry, tied to F-004 F3), code review APPROVE WITH COMMENTS (non-blocking: explicit /metrics field allow-list recommended).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dual-key signing-key rotation window for relay peer HMAC (zero-gap key rotation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Idea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[logged 2026-07-23] Deferred from the D-006 relay HMAC hardening spec (specs/D-006-relay-peer-hmac-and-ssrf-hardening.md, Q7). The initial HMAC rollout uses simple coordinated re-provision+restart signing-key rotation (brief parking-risk window). This feature adds a DUAL-KEY TRANSITION WINDOW for zero-gap rotation: the consumer (cwa) accepts signatures valid under the old OR new EVENT_BUS_PEER_SIGNING_KEY during a window, so the relay can switch keys with no delivery parking. Requires cross-repo coordination (cwa consumer-side dual-key acceptance). Next: /write-feature-brief F-014 -&gt; /prioritize-features.</t>
   </si>
   <si>
     <t xml:space="preserve">DATA DICTIONARY - machine-readable field contract for agents</t>
@@ -4342,10 +4354,16 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="22"/>
-      <c r="B25" s="23"/>
+      <c r="A25" s="22" t="s">
+        <v>286</v>
+      </c>
+      <c r="B25" s="23" t="s">
+        <v>287</v>
+      </c>
       <c r="C25" s="22"/>
-      <c r="D25" s="22"/>
+      <c r="D25" s="22" t="s">
+        <v>288</v>
+      </c>
       <c r="E25" s="22"/>
       <c r="F25" s="22"/>
       <c r="G25" s="25"/>
@@ -4357,7 +4375,9 @@
       <c r="M25" s="25"/>
       <c r="N25" s="25"/>
       <c r="O25" s="27"/>
-      <c r="P25" s="27"/>
+      <c r="P25" s="27" t="s">
+        <v>289</v>
+      </c>
       <c r="Q25" s="28" t="str">
         <f aca="false">IF(V25="Defect","",IF(COUNT(G25:K25)&lt;5,"",ROUND(G25*Config!$B$4+H25*Config!$B$5+I25*Config!$B$6+J25*Config!$B$7+K25*Config!$B$8,2)))</f>
         <v/>
@@ -4378,7 +4398,9 @@
         <f aca="false">IF(T25="","",RANK(T25,$T$4:$T$52))</f>
         <v/>
       </c>
-      <c r="V25" s="36"/>
+      <c r="V25" s="36" t="s">
+        <v>175</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="22"/>
@@ -5493,507 +5515,507 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>286</v>
+        <v>290</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="37" t="s">
-        <v>287</v>
+        <v>291</v>
       </c>
       <c r="B3" s="37" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="C3" s="37" t="s">
-        <v>289</v>
+        <v>293</v>
       </c>
       <c r="D3" s="37" t="s">
-        <v>290</v>
+        <v>294</v>
       </c>
       <c r="E3" s="37" t="s">
-        <v>291</v>
+        <v>295</v>
       </c>
       <c r="F3" s="37" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>293</v>
+        <v>297</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>294</v>
+        <v>298</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>296</v>
+        <v>300</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>298</v>
+        <v>302</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
+        <v>303</v>
+      </c>
+      <c r="B5" s="18" t="s">
+        <v>304</v>
+      </c>
+      <c r="C5" s="18" t="s">
         <v>299</v>
       </c>
-      <c r="B5" s="18" t="s">
-        <v>300</v>
-      </c>
-      <c r="C5" s="18" t="s">
-        <v>295</v>
-      </c>
       <c r="D5" s="18" t="s">
+        <v>305</v>
+      </c>
+      <c r="E5" s="18" t="s">
         <v>301</v>
       </c>
-      <c r="E5" s="18" t="s">
-        <v>297</v>
-      </c>
       <c r="F5" s="18" t="s">
-        <v>302</v>
+        <v>306</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>304</v>
+        <v>308</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>305</v>
+        <v>309</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>306</v>
+        <v>310</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>308</v>
+        <v>312</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
+        <v>317</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>318</v>
+      </c>
+      <c r="C8" s="18" t="s">
         <v>313</v>
       </c>
-      <c r="B8" s="18" t="s">
-        <v>314</v>
-      </c>
-      <c r="C8" s="18" t="s">
-        <v>309</v>
-      </c>
       <c r="D8" s="18" t="s">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>317</v>
+        <v>321</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>318</v>
+        <v>322</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>319</v>
+        <v>323</v>
       </c>
       <c r="C9" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="D9" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="E9" s="18" t="s">
         <v>320</v>
       </c>
-      <c r="D9" s="18" t="s">
-        <v>321</v>
-      </c>
-      <c r="E9" s="18" t="s">
-        <v>316</v>
-      </c>
       <c r="F9" s="18" t="s">
-        <v>322</v>
+        <v>326</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>324</v>
+        <v>328</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
+        <v>333</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>334</v>
+      </c>
+      <c r="C11" s="18" t="s">
         <v>329</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="D11" s="18" t="s">
         <v>330</v>
       </c>
-      <c r="C11" s="18" t="s">
-        <v>325</v>
-      </c>
-      <c r="D11" s="18" t="s">
-        <v>326</v>
-      </c>
       <c r="E11" s="18" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>331</v>
+        <v>335</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="D12" s="18" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="F12" s="18" t="s">
-        <v>334</v>
+        <v>338</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>336</v>
+        <v>340</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>337</v>
+        <v>341</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>301</v>
+        <v>305</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>316</v>
+        <v>320</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
+        <v>368</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>369</v>
+      </c>
+      <c r="C21" s="18" t="s">
         <v>364</v>
       </c>
-      <c r="B21" s="18" t="s">
-        <v>365</v>
-      </c>
-      <c r="C21" s="18" t="s">
-        <v>360</v>
-      </c>
       <c r="D21" s="18" t="s">
+        <v>370</v>
+      </c>
+      <c r="E21" s="18" t="s">
         <v>366</v>
       </c>
-      <c r="E21" s="18" t="s">
-        <v>362</v>
-      </c>
       <c r="F21" s="18" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>297</v>
+        <v>301</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>309</v>
+        <v>313</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>325</v>
+        <v>329</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="F27" s="18" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: add F-015 — admin-console tracking Feature for D-006 HMAC/SSRF spec
Feature row so /implement-spec can run the D-006 hardening spec (D-006 is a
Fixed Defect; /implement-spec hard-stops on Defect rows). brief_ref -> the
spec. Must be implemented IN PARALLEL with customer-web-app F-009 (consumer
HMAC verification) per the 3-step cut-over. Status Brief Drafted (spec-first,
unscored).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSQAV9AspmwvxZ78jg9QNx
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="526" uniqueCount="398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="403">
   <si>
     <t xml:space="preserve">FEATURE VALUE SCORING FRAMEWORK</t>
   </si>
@@ -894,6 +894,21 @@
   </si>
   <si>
     <t xml:space="preserve">[logged 2026-07-23] Deferred from the D-006 relay HMAC hardening spec (specs/D-006-relay-peer-hmac-and-ssrf-hardening.md, Q7). The initial HMAC rollout uses simple coordinated re-provision+restart signing-key rotation (brief parking-risk window). This feature adds a DUAL-KEY TRANSITION WINDOW for zero-gap rotation: the consumer (cwa) accepts signatures valid under the old OR new EVENT_BUS_PEER_SIGNING_KEY during a window, so the relay can switch keys with no delivery parking. Requires cross-repo coordination (cwa consumer-side dual-key acceptance). Next: /write-feature-brief F-014 -&gt; /prioritize-features.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F-015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relay peer HMAC signing + SSRF host allowlist (implements D-006 remaining hardening)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">specs/D-006-relay-peer-hmac-and-ssrf-hardening.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brief Drafted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[logged 2026-07-23] Implementation-tracking Feature for D-006's remaining hardening legs (F-004 review F2 HMAC message-integrity + F4 SSRF host allowlist), spec'd at specs/D-006-relay-peer-hmac-and-ssrf-hardening.md (rev 3, RULED). Created as a FEATURE row because D-006 is a Fixed Defect and /implement-spec hard-stops on Defect rows (item_type=Defect). *** MUST BE IMPLEMENTED IN PARALLEL with customer-web-app F-009 (consumer-side HMAC verification) *** — the 3-step cut-over (cwa accept -&gt; relay sign -&gt; cwa require) parks every delivery if the producer and consumer sides are out of sync. Next: /prioritize-features to score it, or /implement-spec (with explicit go-ahead, spec-first) against the spec path. Unscored on the Feature scale.</t>
   </si>
   <si>
     <t xml:space="preserve">DATA DICTIONARY - machine-readable field contract for agents</t>
@@ -4403,10 +4418,18 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="22"/>
-      <c r="B26" s="23"/>
-      <c r="C26" s="22"/>
-      <c r="D26" s="22"/>
+      <c r="A26" s="22" t="s">
+        <v>290</v>
+      </c>
+      <c r="B26" s="23" t="s">
+        <v>291</v>
+      </c>
+      <c r="C26" s="22" t="s">
+        <v>292</v>
+      </c>
+      <c r="D26" s="22" t="s">
+        <v>293</v>
+      </c>
       <c r="E26" s="22"/>
       <c r="F26" s="22"/>
       <c r="G26" s="25"/>
@@ -4418,7 +4441,9 @@
       <c r="M26" s="25"/>
       <c r="N26" s="25"/>
       <c r="O26" s="27"/>
-      <c r="P26" s="27"/>
+      <c r="P26" s="27" t="s">
+        <v>294</v>
+      </c>
       <c r="Q26" s="28" t="str">
         <f aca="false">IF(V26="Defect","",IF(COUNT(G26:K26)&lt;5,"",ROUND(G26*Config!$B$4+H26*Config!$B$5+I26*Config!$B$6+J26*Config!$B$7+K26*Config!$B$8,2)))</f>
         <v/>
@@ -4439,7 +4464,9 @@
         <f aca="false">IF(T26="","",RANK(T26,$T$4:$T$52))</f>
         <v/>
       </c>
-      <c r="V26" s="36"/>
+      <c r="V26" s="36" t="s">
+        <v>175</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="22"/>
@@ -5515,507 +5542,507 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="37" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="B3" s="37" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="C3" s="37" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="D3" s="37" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="E3" s="37" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="F3" s="37" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="B5" s="18" t="s">
+        <v>309</v>
+      </c>
+      <c r="C5" s="18" t="s">
         <v>304</v>
       </c>
-      <c r="C5" s="18" t="s">
-        <v>299</v>
-      </c>
       <c r="D5" s="18" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="D6" s="18" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="F6" s="18" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="B8" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="C8" s="18" t="s">
         <v>318</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>313</v>
-      </c>
       <c r="D8" s="18" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="D9" s="18" t="s">
+        <v>330</v>
+      </c>
+      <c r="E9" s="18" t="s">
         <v>325</v>
       </c>
-      <c r="E9" s="18" t="s">
-        <v>320</v>
-      </c>
       <c r="F9" s="18" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="B11" s="18" t="s">
+        <v>339</v>
+      </c>
+      <c r="C11" s="18" t="s">
         <v>334</v>
       </c>
-      <c r="C11" s="18" t="s">
-        <v>329</v>
-      </c>
       <c r="D11" s="18" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
+        <v>341</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>342</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>334</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>335</v>
+      </c>
+      <c r="E12" s="18" t="s">
         <v>336</v>
       </c>
-      <c r="B12" s="18" t="s">
-        <v>337</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>329</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>330</v>
-      </c>
-      <c r="E12" s="18" t="s">
-        <v>331</v>
-      </c>
       <c r="F12" s="18" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>342</v>
+        <v>347</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>343</v>
+        <v>348</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>344</v>
+        <v>349</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
-        <v>345</v>
+        <v>350</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>346</v>
+        <v>351</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>347</v>
+        <v>352</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>348</v>
+        <v>353</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>349</v>
+        <v>354</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>350</v>
+        <v>355</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>351</v>
+        <v>356</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
-        <v>352</v>
+        <v>357</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>353</v>
+        <v>358</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>354</v>
+        <v>359</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>355</v>
+        <v>360</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>356</v>
+        <v>361</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>357</v>
+        <v>362</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>358</v>
+        <v>363</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
-        <v>359</v>
+        <v>364</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>361</v>
+        <v>366</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>368</v>
+        <v>373</v>
       </c>
       <c r="B21" s="18" t="s">
+        <v>374</v>
+      </c>
+      <c r="C21" s="18" t="s">
         <v>369</v>
       </c>
-      <c r="C21" s="18" t="s">
-        <v>364</v>
-      </c>
       <c r="D21" s="18" t="s">
-        <v>370</v>
+        <v>375</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>371</v>
+        <v>376</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
-        <v>372</v>
+        <v>377</v>
       </c>
       <c r="B22" s="18" t="s">
-        <v>373</v>
+        <v>378</v>
       </c>
       <c r="C22" s="18" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>374</v>
+        <v>379</v>
       </c>
       <c r="E22" s="18" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>375</v>
+        <v>380</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>376</v>
+        <v>381</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>377</v>
+        <v>382</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>378</v>
+        <v>383</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>379</v>
+        <v>384</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>380</v>
+        <v>385</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>381</v>
+        <v>386</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>382</v>
+        <v>387</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>383</v>
+        <v>388</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>384</v>
+        <v>389</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>385</v>
+        <v>390</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>386</v>
+        <v>391</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>387</v>
+        <v>392</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
-        <v>388</v>
+        <v>393</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>389</v>
+        <v>394</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>390</v>
+        <v>395</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>391</v>
+        <v>396</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>392</v>
+        <v>397</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
-        <v>393</v>
+        <v>398</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>394</v>
+        <v>399</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>395</v>
+        <v>400</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>396</v>
+        <v>401</v>
       </c>
       <c r="F27" s="18" t="s">
-        <v>397</v>
+        <v>402</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: log D-009 In Progress — ingest header-name mismatch (sev 4)
Relay sends X-Event-Auth-Token; cwa ingest requires X-Event-Ingest-Secret ->
every bus-mode delivery 401-parks. GH #47. Fixing via /fix-defect-or-bug:
align producer header to cwa's frozen contract.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSQAV9AspmwvxZ78jg9QNx
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="409">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="415">
   <si>
     <t xml:space="preserve">FEATURE VALUE SCORING FRAMEWORK</t>
   </si>
@@ -927,6 +927,24 @@
   </si>
   <si>
     <t xml:space="preserve">[triage 2026-07-23] severity 2 (internal test-suite health; no user/production impact; blocks e2e verification of the relay credential path). Fix (tests/e2e/ only): make the stub peer serve https (self-signed) + relay trusts it in the spawn harness. Process note: D-006's config guard gates on credential-configured, so it DID affect the credential e2e journeys - the D-006 e2e skip was the miss. || [fix-defect-or-bug 2026-07-23] root cause: e2e stub peer served http:// only, refused by D-006 https guard when a credential is set. Fixed (tests/e2e/ only): stub peer -&gt; node:https with a checked-in self-signed loopback cert; relay child trusts it via NODE_EXTRA_CA_CERTS; journeys use https:// URLs. Relay e2e 16/16 green, 3x stable; code review PASS WITH NOTES (applied). Verified via e2e. No bff/src change; no production impact.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D-009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relay sends shared secret in X-Event-Auth-Token but cwa ingest requires X-Event-Ingest-Secret (bus-mode deliveries 401-park)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/dispatch-derek/admin-console/issues/47</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In Progress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verified 2026-07-23 on main: bff/src/relay/http-peer-transport.ts:18 AUTH_TOKEN_HEADER='X-Event-Auth-Token', :91 attached to each peer POST; customer-web-app bff/src/server/ingest-auth.ts:26 reads 'x-event-ingest-secret' only and 401s otherwise (:48). Header names differ -&gt; cwa 401 -&gt; REQ-F004-055 permanent -&gt; park every admin.* delivery in bus mode. F-010 Q1 flagged this exact 'silent 401 loop' and left the header name provisional/to-be-reconciled with cwa; reconciliation never happened.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[triage 2026-07-23, human-directed immediate fix] severity 4 (major: admin-&gt;cwa event pipeline unusable in bus mode, no config workaround, no data loss - events park/retain). Fix: align producer header X-Event-Auth-Token -&gt; X-Event-Ingest-Secret (cwa's frozen consumer contract, REQ-F005-012). Env var stays EVENT_BUS_PEER_AUTH_TOKEN. Separate cwa defect renames cwa's env var INGEST_SHARED_SECRET -&gt; EVENT_BUS_PEER_AUTH_TOKEN for cross-app naming consistency.</t>
   </si>
   <si>
     <t xml:space="preserve">DATA DICTIONARY - machine-readable field contract for agents</t>
@@ -4546,12 +4564,20 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="22"/>
-      <c r="B28" s="23"/>
-      <c r="C28" s="22"/>
-      <c r="D28" s="22"/>
+      <c r="A28" s="22" t="s">
+        <v>301</v>
+      </c>
+      <c r="B28" s="23" t="s">
+        <v>302</v>
+      </c>
+      <c r="C28" s="22" t="s">
+        <v>303</v>
+      </c>
+      <c r="D28" s="22" t="s">
+        <v>304</v>
+      </c>
       <c r="E28" s="22"/>
-      <c r="F28" s="22"/>
+      <c r="F28" s="32"/>
       <c r="G28" s="25"/>
       <c r="H28" s="25"/>
       <c r="I28" s="25"/>
@@ -4560,8 +4586,12 @@
       <c r="L28" s="25"/>
       <c r="M28" s="25"/>
       <c r="N28" s="25"/>
-      <c r="O28" s="27"/>
-      <c r="P28" s="27"/>
+      <c r="O28" s="27" t="s">
+        <v>305</v>
+      </c>
+      <c r="P28" s="27" t="s">
+        <v>306</v>
+      </c>
       <c r="Q28" s="28" t="str">
         <f aca="false">IF(V28="Defect","",IF(COUNT(G28:K28)&lt;5,"",ROUND(G28*Config!$B$4+H28*Config!$B$5+I28*Config!$B$6+J28*Config!$B$7+K28*Config!$B$8,2)))</f>
         <v/>
@@ -4582,7 +4612,15 @@
         <f aca="false">IF(T28="","",RANK(T28,$T$4:$T$52))</f>
         <v/>
       </c>
-      <c r="V28" s="36"/>
+      <c r="V28" s="36" t="s">
+        <v>199</v>
+      </c>
+      <c r="W28" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="X28" s="1" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="22"/>
@@ -5580,507 +5618,507 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="37" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="B3" s="37" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="C3" s="37" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="D3" s="37" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="E3" s="37" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="F3" s="37" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>316</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="E6" s="18" t="s">
         <v>318</v>
       </c>
-      <c r="B6" s="18" t="s">
-        <v>319</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>310</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>320</v>
-      </c>
-      <c r="E6" s="18" t="s">
-        <v>312</v>
-      </c>
       <c r="F6" s="18" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>326</v>
+        <v>332</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>327</v>
+        <v>333</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
+        <v>353</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>354</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="D12" s="18" t="s">
         <v>347</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="E12" s="18" t="s">
         <v>348</v>
       </c>
-      <c r="C12" s="18" t="s">
-        <v>340</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>341</v>
-      </c>
-      <c r="E12" s="18" t="s">
-        <v>342</v>
-      </c>
       <c r="F12" s="18" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
+        <v>389</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>390</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>381</v>
+      </c>
+      <c r="D22" s="18" t="s">
+        <v>391</v>
+      </c>
+      <c r="E22" s="18" t="s">
         <v>383</v>
       </c>
-      <c r="B22" s="18" t="s">
-        <v>384</v>
-      </c>
-      <c r="C22" s="18" t="s">
-        <v>375</v>
-      </c>
-      <c r="D22" s="18" t="s">
-        <v>385</v>
-      </c>
-      <c r="E22" s="18" t="s">
-        <v>377</v>
-      </c>
       <c r="F22" s="18" t="s">
-        <v>386</v>
+        <v>392</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>403</v>
+        <v>409</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>405</v>
+        <v>411</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>406</v>
+        <v>412</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="F27" s="18" t="s">
-        <v>408</v>
+        <v>414</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: log D-010 In Progress — e2e stub peer http-only vs D-006 https guard
Relay credential e2e journeys can't boot (config refuses http:// peer when a
credential is set); stub peer serves http only. Test-infra regression from
D-006 (e2e phase was skipped). GH #48. Sev 2, no production impact.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSQAV9AspmwvxZ78jg9QNx
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="403">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="409">
   <si>
     <t xml:space="preserve">FEATURE VALUE SCORING FRAMEWORK</t>
   </si>
@@ -909,6 +909,24 @@
   </si>
   <si>
     <t xml:space="preserve">[logged 2026-07-23] Implementation-tracking Feature for D-006's remaining hardening legs (F-004 review F2 HMAC message-integrity + F4 SSRF host allowlist), spec'd at specs/D-006-relay-peer-hmac-and-ssrf-hardening.md (rev 3, RULED). Created as a FEATURE row because D-006 is a Fixed Defect and /implement-spec hard-stops on Defect rows (item_type=Defect). *** MUST BE IMPLEMENTED IN PARALLEL with customer-web-app F-009 (consumer-side HMAC verification) *** — the 3-step cut-over (cwa accept -&gt; relay sign -&gt; cwa require) parks every delivery if the producer and consumer sides are out of sync. Next: /prioritize-features to score it, or /implement-spec (with explicit go-ahead, spec-first) against the spec path. Unscored on the Feature scale.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D-010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relay credential e2e journeys cannot boot — http-only stub peer vs D-006 https enforcement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/dispatch-derek/admin-console/issues/48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In Progress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verified 2026-07-23: D-006 https-only guard (bff/src/relay/config.ts:82-92) refuses boot when a credential is configured and a peer is http://; the e2e stub peer (tests/e2e/relay/fixtures/stubPeer.ts) serves http://127.0.0.1 only. So the 3 credential-configured e2e journeys die at relay boot. tests/e2e/relay red 3/16. Last green commit 7c06073 (pre-D-006). No production impact (real deploys use https cwa). Surfaced during D-009 e2e; D-006's pipeline had skipped its e2e phase.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[triage 2026-07-23] severity 2 (internal test-suite health; no user/production impact; blocks e2e verification of the relay credential path). Fix (tests/e2e/ only): make the stub peer serve https (self-signed) + relay trusts it in the spawn harness. Process note: D-006's config guard gates on credential-configured, so it DID affect the credential e2e journeys - the D-006 e2e skip was the miss.</t>
   </si>
   <si>
     <t xml:space="preserve">DATA DICTIONARY - machine-readable field contract for agents</t>
@@ -4469,12 +4487,20 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="22"/>
-      <c r="B27" s="23"/>
-      <c r="C27" s="22"/>
-      <c r="D27" s="22"/>
+      <c r="A27" s="22" t="s">
+        <v>295</v>
+      </c>
+      <c r="B27" s="23" t="s">
+        <v>296</v>
+      </c>
+      <c r="C27" s="22" t="s">
+        <v>297</v>
+      </c>
+      <c r="D27" s="22" t="s">
+        <v>298</v>
+      </c>
       <c r="E27" s="22"/>
-      <c r="F27" s="22"/>
+      <c r="F27" s="32"/>
       <c r="G27" s="25"/>
       <c r="H27" s="25"/>
       <c r="I27" s="25"/>
@@ -4483,8 +4509,12 @@
       <c r="L27" s="25"/>
       <c r="M27" s="25"/>
       <c r="N27" s="25"/>
-      <c r="O27" s="27"/>
-      <c r="P27" s="27"/>
+      <c r="O27" s="27" t="s">
+        <v>299</v>
+      </c>
+      <c r="P27" s="27" t="s">
+        <v>300</v>
+      </c>
       <c r="Q27" s="28" t="str">
         <f aca="false">IF(V27="Defect","",IF(COUNT(G27:K27)&lt;5,"",ROUND(G27*Config!$B$4+H27*Config!$B$5+I27*Config!$B$6+J27*Config!$B$7+K27*Config!$B$8,2)))</f>
         <v/>
@@ -4505,7 +4535,15 @@
         <f aca="false">IF(T27="","",RANK(T27,$T$4:$T$52))</f>
         <v/>
       </c>
-      <c r="V27" s="36"/>
+      <c r="V27" s="36" t="s">
+        <v>199</v>
+      </c>
+      <c r="W27" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="X27" s="1" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="22"/>
@@ -5542,507 +5580,507 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="37" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="B3" s="37" t="s">
-        <v>297</v>
+        <v>303</v>
       </c>
       <c r="C3" s="37" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="D3" s="37" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="E3" s="37" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
       <c r="F3" s="37" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
+        <v>318</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>319</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>310</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="E6" s="18" t="s">
         <v>312</v>
       </c>
-      <c r="B6" s="18" t="s">
-        <v>313</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>304</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>314</v>
-      </c>
-      <c r="E6" s="18" t="s">
-        <v>306</v>
-      </c>
       <c r="F6" s="18" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>326</v>
+        <v>332</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
+        <v>347</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>348</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>340</v>
+      </c>
+      <c r="D12" s="18" t="s">
         <v>341</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="E12" s="18" t="s">
         <v>342</v>
       </c>
-      <c r="C12" s="18" t="s">
-        <v>334</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>335</v>
-      </c>
-      <c r="E12" s="18" t="s">
-        <v>336</v>
-      </c>
       <c r="F12" s="18" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
+        <v>383</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>375</v>
+      </c>
+      <c r="D22" s="18" t="s">
+        <v>385</v>
+      </c>
+      <c r="E22" s="18" t="s">
         <v>377</v>
       </c>
-      <c r="B22" s="18" t="s">
-        <v>378</v>
-      </c>
-      <c r="C22" s="18" t="s">
-        <v>369</v>
-      </c>
-      <c r="D22" s="18" t="s">
-        <v>379</v>
-      </c>
-      <c r="E22" s="18" t="s">
-        <v>371</v>
-      </c>
       <c r="F22" s="18" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>383</v>
+        <v>389</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>384</v>
+        <v>390</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>385</v>
+        <v>391</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>386</v>
+        <v>392</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="F27" s="18" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: D-010 -> Verified (fix-defect-or-bug write-back)
e2e stub peer now https-capable; relay credential journeys boot and pass
(16/16). Verified via e2e. Provenance appended.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSQAV9AspmwvxZ78jg9QNx
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -920,13 +920,13 @@
     <t xml:space="preserve">https://github.com/dispatch-derek/admin-console/issues/48</t>
   </si>
   <si>
-    <t xml:space="preserve">In Progress</t>
+    <t xml:space="preserve">Verified</t>
   </si>
   <si>
     <t xml:space="preserve">Verified 2026-07-23: D-006 https-only guard (bff/src/relay/config.ts:82-92) refuses boot when a credential is configured and a peer is http://; the e2e stub peer (tests/e2e/relay/fixtures/stubPeer.ts) serves http://127.0.0.1 only. So the 3 credential-configured e2e journeys die at relay boot. tests/e2e/relay red 3/16. Last green commit 7c06073 (pre-D-006). No production impact (real deploys use https cwa). Surfaced during D-009 e2e; D-006's pipeline had skipped its e2e phase.</t>
   </si>
   <si>
-    <t xml:space="preserve">[triage 2026-07-23] severity 2 (internal test-suite health; no user/production impact; blocks e2e verification of the relay credential path). Fix (tests/e2e/ only): make the stub peer serve https (self-signed) + relay trusts it in the spawn harness. Process note: D-006's config guard gates on credential-configured, so it DID affect the credential e2e journeys - the D-006 e2e skip was the miss.</t>
+    <t xml:space="preserve">[triage 2026-07-23] severity 2 (internal test-suite health; no user/production impact; blocks e2e verification of the relay credential path). Fix (tests/e2e/ only): make the stub peer serve https (self-signed) + relay trusts it in the spawn harness. Process note: D-006's config guard gates on credential-configured, so it DID affect the credential e2e journeys - the D-006 e2e skip was the miss. || [fix-defect-or-bug 2026-07-23] root cause: e2e stub peer served http:// only, refused by D-006 https guard when a credential is set. Fixed (tests/e2e/ only): stub peer -&gt; node:https with a checked-in self-signed loopback cert; relay child trusts it via NODE_EXTRA_CA_CERTS; journeys use https:// URLs. Relay e2e 16/16 green, 3x stable; code review PASS WITH NOTES (applied). Verified via e2e. No bff/src change; no production impact.</t>
   </si>
   <si>
     <t xml:space="preserve">DATA DICTIONARY - machine-readable field contract for agents</t>

</xml_diff>

<commit_message>
docs+chore: D-009 runbook/CHANGELOG fix + -> Verified
Corrects the live runbook's peer-verification header to X-Event-Ingest-Secret
(was X-Event-Auth-Token — would mislead on-call curl checks); adds the D-009
CHANGELOG entry; marks D-009 Verified (bff 1328, relay e2e 16/16, security PASS,
code review PASS WITH NOTES).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSQAV9AspmwvxZ78jg9QNx
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="414">
   <si>
     <t xml:space="preserve">FEATURE VALUE SCORING FRAMEWORK</t>
   </si>
@@ -938,13 +938,10 @@
     <t xml:space="preserve">https://github.com/dispatch-derek/admin-console/issues/47</t>
   </si>
   <si>
-    <t xml:space="preserve">In Progress</t>
-  </si>
-  <si>
     <t xml:space="preserve">Verified 2026-07-23 on main: bff/src/relay/http-peer-transport.ts:18 AUTH_TOKEN_HEADER='X-Event-Auth-Token', :91 attached to each peer POST; customer-web-app bff/src/server/ingest-auth.ts:26 reads 'x-event-ingest-secret' only and 401s otherwise (:48). Header names differ -&gt; cwa 401 -&gt; REQ-F004-055 permanent -&gt; park every admin.* delivery in bus mode. F-010 Q1 flagged this exact 'silent 401 loop' and left the header name provisional/to-be-reconciled with cwa; reconciliation never happened.</t>
   </si>
   <si>
-    <t xml:space="preserve">[triage 2026-07-23, human-directed immediate fix] severity 4 (major: admin-&gt;cwa event pipeline unusable in bus mode, no config workaround, no data loss - events park/retain). Fix: align producer header X-Event-Auth-Token -&gt; X-Event-Ingest-Secret (cwa's frozen consumer contract, REQ-F005-012). Env var stays EVENT_BUS_PEER_AUTH_TOKEN. Separate cwa defect renames cwa's env var INGEST_SHARED_SECRET -&gt; EVENT_BUS_PEER_AUTH_TOKEN for cross-app naming consistency.</t>
+    <t xml:space="preserve">[triage 2026-07-23, human-directed immediate fix] severity 4 (major: admin-&gt;cwa event pipeline unusable in bus mode, no config workaround, no data loss - events park/retain). Fix: align producer header X-Event-Auth-Token -&gt; X-Event-Ingest-Secret (cwa's frozen consumer contract, REQ-F005-012). Env var stays EVENT_BUS_PEER_AUTH_TOKEN. Separate cwa defect renames cwa's env var INGEST_SHARED_SECRET -&gt; EVENT_BUS_PEER_AUTH_TOKEN for cross-app naming consistency. || [fix-defect-or-bug 2026-07-23] root cause: AUTH_TOKEN_HEADER=X-Event-Auth-Token (http-peer-transport.ts:18) but cwa ingest requires X-Event-Ingest-Secret. Fixed: header constant -&gt; X-Event-Ingest-Secret (env var EVENT_BUS_PEER_AUTH_TOKEN unchanged); corrected 33 test literals + runbook + README + config comment. Regression: http-peer-transport.d009.test.ts. Verified: bff 1328/1328, relay e2e 16/16 (over D-010 https stub), tsc clean; security PASS, code review PASS WITH NOTES.</t>
   </si>
   <si>
     <t xml:space="preserve">DATA DICTIONARY - machine-readable field contract for agents</t>
@@ -4574,7 +4571,7 @@
         <v>303</v>
       </c>
       <c r="D28" s="22" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="E28" s="22"/>
       <c r="F28" s="32"/>
@@ -4587,10 +4584,10 @@
       <c r="M28" s="25"/>
       <c r="N28" s="25"/>
       <c r="O28" s="27" t="s">
+        <v>304</v>
+      </c>
+      <c r="P28" s="27" t="s">
         <v>305</v>
-      </c>
-      <c r="P28" s="27" t="s">
-        <v>306</v>
       </c>
       <c r="Q28" s="28" t="str">
         <f aca="false">IF(V28="Defect","",IF(COUNT(G28:K28)&lt;5,"",ROUND(G28*Config!$B$4+H28*Config!$B$5+I28*Config!$B$6+J28*Config!$B$7+K28*Config!$B$8,2)))</f>
@@ -5618,507 +5615,507 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="37" t="s">
+        <v>307</v>
+      </c>
+      <c r="B3" s="37" t="s">
         <v>308</v>
       </c>
-      <c r="B3" s="37" t="s">
+      <c r="C3" s="37" t="s">
         <v>309</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="D3" s="37" t="s">
         <v>310</v>
       </c>
-      <c r="D3" s="37" t="s">
+      <c r="E3" s="37" t="s">
         <v>311</v>
       </c>
-      <c r="E3" s="37" t="s">
+      <c r="F3" s="37" t="s">
         <v>312</v>
-      </c>
-      <c r="F3" s="37" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
+        <v>313</v>
+      </c>
+      <c r="B4" s="18" t="s">
         <v>314</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="C4" s="18" t="s">
         <v>315</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="D4" s="18" t="s">
         <v>316</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="E4" s="18" t="s">
         <v>317</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="F4" s="18" t="s">
         <v>318</v>
-      </c>
-      <c r="F4" s="18" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
+        <v>319</v>
+      </c>
+      <c r="B5" s="18" t="s">
         <v>320</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="C5" s="18" t="s">
+        <v>315</v>
+      </c>
+      <c r="D5" s="18" t="s">
         <v>321</v>
       </c>
-      <c r="C5" s="18" t="s">
-        <v>316</v>
-      </c>
-      <c r="D5" s="18" t="s">
+      <c r="E5" s="18" t="s">
+        <v>317</v>
+      </c>
+      <c r="F5" s="18" t="s">
         <v>322</v>
-      </c>
-      <c r="E5" s="18" t="s">
-        <v>318</v>
-      </c>
-      <c r="F5" s="18" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="B6" s="18" t="s">
         <v>324</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="C6" s="18" t="s">
+        <v>315</v>
+      </c>
+      <c r="D6" s="18" t="s">
         <v>325</v>
       </c>
-      <c r="C6" s="18" t="s">
-        <v>316</v>
-      </c>
-      <c r="D6" s="18" t="s">
+      <c r="E6" s="18" t="s">
+        <v>317</v>
+      </c>
+      <c r="F6" s="18" t="s">
         <v>326</v>
-      </c>
-      <c r="E6" s="18" t="s">
-        <v>318</v>
-      </c>
-      <c r="F6" s="18" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
+        <v>327</v>
+      </c>
+      <c r="B7" s="18" t="s">
         <v>328</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="C7" s="18" t="s">
         <v>329</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="D7" s="18" t="s">
         <v>330</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="E7" s="18" t="s">
         <v>331</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="F7" s="18" t="s">
         <v>332</v>
-      </c>
-      <c r="F7" s="18" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
+        <v>333</v>
+      </c>
+      <c r="B8" s="18" t="s">
         <v>334</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="C8" s="18" t="s">
+        <v>329</v>
+      </c>
+      <c r="D8" s="18" t="s">
         <v>335</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>330</v>
-      </c>
-      <c r="D8" s="18" t="s">
+      <c r="E8" s="18" t="s">
         <v>336</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="F8" s="18" t="s">
         <v>337</v>
-      </c>
-      <c r="F8" s="18" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
+        <v>338</v>
+      </c>
+      <c r="B9" s="18" t="s">
         <v>339</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="C9" s="18" t="s">
         <v>340</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="D9" s="18" t="s">
         <v>341</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="E9" s="18" t="s">
+        <v>336</v>
+      </c>
+      <c r="F9" s="18" t="s">
         <v>342</v>
-      </c>
-      <c r="E9" s="18" t="s">
-        <v>337</v>
-      </c>
-      <c r="F9" s="18" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
+        <v>343</v>
+      </c>
+      <c r="B10" s="18" t="s">
         <v>344</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="C10" s="18" t="s">
         <v>345</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="D10" s="18" t="s">
         <v>346</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="E10" s="18" t="s">
         <v>347</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="F10" s="18" t="s">
         <v>348</v>
-      </c>
-      <c r="F10" s="18" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
+        <v>349</v>
+      </c>
+      <c r="B11" s="18" t="s">
         <v>350</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="C11" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>347</v>
+      </c>
+      <c r="F11" s="18" t="s">
         <v>351</v>
-      </c>
-      <c r="C11" s="18" t="s">
-        <v>346</v>
-      </c>
-      <c r="D11" s="18" t="s">
-        <v>347</v>
-      </c>
-      <c r="E11" s="18" t="s">
-        <v>348</v>
-      </c>
-      <c r="F11" s="18" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
+        <v>352</v>
+      </c>
+      <c r="B12" s="18" t="s">
         <v>353</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="C12" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="E12" s="18" t="s">
+        <v>347</v>
+      </c>
+      <c r="F12" s="18" t="s">
         <v>354</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>346</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>347</v>
-      </c>
-      <c r="E12" s="18" t="s">
-        <v>348</v>
-      </c>
-      <c r="F12" s="18" t="s">
-        <v>355</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="B13" s="18" t="s">
         <v>356</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="C13" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>317</v>
+      </c>
+      <c r="F13" s="18" t="s">
         <v>357</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>346</v>
-      </c>
-      <c r="D13" s="18" t="s">
-        <v>347</v>
-      </c>
-      <c r="E13" s="18" t="s">
-        <v>318</v>
-      </c>
-      <c r="F13" s="18" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
+        <v>358</v>
+      </c>
+      <c r="B14" s="18" t="s">
         <v>359</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="C14" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>347</v>
+      </c>
+      <c r="F14" s="18" t="s">
         <v>360</v>
-      </c>
-      <c r="C14" s="18" t="s">
-        <v>346</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>347</v>
-      </c>
-      <c r="E14" s="18" t="s">
-        <v>348</v>
-      </c>
-      <c r="F14" s="18" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
+        <v>361</v>
+      </c>
+      <c r="B15" s="18" t="s">
         <v>362</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="C15" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="E15" s="18" t="s">
+        <v>336</v>
+      </c>
+      <c r="F15" s="18" t="s">
         <v>363</v>
-      </c>
-      <c r="C15" s="18" t="s">
-        <v>346</v>
-      </c>
-      <c r="D15" s="18" t="s">
-        <v>347</v>
-      </c>
-      <c r="E15" s="18" t="s">
-        <v>337</v>
-      </c>
-      <c r="F15" s="18" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
+        <v>364</v>
+      </c>
+      <c r="B16" s="18" t="s">
         <v>365</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="C16" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="E16" s="18" t="s">
         <v>366</v>
       </c>
-      <c r="C16" s="18" t="s">
-        <v>346</v>
-      </c>
-      <c r="D16" s="18" t="s">
-        <v>347</v>
-      </c>
-      <c r="E16" s="18" t="s">
+      <c r="F16" s="18" t="s">
         <v>367</v>
-      </c>
-      <c r="F16" s="18" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
+        <v>368</v>
+      </c>
+      <c r="B17" s="18" t="s">
         <v>369</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="C17" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>317</v>
+      </c>
+      <c r="F17" s="18" t="s">
         <v>370</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>346</v>
-      </c>
-      <c r="D17" s="18" t="s">
-        <v>347</v>
-      </c>
-      <c r="E17" s="18" t="s">
-        <v>318</v>
-      </c>
-      <c r="F17" s="18" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
+        <v>371</v>
+      </c>
+      <c r="B18" s="18" t="s">
         <v>372</v>
       </c>
-      <c r="B18" s="18" t="s">
+      <c r="C18" s="18" t="s">
+        <v>315</v>
+      </c>
+      <c r="D18" s="18" t="s">
         <v>373</v>
       </c>
-      <c r="C18" s="18" t="s">
-        <v>316</v>
-      </c>
-      <c r="D18" s="18" t="s">
+      <c r="E18" s="18" t="s">
+        <v>336</v>
+      </c>
+      <c r="F18" s="18" t="s">
         <v>374</v>
-      </c>
-      <c r="E18" s="18" t="s">
-        <v>337</v>
-      </c>
-      <c r="F18" s="18" t="s">
-        <v>375</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
+        <v>375</v>
+      </c>
+      <c r="B19" s="18" t="s">
         <v>376</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="C19" s="18" t="s">
+        <v>315</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>336</v>
+      </c>
+      <c r="F19" s="18" t="s">
         <v>377</v>
-      </c>
-      <c r="C19" s="18" t="s">
-        <v>316</v>
-      </c>
-      <c r="D19" s="18" t="s">
-        <v>322</v>
-      </c>
-      <c r="E19" s="18" t="s">
-        <v>337</v>
-      </c>
-      <c r="F19" s="18" t="s">
-        <v>378</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
+        <v>378</v>
+      </c>
+      <c r="B20" s="18" t="s">
         <v>379</v>
       </c>
-      <c r="B20" s="18" t="s">
+      <c r="C20" s="18" t="s">
         <v>380</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="D20" s="18" t="s">
         <v>381</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="E20" s="18" t="s">
         <v>382</v>
       </c>
-      <c r="E20" s="18" t="s">
+      <c r="F20" s="18" t="s">
         <v>383</v>
-      </c>
-      <c r="F20" s="18" t="s">
-        <v>384</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="B21" s="18" t="s">
         <v>385</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="C21" s="18" t="s">
+        <v>380</v>
+      </c>
+      <c r="D21" s="18" t="s">
         <v>386</v>
       </c>
-      <c r="C21" s="18" t="s">
-        <v>381</v>
-      </c>
-      <c r="D21" s="18" t="s">
+      <c r="E21" s="18" t="s">
+        <v>382</v>
+      </c>
+      <c r="F21" s="18" t="s">
         <v>387</v>
-      </c>
-      <c r="E21" s="18" t="s">
-        <v>383</v>
-      </c>
-      <c r="F21" s="18" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="B22" s="18" t="s">
         <v>389</v>
       </c>
-      <c r="B22" s="18" t="s">
+      <c r="C22" s="18" t="s">
+        <v>380</v>
+      </c>
+      <c r="D22" s="18" t="s">
         <v>390</v>
       </c>
-      <c r="C22" s="18" t="s">
-        <v>381</v>
-      </c>
-      <c r="D22" s="18" t="s">
+      <c r="E22" s="18" t="s">
+        <v>382</v>
+      </c>
+      <c r="F22" s="18" t="s">
         <v>391</v>
-      </c>
-      <c r="E22" s="18" t="s">
-        <v>383</v>
-      </c>
-      <c r="F22" s="18" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
+        <v>392</v>
+      </c>
+      <c r="B23" s="18" t="s">
         <v>393</v>
       </c>
-      <c r="B23" s="18" t="s">
+      <c r="C23" s="18" t="s">
+        <v>380</v>
+      </c>
+      <c r="D23" s="18" t="s">
         <v>394</v>
       </c>
-      <c r="C23" s="18" t="s">
-        <v>381</v>
-      </c>
-      <c r="D23" s="18" t="s">
+      <c r="E23" s="18" t="s">
+        <v>382</v>
+      </c>
+      <c r="F23" s="18" t="s">
         <v>395</v>
-      </c>
-      <c r="E23" s="18" t="s">
-        <v>383</v>
-      </c>
-      <c r="F23" s="18" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
+        <v>396</v>
+      </c>
+      <c r="B24" s="18" t="s">
         <v>397</v>
       </c>
-      <c r="B24" s="18" t="s">
+      <c r="C24" s="18" t="s">
+        <v>380</v>
+      </c>
+      <c r="D24" s="18" t="s">
         <v>398</v>
       </c>
-      <c r="C24" s="18" t="s">
-        <v>381</v>
-      </c>
-      <c r="D24" s="18" t="s">
+      <c r="E24" s="18" t="s">
+        <v>382</v>
+      </c>
+      <c r="F24" s="18" t="s">
         <v>399</v>
-      </c>
-      <c r="E24" s="18" t="s">
-        <v>383</v>
-      </c>
-      <c r="F24" s="18" t="s">
-        <v>400</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
+        <v>400</v>
+      </c>
+      <c r="B25" s="18" t="s">
         <v>401</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="C25" s="18" t="s">
+        <v>329</v>
+      </c>
+      <c r="D25" s="18" t="s">
         <v>402</v>
       </c>
-      <c r="C25" s="18" t="s">
-        <v>330</v>
-      </c>
-      <c r="D25" s="18" t="s">
+      <c r="E25" s="18" t="s">
+        <v>317</v>
+      </c>
+      <c r="F25" s="18" t="s">
         <v>403</v>
-      </c>
-      <c r="E25" s="18" t="s">
-        <v>318</v>
-      </c>
-      <c r="F25" s="18" t="s">
-        <v>404</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
+        <v>404</v>
+      </c>
+      <c r="B26" s="18" t="s">
         <v>405</v>
       </c>
-      <c r="B26" s="18" t="s">
+      <c r="C26" s="18" t="s">
+        <v>329</v>
+      </c>
+      <c r="D26" s="18" t="s">
         <v>406</v>
       </c>
-      <c r="C26" s="18" t="s">
-        <v>330</v>
-      </c>
-      <c r="D26" s="18" t="s">
+      <c r="E26" s="18" t="s">
         <v>407</v>
       </c>
-      <c r="E26" s="18" t="s">
+      <c r="F26" s="18" t="s">
         <v>408</v>
-      </c>
-      <c r="F26" s="18" t="s">
-        <v>409</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
+        <v>409</v>
+      </c>
+      <c r="B27" s="18" t="s">
         <v>410</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="C27" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="D27" s="18" t="s">
         <v>411</v>
       </c>
-      <c r="C27" s="18" t="s">
-        <v>346</v>
-      </c>
-      <c r="D27" s="18" t="s">
+      <c r="E27" s="18" t="s">
         <v>412</v>
       </c>
-      <c r="E27" s="18" t="s">
+      <c r="F27" s="18" t="s">
         <v>413</v>
-      </c>
-      <c r="F27" s="18" t="s">
-        <v>414</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: log D-011 In Progress — rename relay wire header to X-Event-Bus-Peer-Auth-Token
Supersedes stranded D-009. admin-console main still sends X-Event-Auth-Token
(D-009 never reached main). Final header for both apps: X-Event-Bus-Peer-Auth-Token.
GH #51. Sev 4. Must land with cwa D-003.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSQAV9AspmwvxZ78jg9QNx
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="409">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="415">
   <si>
     <t xml:space="preserve">FEATURE VALUE SCORING FRAMEWORK</t>
   </si>
@@ -927,6 +927,24 @@
   </si>
   <si>
     <t xml:space="preserve">[triage 2026-07-23] severity 2 (internal test-suite health; no user/production impact; blocks e2e verification of the relay credential path). Fix (tests/e2e/ only): make the stub peer serve https (self-signed) + relay trusts it in the spawn harness. Process note: D-006's config guard gates on credential-configured, so it DID affect the credential e2e journeys - the D-006 e2e skip was the miss. || [fix-defect-or-bug 2026-07-23] root cause: e2e stub peer served http:// only, refused by D-006 https guard when a credential is set. Fixed (tests/e2e/ only): stub peer -&gt; node:https with a checked-in self-signed loopback cert; relay child trusts it via NODE_EXTRA_CA_CERTS; journeys use https:// URLs. Relay e2e 16/16 green, 3x stable; code review PASS WITH NOTES (applied). Verified via e2e. No bff/src change; no production impact.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D-011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rename relay wire header to X-Event-Bus-Peer-Auth-Token (supersedes stranded D-009)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/dispatch-derek/admin-console/issues/51</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In Progress</t>
+  </si>
+  <si>
+    <t xml:space="preserve">admin-console main sends header X-Event-Auth-Token (http-peer-transport.ts:18); D-009's fix (-&gt;X-Event-Ingest-Secret) merged into a stacked base, never reached main (PR #50). Product-owner chose final header X-Event-Bus-Peer-Auth-Token for both apps. Pairs with cwa D-003. Pipeline broken on main until both land.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[triage 2026-07-23] sev 4 (admin-&gt;cwa pipeline broken on main). Fix: AUTH_TOKEN_HEADER -&gt; 'X-Event-Bus-Peer-Auth-Token' (env var EVENT_BUS_PEER_AUTH_TOKEN unchanged); update comments/README/runbook/tests. Based on main, no stacking. Supersedes D-009 (#47). MUST land with cwa D-003.</t>
   </si>
   <si>
     <t xml:space="preserve">DATA DICTIONARY - machine-readable field contract for agents</t>
@@ -4546,12 +4564,20 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="22"/>
-      <c r="B28" s="23"/>
-      <c r="C28" s="22"/>
-      <c r="D28" s="22"/>
+      <c r="A28" s="22" t="s">
+        <v>301</v>
+      </c>
+      <c r="B28" s="23" t="s">
+        <v>302</v>
+      </c>
+      <c r="C28" s="22" t="s">
+        <v>303</v>
+      </c>
+      <c r="D28" s="22" t="s">
+        <v>304</v>
+      </c>
       <c r="E28" s="22"/>
-      <c r="F28" s="22"/>
+      <c r="F28" s="32"/>
       <c r="G28" s="25"/>
       <c r="H28" s="25"/>
       <c r="I28" s="25"/>
@@ -4560,8 +4586,12 @@
       <c r="L28" s="25"/>
       <c r="M28" s="25"/>
       <c r="N28" s="25"/>
-      <c r="O28" s="27"/>
-      <c r="P28" s="27"/>
+      <c r="O28" s="27" t="s">
+        <v>305</v>
+      </c>
+      <c r="P28" s="27" t="s">
+        <v>306</v>
+      </c>
       <c r="Q28" s="28" t="str">
         <f aca="false">IF(V28="Defect","",IF(COUNT(G28:K28)&lt;5,"",ROUND(G28*Config!$B$4+H28*Config!$B$5+I28*Config!$B$6+J28*Config!$B$7+K28*Config!$B$8,2)))</f>
         <v/>
@@ -4582,7 +4612,15 @@
         <f aca="false">IF(T28="","",RANK(T28,$T$4:$T$52))</f>
         <v/>
       </c>
-      <c r="V28" s="36"/>
+      <c r="V28" s="36" t="s">
+        <v>199</v>
+      </c>
+      <c r="W28" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="X28" s="1" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="22"/>
@@ -5580,507 +5618,507 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="37" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="B3" s="37" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="C3" s="37" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
       <c r="D3" s="37" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="E3" s="37" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="F3" s="37" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="C5" s="18" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="D5" s="18" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="E5" s="18" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
+        <v>324</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="C6" s="18" t="s">
+        <v>316</v>
+      </c>
+      <c r="D6" s="18" t="s">
+        <v>326</v>
+      </c>
+      <c r="E6" s="18" t="s">
         <v>318</v>
       </c>
-      <c r="B6" s="18" t="s">
-        <v>319</v>
-      </c>
-      <c r="C6" s="18" t="s">
-        <v>310</v>
-      </c>
-      <c r="D6" s="18" t="s">
-        <v>320</v>
-      </c>
-      <c r="E6" s="18" t="s">
-        <v>312</v>
-      </c>
       <c r="F6" s="18" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>326</v>
+        <v>332</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>327</v>
+        <v>333</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="D8" s="18" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="C9" s="18" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D11" s="18" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
+        <v>353</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>354</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="D12" s="18" t="s">
         <v>347</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="E12" s="18" t="s">
         <v>348</v>
       </c>
-      <c r="C12" s="18" t="s">
-        <v>340</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>341</v>
-      </c>
-      <c r="E12" s="18" t="s">
-        <v>342</v>
-      </c>
       <c r="F12" s="18" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D13" s="18" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="F13" s="18" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="B15" s="18" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D15" s="18" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="F15" s="18" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D16" s="18" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
       <c r="B17" s="18" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="C17" s="18" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="F17" s="18" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="B18" s="18" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="C18" s="18" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="F18" s="18" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="B19" s="18" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="F19" s="18" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="B20" s="18" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="D20" s="18" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>378</v>
+        <v>384</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>379</v>
+        <v>385</v>
       </c>
       <c r="B21" s="18" t="s">
-        <v>380</v>
+        <v>386</v>
       </c>
       <c r="C21" s="18" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="D21" s="18" t="s">
-        <v>381</v>
+        <v>387</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="F21" s="18" t="s">
-        <v>382</v>
+        <v>388</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
+        <v>389</v>
+      </c>
+      <c r="B22" s="18" t="s">
+        <v>390</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>381</v>
+      </c>
+      <c r="D22" s="18" t="s">
+        <v>391</v>
+      </c>
+      <c r="E22" s="18" t="s">
         <v>383</v>
       </c>
-      <c r="B22" s="18" t="s">
-        <v>384</v>
-      </c>
-      <c r="C22" s="18" t="s">
-        <v>375</v>
-      </c>
-      <c r="D22" s="18" t="s">
-        <v>385</v>
-      </c>
-      <c r="E22" s="18" t="s">
-        <v>377</v>
-      </c>
       <c r="F22" s="18" t="s">
-        <v>386</v>
+        <v>392</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
-        <v>387</v>
+        <v>393</v>
       </c>
       <c r="B23" s="18" t="s">
-        <v>388</v>
+        <v>394</v>
       </c>
       <c r="C23" s="18" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="D23" s="18" t="s">
-        <v>389</v>
+        <v>395</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="F23" s="18" t="s">
-        <v>390</v>
+        <v>396</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>391</v>
+        <v>397</v>
       </c>
       <c r="B24" s="18" t="s">
-        <v>392</v>
+        <v>398</v>
       </c>
       <c r="C24" s="18" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="D24" s="18" t="s">
-        <v>393</v>
+        <v>399</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>377</v>
+        <v>383</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>394</v>
+        <v>400</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
-        <v>395</v>
+        <v>401</v>
       </c>
       <c r="B25" s="18" t="s">
-        <v>396</v>
+        <v>402</v>
       </c>
       <c r="C25" s="18" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="E25" s="18" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="F25" s="18" t="s">
-        <v>398</v>
+        <v>404</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
-        <v>399</v>
+        <v>405</v>
       </c>
       <c r="B26" s="18" t="s">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="C26" s="18" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="D26" s="18" t="s">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="E26" s="18" t="s">
-        <v>402</v>
+        <v>408</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>403</v>
+        <v>409</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
-        <v>404</v>
+        <v>410</v>
       </c>
       <c r="B27" s="18" t="s">
-        <v>405</v>
+        <v>411</v>
       </c>
       <c r="C27" s="18" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="D27" s="18" t="s">
-        <v>406</v>
+        <v>412</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>407</v>
+        <v>413</v>
       </c>
       <c r="F27" s="18" t="s">
-        <v>408</v>
+        <v>414</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs+chore: D-011 runbook/CHANGELOG/security report + -> Verified
Runbook + CHANGELOG updated to X-Event-Bus-Peer-Auth-Token; adds
security/D-011-security-review.md (PASS); marks D-011 Verified (bff 1327,
relay e2e 16/16, security PASS, code review APPROVE). Supersedes D-009.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PSQAV9AspmwvxZ78jg9QNx
</commit_message>
<xml_diff>
--- a/feature-value-scoring.xlsx
+++ b/feature-value-scoring.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="415">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="414">
   <si>
     <t xml:space="preserve">FEATURE VALUE SCORING FRAMEWORK</t>
   </si>
@@ -938,13 +938,10 @@
     <t xml:space="preserve">https://github.com/dispatch-derek/admin-console/issues/51</t>
   </si>
   <si>
-    <t xml:space="preserve">In Progress</t>
-  </si>
-  <si>
     <t xml:space="preserve">admin-console main sends header X-Event-Auth-Token (http-peer-transport.ts:18); D-009's fix (-&gt;X-Event-Ingest-Secret) merged into a stacked base, never reached main (PR #50). Product-owner chose final header X-Event-Bus-Peer-Auth-Token for both apps. Pairs with cwa D-003. Pipeline broken on main until both land.</t>
   </si>
   <si>
-    <t xml:space="preserve">[triage 2026-07-23] sev 4 (admin-&gt;cwa pipeline broken on main). Fix: AUTH_TOKEN_HEADER -&gt; 'X-Event-Bus-Peer-Auth-Token' (env var EVENT_BUS_PEER_AUTH_TOKEN unchanged); update comments/README/runbook/tests. Based on main, no stacking. Supersedes D-009 (#47). MUST land with cwa D-003.</t>
+    <t xml:space="preserve">[triage 2026-07-23] sev 4 (admin-&gt;cwa pipeline broken on main). Fix: AUTH_TOKEN_HEADER -&gt; 'X-Event-Bus-Peer-Auth-Token' (env var EVENT_BUS_PEER_AUTH_TOKEN unchanged); update comments/README/runbook/tests. Based on main, no stacking. Supersedes D-009 (#47). MUST land with cwa D-003. || [fix-defect-or-bug 2026-07-23] fixed: AUTH_TOKEN_HEADER -&gt; X-Event-Bus-Peer-Auth-Token (http-peer-transport.ts:18); env var EVENT_BUS_PEER_AUTH_TOKEN unchanged. Corrected 32 bff test literals + e2e + runbook + README + config comment. Regression: http-peer-transport.d011.test.ts. Verified: bff 1327/1327, relay e2e 16/16 (3x), tsc clean; security PASS, code review APPROVE. Supersedes stranded D-009. MUST land with cwa D-003 (both sides mismatched until then). Deploy note: rebuild bff/dist (old literal in git-ignored build artifact).</t>
   </si>
   <si>
     <t xml:space="preserve">DATA DICTIONARY - machine-readable field contract for agents</t>
@@ -4574,7 +4571,7 @@
         <v>303</v>
       </c>
       <c r="D28" s="22" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="E28" s="22"/>
       <c r="F28" s="32"/>
@@ -4587,10 +4584,10 @@
       <c r="M28" s="25"/>
       <c r="N28" s="25"/>
       <c r="O28" s="27" t="s">
+        <v>304</v>
+      </c>
+      <c r="P28" s="27" t="s">
         <v>305</v>
-      </c>
-      <c r="P28" s="27" t="s">
-        <v>306</v>
       </c>
       <c r="Q28" s="28" t="str">
         <f aca="false">IF(V28="Defect","",IF(COUNT(G28:K28)&lt;5,"",ROUND(G28*Config!$B$4+H28*Config!$B$5+I28*Config!$B$6+J28*Config!$B$7+K28*Config!$B$8,2)))</f>
@@ -5618,507 +5615,507 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="37" t="s">
+        <v>307</v>
+      </c>
+      <c r="B3" s="37" t="s">
         <v>308</v>
       </c>
-      <c r="B3" s="37" t="s">
+      <c r="C3" s="37" t="s">
         <v>309</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="D3" s="37" t="s">
         <v>310</v>
       </c>
-      <c r="D3" s="37" t="s">
+      <c r="E3" s="37" t="s">
         <v>311</v>
       </c>
-      <c r="E3" s="37" t="s">
+      <c r="F3" s="37" t="s">
         <v>312</v>
-      </c>
-      <c r="F3" s="37" t="s">
-        <v>313</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="18" t="s">
+        <v>313</v>
+      </c>
+      <c r="B4" s="18" t="s">
         <v>314</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="C4" s="18" t="s">
         <v>315</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="D4" s="18" t="s">
         <v>316</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="E4" s="18" t="s">
         <v>317</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="F4" s="18" t="s">
         <v>318</v>
-      </c>
-      <c r="F4" s="18" t="s">
-        <v>319</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
+        <v>319</v>
+      </c>
+      <c r="B5" s="18" t="s">
         <v>320</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="C5" s="18" t="s">
+        <v>315</v>
+      </c>
+      <c r="D5" s="18" t="s">
         <v>321</v>
       </c>
-      <c r="C5" s="18" t="s">
-        <v>316</v>
-      </c>
-      <c r="D5" s="18" t="s">
+      <c r="E5" s="18" t="s">
+        <v>317</v>
+      </c>
+      <c r="F5" s="18" t="s">
         <v>322</v>
-      </c>
-      <c r="E5" s="18" t="s">
-        <v>318</v>
-      </c>
-      <c r="F5" s="18" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="18" t="s">
+        <v>323</v>
+      </c>
+      <c r="B6" s="18" t="s">
         <v>324</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="C6" s="18" t="s">
+        <v>315</v>
+      </c>
+      <c r="D6" s="18" t="s">
         <v>325</v>
       </c>
-      <c r="C6" s="18" t="s">
-        <v>316</v>
-      </c>
-      <c r="D6" s="18" t="s">
+      <c r="E6" s="18" t="s">
+        <v>317</v>
+      </c>
+      <c r="F6" s="18" t="s">
         <v>326</v>
-      </c>
-      <c r="E6" s="18" t="s">
-        <v>318</v>
-      </c>
-      <c r="F6" s="18" t="s">
-        <v>327</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
+        <v>327</v>
+      </c>
+      <c r="B7" s="18" t="s">
         <v>328</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="C7" s="18" t="s">
         <v>329</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="D7" s="18" t="s">
         <v>330</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="E7" s="18" t="s">
         <v>331</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="F7" s="18" t="s">
         <v>332</v>
-      </c>
-      <c r="F7" s="18" t="s">
-        <v>333</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
+        <v>333</v>
+      </c>
+      <c r="B8" s="18" t="s">
         <v>334</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="C8" s="18" t="s">
+        <v>329</v>
+      </c>
+      <c r="D8" s="18" t="s">
         <v>335</v>
       </c>
-      <c r="C8" s="18" t="s">
-        <v>330</v>
-      </c>
-      <c r="D8" s="18" t="s">
+      <c r="E8" s="18" t="s">
         <v>336</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="F8" s="18" t="s">
         <v>337</v>
-      </c>
-      <c r="F8" s="18" t="s">
-        <v>338</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
+        <v>338</v>
+      </c>
+      <c r="B9" s="18" t="s">
         <v>339</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="C9" s="18" t="s">
         <v>340</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="D9" s="18" t="s">
         <v>341</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="E9" s="18" t="s">
+        <v>336</v>
+      </c>
+      <c r="F9" s="18" t="s">
         <v>342</v>
-      </c>
-      <c r="E9" s="18" t="s">
-        <v>337</v>
-      </c>
-      <c r="F9" s="18" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
+        <v>343</v>
+      </c>
+      <c r="B10" s="18" t="s">
         <v>344</v>
       </c>
-      <c r="B10" s="18" t="s">
+      <c r="C10" s="18" t="s">
         <v>345</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="D10" s="18" t="s">
         <v>346</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="E10" s="18" t="s">
         <v>347</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="F10" s="18" t="s">
         <v>348</v>
-      </c>
-      <c r="F10" s="18" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
+        <v>349</v>
+      </c>
+      <c r="B11" s="18" t="s">
         <v>350</v>
       </c>
-      <c r="B11" s="18" t="s">
+      <c r="C11" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="D11" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>347</v>
+      </c>
+      <c r="F11" s="18" t="s">
         <v>351</v>
-      </c>
-      <c r="C11" s="18" t="s">
-        <v>346</v>
-      </c>
-      <c r="D11" s="18" t="s">
-        <v>347</v>
-      </c>
-      <c r="E11" s="18" t="s">
-        <v>348</v>
-      </c>
-      <c r="F11" s="18" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="s">
+        <v>352</v>
+      </c>
+      <c r="B12" s="18" t="s">
         <v>353</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="C12" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="D12" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="E12" s="18" t="s">
+        <v>347</v>
+      </c>
+      <c r="F12" s="18" t="s">
         <v>354</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>346</v>
-      </c>
-      <c r="D12" s="18" t="s">
-        <v>347</v>
-      </c>
-      <c r="E12" s="18" t="s">
-        <v>348</v>
-      </c>
-      <c r="F12" s="18" t="s">
-        <v>355</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
+        <v>355</v>
+      </c>
+      <c r="B13" s="18" t="s">
         <v>356</v>
       </c>
-      <c r="B13" s="18" t="s">
+      <c r="C13" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="D13" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="E13" s="18" t="s">
+        <v>317</v>
+      </c>
+      <c r="F13" s="18" t="s">
         <v>357</v>
-      </c>
-      <c r="C13" s="18" t="s">
-        <v>346</v>
-      </c>
-      <c r="D13" s="18" t="s">
-        <v>347</v>
-      </c>
-      <c r="E13" s="18" t="s">
-        <v>318</v>
-      </c>
-      <c r="F13" s="18" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="18" t="s">
+        <v>358</v>
+      </c>
+      <c r="B14" s="18" t="s">
         <v>359</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="C14" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="D14" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>347</v>
+      </c>
+      <c r="F14" s="18" t="s">
         <v>360</v>
-      </c>
-      <c r="C14" s="18" t="s">
-        <v>346</v>
-      </c>
-      <c r="D14" s="18" t="s">
-        <v>347</v>
-      </c>
-      <c r="E14" s="18" t="s">
-        <v>348</v>
-      </c>
-      <c r="F14" s="18" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="18" t="s">
+        <v>361</v>
+      </c>
+      <c r="B15" s="18" t="s">
         <v>362</v>
       </c>
-      <c r="B15" s="18" t="s">
+      <c r="C15" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="D15" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="E15" s="18" t="s">
+        <v>336</v>
+      </c>
+      <c r="F15" s="18" t="s">
         <v>363</v>
-      </c>
-      <c r="C15" s="18" t="s">
-        <v>346</v>
-      </c>
-      <c r="D15" s="18" t="s">
-        <v>347</v>
-      </c>
-      <c r="E15" s="18" t="s">
-        <v>337</v>
-      </c>
-      <c r="F15" s="18" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="18" t="s">
+        <v>364</v>
+      </c>
+      <c r="B16" s="18" t="s">
         <v>365</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="C16" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="D16" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="E16" s="18" t="s">
         <v>366</v>
       </c>
-      <c r="C16" s="18" t="s">
-        <v>346</v>
-      </c>
-      <c r="D16" s="18" t="s">
-        <v>347</v>
-      </c>
-      <c r="E16" s="18" t="s">
+      <c r="F16" s="18" t="s">
         <v>367</v>
-      </c>
-      <c r="F16" s="18" t="s">
-        <v>368</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="18" t="s">
+        <v>368</v>
+      </c>
+      <c r="B17" s="18" t="s">
         <v>369</v>
       </c>
-      <c r="B17" s="18" t="s">
+      <c r="C17" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="D17" s="18" t="s">
+        <v>346</v>
+      </c>
+      <c r="E17" s="18" t="s">
+        <v>317</v>
+      </c>
+      <c r="F17" s="18" t="s">
         <v>370</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>346</v>
-      </c>
-      <c r="D17" s="18" t="s">
-        <v>347</v>
-      </c>
-      <c r="E17" s="18" t="s">
-        <v>318</v>
-      </c>
-      <c r="F17" s="18" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="s">
+        <v>371</v>
+      </c>
+      <c r="B18" s="18" t="s">
         <v>372</v>
       </c>
-      <c r="B18" s="18" t="s">
+      <c r="C18" s="18" t="s">
+        <v>315</v>
+      </c>
+      <c r="D18" s="18" t="s">
         <v>373</v>
       </c>
-      <c r="C18" s="18" t="s">
-        <v>316</v>
-      </c>
-      <c r="D18" s="18" t="s">
+      <c r="E18" s="18" t="s">
+        <v>336</v>
+      </c>
+      <c r="F18" s="18" t="s">
         <v>374</v>
-      </c>
-      <c r="E18" s="18" t="s">
-        <v>337</v>
-      </c>
-      <c r="F18" s="18" t="s">
-        <v>375</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="18" t="s">
+        <v>375</v>
+      </c>
+      <c r="B19" s="18" t="s">
         <v>376</v>
       </c>
-      <c r="B19" s="18" t="s">
+      <c r="C19" s="18" t="s">
+        <v>315</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>321</v>
+      </c>
+      <c r="E19" s="18" t="s">
+        <v>336</v>
+      </c>
+      <c r="F19" s="18" t="s">
         <v>377</v>
-      </c>
-      <c r="C19" s="18" t="s">
-        <v>316</v>
-      </c>
-      <c r="D19" s="18" t="s">
-        <v>322</v>
-      </c>
-      <c r="E19" s="18" t="s">
-        <v>337</v>
-      </c>
-      <c r="F19" s="18" t="s">
-        <v>378</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="18" t="s">
+        <v>378</v>
+      </c>
+      <c r="B20" s="18" t="s">
         <v>379</v>
       </c>
-      <c r="B20" s="18" t="s">
+      <c r="C20" s="18" t="s">
         <v>380</v>
       </c>
-      <c r="C20" s="18" t="s">
+      <c r="D20" s="18" t="s">
         <v>381</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="E20" s="18" t="s">
         <v>382</v>
       </c>
-      <c r="E20" s="18" t="s">
+      <c r="F20" s="18" t="s">
         <v>383</v>
-      </c>
-      <c r="F20" s="18" t="s">
-        <v>384</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
+        <v>384</v>
+      </c>
+      <c r="B21" s="18" t="s">
         <v>385</v>
       </c>
-      <c r="B21" s="18" t="s">
+      <c r="C21" s="18" t="s">
+        <v>380</v>
+      </c>
+      <c r="D21" s="18" t="s">
         <v>386</v>
       </c>
-      <c r="C21" s="18" t="s">
-        <v>381</v>
-      </c>
-      <c r="D21" s="18" t="s">
+      <c r="E21" s="18" t="s">
+        <v>382</v>
+      </c>
+      <c r="F21" s="18" t="s">
         <v>387</v>
-      </c>
-      <c r="E21" s="18" t="s">
-        <v>383</v>
-      </c>
-      <c r="F21" s="18" t="s">
-        <v>388</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
+        <v>388</v>
+      </c>
+      <c r="B22" s="18" t="s">
         <v>389</v>
       </c>
-      <c r="B22" s="18" t="s">
+      <c r="C22" s="18" t="s">
+        <v>380</v>
+      </c>
+      <c r="D22" s="18" t="s">
         <v>390</v>
       </c>
-      <c r="C22" s="18" t="s">
-        <v>381</v>
-      </c>
-      <c r="D22" s="18" t="s">
+      <c r="E22" s="18" t="s">
+        <v>382</v>
+      </c>
+      <c r="F22" s="18" t="s">
         <v>391</v>
-      </c>
-      <c r="E22" s="18" t="s">
-        <v>383</v>
-      </c>
-      <c r="F22" s="18" t="s">
-        <v>392</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="18" t="s">
+        <v>392</v>
+      </c>
+      <c r="B23" s="18" t="s">
         <v>393</v>
       </c>
-      <c r="B23" s="18" t="s">
+      <c r="C23" s="18" t="s">
+        <v>380</v>
+      </c>
+      <c r="D23" s="18" t="s">
         <v>394</v>
       </c>
-      <c r="C23" s="18" t="s">
-        <v>381</v>
-      </c>
-      <c r="D23" s="18" t="s">
+      <c r="E23" s="18" t="s">
+        <v>382</v>
+      </c>
+      <c r="F23" s="18" t="s">
         <v>395</v>
-      </c>
-      <c r="E23" s="18" t="s">
-        <v>383</v>
-      </c>
-      <c r="F23" s="18" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
+        <v>396</v>
+      </c>
+      <c r="B24" s="18" t="s">
         <v>397</v>
       </c>
-      <c r="B24" s="18" t="s">
+      <c r="C24" s="18" t="s">
+        <v>380</v>
+      </c>
+      <c r="D24" s="18" t="s">
         <v>398</v>
       </c>
-      <c r="C24" s="18" t="s">
-        <v>381</v>
-      </c>
-      <c r="D24" s="18" t="s">
+      <c r="E24" s="18" t="s">
+        <v>382</v>
+      </c>
+      <c r="F24" s="18" t="s">
         <v>399</v>
-      </c>
-      <c r="E24" s="18" t="s">
-        <v>383</v>
-      </c>
-      <c r="F24" s="18" t="s">
-        <v>400</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="18" t="s">
+        <v>400</v>
+      </c>
+      <c r="B25" s="18" t="s">
         <v>401</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="C25" s="18" t="s">
+        <v>329</v>
+      </c>
+      <c r="D25" s="18" t="s">
         <v>402</v>
       </c>
-      <c r="C25" s="18" t="s">
-        <v>330</v>
-      </c>
-      <c r="D25" s="18" t="s">
+      <c r="E25" s="18" t="s">
+        <v>317</v>
+      </c>
+      <c r="F25" s="18" t="s">
         <v>403</v>
-      </c>
-      <c r="E25" s="18" t="s">
-        <v>318</v>
-      </c>
-      <c r="F25" s="18" t="s">
-        <v>404</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="18" t="s">
+        <v>404</v>
+      </c>
+      <c r="B26" s="18" t="s">
         <v>405</v>
       </c>
-      <c r="B26" s="18" t="s">
+      <c r="C26" s="18" t="s">
+        <v>329</v>
+      </c>
+      <c r="D26" s="18" t="s">
         <v>406</v>
       </c>
-      <c r="C26" s="18" t="s">
-        <v>330</v>
-      </c>
-      <c r="D26" s="18" t="s">
+      <c r="E26" s="18" t="s">
         <v>407</v>
       </c>
-      <c r="E26" s="18" t="s">
+      <c r="F26" s="18" t="s">
         <v>408</v>
-      </c>
-      <c r="F26" s="18" t="s">
-        <v>409</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
+        <v>409</v>
+      </c>
+      <c r="B27" s="18" t="s">
         <v>410</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="C27" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="D27" s="18" t="s">
         <v>411</v>
       </c>
-      <c r="C27" s="18" t="s">
-        <v>346</v>
-      </c>
-      <c r="D27" s="18" t="s">
+      <c r="E27" s="18" t="s">
         <v>412</v>
       </c>
-      <c r="E27" s="18" t="s">
+      <c r="F27" s="18" t="s">
         <v>413</v>
-      </c>
-      <c r="F27" s="18" t="s">
-        <v>414</v>
       </c>
     </row>
   </sheetData>

</xml_diff>